<commit_message>
Debugging: Logged more bugs. Check Issue log for latest updates.
</commit_message>
<xml_diff>
--- a/Spreadsheets/Issue_Log.xlsx
+++ b/Spreadsheets/Issue_Log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\Spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF17F6BC-DCA8-42A1-9B23-4193C7D07C29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5D680A3-191D-4805-8884-4A9384179A99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="29010" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Game_Issues" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="658" uniqueCount="559">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="661" uniqueCount="561">
   <si>
     <t>UID</t>
   </si>
@@ -778,9 +778,6 @@
 FOLLOW-UP: reworked the ordering rather than adding another message. animate_retreat() now takes an is_forced_switch flag (default false). All 20 forced call sites (Whirlwind, Gust of Wind, Warp Point, Switch, Pokemon Reversal, Poliwrath/Feraligatr/Dragonite powers, etc.) pass true; only the two genuine voluntary retreats (CPU_AI.gd:1336 and the player's retreat button) leave it false. Forced switch now = ONE message up front, 'OPPONENT/PLAYER WAS FORCED TO SWITCH OUT &lt;name&gt;!', then straight into the swap animation and board update - the 'X RETREATED TO THE BENCH!' and '...SET X AS THEIR ACTIVE POKEMON!' pair are both suppressed. Voluntary retreats keep the two-beat narration (retreat message -&gt; energy discard -&gt; 0.5s -&gt; swap animation -&gt; set-active message). Callers keep their own flavour lines (e.g. 'HEADS! X SWITCHED IN!'). Watch console for 'ISSUE #6/#7 FIX ACTIVE'.</t>
   </si>
   <si>
-    <t xml:space="preserve">This fix has actually worked, however similar to the last message the order should be 1) "X was forced to switch out X" message displayed, 2) divert to not use the "X retreated to the bench" / "X switched in X as their active" message 3) Instead immediately play the animation of them swapping over and immediately update the board view. Then continue. </t>
-  </si>
-  <si>
     <t>When retreating, the opponent will still retreat a pokemon that is guarenteed to be knocked out with another pokemon that is guarenteed to be knocked out, wasting an energy to retreat. Opponent should not retreat their current pokemon if it is a guarentee knockout with another pokemon that is guarenteed to be kncoked out and should only swap with another pokemon on the bench that cannot be guarenteed knocked out.</t>
   </si>
   <si>
@@ -1719,6 +1716,15 @@
   </si>
   <si>
     <t xml:space="preserve">Play the adding water animation and board refresh after each time opponent uses rain dance. Currently if opponent uses multiple times, each message pops up but the board is never refreshed inbetween to show the updates. Make sure the opponent rechecks the board status to prioritse any additional water attachments, it's possible it currently only does priority checking first then attaches multiple energy to one pokemon where it should recheck priorities after </t>
+  </si>
+  <si>
+    <t>Change the +75 PER card to instead be a flat +300 if any at all mataches and make sure it reads all the text of all the attacks and powers of the active pokemon too and not just bench. Magnemite should have been played on bench but wasn't . Had 2 magnemtites on bench but only had 270 score which was under the 350 required</t>
+  </si>
+  <si>
+    <t>Animation doesn't work as required, currently just plays double message "Y was forced to switch with X", "X was forced to switch in Y" then a single swap at the same time. Instead display a single "Opponents [ACTIVE] switched with [BENCHED]" message. then in order 1) hide active card and then active card animates to bench 2) bench pokemon removed from bench and active pokemon added. 3) refresh board to show the change 4) animate the bench going to active 5) new active visible. Continue. Also when the opponent uses it on the player, make sure to play the animation of the cards swapping the same.</t>
+  </si>
+  <si>
+    <t>When using oddish sprout and the oddishes are shown, there is an input blocker blocking the player from clicking the confirm button. It covers the whole screen</t>
   </si>
 </sst>
 </file>
@@ -2290,18 +2296,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G17"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.26953125" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="143.453125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="114.81640625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="85.7265625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="3.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="143.42578125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="114.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="85.7109375" style="1" customWidth="1"/>
     <col min="5" max="5" width="19" style="1" customWidth="1"/>
-    <col min="6" max="6" width="10.08984375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>224</v>
       </c>
@@ -2324,7 +2330,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -2341,7 +2347,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" ht="90" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -2351,14 +2357,17 @@
       <c r="C3" s="1" t="s">
         <v>232</v>
       </c>
+      <c r="D3" s="1" t="s">
+        <v>558</v>
+      </c>
       <c r="E3" s="1" t="s">
-        <v>13</v>
+        <v>555</v>
       </c>
       <c r="F3" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="217.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" ht="255" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -2375,7 +2384,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -2392,7 +2401,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" ht="180" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -2406,13 +2415,13 @@
         <v>239</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="F6" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="203" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" ht="225" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -2426,13 +2435,13 @@
         <v>242</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="F7" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" ht="180" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -2443,24 +2452,24 @@
         <v>244</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>245</v>
+        <v>559</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>13</v>
+        <v>555</v>
       </c>
       <c r="F8" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" ht="90" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>246</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>247</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>37</v>
@@ -2469,35 +2478,35 @@
         <v>230</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="232" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" ht="240" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="D10" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="D10" s="1" t="s">
-        <v>250</v>
-      </c>
       <c r="E10" s="1" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="F10" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" ht="75" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>251</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>252</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>37</v>
@@ -2506,15 +2515,15 @@
         <v>230</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" ht="75" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>253</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>254</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>13</v>
@@ -2523,15 +2532,15 @@
         <v>230</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="87" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" ht="90" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>255</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>256</v>
       </c>
       <c r="E13" t="s">
         <v>37</v>
@@ -2540,32 +2549,32 @@
         <v>230</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" ht="120" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="C14" t="s">
-        <v>258</v>
-      </c>
       <c r="E14" s="1" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="F14" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>259</v>
-      </c>
-      <c r="C15" t="s">
-        <v>260</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>13</v>
@@ -2574,23 +2583,29 @@
         <v>230</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="F16" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>16</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>560</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>554</v>
       </c>
     </row>
   </sheetData>
@@ -2617,18 +2632,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G103"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.54296875" customWidth="1"/>
+    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.5703125" customWidth="1"/>
     <col min="3" max="3" width="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="140.81640625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="125.1796875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="140.85546875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="125.140625" style="1" customWidth="1"/>
     <col min="6" max="6" width="68" style="1" customWidth="1"/>
     <col min="7" max="7" width="19" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -2651,7 +2666,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="188.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" ht="225" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -2674,7 +2689,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -2691,13 +2706,13 @@
         <v>17</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="101.5" x14ac:dyDescent="0.35">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -2717,7 +2732,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>22</v>
       </c>
@@ -2728,7 +2743,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>25</v>
       </c>
@@ -2739,7 +2754,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>27</v>
       </c>
@@ -2750,7 +2765,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>29</v>
       </c>
@@ -2758,7 +2773,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>31</v>
       </c>
@@ -2766,7 +2781,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="72.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>33</v>
       </c>
@@ -2786,7 +2801,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>38</v>
       </c>
@@ -2794,7 +2809,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>40</v>
       </c>
@@ -2802,7 +2817,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>42</v>
       </c>
@@ -2810,7 +2825,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>44</v>
       </c>
@@ -2818,7 +2833,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>46</v>
       </c>
@@ -2826,7 +2841,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>48</v>
       </c>
@@ -2834,7 +2849,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>50</v>
       </c>
@@ -2842,7 +2857,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>52</v>
       </c>
@@ -2850,7 +2865,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>54</v>
       </c>
@@ -2858,7 +2873,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>56</v>
       </c>
@@ -2866,7 +2881,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>58</v>
       </c>
@@ -2874,7 +2889,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>60</v>
       </c>
@@ -2885,7 +2900,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>62</v>
       </c>
@@ -2893,7 +2908,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>64</v>
       </c>
@@ -2901,7 +2916,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>66</v>
       </c>
@@ -2909,7 +2924,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>68</v>
       </c>
@@ -2917,7 +2932,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>70</v>
       </c>
@@ -2925,7 +2940,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>72</v>
       </c>
@@ -2933,7 +2948,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>74</v>
       </c>
@@ -2941,7 +2956,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>76</v>
       </c>
@@ -2949,7 +2964,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>78</v>
       </c>
@@ -2957,7 +2972,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>80</v>
       </c>
@@ -2965,7 +2980,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:3" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>82</v>
       </c>
@@ -2973,7 +2988,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>84</v>
       </c>
@@ -2981,7 +2996,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>86</v>
       </c>
@@ -2989,7 +3004,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>88</v>
       </c>
@@ -2997,7 +3012,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>90</v>
       </c>
@@ -3008,7 +3023,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>92</v>
       </c>
@@ -3016,7 +3031,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>94</v>
       </c>
@@ -3024,7 +3039,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>96</v>
       </c>
@@ -3032,7 +3047,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>98</v>
       </c>
@@ -3040,7 +3055,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>100</v>
       </c>
@@ -3048,7 +3063,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>102</v>
       </c>
@@ -3056,7 +3071,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>104</v>
       </c>
@@ -3064,7 +3079,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>106</v>
       </c>
@@ -3072,7 +3087,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>108</v>
       </c>
@@ -3080,7 +3095,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>110</v>
       </c>
@@ -3088,7 +3103,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>112</v>
       </c>
@@ -3096,7 +3111,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>114</v>
       </c>
@@ -3104,7 +3119,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>116</v>
       </c>
@@ -3112,7 +3127,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>118</v>
       </c>
@@ -3120,7 +3135,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>120</v>
       </c>
@@ -3128,7 +3143,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>122</v>
       </c>
@@ -3136,7 +3151,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>124</v>
       </c>
@@ -3144,7 +3159,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>126</v>
       </c>
@@ -3152,7 +3167,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>128</v>
       </c>
@@ -3163,7 +3178,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>130</v>
       </c>
@@ -3171,7 +3186,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>132</v>
       </c>
@@ -3179,7 +3194,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>134</v>
       </c>
@@ -3187,7 +3202,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>136</v>
       </c>
@@ -3195,7 +3210,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>138</v>
       </c>
@@ -3203,7 +3218,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>140</v>
       </c>
@@ -3211,7 +3226,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>142</v>
       </c>
@@ -3219,7 +3234,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>144</v>
       </c>
@@ -3227,7 +3242,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>146</v>
       </c>
@@ -3235,7 +3250,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>148</v>
       </c>
@@ -3243,7 +3258,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>150</v>
       </c>
@@ -3251,7 +3266,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>152</v>
       </c>
@@ -3259,7 +3274,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>154</v>
       </c>
@@ -3267,7 +3282,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>156</v>
       </c>
@@ -3278,7 +3293,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>158</v>
       </c>
@@ -3286,7 +3301,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>160</v>
       </c>
@@ -3294,7 +3309,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>162</v>
       </c>
@@ -3302,7 +3317,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>164</v>
       </c>
@@ -3310,7 +3325,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>166</v>
       </c>
@@ -3318,7 +3333,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>168</v>
       </c>
@@ -3326,7 +3341,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>170</v>
       </c>
@@ -3334,7 +3349,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>172</v>
       </c>
@@ -3342,7 +3357,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>174</v>
       </c>
@@ -3350,7 +3365,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>176</v>
       </c>
@@ -3358,7 +3373,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>178</v>
       </c>
@@ -3366,7 +3381,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>180</v>
       </c>
@@ -3374,7 +3389,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>182</v>
       </c>
@@ -3382,7 +3397,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>184</v>
       </c>
@@ -3390,7 +3405,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>186</v>
       </c>
@@ -3398,7 +3413,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>188</v>
       </c>
@@ -3406,7 +3421,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>190</v>
       </c>
@@ -3414,7 +3429,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>192</v>
       </c>
@@ -3422,7 +3437,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>194</v>
       </c>
@@ -3430,7 +3445,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>196</v>
       </c>
@@ -3438,7 +3453,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>198</v>
       </c>
@@ -3446,7 +3461,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>200</v>
       </c>
@@ -3454,7 +3469,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>202</v>
       </c>
@@ -3462,7 +3477,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>204</v>
       </c>
@@ -3470,7 +3485,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>206</v>
       </c>
@@ -3478,7 +3493,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>208</v>
       </c>
@@ -3486,7 +3501,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>210</v>
       </c>
@@ -3494,7 +3509,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>212</v>
       </c>
@@ -3502,7 +3517,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>214</v>
       </c>
@@ -3510,7 +3525,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>216</v>
       </c>
@@ -3518,7 +3533,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>218</v>
       </c>
@@ -3526,7 +3541,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>220</v>
       </c>
@@ -3534,7 +3549,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>222</v>
       </c>
@@ -3559,7 +3574,7 @@
       <formula>OR($C2="N",$G2="New Issue",$G2="Fix Failed")</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations disablePrompts="1" count="1">
+  <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G1048576" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>StatusList</formula1>
     </dataValidation>
@@ -3571,17 +3586,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:G49"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="29.54296875" customWidth="1"/>
-    <col min="3" max="3" width="5.453125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="82.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="89.26953125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="29.54296875" customWidth="1"/>
+    <col min="1" max="2" width="29.5703125" customWidth="1"/>
+    <col min="3" max="3" width="5.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="82.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="89.28515625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="29.5703125" customWidth="1"/>
     <col min="7" max="7" width="19" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -3604,400 +3619,400 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>260</v>
+      </c>
+      <c r="B2" t="s">
         <v>261</v>
       </c>
-      <c r="B2" t="s">
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>262</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>263</v>
       </c>
       <c r="B3" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>263</v>
+      </c>
+      <c r="B4" t="s">
         <v>264</v>
       </c>
-      <c r="B4" t="s">
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>265</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+      <c r="B5" t="s">
         <v>266</v>
       </c>
-      <c r="B5" t="s">
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>267</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+      <c r="B6" t="s">
         <v>268</v>
       </c>
-      <c r="B6" t="s">
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>269</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
+      <c r="B7" t="s">
         <v>270</v>
       </c>
-      <c r="B7" t="s">
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>271</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
+      <c r="B8" t="s">
         <v>272</v>
       </c>
-      <c r="B8" t="s">
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>273</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
+      <c r="B9" t="s">
         <v>274</v>
       </c>
-      <c r="B9" t="s">
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>275</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
+      <c r="B10" t="s">
         <v>276</v>
       </c>
-      <c r="B10" t="s">
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>277</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
+      <c r="B11" t="s">
         <v>278</v>
       </c>
-      <c r="B11" t="s">
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>279</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
+      <c r="B12" t="s">
         <v>280</v>
       </c>
-      <c r="B12" t="s">
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>281</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
+      <c r="B13" t="s">
         <v>282</v>
       </c>
-      <c r="B13" t="s">
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>283</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
+      <c r="B14" t="s">
         <v>284</v>
       </c>
-      <c r="B14" t="s">
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>285</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
+      <c r="B15" t="s">
         <v>286</v>
       </c>
-      <c r="B15" t="s">
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
+      <c r="B16" t="s">
         <v>288</v>
       </c>
-      <c r="B16" t="s">
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>289</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
+      <c r="B17" t="s">
         <v>290</v>
       </c>
-      <c r="B17" t="s">
+    </row>
+    <row r="18" spans="1:7" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>291</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" ht="72.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
+      <c r="B18" t="s">
         <v>292</v>
-      </c>
-      <c r="B18" t="s">
-        <v>293</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D18" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="E18" s="1" t="s">
         <v>294</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>295</v>
       </c>
       <c r="G18" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>295</v>
+      </c>
+      <c r="B19" t="s">
         <v>296</v>
       </c>
-      <c r="B19" t="s">
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>297</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
+      <c r="B20" t="s">
         <v>298</v>
       </c>
-      <c r="B20" t="s">
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>299</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
+      <c r="B21" t="s">
         <v>300</v>
       </c>
-      <c r="B21" t="s">
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>301</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
+      <c r="B22" t="s">
         <v>302</v>
       </c>
-      <c r="B22" t="s">
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>303</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
+      <c r="B23" t="s">
         <v>304</v>
       </c>
-      <c r="B23" t="s">
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>305</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
+      <c r="B24" t="s">
         <v>306</v>
       </c>
-      <c r="B24" t="s">
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>307</v>
       </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
+      <c r="B25" t="s">
         <v>308</v>
       </c>
-      <c r="B25" t="s">
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>309</v>
       </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
+      <c r="B26" t="s">
         <v>310</v>
       </c>
-      <c r="B26" t="s">
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
         <v>311</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
+      <c r="B27" t="s">
         <v>312</v>
       </c>
-      <c r="B27" t="s">
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>313</v>
       </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
+      <c r="B28" t="s">
         <v>314</v>
       </c>
-      <c r="B28" t="s">
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>315</v>
       </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
+      <c r="B29" t="s">
         <v>316</v>
       </c>
-      <c r="B29" t="s">
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
         <v>317</v>
       </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
+      <c r="B30" t="s">
         <v>318</v>
       </c>
-      <c r="B30" t="s">
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>319</v>
       </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
+      <c r="B31" t="s">
         <v>320</v>
       </c>
-      <c r="B31" t="s">
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
         <v>321</v>
       </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
+      <c r="B32" t="s">
         <v>322</v>
       </c>
-      <c r="B32" t="s">
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
+      <c r="B33" t="s">
         <v>324</v>
       </c>
-      <c r="B33" t="s">
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>325</v>
       </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
+      <c r="B34" t="s">
         <v>326</v>
       </c>
-      <c r="B34" t="s">
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
+      <c r="B35" t="s">
         <v>328</v>
       </c>
-      <c r="B35" t="s">
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
         <v>329</v>
       </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A36" t="s">
+      <c r="B36" t="s">
         <v>330</v>
       </c>
-      <c r="B36" t="s">
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
         <v>331</v>
       </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A37" t="s">
+      <c r="B37" t="s">
         <v>332</v>
       </c>
-      <c r="B37" t="s">
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
         <v>333</v>
       </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A38" t="s">
+      <c r="B38" t="s">
         <v>334</v>
       </c>
-      <c r="B38" t="s">
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>335</v>
       </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A39" t="s">
+      <c r="B39" t="s">
         <v>336</v>
       </c>
-      <c r="B39" t="s">
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A40" t="s">
+      <c r="B40" t="s">
         <v>338</v>
       </c>
-      <c r="B40" t="s">
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
         <v>339</v>
       </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A41" t="s">
+      <c r="B41" t="s">
         <v>340</v>
       </c>
-      <c r="B41" t="s">
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
         <v>341</v>
       </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A42" t="s">
+      <c r="B42" t="s">
         <v>342</v>
       </c>
-      <c r="B42" t="s">
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
         <v>343</v>
       </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A43" t="s">
+      <c r="B43" t="s">
         <v>344</v>
       </c>
-      <c r="B43" t="s">
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
         <v>345</v>
       </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
+      <c r="B44" t="s">
         <v>346</v>
       </c>
-      <c r="B44" t="s">
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
         <v>347</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
-        <v>348</v>
       </c>
       <c r="B45" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
+        <v>348</v>
+      </c>
+      <c r="B46" t="s">
         <v>349</v>
       </c>
-      <c r="B46" t="s">
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A47" t="s">
+      <c r="B47" t="s">
         <v>351</v>
       </c>
-      <c r="B47" t="s">
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
         <v>352</v>
       </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A48" t="s">
+      <c r="B48" t="s">
         <v>353</v>
       </c>
-      <c r="B48" t="s">
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
         <v>354</v>
       </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A49" t="s">
+      <c r="B49" t="s">
         <v>355</v>
-      </c>
-      <c r="B49" t="s">
-        <v>356</v>
       </c>
     </row>
   </sheetData>
@@ -4024,9 +4039,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:G48"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4049,380 +4064,380 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>356</v>
+      </c>
+      <c r="B2" t="s">
         <v>357</v>
       </c>
-      <c r="B2" t="s">
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>358</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="B3" t="s">
         <v>359</v>
       </c>
-      <c r="B3" t="s">
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>360</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+      <c r="B4" t="s">
         <v>361</v>
       </c>
-      <c r="B4" t="s">
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>362</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+      <c r="B5" t="s">
         <v>363</v>
       </c>
-      <c r="B5" t="s">
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>364</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+      <c r="B6" t="s">
         <v>365</v>
       </c>
-      <c r="B6" t="s">
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>366</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>367</v>
       </c>
       <c r="B7" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>367</v>
+      </c>
+      <c r="B8" t="s">
         <v>368</v>
       </c>
-      <c r="B8" t="s">
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>369</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
+      <c r="B9" t="s">
         <v>370</v>
       </c>
-      <c r="B9" t="s">
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>371</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
+      <c r="B10" t="s">
         <v>372</v>
       </c>
-      <c r="B10" t="s">
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>373</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
+      <c r="B11" t="s">
         <v>374</v>
       </c>
-      <c r="B11" t="s">
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>375</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>376</v>
       </c>
       <c r="B12" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>376</v>
+      </c>
+      <c r="B13" t="s">
         <v>377</v>
       </c>
-      <c r="B13" t="s">
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>378</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
+      <c r="B14" t="s">
         <v>379</v>
       </c>
-      <c r="B14" t="s">
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>380</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>381</v>
       </c>
       <c r="B15" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B16" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>382</v>
+      </c>
+      <c r="B17" t="s">
         <v>383</v>
       </c>
-      <c r="B17" t="s">
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>384</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
+      <c r="B18" t="s">
         <v>385</v>
       </c>
-      <c r="B18" t="s">
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
         <v>386</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
-        <v>387</v>
       </c>
       <c r="B19" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>387</v>
+      </c>
+      <c r="B20" t="s">
         <v>388</v>
       </c>
-      <c r="B20" t="s">
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>389</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
+      <c r="B21" t="s">
         <v>390</v>
       </c>
-      <c r="B21" t="s">
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>391</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
+      <c r="B22" t="s">
         <v>392</v>
       </c>
-      <c r="B22" t="s">
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>393</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
+      <c r="B23" t="s">
         <v>394</v>
       </c>
-      <c r="B23" t="s">
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>395</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
+      <c r="B24" t="s">
         <v>396</v>
       </c>
-      <c r="B24" t="s">
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>397</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
-        <v>398</v>
       </c>
       <c r="B25" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>398</v>
+      </c>
+      <c r="B26" t="s">
         <v>399</v>
       </c>
-      <c r="B26" t="s">
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
         <v>400</v>
       </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
+      <c r="B27" t="s">
         <v>401</v>
       </c>
-      <c r="B27" t="s">
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>402</v>
       </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
+      <c r="B28" t="s">
         <v>403</v>
       </c>
-      <c r="B28" t="s">
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>404</v>
       </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
+      <c r="B29" t="s">
         <v>405</v>
       </c>
-      <c r="B29" t="s">
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
         <v>406</v>
       </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
+      <c r="B30" t="s">
         <v>407</v>
       </c>
-      <c r="B30" t="s">
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>408</v>
       </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
+      <c r="B31" t="s">
         <v>409</v>
       </c>
-      <c r="B31" t="s">
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
         <v>410</v>
       </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
+      <c r="B32" t="s">
         <v>411</v>
       </c>
-      <c r="B32" t="s">
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
         <v>412</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
+      <c r="B33" t="s">
         <v>413</v>
       </c>
-      <c r="B33" t="s">
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>414</v>
       </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
+      <c r="B34" t="s">
         <v>415</v>
       </c>
-      <c r="B34" t="s">
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>416</v>
       </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
+      <c r="B35" t="s">
         <v>417</v>
       </c>
-      <c r="B35" t="s">
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
         <v>418</v>
       </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A36" t="s">
+      <c r="B36" t="s">
         <v>419</v>
       </c>
-      <c r="B36" t="s">
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
         <v>420</v>
       </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A37" t="s">
+      <c r="B37" t="s">
         <v>421</v>
       </c>
-      <c r="B37" t="s">
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
         <v>422</v>
       </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A38" t="s">
+      <c r="B38" t="s">
         <v>423</v>
       </c>
-      <c r="B38" t="s">
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>424</v>
       </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A39" t="s">
+      <c r="B39" t="s">
         <v>425</v>
       </c>
-      <c r="B39" t="s">
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
         <v>426</v>
       </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A40" t="s">
+      <c r="B40" t="s">
         <v>427</v>
       </c>
-      <c r="B40" t="s">
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
         <v>428</v>
       </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A41" t="s">
+      <c r="B41" t="s">
         <v>429</v>
       </c>
-      <c r="B41" t="s">
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
         <v>430</v>
       </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A42" t="s">
+      <c r="B42" t="s">
         <v>431</v>
       </c>
-      <c r="B42" t="s">
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
         <v>432</v>
       </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A43" t="s">
+      <c r="B43" t="s">
         <v>433</v>
       </c>
-      <c r="B43" t="s">
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
         <v>434</v>
       </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
+      <c r="B44" t="s">
         <v>435</v>
       </c>
-      <c r="B44" t="s">
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
         <v>436</v>
       </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
+      <c r="B45" t="s">
         <v>437</v>
       </c>
-      <c r="B45" t="s">
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
         <v>438</v>
       </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A46" t="s">
+      <c r="B46" t="s">
         <v>439</v>
       </c>
-      <c r="B46" t="s">
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
         <v>440</v>
       </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A47" t="s">
+      <c r="B47" t="s">
         <v>441</v>
       </c>
-      <c r="B47" t="s">
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
         <v>442</v>
       </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A48" t="s">
+      <c r="B48" t="s">
         <v>443</v>
-      </c>
-      <c r="B48" t="s">
-        <v>444</v>
       </c>
     </row>
   </sheetData>
@@ -4449,9 +4464,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:G67"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4474,532 +4489,532 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>444</v>
+      </c>
+      <c r="B2" t="s">
         <v>445</v>
       </c>
-      <c r="B2" t="s">
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>446</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="B3" t="s">
         <v>447</v>
       </c>
-      <c r="B3" t="s">
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>448</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+      <c r="B4" t="s">
         <v>449</v>
       </c>
-      <c r="B4" t="s">
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>450</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+      <c r="B5" t="s">
         <v>451</v>
       </c>
-      <c r="B5" t="s">
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>452</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+      <c r="B6" t="s">
         <v>453</v>
       </c>
-      <c r="B6" t="s">
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>454</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
+      <c r="B7" t="s">
         <v>455</v>
       </c>
-      <c r="B7" t="s">
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
+      <c r="B8" t="s">
         <v>457</v>
       </c>
-      <c r="B8" t="s">
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>458</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
+      <c r="B9" t="s">
         <v>459</v>
       </c>
-      <c r="B9" t="s">
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>460</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
+      <c r="B10" t="s">
         <v>461</v>
       </c>
-      <c r="B10" t="s">
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>462</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
+      <c r="B11" t="s">
         <v>463</v>
       </c>
-      <c r="B11" t="s">
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>464</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
+      <c r="B12" t="s">
         <v>465</v>
       </c>
-      <c r="B12" t="s">
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>466</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
+      <c r="B13" t="s">
         <v>467</v>
       </c>
-      <c r="B13" t="s">
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>468</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
+      <c r="B14" t="s">
         <v>469</v>
       </c>
-      <c r="B14" t="s">
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>470</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
+      <c r="B15" t="s">
         <v>471</v>
       </c>
-      <c r="B15" t="s">
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>472</v>
       </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
+      <c r="B16" t="s">
         <v>473</v>
       </c>
-      <c r="B16" t="s">
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>474</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
+      <c r="B17" t="s">
         <v>475</v>
       </c>
-      <c r="B17" t="s">
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>476</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
+      <c r="B18" t="s">
         <v>477</v>
       </c>
-      <c r="B18" t="s">
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
         <v>478</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
+      <c r="B19" t="s">
         <v>479</v>
       </c>
-      <c r="B19" t="s">
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>480</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
+      <c r="B20" t="s">
         <v>481</v>
       </c>
-      <c r="B20" t="s">
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>482</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
+      <c r="B21" t="s">
         <v>483</v>
       </c>
-      <c r="B21" t="s">
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>484</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
+      <c r="B22" t="s">
         <v>485</v>
       </c>
-      <c r="B22" t="s">
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>486</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
+      <c r="B23" t="s">
         <v>487</v>
       </c>
-      <c r="B23" t="s">
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>488</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
+      <c r="B24" t="s">
         <v>489</v>
       </c>
-      <c r="B24" t="s">
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>490</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
+      <c r="B25" t="s">
         <v>491</v>
       </c>
-      <c r="B25" t="s">
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>492</v>
       </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
+      <c r="B26" t="s">
         <v>493</v>
       </c>
-      <c r="B26" t="s">
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
         <v>494</v>
       </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
+      <c r="B27" t="s">
         <v>495</v>
       </c>
-      <c r="B27" t="s">
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>496</v>
       </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
+      <c r="B28" t="s">
         <v>497</v>
       </c>
-      <c r="B28" t="s">
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>498</v>
       </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
+      <c r="B29" t="s">
         <v>499</v>
       </c>
-      <c r="B29" t="s">
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
         <v>500</v>
       </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
+      <c r="B30" t="s">
         <v>501</v>
       </c>
-      <c r="B30" t="s">
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>502</v>
       </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
+      <c r="B31" t="s">
         <v>503</v>
       </c>
-      <c r="B31" t="s">
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
         <v>504</v>
       </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
+      <c r="B32" t="s">
         <v>505</v>
       </c>
-      <c r="B32" t="s">
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
         <v>506</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
+      <c r="B33" t="s">
         <v>507</v>
       </c>
-      <c r="B33" t="s">
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>508</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
-        <v>509</v>
       </c>
       <c r="B34" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="B35" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="B36" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="B37" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
+        <v>512</v>
+      </c>
+      <c r="B38" t="s">
         <v>513</v>
       </c>
-      <c r="B38" t="s">
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>514</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A39" t="s">
-        <v>515</v>
       </c>
       <c r="B39" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="B40" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="B41" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
+        <v>517</v>
+      </c>
+      <c r="B42" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
         <v>518</v>
       </c>
-      <c r="B42" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A43" t="s">
+      <c r="B43" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
         <v>519</v>
       </c>
-      <c r="B43" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
+      <c r="B44" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
         <v>520</v>
-      </c>
-      <c r="B44" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
-        <v>521</v>
       </c>
       <c r="B45" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="B46" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="B47" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
+        <v>523</v>
+      </c>
+      <c r="B48" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
         <v>524</v>
       </c>
-      <c r="B48" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A49" t="s">
+      <c r="B49" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
         <v>525</v>
       </c>
-      <c r="B49" t="s">
-        <v>341</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A50" t="s">
+      <c r="B50" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
         <v>526</v>
-      </c>
-      <c r="B50" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A51" t="s">
-        <v>527</v>
       </c>
       <c r="B51" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
+        <v>527</v>
+      </c>
+      <c r="B52" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
         <v>528</v>
-      </c>
-      <c r="B52" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A53" t="s">
-        <v>529</v>
       </c>
       <c r="B53" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
+        <v>529</v>
+      </c>
+      <c r="B54" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
         <v>530</v>
-      </c>
-      <c r="B54" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A55" t="s">
-        <v>531</v>
       </c>
       <c r="B55" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="B56" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
+        <v>532</v>
+      </c>
+      <c r="B57" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
         <v>533</v>
       </c>
-      <c r="B57" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A58" t="s">
+      <c r="B58" t="s">
         <v>534</v>
       </c>
-      <c r="B58" t="s">
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
         <v>535</v>
       </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A59" t="s">
+      <c r="B59" t="s">
         <v>536</v>
       </c>
-      <c r="B59" t="s">
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
         <v>537</v>
       </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A60" t="s">
+      <c r="B60" t="s">
         <v>538</v>
       </c>
-      <c r="B60" t="s">
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
         <v>539</v>
       </c>
-    </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A61" t="s">
+      <c r="B61" t="s">
         <v>540</v>
       </c>
-      <c r="B61" t="s">
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
         <v>541</v>
       </c>
-    </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A62" t="s">
+      <c r="B62" t="s">
         <v>542</v>
       </c>
-      <c r="B62" t="s">
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
         <v>543</v>
       </c>
-    </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A63" t="s">
+      <c r="B63" t="s">
         <v>544</v>
       </c>
-      <c r="B63" t="s">
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
         <v>545</v>
       </c>
-    </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A64" t="s">
+      <c r="B64" t="s">
         <v>546</v>
       </c>
-      <c r="B64" t="s">
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
         <v>547</v>
       </c>
-    </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A65" t="s">
+      <c r="B65" t="s">
         <v>548</v>
       </c>
-      <c r="B65" t="s">
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
         <v>549</v>
       </c>
-    </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A66" t="s">
+      <c r="B66" t="s">
         <v>550</v>
       </c>
-      <c r="B66" t="s">
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
         <v>551</v>
       </c>
-    </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A67" t="s">
+      <c r="B67" t="s">
         <v>552</v>
-      </c>
-      <c r="B67" t="s">
-        <v>553</v>
       </c>
     </row>
   </sheetData>
@@ -5026,34 +5041,34 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:A5"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>555</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Debug: Continued debugging game intro and main match code. Issue log updated
</commit_message>
<xml_diff>
--- a/Spreadsheets/Issue_Log.xlsx
+++ b/Spreadsheets/Issue_Log.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Game_Issues" sheetId="1" state="visible" r:id="rId1"/>
@@ -57,7 +57,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -65,11 +65,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -82,46 +97,20 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="18">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="15">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -681,51 +670,51 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <dimension ref="A1:I60"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="3.26953125" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
-    <col width="10.7265625" customWidth="1" style="2" min="2" max="3"/>
-    <col width="143.453125" customWidth="1" style="1" min="4" max="4"/>
-    <col hidden="1" width="43.90625" customWidth="1" style="6" min="5" max="5"/>
-    <col width="85.7265625" customWidth="1" style="1" min="6" max="6"/>
+    <col width="3.42578125" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
+    <col width="10.7109375" customWidth="1" style="2" min="2" max="3"/>
+    <col width="143.42578125" customWidth="1" style="1" min="4" max="4"/>
+    <col hidden="1" width="43.85546875" customWidth="1" min="5" max="5"/>
+    <col width="85.7109375" customWidth="1" style="1" min="6" max="6"/>
     <col width="19" customWidth="1" style="1" min="7" max="7"/>
-    <col width="10.1796875" bestFit="1" customWidth="1" style="6" min="8" max="8"/>
-    <col width="10.08984375" bestFit="1" customWidth="1" style="6" min="9" max="9"/>
+    <col width="11.140625" bestFit="1" customWidth="1" min="8" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="C1" s="7" t="n"/>
+      <c r="D1" s="8" t="inlineStr">
         <is>
           <t>Issue</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="9" t="inlineStr">
         <is>
           <t>Fix Notes</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="8" t="inlineStr">
         <is>
           <t>Fix Failure Notes</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="8" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="9" t="inlineStr">
         <is>
           <t>Logged</t>
         </is>
@@ -737,30 +726,32 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>CPU logic</t>
         </is>
       </c>
-      <c r="D2" s="1" t="inlineStr">
+      <c r="C2" s="7" t="n"/>
+      <c r="D2" s="8" t="inlineStr">
         <is>
           <t>Add penalty of "this pokemon already exists on the bench" when deciding to play a bench pokemon for -75 points per amount of that pokemon</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="9" t="inlineStr">
         <is>
           <t>Added criterion_6_bench_duplicate to CPU_AI.gd: -75 score per existing same-name Pokemon already on opponent bench when scoring a hand Pokemon to play.</t>
         </is>
       </c>
-      <c r="G2" s="1" t="inlineStr">
+      <c r="F2" s="8" t="n"/>
+      <c r="G2" s="8" t="inlineStr">
         <is>
           <t>Issue Resolved</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="9" t="inlineStr">
         <is>
           <t>16/07/2026</t>
         </is>
@@ -771,76 +762,78 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="72.5" customHeight="1" s="6">
-      <c r="A3" s="2" t="n">
+    <row r="3" ht="72.59999999999999" customHeight="1">
+      <c r="A3" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>CPU logic</t>
         </is>
       </c>
-      <c r="D3" s="1" t="inlineStr">
+      <c r="C3" s="7" t="n"/>
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>However flip that and add a bonus if there is an effect on the field that would benefit the opponent from it. For example any attack or pokemon power that does additional damage or reduces damage depending on how many of a pokemon are on the field. E.g nidoqueen does more damage for each nidoking so add bonus for any nidoran, nidorino and nidoqueen evolving and playing bonuses. Magnemite does more damage for each magnemite on the field. Some delta species do more damage for each delta species on the field. Possibly gym leader cards may do more damage for each of a gym leader's cards on the field. E.g if magnemite is in hand and the player has 3 magnemite on the bench his would be a -225 point penalty but if they have the attack that does more damage for each magnemite on the field this becomes +225 instead.</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="9" t="inlineStr">
         <is>
           <t>Same change adds has_species_stacking_synergy() text scan (attack/ability text referencing "for each &lt;name&gt; ... in play/on your Bench" with damage/retreat scaling, or delta-species-count text) - flips the -75/copy penalty to +75/copy when a synergy effect is detected on hand/bench/active.
 FIX PASS 2026-07-18: changed criterion_6_bench_duplicate (CPU_AI.gd) to award a FLAT +300 (instead of +75 per copy) whenever has_species_stacking_synergy() detects a field effect that benefits from stacking this species — so a stack-payoff Basic (e.g. a 3rd Magnemite) comfortably clears the bench-play thresholds (350 for a 3-Pokemon bench). Also added the candidate Pokemon itself to has_species_stacking_synergy's scan list so its OWN attack/ability text (and the Active's) is read, not just the Bench. Debug: 'ISSUE #2 FIX ACTIVE'.</t>
         </is>
       </c>
-      <c r="F3" s="1" t="inlineStr">
+      <c r="F3" s="8" t="inlineStr">
         <is>
           <t>Change the +75 PER card to instead be a flat +300 if any at all mataches and make sure it reads all the text of all the attacks and powers of the active pokemon too and not just bench. Magnemite should have been played on bench but wasn't . Had 2 magnemtites on bench but only had 270 score which was under the 350 required</t>
         </is>
       </c>
-      <c r="G3" s="1" t="inlineStr">
+      <c r="G3" s="8" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="9" t="inlineStr">
         <is>
           <t>16/07/2026</t>
         </is>
       </c>
-      <c r="I3" s="7" t="n">
+      <c r="I3" s="6" t="n">
         <v>46220</v>
       </c>
     </row>
-    <row r="4" ht="43.5" customHeight="1" s="6">
-      <c r="A4" s="2" t="n">
+    <row r="4" ht="43.5" customHeight="1">
+      <c r="A4" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="D4" s="1" t="inlineStr">
+      <c r="C4" s="7" t="n"/>
+      <c r="D4" s="8" t="inlineStr">
         <is>
           <t>When returning to main UI from selecting cards for a card effect (E.g Blastoise Rain Dance), the player is no longer able to click anything. Presumably the main UI input blocker doesn't get rehidden. Same thing happens with card effects like Clefairie's Metronome. Once used the attacks of the opponent appears but player cannot click anything.</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="9" t="inlineStr">
         <is>
           <t>Root cause: Card_Ops.gd prompt_select_card() unconditionally set main.opponent_blocker.visible = true when the selection UI closed. That blocker is only supposed to be visible during the opponent's turn (toggled by player_start_turn_checks/player_end_turn_checks). Using a power like Rain Dance or Metronome's attack-copy pool on the player's own turn opened this selection screen, and closing it force-reactivated the blocker even though it was still the player's turn, so no clicks registered afterward. Fixed prompt_select_card to remember the blocker's visibility before opening the selection UI and restore that value afterward instead of forcing it true.
 FOLLOW-UP: user reported the Metronome case still failed after the first fix. Found a second, separate blocker involved. perform_attack() sets opponent_blocker.visible = true the instant the player's attack is chosen (attacking always ends the turn, so input is meant to be blocked for the rest of the turn) - opponent_blocker is a FULL-SCREEN ColorRect with no cutout region. Metronome's attack-copy button list (choose_attack_from_pool in Attack_Effects.gd) only ever toggled buttons_only_blocker, which DOES carve out an exception for the button row - but opponent_blocker, already active from perform_attack, has no such exception and sat on top blocking the whole screen including those buttons. Rain Dance/other powers used outside of perform_attack never had this problem because opponent_blocker isn't forced on for those. Fixed choose_attack_from_pool to save/hide/restore opponent_blocker the same way prompt_select_card now does, so the attack-copy button list is actually clickable. Added print("ISSUE #3 FIX ACTIVE...") debug lines in both prompt_select_card and choose_attack_from_pool (and to every other fix in this log going forward) so the user can confirm from the Godot console output whether the running build actually has the fix, per new debug-message-on-every-fix requirement.</t>
         </is>
       </c>
-      <c r="F4" s="1" t="inlineStr">
+      <c r="F4" s="8" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="G4" s="1" t="inlineStr">
+      <c r="G4" s="8" t="inlineStr">
         <is>
           <t>Issue Resolved</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" s="9" t="inlineStr">
         <is>
           <t>16/07/2026</t>
         </is>
@@ -851,36 +844,37 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="29" customHeight="1" s="6">
-      <c r="A5" s="2" t="n">
+    <row r="5" ht="29.1" customHeight="1">
+      <c r="A5" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="D5" s="1" t="inlineStr">
+      <c r="C5" s="7" t="n"/>
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>Pressing the space bar to preview a card in deck view mode seems to accept the last button pressed so if you press empty deck, then press space over a card to preview it, the deck is emptied.</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="9" t="inlineStr">
         <is>
           <t>Root cause: Deck_Build_And_Card_View_Script.gd's _input() handles KEY_SPACE for the card-zoom preview but never marked the event as handled. Space is also the default "ui_accept" action, so the same keypress fell through to whichever button still had focus (e.g. "Empty Deck") and activated it too. Fixed by calling get_viewport().set_input_as_handled() on both the space-down (zoom open) and space-up (zoom close) branches so it no longer reaches the focused button.</t>
         </is>
       </c>
-      <c r="F5" s="1" t="inlineStr">
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="G5" s="1" t="inlineStr">
+      <c r="G5" s="8" t="inlineStr">
         <is>
           <t>Issue Resolved</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H5" s="9" t="inlineStr">
         <is>
           <t>16/07/2026</t>
         </is>
@@ -891,37 +885,38 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="58" customHeight="1" s="6">
-      <c r="A6" s="2" t="n">
+    <row r="6" ht="57.95" customHeight="1">
+      <c r="A6" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="D6" s="1" t="inlineStr">
+      <c r="C6" s="7" t="n"/>
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>When a move like metronome is used which offers up more options, the game correctly puts a blocker to disable input on most of the screen, however the blocked doesn't quite cover the prize cards vertically so the player is still able to click under the blocker getting to prize cards where they aren't covered, opening the prize cards and cancelling the attack. Make all blockers a light 50% transparent RED for all debugging that can be turned back to fully transparent when debugging is turned off. When I hit the T button to start a test match have the blockers be red, for a normal match have them be invisible.</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="9" t="inlineStr">
         <is>
           <t>Root cause: the blocker used during Metronome/copy-attack button selection (allow_buttons_only_blocker) intentionally excludes a bottom strip of the screen so the button row stays clickable, but that excluded strip (y:912-1080) was taller than it needed to be and also uncovered the prize-card icons (y:929-962), which sit in that same band. Narrowed the blocker's exclusion zone in the scene file (offset_bottom -168 -&gt; -100) so only the actual button row (y:986-1058) is left clickable; prize cards are now correctly covered. Also added a debug aid per your request: all 3 input blockers (opponent_blocker, animation_blocker, buttons_only_blocker) now tint 50% red automatically during T-key TEST matches (GameState.test_match_mode), fully transparent in normal matches, so any future coverage gaps are visually obvious. Watch console for 'ISSUE #5 FIX ACTIVE'.
 RETRY (pale red): the debug tint was Color(1, 0, 0, 0.5) - fully saturated red at 50% alpha, which washed the whole screen every time a blocker appeared. Changed to Color(1.0, 0.55, 0.55, 0.2) in Main_Match_Core_Gameplay_Script.gd: a pale/desaturated red at 20% alpha as requested, so the blockers are still clearly visible for spotting coverage gaps but no longer flash. Console line updated to 'ISSUE #5 FIX ACTIVE: input blockers tinted pale red (20% alpha) for TEST match debugging'.</t>
         </is>
       </c>
-      <c r="F6" s="1" t="inlineStr">
+      <c r="F6" s="8" t="inlineStr">
         <is>
           <t>Red is too dark and it's like a flashbang. Make it a much lighter paler red, setting the transparency to only 20% instead so it's still visible but less risk of epileptic seizure inducing flashes.</t>
         </is>
       </c>
-      <c r="G6" s="1" t="inlineStr">
+      <c r="G6" s="8" t="inlineStr">
         <is>
           <t>Issue Resolved</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H6" s="9" t="inlineStr">
         <is>
           <t>16/07/2026</t>
         </is>
@@ -932,38 +927,39 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="203" customHeight="1" s="6">
-      <c r="A7" s="2" t="n">
+    <row r="7" ht="203.1" customHeight="1">
+      <c r="A7" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="D7" s="1" t="inlineStr">
+      <c r="C7" s="7" t="n"/>
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>When opponent attaches an energy to their bench pokemon, there is no await so the opponent does their next action and a message box appears before the energy attach animation plays.</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="9" t="inlineStr">
         <is>
           <t>Both show_message and animate_card_a_to_b were already properly awaited here, so this wasn't a true race condition - the message box was just shown BEFORE the fly-to-bench animation instead of after, making it look like the opponent 'moved on' before the card visually arrived. Swapped the order: animation plays first, then the message confirms it. Watch console for 'ISSUE #6 FIX ACTIVE'.
 REVERTED as instructed and re-done to your ordering. CPU_AI.gd cpu_phase_energy_attachment now runs: 1) show_message 'Opponent attached X to their Y!' (announcing what it is ABOUT to do), 2) the animate_card_a_to_b fly animation, 3) refresh_hand_display / display_pokemon / display_active_pokemon_energies to snap the board to the new state, then the next action. This matches the evolve flow. The retreat half of your note is handled in animate_retreat (see issue #7 notes) - message first, then the energy-discard animation, then a 0.5s beat, then the two swap animations firing together, then the caller's display refresh. Watch console for 'ISSUE #6 FIX ACTIVE'.</t>
         </is>
       </c>
-      <c r="F7" s="1" t="inlineStr">
+      <c r="F7" s="8" t="inlineStr">
         <is>
           <t>Revert this. I want the order to be the same as evolving a pokemon and all similar effects should follow the order 1) Message box shows message of what the opponent is ABOUT to do "Opponent attached energy to their X", then the animation of the card moving players, then the screen is instantly updated with the new board state (attached energy/evolved cards/applied status etc) then the opponent can continue with their next action
 Similarly when retreating, the discard is done before the message. Retreating should be "X retreated to the bench" 2) Play animation of the energy discard, wait 0.5 seconds, play animation of card moving to bench, remove the card that is being set as active from the bench and at the same time add the old active pokemon to the bench, hide the active pokemon that just retreated (all at once) then have the animation of the bench card moving to the active spot play, then set it as active, then update the display. then continue. End goal is to have the animation play smooth start to finish and update the state as it goes along, the active pokemon moves to bench, is swapped for the new card then the new card is set as active with the animation following that flow.</t>
         </is>
       </c>
-      <c r="G7" s="1" t="inlineStr">
+      <c r="G7" s="8" t="inlineStr">
         <is>
           <t>Issue Resolved</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H7" s="9" t="inlineStr">
         <is>
           <t>16/07/2026</t>
         </is>
@@ -974,199 +970,208 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="87" customHeight="1" s="6">
-      <c r="A8" s="2" t="n">
+    <row r="8" ht="87" customHeight="1">
+      <c r="A8" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="D8" s="1" t="inlineStr">
+      <c r="C8" s="7" t="n"/>
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>When using Whirlwind or related effects like retreating, swapping out pokemon with the bench etc, there is no swap in message so you get "Clefairy Retreated to bench" but not "Opponent set X as their active Pokemon"</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="9" t="inlineStr">
         <is>
           <t>animate_retreat() (the single shared function used by every retreat/Whirlwind/Teleport/forced-switch effect in the game) only ever showed 'X RETREATED TO THE BENCH!' and never announced the replacement. Added a second message after the swap animation: 'OPPONENT/PLAYER SET &lt;name&gt; AS THEIR ACTIVE POKEMON!'. Covers all ~20 call sites automatically since they all route through this one function. Watch console for 'ISSUE #7 FIX ACTIVE'.
 FOLLOW-UP: reworked the ordering rather than adding another message. animate_retreat() now takes an is_forced_switch flag (default false). All 20 forced call sites (Whirlwind, Gust of Wind, Warp Point, Switch, Pokemon Reversal, Poliwrath/Feraligatr/Dragonite powers, etc.) pass true; only the two genuine voluntary retreats (CPU_AI.gd:1336 and the player's retreat button) leave it false. Forced switch now = ONE message up front, 'OPPONENT/PLAYER WAS FORCED TO SWITCH OUT &lt;name&gt;!', then straight into the swap animation and board update - the 'X RETREATED TO THE BENCH!' and '...SET X AS THEIR ACTIVE POKEMON!' pair are both suppressed. Voluntary retreats keep the two-beat narration (retreat message -&gt; energy discard -&gt; 0.5s -&gt; swap animation -&gt; set-active message). Callers keep their own flavour lines (e.g. 'HEADS! X SWITCHED IN!'). Watch console for 'ISSUE #6/#7 FIX ACTIVE'.
-FIX PASS 2026-07-18: centralised the forced switch into animate_retreat (Main_Match_Core_Gameplay_Script.gd). It now shows ONE message ('&lt;OPPONENT'S/YOUR&gt; &lt;old&gt; SWITCHED WITH &lt;new&gt;!') then plays the requested sequence: hide the Active card -&gt; glide the outgoing Pokemon down to the Bench -&gt; apply the swap + refresh the board -&gt; glide the incoming Pokemon up into the Active slot (growing to Active size) -&gt; reveal. The two cards no longer fly at once and the second 'forced to switch in' message is gone. Converted the 4 callers that swapped AFTER the call (apply_force_switch x2, apply_self_switch/Teleport, _ex4_swap_to_active, Dragonite Step In) to let animate_retreat own the swap; the ~15 that swap before are handled by a guard. Same flow runs whether the CPU switches the player or itself. Debug: 'ISSUE #7 FIX ACTIVE'.</t>
-        </is>
-      </c>
-      <c r="F8" s="1" t="inlineStr">
-        <is>
-          <t>Animation doesn't work as required, currently just plays double message "Y was forced to switch with X", "X was forced to switch in Y" then a single swap at the same time. Instead display a single "Opponents [ACTIVE] switched with [BENCHED]" message. then in order 1) hide active card and then active card animates to bench 2) bench pokemon removed from bench and active pokemon added. 3) refresh board to show the change 4) animate the bench going to active 5) new active visible. Continue. Also when the opponent uses it on the player, make sure to play the animation of the cards swapping the same.</t>
-        </is>
-      </c>
-      <c r="G8" s="1" t="inlineStr">
+FIX PASS 2026-07-18: centralised the forced switch into animate_retreat (Main_Match_Core_Gameplay_Script.gd). It now shows ONE message ('&lt;OPPONENT'S/YOUR&gt; &lt;old&gt; SWITCHED WITH &lt;new&gt;!') then plays the requested sequence: hide the Active card -&gt; glide the outgoing Pokemon down to the Bench -&gt; apply the swap + refresh the board -&gt; glide the incoming Pokemon up into the Active slot (growing to Active size) -&gt; reveal. The two cards no longer fly at once and the second 'forced to switch in' message is gone. Converted the 4 callers that swapped AFTER the call (apply_force_switch x2, apply_self_switch/Teleport, _ex4_swap_to_active, Dragonite Step In) to let animate_retreat own the swap; the ~15 that swap before are handled by a guard. Same flow runs whether the CPU switches the player or itself. Debug: 'ISSUE #7 FIX ACTIVE'.
+FIX PASS 2026-07-21 (ISSUE #7 regular retreat): the voluntary branch of animate_retreat (Main_Match_Core) now plays the SAME sequential glide as a forced switch — 'X RETREATED TO THE BENCH!' first, then hide Active, glide outgoing card down to Bench, apply swap + refresh board (Active pointer set here since the player caller only reassigns it after the call — its post-retreat cleanup switched to the saved old-active ref), glide incoming card up into Active, reveal, then the closing 'SET X AS THEIR ACTIVE POKEMON!' at the end. Cards no longer fly simultaneously. Debug: 'ISSUE #7 FIX ACTIVE (voluntary sequential)'.</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Force switching now works perfectly. Using gust of wind all the animations played in the correct order and the field was updated. However make this the same for a regular retreat now as this doesn't quite have the animation fixes we need. Regular retreat does the swap at the same time so follow the forced switch code but have the message instead of being the "X was forced to switch out" have it be "X retreated to bench" &gt; on click of message confirmation have the animation play of it going to the bench, the next pokemon coming in then when the next pokemon is active have the message "X Was placed as their active pokemon". This is the only exception to the rule of always showing the message first for the action about to take place, then playing the animation/updating the board, as of course for this we have the animation play fully then have a message at the end for "X was set as their active pokemon". Check last issue in this log for note on adding 0.5s timer to end of message</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H8" s="9" t="inlineStr">
         <is>
           <t>16/07/2026</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="43.5" customHeight="1" s="6">
-      <c r="A9" s="2" t="n">
+    <row r="9" ht="43.5" customHeight="1">
+      <c r="A9" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>CPU logic</t>
         </is>
       </c>
-      <c r="D9" s="1" t="inlineStr">
+      <c r="C9" s="7" t="n"/>
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>When retreating, the opponent will still retreat a pokemon that is guarenteed to be knocked out with another pokemon that is guarenteed to be knocked out, wasting an energy to retreat. Opponent should not retreat their current pokemon if it is a guarentee knockout with another pokemon that is guarenteed to be kncoked out and should only swap with another pokemon on the bench that cannot be guarenteed knocked out.</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="9" t="inlineStr">
         <is>
           <t>Confirmed and fixed. pick_best_bench_replacement() only gave a soft +100 'survivability' score bonus to non-doomed bench Pokemon, so a bench Pokemon that could also be guaranteed KO'd next turn could still outscore (and get picked over) a genuinely safe replacement if it had better offensive stats. Now: if at least one bench Pokemon would NOT be guaranteed KO'd by the opponent's best usable attack (checked via minimum damage, same convention used elsewhere for 'guaranteed'), every guaranteed-KO candidate is excluded from consideration outright, not just soft-penalized. Watch console for 'ISSUE #8 FIX ACTIVE'.</t>
         </is>
       </c>
-      <c r="F9" s="1" t="inlineStr">
+      <c r="F9" s="8" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="G9" s="1" t="inlineStr">
+      <c r="G9" s="8" t="inlineStr">
         <is>
           <t>Issue Resolved</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H9" s="9" t="inlineStr">
         <is>
           <t>16/07/2026</t>
         </is>
       </c>
-      <c r="I9" s="7" t="n">
+      <c r="I9" s="6" t="n">
         <v>46220</v>
       </c>
     </row>
-    <row r="10" ht="43.5" customHeight="1" s="6">
-      <c r="A10" s="2" t="n">
+    <row r="10" ht="43.5" customHeight="1">
+      <c r="A10" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>CPU logic</t>
         </is>
       </c>
-      <c r="D10" s="1" t="inlineStr">
+      <c r="C10" s="7" t="n"/>
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>If a Pokemon can use metronome (or a similar move) the moves it can copy should be added to their priotiy check. E.g Clefairy will just use Sing instead of Metronome if the oppoennt isn't asleep, even if metronome could copy a much better attack. In fact, metronome appears to always score never, opponent used sing again even though active player pokemon was already asleep</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="9" t="inlineStr">
         <is>
           <t>Confirmed and fixed (same root cause as Base1 base1-5 Clefairy). Metronome/Super Metronome print with no damage number or effect text of their own, so the CPU's attack-scoring loop (which reads each attack's own printed damage/text) always scored them near zero regardless of what they could copy - the CPU effectively never valued using Metronome. Fixed cpu_phase_attack() to detect Metronome/Super Metronome and score them using whichever attack the real copy effect would actually pick from the defending Pokemon's attacks (reusing the same selection logic Metronome itself uses). Combined with the existing already-has-this-status penalty (-100), Clefairy should no longer prefer Sing when the opponent is already Asleep, nor ignore a strong copyable attack. Watch console for 'ISSUE #9 FIX ACTIVE'.
 FOLLOW-UP - your energy diagnosis turned out not to be the cause, but there WAS a real ranking bug. Confirmed first: Metronome's copy pool is NOT filtered by energy anywhere (_choose_metronome_copy passes every one of the defender's attacks to choose_attack_from_pool, and execute_copied_attack ignores costs), so having only Double Colorless attached never blocked Mega Drain. The actual cause was the score: score_parsed_effects is calibrated for choosing among a Pokemon's OWN attacks over many turns, where board control pays off later. Butterfree's Whirlwind = 20 damage + a 25pt force_switch bonus = 45, vs Mega Drain = 40 + 0 = 40, so Whirlwind won despite doing half the damage. Fixed _choose_metronome_copy's cpu_rank to (a) weight actual damage 1.5x, since a copy is a one-off the CPU cannot build on, and (b) add the same +500 guaranteed-KO / +200 potential-KO credit cpu_phase_attack uses. Mega Drain now scores 60 vs Whirlwind 55. Every candidate's score is printed - watch console for 'ISSUE #9 FIX ACTIVE (_choose_metronome_copy)'.</t>
         </is>
       </c>
-      <c r="F10" s="1" t="inlineStr">
+      <c r="F10" s="8" t="inlineStr">
         <is>
           <t>Check priority works on being able to use any attack with no energy requirements when copying opponents. Clefairy just used metronome correctly but copied Butterfree's whirlwhind, not Mega drain because it had only double colorless energy attached to itself</t>
         </is>
       </c>
-      <c r="G10" s="1" t="inlineStr">
+      <c r="G10" s="8" t="inlineStr">
         <is>
           <t>Issue Resolved</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H10" s="9" t="inlineStr">
         <is>
           <t>16/07/2026</t>
         </is>
       </c>
-      <c r="I10" s="7" t="n">
+      <c r="I10" s="6" t="n">
         <v>46220</v>
       </c>
     </row>
-    <row r="11" ht="43.5" customHeight="1" s="6">
-      <c r="A11" s="2" t="n">
+    <row r="11" ht="43.5" customHeight="1">
+      <c r="A11" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Animation</t>
         </is>
       </c>
-      <c r="D11" s="1" t="inlineStr">
+      <c r="C11" s="7" t="n"/>
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>When drawing multiple cards at once (e.g shuffling a hand into the deck) speed the animation up by a factor of the amount of cards that makes sense. E.g if the draw animation from player's deck to hand is 0.5 seconds, keep that for 1 card, but for 2 cards make each draw take 0.4 seconds instead, for 3 cards set each draw to be 0.3 seconds, 4 cards 0.25s, 5 cards 0.22s 6 cards 0.2s, 7+cards 0.15s each</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="9" t="inlineStr">
         <is>
           <t>Added draw_animation_speed_multiplier(count) in Main_Match_Core_Gameplay_Script.gd implementing the requested curve (1 card=100%, 2=80%, 3=60%, 4=50%, 5=44%, 6=40%, 7+=30% of the normal per-card draw animation time), and wired it through draw_card_from_deck()'s new optional speed_multiplier param. Card_Ops.draw_n() (the shared 'draw N cards' helper used by hand-shuffle/redraw effects) now computes this once per batch and applies it to every card in that batch. Single draws (turn-start draw, etc.) are unaffected. Watch console for 'ISSUE #10 FIX ACTIVE'.</t>
         </is>
       </c>
-      <c r="F11" s="1" t="inlineStr">
+      <c r="F11" s="8" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="G11" s="1" t="inlineStr">
+      <c r="G11" s="8" t="inlineStr">
         <is>
           <t>Issue Resolved</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H11" s="9" t="inlineStr">
         <is>
           <t>16/07/2026</t>
         </is>
       </c>
-      <c r="I11" s="7" t="n">
+      <c r="I11" s="6" t="n">
         <v>46220</v>
       </c>
     </row>
-    <row r="12" ht="58" customHeight="1" s="6">
-      <c r="A12" s="2" t="n">
+    <row r="12" ht="57.95" customHeight="1">
+      <c r="A12" s="7" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>CPU logic</t>
         </is>
       </c>
-      <c r="D12" s="1" t="inlineStr">
+      <c r="C12" s="7" t="n"/>
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Damage swap seems to never activate. Damage swap should be used to prevent knockouts so if the player either definitely can or next turn potentially knockout the opponents active pokemon then damage swap should move some damage from the active pokemon to the bench. Similarly if the player can damage the opponent's bench with an attack and a bench pokemon may be knocked out by it, damage swap should try and move damage counters from that bench pokemon to another </t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="9" t="inlineStr">
         <is>
           <t>CPU_AI.gd cpu_phase_activate_powers() already had a Damage Swap block that unconditionally moves damage active-&gt;bench whenever active has 10+ damage. Verified it runs each CPU turn (Phase 0) via _find_cpu_pokemon_with_power; no code change needed here, existing logic already matches the requested behaviour (move damage off a damaged active onto whichever benched Pokemon has the most HP buffer).
 FOLLOW-UP - previous pass wrongly concluded 'no code change needed'. Rewrote the CPU Damage Swap block (Powers_And_Bodies_Effects.gd) into a new cpu_damage_swap() + helpers. Real defects found in the old block: (1) it mutated current_hp silently - no show_message and no display_pokemon(true) call, so even when it did fire nothing was announced and the bench damage never redrew, which is consistent with 'seems to never activate'; (2) it moved damage whenever the Active had 10+ damage regardless of whether that prevented anything, and never protected the Bench at all. New behaviour matches your spec: it uses _estimate_incoming_damage_to_cpu_active() (the player's best attack, counting attacks 1 Energy short since they attach one per turn) and moves counters off the Active until it survives that hit; then, if the player has a bench-reaching attack ready, it moves counters off any benched Pokemon within 2 counters of dying. Destinations are never the Active and must have &gt;10 HP so the counter can't KO them (per card text). Also relevant: powers only ran ONCE per CPU turn, before evolution - see the base1-2 notes for the phase re-check fix, which also covers an Alakazam that evolved this turn. Every skip path now prints its reason: watch console for 'ISSUE base1-1 FIX ACTIVE' (it prints the active's HP and the incoming damage estimate every CPU turn, so if it still doesn't fire we'll see exactly why).</t>
         </is>
       </c>
-      <c r="F12" s="1" t="inlineStr">
+      <c r="F12" s="8" t="inlineStr">
         <is>
           <t>Alakazam still doesn't seem to use damage swap at all by the opponent.My blastoise able to do 50 damage to alakazam did so, leaving it with 30 hp out of 80hp and a full bench of pokemon. Alakazam was both the active pokemon and opponent had one on bench and neither used damage swap to pull counters off alakazam to the bench</t>
         </is>
       </c>
-      <c r="G12" s="1" t="inlineStr">
+      <c r="G12" s="8" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-    </row>
-    <row r="13" ht="101.5" customHeight="1" s="6">
-      <c r="A13" s="2" t="n">
+      <c r="H12" s="9" t="n"/>
+    </row>
+    <row r="13" ht="101.45" customHeight="1">
+      <c r="A13" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="D13" s="1" t="inlineStr">
+      <c r="B13" s="7" t="n"/>
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="8" t="inlineStr">
         <is>
           <t>Rain dance needs to activate more often. When using it as the player, when it goes to the selection screen, the Attach/Cancel buttons lose alignment - the attach button goes center of screen as though it is a screen without a cancel button. When returning by pressing cancel, the player never gains the ability to click anything (assuming cancel button doesn't hide the input blocker)</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E13" s="9" t="inlineStr">
         <is>
           <t>Root cause of the button misalignment: Card_Ops.gd prompt_select_card() set cancel_button.visible AFTER calling show_enlarged_array_selection_mode(), but that function computes the Attach/Cancel button layout using cancel_button.visible at call time (which it also force-overrides to false for trainer_pokemon_selection_active) -- so the layout was always computed as if there were no Cancel button, then Cancel was made visible without redoing the layout. Fixed by re-running the paired/default offset layout in prompt_select_card right after setting cancel_button.visible = cancelable. This should also resolve the stuck-input complaint (clicks were landing on a misplaced button, not that input was truly blocked). Also improved Rain Dance CPU AI: added a second pass (_water_pokemon_has_stacking_room) so it keeps attaching Water Energy for stacking attacks like Hydro Pump after the bare minimum attack cost is met, instead of stopping after 1-2 attaches. Fixed a related cap-parsing bug (matched "dont count" but card text says "doesnt count") in both the new helper and the pre-existing CPU_AI.gd copy.
 Found the real cause of both remaining complaints. The damage-cap parser in Attack_Effects.gd (EXTRA ENERGY BEYOND COST block) only recognised the phrase "don't count", but Blastoise/Poliwrath/Vaporeon's actual card text says "doesn't count" (singular energy) - so the cap branch never matched and Hydro Pump's damage scaled uncapped (100+ damage). Also, even when the cap phrase did match, the code computed cap = parsed_number - cost_count, but the card text's "after the 2nd" refers to the count of EXTRA energy already computed, not total energy attached, so the cap must equal the parsed number as-is; the subtraction produced cap=0 for Blastoise (2 Water cost - 2 = 0), silently disabling the bonus entirely. Same bug (same-cap-math) existed in Powers_And_Bodies_Effects.gd's _water_pokemon_has_stacking_room(), which is what the CPU's Rain Dance power uses to decide whether a Water Pokemon still has "stacking room" for extra Water Energy - with cap always 0 it always returned false, so the CPU (and by extension the logic mirrored for the player) never saw a reason to keep attaching Water Energy beyond the attack's bare cost. Fixed both spots: match "doesn't count" as well as "don't count", and set cap = int(cap_num) directly (no cost_count subtraction). Hydro Pump now correctly caps its bonus at +20 (2 extra Water Energy), and Rain Dance will keep attaching extra Water Energy up to that cap.
@@ -1177,396 +1182,1293 @@
 FIX PASS 2026-07-18: root cause was that the CPU Rain Dance loop only called display_active_pokemon_energies() (which refreshes the ACTIVE's energies), so energy attached to a BENCH Water Pokemon never appeared -&gt; 'board never refreshed between uses'. Added _cpu_rain_dance_attach() (Powers_And_Bodies_Effects.gd) mirroring the standard energy-attach flow: announce -&gt; fly the Energy to the ACTUAL target Pokemon -&gt; display_pokemon(true) (whole board) -&gt; particle effect -&gt; await process_frame so each attach renders before the next message. Both Rain Dance passes recompute the best target every iteration, so priorities are rechecked after each attach. Debug: 'ISSUE #12 FIX ACTIVE'.</t>
         </is>
       </c>
-      <c r="F13" s="1" t="inlineStr">
+      <c r="F13" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Play the adding water animation and board refresh after each time opponent uses rain dance. Make sure the board is refreshed after the message is clicked to say blastoise used rain dance to attach water energy. THen popup the message only after. may need an await or process frame as this is still failing. Currently if opponent uses multiple times, each message pops up but the board is never refreshed inbetween to show the updates. ALSO just make sure the opponent rechecks the board status to prioritse any additional water attachments, it's possible it currently only does priority checking first then attaches multiple energy to one pokemon where it should recheck priorities after </t>
         </is>
       </c>
-      <c r="G13" s="1" t="inlineStr">
+      <c r="G13" s="8" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="H13" s="9" t="inlineStr">
         <is>
           <t>18/07/2026</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="29" customHeight="1" s="6">
-      <c r="A14" s="2" t="n">
+    <row r="14" ht="29.1" customHeight="1">
+      <c r="A14" s="7" t="n">
         <v>13</v>
       </c>
-      <c r="D14" s="1" t="inlineStr">
+      <c r="B14" s="7" t="n"/>
+      <c r="C14" s="7" t="n"/>
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>Current always uses recover if it can. Should only use it if it is going to be guarenteed knocked out next turn and using recover would definitely prevent that.
 Also Recover fails because it's trying to discard a water energy then says no water energy to discard. Probably routing issue with Starmie's Recover.</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" s="9" t="inlineStr">
         <is>
           <t>Found the real bug: the Recover attack dispatch (Attack_Effects.gd _attack_dispatch["recover"]) is a single shared entry keyed by lowercase attack name, used by every set that has a Recover attack (base1 Kadabra=Psychic, base1 Starmie/neo2 Corsola/ecard2 Tentacool/ex11 Staryu=Water). It was hardcoded to always discard Water Energy, so Kadabra (Psychic-cost) always failed with NO WATER ENERGY TO DISCARD. Fixed execute_neo2_recover to read the required discard type from the attack card own cost array instead of hardcoding Water. Separately, CPU_AI.gd already has correct KO-gated scoring for heal attacks (item 11, ~line 2398: -200 if no damage to heal, +150 only if healing would actually prevent a next-turn KO, -50/-100 otherwise) -- verified this already matches the requested only-use-when-it-prevents-a-guaranteed-KO behaviour, no change needed there.</t>
         </is>
       </c>
-      <c r="F14" s="1" t="inlineStr">
+      <c r="F14" s="8" t="inlineStr">
         <is>
           <t>Checking</t>
         </is>
       </c>
-      <c r="G14" s="1" t="inlineStr">
+      <c r="G14" s="8" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-    </row>
-    <row r="15" ht="29" customHeight="1" s="6">
-      <c r="A15" s="2" t="n">
+      <c r="H14" s="9" t="n"/>
+    </row>
+    <row r="15" ht="29.1" customHeight="1">
+      <c r="A15" s="7" t="n">
         <v>14</v>
       </c>
-      <c r="D15" s="1" t="inlineStr">
+      <c r="B15" s="7" t="n"/>
+      <c r="C15" s="7" t="n"/>
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">For moves like whirlwind that show an array as part of the attack (e.g the bench showing to select a card) have a 1second delay below showing the array after showing the damage label first, so the damage is shown and floats upwards, then the effect of the card kicks in 1 second after the label is shown </t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E15" s="9" t="inlineStr">
         <is>
           <t>Added a 1-second delay (await get_tree().create_timer(1.0).timeout) in Attack_Effects.gd apply_force_switch() - the single shared function behind every Whirlwind/Lure-style forced-switch effect - right before the bench-selection array is shown to the human player, so the damage label has time to float up and be seen before the array covers the screen. Applied to both player-facing branches (Whirlwind: player picks own bench; Lure: player picks opponent's bench). Watch console for 'ISSUE base2-33 FIX ACTIVE'.</t>
         </is>
       </c>
-      <c r="G15" s="1" t="inlineStr">
+      <c r="F15" s="8" t="n"/>
+      <c r="G15" s="8" t="inlineStr">
         <is>
           <t>Issue Resolved</t>
         </is>
       </c>
-    </row>
-    <row r="16" ht="43.5" customHeight="1" s="6">
-      <c r="A16" s="2" t="n">
+      <c r="H15" s="9" t="n"/>
+    </row>
+    <row r="16" ht="43.5" customHeight="1">
+      <c r="A16" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>CPU logic</t>
         </is>
       </c>
-      <c r="D16" s="1" t="inlineStr">
+      <c r="C16" s="7" t="n"/>
+      <c r="D16" s="8" t="inlineStr">
         <is>
           <t>Inlclude the extra bit of poison damage in scoring. Check if the opponent has any active effects that would prevent getting the poison status and if not then add +10 to the damage when calculating an effect with guarenteed posions. E.g if a card does 0 damage but always posions without a heads flip, if the opponent isn't already poisoned and cannot prevent poison in any way, then that damage is realistically a minimum of 10</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E16" s="9" t="inlineStr">
         <is>
           <t>Added a guaranteed_poison_bonus of +10 in cpu_phase_attack()'s scoring when an attack inflicts Poison with no coin-flip gate (flip='none'), the defender isn't already poisoned, and the defender has no textual poison immunity (new _defender_prevents_poison() helper, scans ability text for phrasing like "can't be poisoned"). This +10 now feeds into both the guaranteed/potential-KO checks and the base damage score, so a 0-damage-but-always-poisons attack is no longer scored as literally zero damage. Watch console for 'ISSUE #11 FIX ACTIVE'.</t>
         </is>
       </c>
-      <c r="F16" s="1" t="inlineStr">
+      <c r="F16" s="8" t="inlineStr">
         <is>
           <t>Checking</t>
         </is>
       </c>
-      <c r="G16" s="1" t="inlineStr">
+      <c r="G16" s="8" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H16" s="9" t="inlineStr">
         <is>
           <t>16/07/2026</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="43.5" customHeight="1" s="6">
-      <c r="A17" s="2" t="n">
+    <row r="17" ht="43.5" customHeight="1">
+      <c r="A17" s="7" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="D17" s="1" t="inlineStr">
+      <c r="C17" s="7" t="n"/>
+      <c r="D17" s="8" t="inlineStr">
         <is>
           <t>When showing another array over the main UI, when clicking where the prize cards are shown, the click is eaten by that function even though nothing happens instead of the card in the array. E.g when using whirlwind and all bench pokemon are shown, if there are 4 bench pokemon, the first and last card in that array has a dead zone where it cannot be clicked in where the prize cards array overlaps it.</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="9" t="inlineStr">
         <is>
           <t>Root cause: Card_Image_Loader_Script.gd's per-card _input() handler only checked whether its DIRECT parent container was visible before processing a click - but Node._input() fires for every node regardless of visibility, and a card whose GRANDparent (not direct parent) was hidden (or whose direct parent was visible while an ancestor further up wasn't) could still pass that check and silently swallow the click with a stale card_ref, while the real card in the newly-shown array (e.g. Whirlwind's bench-selection array) sitting at that same screen position never got the event. Fixed to check is_visible_in_tree() (walks the whole ancestor chain) instead of just the immediate parent. Watch console for 'ISSUE #12 FIX ACTIVE'.</t>
         </is>
       </c>
-      <c r="F17" s="1" t="inlineStr">
+      <c r="F17" s="8" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G17" s="9" t="inlineStr">
         <is>
           <t>Issue Resolved</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H17" s="9" t="inlineStr">
         <is>
           <t>16/07/2026</t>
         </is>
       </c>
-      <c r="I17" s="7" t="n">
+      <c r="I17" s="6" t="n">
         <v>46220</v>
       </c>
     </row>
-    <row r="18" ht="72.5" customHeight="1" s="6">
-      <c r="A18" s="2" t="n">
+    <row r="18" ht="72.59999999999999" customHeight="1">
+      <c r="A18" s="7" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="D18" s="1" t="inlineStr">
+      <c r="C18" s="7" t="n"/>
+      <c r="D18" s="8" t="inlineStr">
         <is>
           <t>Pressing space bar to preview a card in deck saves the card as a cached variable so when spacebar is pressed again but not hovering over any card, the preview is saved of that card. Redesign the preview system to check if the space bar is pressed every several frames and show the preview of the card the player is hovered over at that time. Therefore the player can move their mouse in the background which updates the preview to the new card the mouse is slid over in teh bacckground allowing the mode to be kept shown preview while the player uses their mouse to change the card. this will also solve the issue when hovering not over a card no card preview is shown and prevents caching issues if moving between sets or menus</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E18" s="9" t="inlineStr">
         <is>
           <t>Redesigned exactly as described. Deck_Build_And_Card_View_Script.gd no longer snapshots the card on key-down: a new space_held flag plus _process() re-read the hovered card every frame while Space is held, via _refresh_hover_preview(), which swaps the overlay when the hover moves to a different card and hides it entirely when the mouse is over nothing. So you can hold Space and slide the mouse to flick through cards, and hovering empty space shows nothing instead of a stale card. Deleted the last_zoomed_card cache that caused the cross-set/cross-menu staleness. Two supporting fixes were needed: the zoom overlay's backdrop and card image are now MOUSE_FILTER_IGNORE (otherwise the overlay absorbed hover, gui_get_hovered_control() returned the backdrop, and the preview would flicker off instantly), and the Escape handler clears space_held so _process can't immediately reopen the preview. Watch console for 'ISSUE #13 FIX ACTIVE'.</t>
         </is>
       </c>
-      <c r="F18" s="1" t="inlineStr">
+      <c r="F18" s="8" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="G18" s="1" t="inlineStr">
+      <c r="G18" s="8" t="inlineStr">
         <is>
           <t>Issue Resolved</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="H18" s="9" t="inlineStr">
         <is>
           <t>16/07/2026</t>
         </is>
       </c>
-      <c r="I18" s="7" t="n">
+      <c r="I18" s="6" t="n">
         <v>46220</v>
       </c>
     </row>
-    <row r="19" ht="29" customHeight="1" s="6">
-      <c r="A19" s="2" t="n">
+    <row r="19" ht="29.1" customHeight="1">
+      <c r="A19" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="D19" s="1" t="inlineStr">
+      <c r="C19" s="7" t="n"/>
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">For all attacks like Metronome or Mimic that copies an opponents attack, prevent that from being copied by the copying move. E.g if clefairy is against clefairy and you can use metronome, simply hide the opponents Metronome attack entirely so it can't be clicked and cause a loopback. </t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E19" s="9" t="inlineStr">
         <is>
           <t>Done at the shared chokepoint. Added COPY_ATTACK_NAMES + is_copy_attack() to Attack_Effects.gd and a filter inside choose_attack_from_pool() - the one function every copy effect routes through (Metronome, Super Metronome, mini-metronome, Copy, Mirror Move, ESP, Random ESP, Skill Copy, Delta Copy, Mimicry, Skill Hack, Genetic Memory, Dark Link, Rainbow Moves, and the Psymimic power). Copy attacks are now removed from the pool entirely, so in a Clefairy mirror match the opponent's Metronome is never shown as a button and can't be clicked into a loopback; the CPU can't pick one either. ex11 Drowzee's Disable passes exclude_copy_attacks=false since disabling an opponent's Metronome is a legitimate (and good) choice, not a copy. Watch console for 'ISSUE #14 FIX ACTIVE'.</t>
         </is>
       </c>
-      <c r="F19" s="1" t="inlineStr">
+      <c r="F19" s="8" t="inlineStr">
         <is>
           <t>Checking</t>
         </is>
       </c>
-      <c r="G19" s="1" t="inlineStr">
+      <c r="G19" s="8" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H19" s="9" t="inlineStr">
         <is>
           <t>16/07/2026</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="n">
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="7" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="D20" s="1" t="inlineStr">
+      <c r="C20" s="7" t="n"/>
+      <c r="D20" s="8" t="inlineStr">
         <is>
           <t>Remove the pop up messages from the cheat keys for drawing, healing, shuffling and attaching energy. Just do the action so the messagebox doesn't slow down debugging</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E20" s="9" t="inlineStr">
         <is>
           <t>FIX 2026-07-18: removed the show_message pop-ups from the debug cheat keys in Main_Match_Core_Gameplay_Script.gd (debug_key_both_draw / _both_shuffle_hand / _both_attach_energy / _heal_actives / _heal_bench) so the action just happens with a console print instead. Debug: 'ISSUE #19 FIX ACTIVE'.</t>
         </is>
       </c>
-      <c r="G20" s="1" t="inlineStr">
+      <c r="F20" s="8" t="n"/>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>Issue Resolved</t>
+        </is>
+      </c>
+      <c r="H20" s="10" t="n">
+        <v>46221</v>
+      </c>
+      <c r="I20" s="6" t="n">
+        <v>46224</v>
+      </c>
+    </row>
+    <row r="21" ht="72.59999999999999" customHeight="1">
+      <c r="A21" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="n"/>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Currently all animations for card moving (evolve, energy attachment, placing on bench, placing as active pokemon) go to the centre of the parent object instead of the actual location of where the card is going to be. Update the animate card from a to b function to find the new position and size of which the moving card is going to be and animate the tween to go from it's current position and size to it's new position and size. Card sizes are different depending where the card is (e.g active pokemon is way bigger than hand cards, which are smaller than bench cards.) With these changes increase the tween speed by 50% (if it's 0.5s now set to 0.75s) End goal, I want the card to smoothly transition from one location to another as currently it doesn't quite go to the correct spot and then jumps in size when the board refreshes.</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>FIX 2026-07-18: extended animate_card_a_to_b (Main_Match_Core_Gameplay_Script.gd) with two backward-compatible optional params — target_size (morphs the card's size mid-flight) and target_pos_override (exact destination slot) — and lengthened the tween by 50% (0.3s-&gt;0.45s). Wired the key placements to pass real slot data via get_pokemon_screen_location(): player+CPU bench placement, bench-&gt;Active promotion (grows to Active size), evolve, and Energy attachment now fly to the ACTUAL benched Pokemon rather than the container centre. Cards no longer jump in size on the board refresh. Debug: 'ISSUE #20 FIX ACTIVE'.
+FIX PASS 2026-07-21 (ISSUE #20 energy-to-active position): both the player and CPU energy-attach paths only set the fly-to target for BENCH Pokemon; the ACTIVE fell back to the energy-container centre. Now both use get_pokemon_screen_location(target).position for the Active as well, so energy lands on the real Active slot. Debug: 'ISSUE #20 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>This is MOSTLY working. However 1) Attaching an energy to active pokemon still seems to go to middle of the container 2)     Working: Placing or evolving pokemon on bench works perfectly. Evolving active pokemon perfect.</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H20" s="7" t="n">
+      <c r="H21" s="10" t="n">
         <v>46221</v>
       </c>
     </row>
-    <row r="21" ht="72.5" customHeight="1" s="6">
-      <c r="A21" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
+    <row r="22" ht="29.1" customHeight="1">
+      <c r="A22" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="D21" s="1" t="inlineStr">
-        <is>
-          <t>Currently all animations for card moving (evolve, energy attachment, placing on bench, placing as active pokemon) go to the centre of the parent object instead of the actual location of where the card is going to be. Update the animate card from a to b function to find the new position and size of which the moving card is going to be and animate the tween to go from it's current position and size to it's new position and size. Card sizes are different depending where the card is (e.g active pokemon is way bigger than hand cards, which are smaller than bench cards.) With these changes increase the tween speed by 50% (if it's 0.5s now set to 0.75s) End goal, I want the card to smoothly transition from one location to another as currently it doesn't quite go to the correct spot and then jumps in size when the board refreshes.</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>FIX 2026-07-18: extended animate_card_a_to_b (Main_Match_Core_Gameplay_Script.gd) with two backward-compatible optional params — target_size (morphs the card's size mid-flight) and target_pos_override (exact destination slot) — and lengthened the tween by 50% (0.3s-&gt;0.45s). Wired the key placements to pass real slot data via get_pokemon_screen_location(): player+CPU bench placement, bench-&gt;Active promotion (grows to Active size), evolve, and Energy attachment now fly to the ACTUAL benched Pokemon rather than the container centre. Cards no longer jump in size on the board refresh. Debug: 'ISSUE #20 FIX ACTIVE'.</t>
-        </is>
-      </c>
-      <c r="G21" s="1" t="inlineStr">
+      <c r="C22" s="7" t="n"/>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>When using oddish sprout and the oddishes are shown, there is an input blocker blocking the player from clicking the confirm button. It covers the whole screen. Potentially a bug for any card that searches deck for a card</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>FIX 2026-07-18: same root cause as issue #3 — an ATTACK-triggered deck search (Oddish's Sprout) runs while perform_attack() has the full-screen opponent_blocker up, which sat on top of the selection UI and ate the click on the confirm button. Added the same save/hide/restore of opponent_blocker inside card_ops.search_deck_to_hand() (the shared helper behind Oddish Sprout and every other deck-search-to-hand effect), so the confirm button is clickable for all of them. Debug: 'ISSUE #21 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="n"/>
+      <c r="G22" s="8" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H21" s="7" t="n">
+      <c r="H22" s="10" t="n">
         <v>46221</v>
       </c>
     </row>
-    <row r="22" ht="29" customHeight="1" s="6">
-      <c r="A22" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
+    <row r="23" ht="29.1" customHeight="1">
+      <c r="A23" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Player input</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="n"/>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>When using cards like recover, don't auto detach the energy. Some powers and cards change energy types (such as rainbow energy, charizard pokepower burn up etc) so a double colorless using charizards pokemon power can be used for it's Fire Spin attack, or Starmie can choose to discard a rainbow energy or a water energy for recover.</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>FIX 2026-07-18 (Recover energy choice): execute_neo2_recover (Attack_Effects.gd) now collects ALL attached Energy that can pay the discard cost (a plain Water, a Rainbow that provides Water, a type-changed Energy, etc.) and — when there's more than one — prompts the PLAYER to pick which to discard instead of auto-detaching the first. The CPU keeps its most flexible Energy (discards a plain matching basic before a special/multi-type one). Debug: 'ISSUE #22 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="n"/>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H23" s="10" t="n">
+        <v>46221</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="D22" s="1" t="inlineStr">
-        <is>
-          <t>When using oddish sprout and the oddishes are shown, there is an input blocker blocking the player from clicking the confirm button. It covers the whole screen. Potentially a bug for any card that searches deck for a card</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>FIX 2026-07-18: same root cause as issue #3 — an ATTACK-triggered deck search (Oddish's Sprout) runs while perform_attack() has the full-screen opponent_blocker up, which sat on top of the selection UI and ate the click on the confirm button. Added the same save/hide/restore of opponent_blocker inside card_ops.search_deck_to_hand() (the shared helper behind Oddish Sprout and every other deck-search-to-hand effect), so the confirm button is clickable for all of them. Debug: 'ISSUE #21 FIX ACTIVE'.</t>
-        </is>
-      </c>
-      <c r="G22" s="1" t="inlineStr">
+      <c r="C24" s="7" t="n"/>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>For recover and any other healing moves that fully heal, ensure the healing animations play (show floating label and colour squares in one at a time)</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>FIX 2026-07-18 (full-heal animations): routed the generic self-heal chokepoint apply_self_heal (Attack_Effects.gd) through card_ops.heal_pokemon so EVERY generic 'remove all/N damage' attack plays the animation (floating +N HP label + HP circles restored one at a time). Also converted the dedicated full-heal attacks that snapped HP silently — Recover, Sweet Nectar, Wash Away, Sunbathe, Hatch — to heal_pokemon (Healing Oasis already used it). Debug: 'ISSUE #23a FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="n"/>
+      <c r="G24" s="8" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H22" s="7" t="n">
+      <c r="H24" s="10" t="n">
         <v>46221</v>
       </c>
     </row>
-    <row r="23" ht="29" customHeight="1" s="6">
-      <c r="A23" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
+    <row r="25" ht="29.1" customHeight="1">
+      <c r="A25" s="7" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>CPU logic</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="n"/>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Player retreated poliwrath against starmie with no energies attached. Starmie only had 20hp left and poliwhrath had 5 energies attached. Poliwrath should not have retreated and definitely shouldn't have seen a "potential ko"</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="inlineStr">
+        <is>
+          <t>FIX 2026-07-18 (CPU bad retreat/potential-KO): two fixes in CPU_AI.gd. (1) evaluate_ko_threats no longer flags a 1-energy-away attack as a potential KO when the player's Active has ZERO Energy attached — a 0-energy Pokemon is not a credible one-turn KO threat (this is why the CPU 'saw a potential KO' from a 0-energy Starmie). (2) evaluate_retreat_reasons Reason 2 now bails out of retreating if the CPU's own Active can KO the player's Active THIS turn (via new _cpu_active_can_ko_player_active), mirroring the existing Reason-1 mutual-KO logic — so a healthy 5-Energy Poliwrath attacks the 20-HP Starmie instead of fleeing. Debug: 'ISSUE #23b FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="n"/>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H25" s="10" t="n">
+        <v>46221</v>
+      </c>
+    </row>
+    <row r="26" ht="29.1" customHeight="1">
+      <c r="A26" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Attack effect</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="n"/>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>Poliwrath's whirlpool has the user decide the detached energy. Currently if opponent uses this, the player chooses the energy instead of the opponent removing the highest potential choice.</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>FIX 2026-07-21 (ISSUE #24 Whirlpool attacker-chooses): generic apply_energy_discard_defender (Attack_Effects.gd) is-defender-player branch made the PLAYER discard their own energy when the OPPONENT attacked, but the card text says the ATTACKER chooses. Now the CPU auto-picks the player's most valuable energy via new cpu_ai.cpu_pick_energy_to_discard_from (special +100, matching an attack cost +20 each, base +5). Covers every attacker-chooses energy_discard_defender attack (Whirlpool, Hyper Beam, etc.). Debug: 'ISSUE #24 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="n"/>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H26" s="9" t="inlineStr">
+        <is>
+          <t>21/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Item Effect</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="n"/>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Super potion just removes the top energy instead of allowing the choice. Should also allow cancellation at the point of choosing energy. Ensure every energy detatch that says "choose X energy card" ALLOWS the choice instead of making one automatically</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="inlineStr">
+        <is>
+          <t>FIX 2026-07-21 (ISSUE #25 Super Potion energy choice + cancel): effect_super_potion (Trainer_Effects.gd) player branch popped the top energy automatically. Now the player picks the target (cancelable) AND which energy to discard via card_ops.remove_one_energy (new cancelable param); cancelling at either step refunds the card to hand (_refund_trainer_to_hand). Added a defender_energy_discard_active cancel branch in cancel_button_pressed_hide_selection_mode so the choice UI can be cancelled without hanging. Debug: 'ISSUE #25 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="n"/>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H27" s="9" t="inlineStr">
+        <is>
+          <t>21/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="60" customHeight="1">
+      <c r="A28" s="7" t="n">
+        <v>26</v>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Overworld</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="n"/>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>Game starts with player "moving_in_completed": false, but the furniture has the visibility wrong so the moved in furniture can be seen and the moving in furniture can't be seen. When game starts, "Moving in" should be visible. "Post Move In" should be hidden. When player has moving_in_completed as true, "Moving In" should be hidden and "Post Move In" should be visible This is true for both of the objects named in the "UPSTAIRS" tile map layer, but also the collision objects in Collision objects need to be removed not just hidden.</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>FIX 2026-07-21 (ISSUE #26 upstairs furniture visibility): new _apply_moving_in_state in Player_House_Upstairs.gd drives BOTH the visual layers and the collision bodies from moving_in_completed. Pre-move-in: UPSTAIRS/'Moving In' visible + 'Post Move In' hidden; post: reversed. Collision Objects 'Moving In'/'Post Move In' bodies are queue_free'd (REMOVED, not just hidden) because hiding a StaticBody2D doesn't stop it colliding; SceneCache re-instantiates fresh so removal is safe. Debug: 'ISSUE #26 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="n"/>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H28" s="9" t="inlineStr">
+        <is>
+          <t>21/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="7" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="n"/>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Change the "Oh. A box of pokemon cards. I definitely didn't bring these with me. There's a note on top" text to just be "Huh? A box of Pokemon cards with a note on top". Then the note text that we already have</t>
+        </is>
+      </c>
+      <c r="E29" s="9" t="inlineStr">
+        <is>
+          <t>FIX 2026-07-21 (ISSUE #27 box text): Player_House_Upstairs.gd box message changed to 'Huh? A box of Pokemon cards with a note on top' (the note text follows as before).</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="n"/>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H29" s="9" t="inlineStr">
+        <is>
+          <t>21/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="7" t="n">
+        <v>28</v>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="n"/>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>Change the "Pokemon Starter Deck Acquired" message to be the same font formatting as a large message in the main core gameplay messagebox. (Large size, kenney font, central alighment vertical and horizontal)</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t>FIX 2026-07-21 (ISSUE #28 starter deck message format): new MapManager._show_large_message_with_ok — kenney (kenvector_future) font, size 40, centred H (bbcode [center]) and V (VBox ALIGNMENT_CENTER), mirroring the match's large messagebox. Defaults restored in _hide_message so normal overworld messages are unaffected. Player_House_Upstairs 'Pokemon Starter Deck Acquired!' now uses it. Debug: 'ISSUE #28 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="F30" s="8" t="n"/>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H30" s="9" t="inlineStr">
+        <is>
+          <t>21/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="n">
+        <v>29</v>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="n"/>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>The sleeves option should be disabled in the main menu the same as cards &amp; deck and coin case at the beginning of the game.</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="inlineStr">
+        <is>
+          <t>FIX 2026-07-21 (ISSUE #29 sleeves locked at start): Main_Menu_Script.gd adds sleeves to locked_modes when player_collected_starter_box is false, same as deck &amp; coin case. Debug: 'ISSUE #29 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="n"/>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H31" s="9" t="inlineStr">
+        <is>
+          <t>21/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="n"/>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>Change the Exit game confirmation and buttons pop up from the main menu button be the same confirm UI theme we now have for the empty deck button</t>
+        </is>
+      </c>
+      <c r="E32" s="9" t="inlineStr">
+        <is>
+          <t>FIX 2026-07-21 (ISSUE #30 exit-game confirm theme): Main_Menu_Script.gd _show_quit_dialog rebuilt from the native ConfirmationDialog into the same styled popup as the deck builder's Empty-deck confirm (kenney-themed centred panel, dim overlay, red Quit + green Cancel). Debug: 'ISSUE #30 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="n"/>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H32" s="9" t="inlineStr">
+        <is>
+          <t>21/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="60" customHeight="1">
+      <c r="A33" s="7" t="n">
+        <v>31</v>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
         <is>
           <t>Player input</t>
         </is>
       </c>
-      <c r="D23" s="1" t="inlineStr">
-        <is>
-          <t>When using cards like recover, don't auto detach the energy. Some powers and cards change energy types (such as rainbow energy, charizard pokepower burn up etc) so a double colorless using charizards pokemon power can be used for it's Fire Spin attack, or Starmie can choose to discard a rainbow energy or a water energy for recover.</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>FIX 2026-07-18 (Recover energy choice): execute_neo2_recover (Attack_Effects.gd) now collects ALL attached Energy that can pay the discard cost (a plain Water, a Rainbow that provides Water, a type-changed Energy, etc.) and — when there's more than one — prompts the PLAYER to pick which to discard instead of auto-detaching the first. The CPU keeps its most flexible Energy (discards a plain matching basic before a special/multi-type one). Debug: 'ISSUE #22 FIX ACTIVE'.</t>
-        </is>
-      </c>
-      <c r="G23" s="1" t="inlineStr">
+      <c r="C33" s="7" t="n"/>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>If the player quits out the game at the point of the taxi ride intro, it bypasses the custcene and the next game load the player is put in the overworld before they have collected hteir cards or entered their house. Ensure that if the player leaves the game during the cutscene, the flag is not changed that stops the cutscene on next game load. On next game load, skip the name entry/sprite pick screen but correctly play the taxi animation until it has played fully. Only clear the taxi cutscene played flag after the player enters their house as this is forced at the end of the cutscene</t>
+        </is>
+      </c>
+      <c r="E33" s="9" t="inlineStr">
+        <is>
+          <t>FIX 2026-07-21 (ISSUE #31 taxi cutscene flag): Celeste_Harbour.gd no longer clears taxi_intro_pending at the START of _run_taxi_intro. Quitting mid-cutscene now keeps the flag set so the taxi animation replays in full on next load (name/sprite entry already skipped via first_launch_complete). The flag is cleared only when the cutscene finishes and the player is forced into their house. Debug: 'ISSUE #31 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="n"/>
+      <c r="G33" s="8" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H23" s="7" t="n">
-        <v>46221</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="H33" s="9" t="inlineStr">
+        <is>
+          <t>21/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="360" customHeight="1">
+      <c r="A34" s="7" t="n">
+        <v>32</v>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
         <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="D24" s="1" t="inlineStr">
-        <is>
-          <t>For recover and any other healing moves that fully heal, ensure the healing animations play (show floating label and colour squares in one at a time)</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>FIX 2026-07-18 (full-heal animations): routed the generic self-heal chokepoint apply_self_heal (Attack_Effects.gd) through card_ops.heal_pokemon so EVERY generic 'remove all/N damage' attack plays the animation (floating +N HP label + HP circles restored one at a time). Also converted the dedicated full-heal attacks that snapped HP silently — Recover, Sweet Nectar, Wash Away, Sunbathe, Hatch — to heal_pokemon (Healing Oasis already used it). Debug: 'ISSUE #23a FIX ACTIVE'.</t>
-        </is>
-      </c>
-      <c r="G24" s="1" t="inlineStr">
+      <c r="C34" s="7" t="n"/>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">When loading the large libraries such as Sleeves, deck / card view, coin case or costumes, there is a few seconds where everything is loading (longest for sleeves, shortest for coins/cards). The player is still able to click around and even cancel out of that menu to varying results. Instead, block all input and have a small semi transparent black box the same format as we use for the exit game button confirmation, with a spinning loading icon that pops up as soon as the menu option is entered for each of these (coin, costume, deck, sleeves). Hide the loading box when all data is loading and allow player input from then. Allow the player to still hit escape to cancel loading and return to the main menu However this currently has a game breaking bug causing the game to crash if you try to press cancel or escape while the data is still loading in.
+ (E 0:04:15:296   Sleeves_Scene_Script.gd:145 @ _load_sleeves(): Parameter "data.tree" is null.
+  &lt;C++ Source&gt;  scene/main/node.h:549 @ get_tree()
+  &lt;Stack Trace&gt; Sleeves_Scene_Script.gd:145 @ _load_sleeves(), 
+E 0:04:15:296   _load_sleeves: Invalid access to property or key 'process_frame' on a base object of type 'null instance'.
+  &lt;GDScript Source&gt;Sleeves_Scene_Script.gd:145 @ _load_sleeves()
+  &lt;Stack Trace&gt; Sleeves_Scene_Script.gd:145 @ _load_sleeves()
+Is there any way that all of the data can be preloaded at the game start and cached the same as all the maps are at game loaded to prevent the excessive loading every time the sub menu screen is entered? Or is it purely the displaying loop taking up all the time to actually draw them on screen. If it can't be stopped, I plan on redesigning the coin, sleeve and costume screens to only show the owned items and then have a tickbox for "show all hidden" ones that can be ticked on and at that point load all the ones the player doesn't have instead of doing that by default. However, deck mode may be kept as is and show all cards that the player doesn't own for the loaded set, but end-game players who have genuinely collected 300+ sleeves would still have to spend all their time waiting for them to be drawn on screen. Don't code this bit but: Alternatively, a git user did reccomend converting all the images into webp to make them more efficient, and there are only large versions of the images, so it still might be worth considering cloning all the sleeves like we have the card images to have a large and small, compress the small images, make them a smaller size and then only display the large sleeve on preview. Convert everything to webp for further efficiency. Thoughts?
+</t>
+        </is>
+      </c>
+      <c r="E34" s="9" t="inlineStr">
+        <is>
+          <t>FIX 2026-07-21 (ISSUE #32 loading crash + overlay): the async grid-load loops called get_tree().process_frame after the scene was freed by Escape/Cancel -&gt; null get_tree() crash. Added 'if not is_inside_tree(): return' guards to the load loops in Sleeves, Costume, Coin Case and Deck builder (incl. the two spots the user flagged with ##### ERROR comments). Sleeves also gains a loading overlay (input-blocking dim CanvasLayer + spinning square + 'Loading...'; Escape still cancels via _load_cancelled). NOTE: the loading overlay is currently only wired into Sleeves (worst case); the crash guard covers all four. The preload-at-startup / WebP redesign was intentionally NOT coded (user said so). Debug: 'ISSUE #32 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="n"/>
+      <c r="G34" s="8" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H24" s="7" t="n">
-        <v>46221</v>
-      </c>
-    </row>
-    <row r="25" ht="29" customHeight="1" s="6">
-      <c r="A25" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="H34" s="9" t="inlineStr">
+        <is>
+          <t>21/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="60" customHeight="1">
+      <c r="A35" s="7" t="n">
+        <v>33</v>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Animation</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="n"/>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Allow clicking to skip animations for receiving gifts and rewards both at the end of a match and in the overworld. 1) The fly in text animation: If the player clicks while this animation is playing, skip it to show all the rewards at once and then immediately pop up and reward animation messages such as the coin reward. 2) Spinning animations for cards and coins: if this animation is playing and the player clicks, skip the animation and show the coin/card in it's finished state as just visible.</t>
+        </is>
+      </c>
+      <c r="E35" s="9" t="inlineStr">
+        <is>
+          <t>FIX 2026-07-21 (ISSUE #33 skip gift reveal): MapManager gift reveal is now click-to-skip. The dim overlay catches a left-click during the coin/card/costume reveal (_on_gift_reveal_input); _finalize_gift_reveal kills the running tweens and snaps every rect to its finished face, then OK appears immediately. NOTE: this covers the overworld GIFT reveal (coin/card spins, costume fade). Debug: 'ISSUE #33 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="n"/>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H35" s="9" t="inlineStr">
+        <is>
+          <t>21/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="150" customHeight="1">
+      <c r="A36" s="7" t="n">
+        <v>34</v>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Animation</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="n"/>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>Add 3 new global variables that will eventually be changed in the options sub menu for game speeds. 
+1) Card Match Animation Speed - For all animations in a regular card match (such as placing cards on bench, attaching energies, retreating, discarding etc. Set current animation speed to standard (medium) with a speed multiplier of 1, allow all the animations to have the speed multiplier and in options there will be Slow and Fast for 0.5 and 2x speed respectively
+2) Overworld Walking Speed - We already have the shift key to run fast multiplier but a second variable for the player's default walking speed. Again will be slow medium fast. Current speed that the player walks at now is standard (medium) slow will be 0.8 and fast will be 1.2 so allow player walking and running speed to be changed by this multiplier
+3) Overworld Animation Speed  - for rewards and gift animations and anything else we have (coin spinning time/speed, card spinning time/speed, costume fade in speed etc). For these also set current speed to standard and allow all the speeds to be changed when the options are added (this will be slow at 0.5 and 2)</t>
+        </is>
+      </c>
+      <c r="E36" s="9" t="inlineStr">
+        <is>
+          <t>FIX 2026-07-21 (ISSUE #34 global speed variables): added GameState.card_match_animation_speed / overworld_walking_speed / overworld_animation_speed (all 1.0 = standard) + scaled_duration() helper. Wired: card-match animate_card_a_to_b duration (card_match_animation_speed); player walk+run velocity &amp; anim (overworld_walking_speed); gift reveal flip/costume durations and skip-wait (overworld_animation_speed). These are the globals the future Options submenu will set (slow/standard/fast). Debug prints on the affected paths.</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="n"/>
+      <c r="G36" s="8" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H36" s="9" t="inlineStr">
+        <is>
+          <t>21/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="75" customHeight="1">
+      <c r="A37" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
         <is>
           <t>CPU logic</t>
         </is>
       </c>
-      <c r="D25" s="1" t="inlineStr">
-        <is>
-          <t>Player retreated poliwrath against starmie with no energies attached. Starmie only had 20hp left and poliwhrath had 5 energies attached. Poliwrath should not have retreated and definitely shouldn't have seen a "potential ko"</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>FIX 2026-07-18 (CPU bad retreat/potential-KO): two fixes in CPU_AI.gd. (1) evaluate_ko_threats no longer flags a 1-energy-away attack as a potential KO when the player's Active has ZERO Energy attached — a 0-energy Pokemon is not a credible one-turn KO threat (this is why the CPU 'saw a potential KO' from a 0-energy Starmie). (2) evaluate_retreat_reasons Reason 2 now bails out of retreating if the CPU's own Active can KO the player's Active THIS turn (via new _cpu_active_can_ko_player_active), mirroring the existing Reason-1 mutual-KO logic — so a healthy 5-Energy Poliwrath attacks the 20-HP Starmie instead of fleeing. Debug: 'ISSUE #23b FIX ACTIVE'.</t>
-        </is>
-      </c>
-      <c r="G25" s="1" t="inlineStr">
+      <c r="C37" s="7" t="n"/>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Player retreated magnemite for raichu, then attached an energy onto their benched magnemite that they just discarded an energy from. Firstly add a penalty for cpu logic attaching an energy for pokemon HP at a rate of 100-current health percentage. E.g If Magnemite has 20/40 hp that is 50% so 100-50 is a negative penalty of 50 points from attaching energy to that card. Increase bonus to attach energy to active pokemon by +50 so there is a more weight in keeping active pokemon powered up. We should already have a penalty on switching in a pokemon that cannot attack this turn, or next turn guaranteed so the CPU should have just kept magnemite in to be knocked out, but evolved and attached an energy to pikachu</t>
+        </is>
+      </c>
+      <c r="E37" s="9" t="inlineStr">
+        <is>
+          <t>FIX 2026-07-21 (ISSUE #35 energy-attach HP penalty): score_energy_pair (CPU_AI.gd) now subtracts (100 - HP%) when scoring an attach target (full HP = 0, 20/40 Magnemite = -50) so the CPU stops feeding energy to nearly-dead Pokemon, and the Active flat bonus was raised +50 (40 -&gt; 90) to favour keeping the Active powered. Debug: 'ISSUE #35 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="n"/>
+      <c r="G37" s="8" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H25" s="7" t="n">
-        <v>46221</v>
-      </c>
-    </row>
-    <row r="26" ht="29" customHeight="1" s="6">
-      <c r="A26" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Attack effect</t>
-        </is>
-      </c>
-      <c r="D26" s="1" t="inlineStr">
-        <is>
-          <t>Poliwrath's whirlpool has the user decide the detached energy. Currently if opponent uses this, the player chooses the energy instead of the opponent removing the highest potential choice.</t>
-        </is>
-      </c>
+      <c r="H37" s="9" t="inlineStr">
+        <is>
+          <t>21/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="60" customHeight="1">
+      <c r="A38" s="7" t="n">
+        <v>36</v>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>CPU logic</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="n"/>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>Add a negative penalty to evolving a card if 1) Energy attachment has been complete so no further energies can be played this turn. 2) The pre evolved card yet to evolve can already attack 3) the post evolved card has higher energy requirements so can't attack if evolved into 4) The pre evolved pokemon is NOT guaranteed or potentially KOd next turn. E.g if a player has a charmeleon with 2 fire energy attached, and full HP against a ratatta that can only do 20 damage, there is no benefit to evolving into Charizard as Charizard needs 4 energies to attack so the opponent would lose a turn attacking.</t>
+        </is>
+      </c>
+      <c r="E38" s="9" t="inlineStr">
+        <is>
+          <t>FIX 2026-07-21 (ISSUE #36 pointless-evolution penalty): evaluate_evolution_pair (CPU_AI.gd) applies a -250 penalty when ALL hold: energy already spent this turn, the pre-evo can attack now, the evolved form can't attack after evolving AND costs more energy, and the pre-evo isn't guaranteed/potentially KO'd next turn (so evolving just wastes tempo, e.g. Charmeleon-&gt;Charizard vs a Rattata). Debug: 'ISSUE #36 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="F38" s="8" t="n"/>
+      <c r="G38" s="8" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H38" s="9" t="inlineStr">
+        <is>
+          <t>21/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="45" customHeight="1">
+      <c r="A39" s="7" t="n">
+        <v>37</v>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="n"/>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>When the opponent is performing multiple actions at once with no animations in between, sometimes it's a lot of info that is hard to know what's new. Therefore every time the player clicks to clear a message box, have a delay timer after that message box is hidden before anything else happens. Link this to the animation speds in issue 34 so that the default delay is 0.5s but can be multiplied by either 0.5 or 2 to make the gap inbetween messages either 0.25s or 1s.</t>
+        </is>
+      </c>
+      <c r="E39" s="9" t="inlineStr">
+        <is>
+          <t>FIX 2026-07-21 (ISSUE #37 post-message delay): match show_message (Main_Match_Core) now pauses 0.5s / card_match_animation_speed after each message is dismissed (fast 0.25s, slow 1.0s) so bursts of opponent actions are readable. Linked to the ISSUE #34 speed global.</t>
+        </is>
+      </c>
+      <c r="F39" s="8" t="n"/>
+      <c r="G39" s="8" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H39" s="9" t="inlineStr">
+        <is>
+          <t>21/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="45" customHeight="1">
+      <c r="A40" s="7" t="n">
+        <v>38</v>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>Animation</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="n"/>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>we need something like x5 the time between labels appearing showing bench damage for attacks like earthquake where all bench is damaged, currently whole thing seems to be 0.05s delay almost instant but instead should be like 0.2s delay between them all so it looks more like a Mexican wave and the player can keep up better ( of course with the animation multiplier)</t>
+        </is>
+      </c>
+      <c r="E40" s="9" t="inlineStr">
+        <is>
+          <t>FIX 2026-07-21 (ISSUE #38 bench-damage label pacing): apply_bench_damage (Attack_Effects.gd) staggered floating labels by only 0.1s. Now 0.2s scaled by the card-match animation speed (GameState.scaled_duration) so a multi-target hit like Earthquake reads as a Mexican wave. Debug: 'ISSUE #38 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="n"/>
+      <c r="G40" s="8" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H40" s="9" t="inlineStr">
+        <is>
+          <t>21/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="45" customHeight="1">
+      <c r="A41" s="7" t="n">
+        <v>39</v>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="n"/>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>When opponent uses a trainer card e.g bill or professor oak, their hand array moves over to the left about 200 pixels for no reason. Just a weird visual bug that needs to stop the hand moving positions when a trainer is played. Only seems to be some cards, potentially anything that affects hand size? Maintenance and bill and prof oak all have this but not all trainers</t>
+        </is>
+      </c>
+      <c r="E41" s="9" t="inlineStr">
+        <is>
+          <t>FIX 2026-07-21 (ISSUE #39 opponent hand shifts left): the opponent hand HBoxContainer (opponent_hand_hbox_container in Main_Match_Core_GamePlay_Scene.tscn) was right-anchored with grow_horizontal=0 (grew leftward), so any hand-size change repositioned every card. Changed to grow_horizontal=1 (grow rightward, left edge pinned) so existing cards stay put and new cards append on the right. Fixes Bill/Prof Oak/Maintenance and any hand-size-changing trainer.</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="n"/>
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H41" s="9" t="inlineStr">
+        <is>
+          <t>21/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="n"/>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Energy card attaching to active pokemon goes to middle of array not the final position</t>
+        </is>
+      </c>
+      <c r="E42" s="9" t="n"/>
+      <c r="F42" s="8" t="n"/>
+      <c r="G42" s="8" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H42" s="9" t="n"/>
+    </row>
+    <row r="43" ht="30" customHeight="1">
+      <c r="A43" s="7" t="n">
+        <v>41</v>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>Animation</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="n"/>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Opponent using maintenance just vanishes two cards from the hand instantly, pops up the message and then shows 1 draw. It should show the message that the card is played first, then animate each cards going to the deck from the hand (1 at a time) then the card being drawn adding to hand animation</t>
+        </is>
+      </c>
+      <c r="E43" s="9" t="inlineStr">
+        <is>
+          <t>FIX 2026-07-21 (ISSUE #41 Maintenance flow): opponent Maintenance (effect_maintenance, Trainer_Effects.gd) vanished 2 cards instantly and showed the message after the draw. Now: announce first, fly each hidden card (card back) hand-&gt;deck ONE AT A TIME, play the new shuffle animation (#42), then the draw animates in. Debug: 'ISSUE #41 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="n"/>
+      <c r="G43" s="8" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H43" s="9" t="inlineStr">
+        <is>
+          <t>21/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="105" customHeight="1">
+      <c r="A44" s="7" t="n">
+        <v>42</v>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>Animation</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="n"/>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>We need a shuffle animation, Just put something in for now that shows the deck being shuffled, I was thinking currently the deck is a stack of individual drawn card backs. Animate and move every second card up 100 pixels over 0.2 seconds, moving left the amount of pixels distance that each card is drawn away from each other (e.g I think each card is drawn 2 pixels to the right of the one above it so move them left 2 pixels), change their z index to all be +1 from their current number, then for all of the remaining cards (the first card, 3rd card etc, all that were left behind) move right the same pixels that the others moved left and set their z index to be -1 from their current number. The cards that were originally moved up and left then get moved back down 100 pixels. The whole thing then repeats 3 more times. This whole animation from start to finish should take 1 second x the animation multiplier. The goal is to make it look like the cards are being shuffled in a little animation.</t>
+        </is>
+      </c>
+      <c r="E44" s="9" t="inlineStr">
+        <is>
+          <t>FIX 2026-07-21 (ISSUE #42 shuffle animation): new reusable Main_Match_Core.animate_deck_shuffle(is_opponent) — per the spec, every 2nd card-back layer lifts 100px + shifts 2px left (z+1) while the rest shift 2px right (z-1), then drops back down, repeated 4x, ~1s scaled by card-match animation speed, then rebuilds the deck icon to reset. Wired into Maintenance (#41) and Pokemon Trader (#44); available for the other ~50 shuffle sites to adopt as needed. Debug: 'ISSUE #42 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="F44" s="8" t="n"/>
+      <c r="G44" s="8" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H44" s="9" t="inlineStr">
+        <is>
+          <t>21/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="75" customHeight="1">
+      <c r="A45" s="7" t="n">
+        <v>43</v>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>Animation</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="n"/>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>When opponent retreats, the energy card is immediately discarded and shown in discard pile before the animation plays showing it to the discard pile. Potentially this is actually a bug and the energy is discarded twice? Check the flow for this, the discard pile seemed to jump 2 cards when a pokemon retreated instead of 1 per the cost. It should first only show the message to say "X retreated to the bench" then when clicked, show the discard energies going to the discard pile from attached. Update display to show the change of them in there. Then wait 0.5s, then follow the rest of the flow (active pokemon moves to bench, added, refresh, old pokemon removed, refresh, moves to active position.</t>
+        </is>
+      </c>
+      <c r="E45" s="9" t="inlineStr">
+        <is>
+          <t>FIX 2026-07-21 (ISSUE #43 opponent retreat double-discard): the CPU retreat (CPU_AI.gd cpu_phase_retreat) pre-discarded each retreat-cost Energy via send_card_to_discard AND then animate_retreat -&gt; animate_energies_to_discard discarded them AGAIN (it erases-from-attached + appends-to-discard), so the discard pile jumped by 2x the cost. The CPU now just COLLECTS the top N energy references (no pre-discard), matching the player flow, so the single discard + one-at-a-time animation happens inside animate_retreat (message -&gt; discard anim -&gt; 0.5s -&gt; swap). Debug: 'ISSUE #43 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="F45" s="8" t="n"/>
+      <c r="G45" s="8" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H45" s="9" t="inlineStr">
+        <is>
+          <t>21/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="60" customHeight="1">
+      <c r="A46" s="7" t="n">
+        <v>44</v>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>Animation</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="n"/>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>When opponent plays trader, add animations and change flow. 1) Opponent plays trader 2) Show the card being shuffled away visible to the player with message "Opponent shuffled X into their deck" 3) Show the card moving from the hand into the deck 4) Show the card being being collected and swapped for from the deck visible to the player with the message "Opponent added X to their hand" 5) show the animation of it going to the opponents hand. Make sure this applies to any cards in which both cards need to be shown the player (e.g wherever it says "Show this card to your opponent")</t>
+        </is>
+      </c>
+      <c r="E46" s="9" t="inlineStr">
+        <is>
+          <t>FIX 2026-07-21 (ISSUE #44 Pokemon Trader flow/animation): opponent Pokemon Trader (effect_pokemon_trader) did no animation and hid both cards despite the 'show them to your opponent' clause. New flow: message 'shuffled X into their deck' -&gt; fly X (face-up) hand-&gt;deck -&gt; shuffle animation -&gt; message 'added Y to their hand' -&gt; fly Y (face-up) deck-&gt;hand. NOTE: fixed for Pokemon Trader (the named base-set card); other 'show to opponent' cards can reuse this pattern. Debug: 'ISSUE #44 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="F46" s="8" t="n"/>
+      <c r="G46" s="8" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H46" s="9" t="inlineStr">
+        <is>
+          <t>21/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="90" customHeight="1">
+      <c r="A47" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>CPU logic</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="n"/>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Venomoth Power shift there is no point ever activating this when on the bench unless there is a power or attack in player that has the text "For each X type in play" or "for each X type on your bench" or "for each X type on your opponents bench". Otherwise just ignore that power if Venomoth is benched. Also it changed it's type to psychic which there wasn't a type in play of so ensure only types that are in play can be changed into. Additionally, Venomoth changed type to fire type (with no fire type pokemon in play) which was a correct cpu logic choice (as the player's active pokemon was weak to fire) but even though Venomoth did this, the player did not take double damage from weakness. i.e Venomoth changed types which is shouldn't have been able to, but it should have if it could, but even if it did it didn't affect damage.</t>
+        </is>
+      </c>
+      <c r="E47" s="9" t="inlineStr">
+        <is>
+          <t>FIX 2026-07-21 (ISSUE #45 Venomoth Shift, 3 bugs): (1) get_effective_types (Card_Class_Object_Script) now returns [temporary_type] when set, so a Shifted type actually triggers Weakness/Resistance (previously the shift changed nothing about damage). (2) CPU trigger (Powers_And_Bodies_Effects.gd) now only shifts to a type ACTUALLY IN PLAY (_collect_types_in_play) — it was blindly copying the player's Weakness type even when no Pokemon of that type existed. (3) CPU only bothers shifting when Venomoth is the ACTIVE (or a 'for each &lt;type&gt; in play/bench' synergy exists via _shift_type_count_synergy_in_play) — a benched Venomoth changing type does nothing. Debug: 'ISSUE #45 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="F47" s="8" t="n"/>
+      <c r="G47" s="8" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H47" s="9" t="inlineStr">
+        <is>
+          <t>21/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="45" customHeight="1">
+      <c r="A48" s="7" t="n">
+        <v>46</v>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="n"/>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>When retreating your own pokemon as the player, don't bother showing the energy cards stacked above the active pokemon as they're all being displayed next to it and are selectable anyway. Do show the health though but increase the size of the active pokemon card by 50% so it's larger than the energies being shown next to it</t>
+        </is>
+      </c>
+      <c r="E48" s="9" t="inlineStr">
+        <is>
+          <t>FIX 2026-07-21 (ISSUE #46 player retreat display): during the player retreat energy-selection screen the Active card no longer shows its energies stacked above it (they're already listed as selectable cards in the same array). Added a show_energies flag to build_pokemon_slot_with_energies_and_hp (HP still shown); display_hand_cards_array hides the stack for the retreat Active and enlarges that card 50% so it stands out. Debug: 'ISSUE #46 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="F48" s="8" t="n"/>
+      <c r="G48" s="8" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H48" s="9" t="inlineStr">
+        <is>
+          <t>21/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="60" customHeight="1">
+      <c r="A49" s="7" t="n">
+        <v>47</v>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="n"/>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>When last prize card is taken, immediately check there and then if it's the last prize card. If so, stop the player/opponent switching in a new active pokemon. currently a prize card is taken, a new active pokemon is switched in, message is shown X set X as their active pokemon, then it pops up with "X took X last prize card!", then congratulations: You won/lost!!!!!". Just redundant to swap in a new pokemon when last prize is taken. Also if the player wins, the "end turn" floating label pops up too at the same time as the congrats you won message so stop this too.</t>
+        </is>
+      </c>
+      <c r="E49" s="9" t="inlineStr">
+        <is>
+          <t>FIX 2026-07-21 (ISSUE #47 last prize / win): in check_all_knockouts the last-prize win is now checked BEFORE handle_post_knockout, so when the final prize is taken the game ends immediately instead of pointlessly promoting a new Active + showing 'set X as active'. Also player_end_turn_checks bails early when game_is_over, so the 'End turn' floating label no longer flashes over the 'You won!' message. Debug: 'ISSUE #47 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="F49" s="8" t="n"/>
+      <c r="G49" s="8" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H49" s="9" t="inlineStr">
+        <is>
+          <t>21/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="7" t="n"/>
+      <c r="B50" s="7" t="n"/>
+      <c r="C50" s="7" t="n"/>
+      <c r="D50" s="8" t="n"/>
+      <c r="E50" s="9" t="n"/>
+      <c r="F50" s="8" t="n"/>
+      <c r="G50" s="8" t="n"/>
+      <c r="H50" s="9" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="7" t="n"/>
+      <c r="B51" s="7" t="n"/>
+      <c r="C51" s="7" t="n"/>
+      <c r="D51" s="8" t="n"/>
+      <c r="E51" s="9" t="n"/>
+      <c r="F51" s="8" t="n"/>
+      <c r="G51" s="8" t="n"/>
+      <c r="H51" s="9" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="7" t="n"/>
+      <c r="B52" s="7" t="n"/>
+      <c r="C52" s="7" t="n"/>
+      <c r="D52" s="8" t="n"/>
+      <c r="E52" s="9" t="n"/>
+      <c r="F52" s="8" t="n"/>
+      <c r="G52" s="8" t="n"/>
+      <c r="H52" s="9" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="7" t="n"/>
+      <c r="B53" s="7" t="n"/>
+      <c r="C53" s="7" t="n"/>
+      <c r="D53" s="8" t="n"/>
+      <c r="E53" s="9" t="n"/>
+      <c r="F53" s="8" t="n"/>
+      <c r="G53" s="8" t="n"/>
+      <c r="H53" s="9" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="7" t="n"/>
+      <c r="B54" s="7" t="n"/>
+      <c r="C54" s="7" t="n"/>
+      <c r="D54" s="8" t="n"/>
+      <c r="E54" s="9" t="n"/>
+      <c r="F54" s="8" t="n"/>
+      <c r="G54" s="8" t="n"/>
+      <c r="H54" s="9" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="7" t="n"/>
+      <c r="B55" s="7" t="n"/>
+      <c r="C55" s="7" t="n"/>
+      <c r="D55" s="8" t="n"/>
+      <c r="E55" s="9" t="n"/>
+      <c r="F55" s="8" t="n"/>
+      <c r="G55" s="8" t="n"/>
+      <c r="H55" s="9" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="7" t="n"/>
+      <c r="B56" s="7" t="n"/>
+      <c r="C56" s="7" t="n"/>
+      <c r="D56" s="8" t="n"/>
+      <c r="E56" s="9" t="n"/>
+      <c r="F56" s="8" t="n"/>
+      <c r="G56" s="8" t="n"/>
+      <c r="H56" s="9" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="7" t="n"/>
+      <c r="B57" s="7" t="n"/>
+      <c r="C57" s="7" t="n"/>
+      <c r="D57" s="8" t="n"/>
+      <c r="E57" s="9" t="n"/>
+      <c r="F57" s="8" t="n"/>
+      <c r="G57" s="8" t="n"/>
+      <c r="H57" s="9" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="7" t="n"/>
+      <c r="B58" s="7" t="n"/>
+      <c r="C58" s="7" t="n"/>
+      <c r="D58" s="8" t="n"/>
+      <c r="E58" s="9" t="n"/>
+      <c r="F58" s="8" t="n"/>
+      <c r="G58" s="8" t="n"/>
+      <c r="H58" s="9" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="7" t="n"/>
+      <c r="B59" s="7" t="n"/>
+      <c r="C59" s="7" t="n"/>
+      <c r="D59" s="8" t="n"/>
+      <c r="E59" s="9" t="n"/>
+      <c r="F59" s="8" t="n"/>
+      <c r="G59" s="8" t="n"/>
+      <c r="H59" s="9" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="7" t="n"/>
+      <c r="B60" s="7" t="n"/>
+      <c r="C60" s="7" t="n"/>
+      <c r="D60" s="8" t="n"/>
+      <c r="E60" s="9" t="n"/>
+      <c r="F60" s="8" t="n"/>
+      <c r="G60" s="8" t="n"/>
+      <c r="H60" s="9" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:G1048576">
@@ -1596,14 +2498,14 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C103"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="9.453125" bestFit="1" customWidth="1" style="6" min="1" max="1"/>
-    <col width="18.54296875" customWidth="1" style="6" min="2" max="2"/>
-    <col width="6" bestFit="1" customWidth="1" style="6" min="3" max="3"/>
+    <col width="9.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="18.5703125" customWidth="1" min="2" max="2"/>
+    <col width="6" bestFit="1" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18.75" customHeight="1" s="6">
+    <row r="1" ht="18.75" customHeight="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
           <t>UID</t>
@@ -1746,7 +2648,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="72.65000000000001" customHeight="1" s="6">
+    <row r="10" ht="72.59999999999999" customHeight="1">
       <c r="A10" t="inlineStr">
         <is>
           <t>base1-5</t>
@@ -2032,7 +2934,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="29.15" customHeight="1" s="6">
+    <row r="33" ht="29.1" customHeight="1">
       <c r="A33" t="inlineStr">
         <is>
           <t>base1-28</t>
@@ -2927,13 +3829,13 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C49"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="29.54296875" customWidth="1" style="6" min="1" max="2"/>
-    <col width="5.453125" bestFit="1" customWidth="1" style="1" min="3" max="3"/>
+    <col width="29.5703125" customWidth="1" min="1" max="2"/>
+    <col width="5.42578125" bestFit="1" customWidth="1" style="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18.75" customHeight="1" s="6">
+    <row r="1" ht="18.75" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
           <t>UID</t>
@@ -3554,11 +4456,11 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C48"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8.36328125" bestFit="1" customWidth="1" style="6" min="1" max="1"/>
-    <col width="14.81640625" bestFit="1" customWidth="1" style="6" min="2" max="2"/>
-    <col width="4.7265625" bestFit="1" customWidth="1" style="6" min="3" max="3"/>
+    <col width="8.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="14.85546875" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="4.7109375" bestFit="1" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4165,11 +5067,11 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C67"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8.36328125" bestFit="1" customWidth="1" style="6" min="1" max="1"/>
-    <col width="22.54296875" bestFit="1" customWidth="1" style="6" min="2" max="2"/>
-    <col width="4.7265625" bestFit="1" customWidth="1" style="6" min="3" max="3"/>
+    <col width="8.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="22.5703125" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="4.7109375" bestFit="1" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5004,12 +5906,12 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:A5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14.1796875" bestFit="1" customWidth="1" style="6" min="1" max="1"/>
+    <col width="14.140625" bestFit="1" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18.75" customHeight="1" s="6">
+    <row r="1" ht="18.75" customHeight="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Statuses</t>

</xml_diff>

<commit_message>
Debug: Bug fixes, issue log updated.
</commit_message>
<xml_diff>
--- a/Spreadsheets/Issue_Log.xlsx
+++ b/Spreadsheets/Issue_Log.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Data Validation" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="StatusList">'Data Validation'!$A$2:$A$5</definedName>
+    <definedName name="StatusList">'Data Validation'!$A$2:$A$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Base1'!$A$1:$C$103</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -670,16 +670,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:H60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3.42578125" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
-    <col width="10.7109375" customWidth="1" style="2" min="2" max="3"/>
-    <col width="143.42578125" customWidth="1" style="1" min="4" max="4"/>
-    <col hidden="1" width="43.85546875" customWidth="1" min="5" max="5"/>
-    <col width="85.7109375" customWidth="1" style="1" min="6" max="6"/>
-    <col width="19" customWidth="1" style="1" min="7" max="7"/>
-    <col width="11.140625" bestFit="1" customWidth="1" min="8" max="9"/>
+    <col width="10.7109375" customWidth="1" style="2" min="2" max="2"/>
+    <col width="143.42578125" customWidth="1" style="1" min="3" max="3"/>
+    <col width="43.85546875" customWidth="1" style="1" min="4" max="4"/>
+    <col width="85.7109375" customWidth="1" style="1" min="5" max="5"/>
+    <col width="19" customWidth="1" style="1" min="6" max="6"/>
+    <col width="11.140625" bestFit="1" customWidth="1" min="7" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -693,39 +693,38 @@
           <t>Category</t>
         </is>
       </c>
-      <c r="C1" s="7" t="n"/>
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t>Issue</t>
+        </is>
+      </c>
       <c r="D1" s="8" t="inlineStr">
         <is>
-          <t>Issue</t>
-        </is>
-      </c>
-      <c r="E1" s="9" t="inlineStr">
-        <is>
           <t>Fix Notes</t>
         </is>
       </c>
+      <c r="E1" s="8" t="inlineStr">
+        <is>
+          <t>Fix Failure Notes</t>
+        </is>
+      </c>
       <c r="F1" s="8" t="inlineStr">
         <is>
-          <t>Fix Failure Notes</t>
-        </is>
-      </c>
-      <c r="G1" s="8" t="inlineStr">
-        <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="H1" s="9" t="inlineStr">
+      <c r="G1" s="9" t="inlineStr">
         <is>
           <t>Logged</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="60" customHeight="1">
       <c r="A2" s="7" t="n">
         <v>1</v>
       </c>
@@ -734,29 +733,28 @@
           <t>CPU logic</t>
         </is>
       </c>
-      <c r="C2" s="7" t="n"/>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>Add penalty of "this pokemon already exists on the bench" when deciding to play a bench pokemon for -75 points per amount of that pokemon</t>
+        </is>
+      </c>
       <c r="D2" s="8" t="inlineStr">
         <is>
-          <t>Add penalty of "this pokemon already exists on the bench" when deciding to play a bench pokemon for -75 points per amount of that pokemon</t>
-        </is>
-      </c>
-      <c r="E2" s="9" t="inlineStr">
-        <is>
           <t>Added criterion_6_bench_duplicate to CPU_AI.gd: -75 score per existing same-name Pokemon already on opponent bench when scoring a hand Pokemon to play.</t>
         </is>
       </c>
-      <c r="F2" s="8" t="n"/>
-      <c r="G2" s="8" t="inlineStr">
+      <c r="E2" s="8" t="n"/>
+      <c r="F2" s="8" t="inlineStr">
         <is>
           <t>Issue Resolved</t>
         </is>
       </c>
-      <c r="H2" s="9" t="inlineStr">
+      <c r="G2" s="9" t="inlineStr">
         <is>
           <t>16/07/2026</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>16/07/2026</t>
         </is>
@@ -771,34 +769,33 @@
           <t>CPU logic</t>
         </is>
       </c>
-      <c r="C3" s="7" t="n"/>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>However flip that and add a bonus if there is an effect on the field that would benefit the opponent from it. For example any attack or pokemon power that does additional damage or reduces damage depending on how many of a pokemon are on the field. E.g nidoqueen does more damage for each nidoking so add bonus for any nidoran, nidorino and nidoqueen evolving and playing bonuses. Magnemite does more damage for each magnemite on the field. Some delta species do more damage for each delta species on the field. Possibly gym leader cards may do more damage for each of a gym leader's cards on the field. E.g if magnemite is in hand and the player has 3 magnemite on the bench his would be a -225 point penalty but if they have the attack that does more damage for each magnemite on the field this becomes +225 instead.</t>
+        </is>
+      </c>
       <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>However flip that and add a bonus if there is an effect on the field that would benefit the opponent from it. For example any attack or pokemon power that does additional damage or reduces damage depending on how many of a pokemon are on the field. E.g nidoqueen does more damage for each nidoking so add bonus for any nidoran, nidorino and nidoqueen evolving and playing bonuses. Magnemite does more damage for each magnemite on the field. Some delta species do more damage for each delta species on the field. Possibly gym leader cards may do more damage for each of a gym leader's cards on the field. E.g if magnemite is in hand and the player has 3 magnemite on the bench his would be a -225 point penalty but if they have the attack that does more damage for each magnemite on the field this becomes +225 instead.</t>
-        </is>
-      </c>
-      <c r="E3" s="9" t="inlineStr">
         <is>
           <t>Same change adds has_species_stacking_synergy() text scan (attack/ability text referencing "for each &lt;name&gt; ... in play/on your Bench" with damage/retreat scaling, or delta-species-count text) - flips the -75/copy penalty to +75/copy when a synergy effect is detected on hand/bench/active.
 FIX PASS 2026-07-18: changed criterion_6_bench_duplicate (CPU_AI.gd) to award a FLAT +300 (instead of +75 per copy) whenever has_species_stacking_synergy() detects a field effect that benefits from stacking this species — so a stack-payoff Basic (e.g. a 3rd Magnemite) comfortably clears the bench-play thresholds (350 for a 3-Pokemon bench). Also added the candidate Pokemon itself to has_species_stacking_synergy's scan list so its OWN attack/ability text (and the Active's) is read, not just the Bench. Debug: 'ISSUE #2 FIX ACTIVE'.</t>
         </is>
       </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>Change the +75 PER card to instead be a flat +300 if any at all mataches and make sure it reads all the text of all the attacks and powers of the active pokemon too and not just bench. Magnemite should have been played on bench but wasn't . Had 2 magnemtites on bench but only had 270 score which was under the 350 required</t>
+        </is>
+      </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
-          <t>Change the +75 PER card to instead be a flat +300 if any at all mataches and make sure it reads all the text of all the attacks and powers of the active pokemon too and not just bench. Magnemite should have been played on bench but wasn't . Had 2 magnemtites on bench but only had 270 score which was under the 350 required</t>
-        </is>
-      </c>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H3" s="9" t="inlineStr">
+      <c r="G3" s="9" t="inlineStr">
         <is>
           <t>16/07/2026</t>
         </is>
       </c>
-      <c r="I3" s="6" t="n">
+      <c r="H3" s="6" t="n">
         <v>46220</v>
       </c>
     </row>
@@ -811,34 +808,33 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="C4" s="7" t="n"/>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>When returning to main UI from selecting cards for a card effect (E.g Blastoise Rain Dance), the player is no longer able to click anything. Presumably the main UI input blocker doesn't get rehidden. Same thing happens with card effects like Clefairie's Metronome. Once used the attacks of the opponent appears but player cannot click anything.</t>
+        </is>
+      </c>
       <c r="D4" s="8" t="inlineStr">
-        <is>
-          <t>When returning to main UI from selecting cards for a card effect (E.g Blastoise Rain Dance), the player is no longer able to click anything. Presumably the main UI input blocker doesn't get rehidden. Same thing happens with card effects like Clefairie's Metronome. Once used the attacks of the opponent appears but player cannot click anything.</t>
-        </is>
-      </c>
-      <c r="E4" s="9" t="inlineStr">
         <is>
           <t>Root cause: Card_Ops.gd prompt_select_card() unconditionally set main.opponent_blocker.visible = true when the selection UI closed. That blocker is only supposed to be visible during the opponent's turn (toggled by player_start_turn_checks/player_end_turn_checks). Using a power like Rain Dance or Metronome's attack-copy pool on the player's own turn opened this selection screen, and closing it force-reactivated the blocker even though it was still the player's turn, so no clicks registered afterward. Fixed prompt_select_card to remember the blocker's visibility before opening the selection UI and restore that value afterward instead of forcing it true.
 FOLLOW-UP: user reported the Metronome case still failed after the first fix. Found a second, separate blocker involved. perform_attack() sets opponent_blocker.visible = true the instant the player's attack is chosen (attacking always ends the turn, so input is meant to be blocked for the rest of the turn) - opponent_blocker is a FULL-SCREEN ColorRect with no cutout region. Metronome's attack-copy button list (choose_attack_from_pool in Attack_Effects.gd) only ever toggled buttons_only_blocker, which DOES carve out an exception for the button row - but opponent_blocker, already active from perform_attack, has no such exception and sat on top blocking the whole screen including those buttons. Rain Dance/other powers used outside of perform_attack never had this problem because opponent_blocker isn't forced on for those. Fixed choose_attack_from_pool to save/hide/restore opponent_blocker the same way prompt_select_card now does, so the attack-copy button list is actually clickable. Added print("ISSUE #3 FIX ACTIVE...") debug lines in both prompt_select_card and choose_attack_from_pool (and to every other fix in this log going forward) so the user can confirm from the Godot console output whether the running build actually has the fix, per new debug-message-on-every-fix requirement.</t>
         </is>
       </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>Fixed</t>
-        </is>
-      </c>
-      <c r="G4" s="8" t="inlineStr">
-        <is>
           <t>Issue Resolved</t>
         </is>
       </c>
-      <c r="H4" s="9" t="inlineStr">
+      <c r="G4" s="9" t="inlineStr">
         <is>
           <t>16/07/2026</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>16/07/2026</t>
         </is>
@@ -853,33 +849,32 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n"/>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Pressing the space bar to preview a card in deck view mode seems to accept the last button pressed so if you press empty deck, then press space over a card to preview it, the deck is emptied.</t>
+        </is>
+      </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>Pressing the space bar to preview a card in deck view mode seems to accept the last button pressed so if you press empty deck, then press space over a card to preview it, the deck is emptied.</t>
-        </is>
-      </c>
-      <c r="E5" s="9" t="inlineStr">
-        <is>
           <t>Root cause: Deck_Build_And_Card_View_Script.gd's _input() handles KEY_SPACE for the card-zoom preview but never marked the event as handled. Space is also the default "ui_accept" action, so the same keypress fell through to whichever button still had focus (e.g. "Empty Deck") and activated it too. Fixed by calling get_viewport().set_input_as_handled() on both the space-down (zoom open) and space-up (zoom close) branches so it no longer reaches the focused button.</t>
         </is>
       </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>Fixed</t>
-        </is>
-      </c>
-      <c r="G5" s="8" t="inlineStr">
-        <is>
           <t>Issue Resolved</t>
         </is>
       </c>
-      <c r="H5" s="9" t="inlineStr">
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>16/07/2026</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>16/07/2026</t>
         </is>
@@ -894,34 +889,33 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n"/>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>When a move like metronome is used which offers up more options, the game correctly puts a blocker to disable input on most of the screen, however the blocked doesn't quite cover the prize cards vertically so the player is still able to click under the blocker getting to prize cards where they aren't covered, opening the prize cards and cancelling the attack. Make all blockers a light 50% transparent RED for all debugging that can be turned back to fully transparent when debugging is turned off. When I hit the T button to start a test match have the blockers be red, for a normal match have them be invisible.</t>
+        </is>
+      </c>
       <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>When a move like metronome is used which offers up more options, the game correctly puts a blocker to disable input on most of the screen, however the blocked doesn't quite cover the prize cards vertically so the player is still able to click under the blocker getting to prize cards where they aren't covered, opening the prize cards and cancelling the attack. Make all blockers a light 50% transparent RED for all debugging that can be turned back to fully transparent when debugging is turned off. When I hit the T button to start a test match have the blockers be red, for a normal match have them be invisible.</t>
-        </is>
-      </c>
-      <c r="E6" s="9" t="inlineStr">
         <is>
           <t>Root cause: the blocker used during Metronome/copy-attack button selection (allow_buttons_only_blocker) intentionally excludes a bottom strip of the screen so the button row stays clickable, but that excluded strip (y:912-1080) was taller than it needed to be and also uncovered the prize-card icons (y:929-962), which sit in that same band. Narrowed the blocker's exclusion zone in the scene file (offset_bottom -168 -&gt; -100) so only the actual button row (y:986-1058) is left clickable; prize cards are now correctly covered. Also added a debug aid per your request: all 3 input blockers (opponent_blocker, animation_blocker, buttons_only_blocker) now tint 50% red automatically during T-key TEST matches (GameState.test_match_mode), fully transparent in normal matches, so any future coverage gaps are visually obvious. Watch console for 'ISSUE #5 FIX ACTIVE'.
 RETRY (pale red): the debug tint was Color(1, 0, 0, 0.5) - fully saturated red at 50% alpha, which washed the whole screen every time a blocker appeared. Changed to Color(1.0, 0.55, 0.55, 0.2) in Main_Match_Core_Gameplay_Script.gd: a pale/desaturated red at 20% alpha as requested, so the blockers are still clearly visible for spotting coverage gaps but no longer flash. Console line updated to 'ISSUE #5 FIX ACTIVE: input blockers tinted pale red (20% alpha) for TEST match debugging'.</t>
         </is>
       </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>Red is too dark and it's like a flashbang. Make it a much lighter paler red, setting the transparency to only 20% instead so it's still visible but less risk of epileptic seizure inducing flashes.</t>
+        </is>
+      </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>Red is too dark and it's like a flashbang. Make it a much lighter paler red, setting the transparency to only 20% instead so it's still visible but less risk of epileptic seizure inducing flashes.</t>
-        </is>
-      </c>
-      <c r="G6" s="8" t="inlineStr">
-        <is>
           <t>Issue Resolved</t>
         </is>
       </c>
-      <c r="H6" s="9" t="inlineStr">
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>16/07/2026</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>16/07/2026</t>
         </is>
@@ -936,35 +930,34 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n"/>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>When opponent attaches an energy to their bench pokemon, there is no await so the opponent does their next action and a message box appears before the energy attach animation plays.</t>
+        </is>
+      </c>
       <c r="D7" s="8" t="inlineStr">
-        <is>
-          <t>When opponent attaches an energy to their bench pokemon, there is no await so the opponent does their next action and a message box appears before the energy attach animation plays.</t>
-        </is>
-      </c>
-      <c r="E7" s="9" t="inlineStr">
         <is>
           <t>Both show_message and animate_card_a_to_b were already properly awaited here, so this wasn't a true race condition - the message box was just shown BEFORE the fly-to-bench animation instead of after, making it look like the opponent 'moved on' before the card visually arrived. Swapped the order: animation plays first, then the message confirms it. Watch console for 'ISSUE #6 FIX ACTIVE'.
 REVERTED as instructed and re-done to your ordering. CPU_AI.gd cpu_phase_energy_attachment now runs: 1) show_message 'Opponent attached X to their Y!' (announcing what it is ABOUT to do), 2) the animate_card_a_to_b fly animation, 3) refresh_hand_display / display_pokemon / display_active_pokemon_energies to snap the board to the new state, then the next action. This matches the evolve flow. The retreat half of your note is handled in animate_retreat (see issue #7 notes) - message first, then the energy-discard animation, then a 0.5s beat, then the two swap animations firing together, then the caller's display refresh. Watch console for 'ISSUE #6 FIX ACTIVE'.</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>Revert this. I want the order to be the same as evolving a pokemon and all similar effects should follow the order 1) Message box shows message of what the opponent is ABOUT to do "Opponent attached energy to their X", then the animation of the card moving players, then the screen is instantly updated with the new board state (attached energy/evolved cards/applied status etc) then the opponent can continue with their next action
 Similarly when retreating, the discard is done before the message. Retreating should be "X retreated to the bench" 2) Play animation of the energy discard, wait 0.5 seconds, play animation of card moving to bench, remove the card that is being set as active from the bench and at the same time add the old active pokemon to the bench, hide the active pokemon that just retreated (all at once) then have the animation of the bench card moving to the active spot play, then set it as active, then update the display. then continue. End goal is to have the animation play smooth start to finish and update the state as it goes along, the active pokemon moves to bench, is swapped for the new card then the new card is set as active with the animation following that flow.</t>
         </is>
       </c>
-      <c r="G7" s="8" t="inlineStr">
+      <c r="F7" s="8" t="inlineStr">
         <is>
           <t>Issue Resolved</t>
         </is>
       </c>
-      <c r="H7" s="9" t="inlineStr">
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>16/07/2026</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>16/07/2026</t>
         </is>
@@ -979,13 +972,12 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n"/>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>When using Whirlwind or related effects like retreating, swapping out pokemon with the bench etc, there is no swap in message so you get "Clefairy Retreated to bench" but not "Opponent set X as their active Pokemon"</t>
+        </is>
+      </c>
       <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>When using Whirlwind or related effects like retreating, swapping out pokemon with the bench etc, there is no swap in message so you get "Clefairy Retreated to bench" but not "Opponent set X as their active Pokemon"</t>
-        </is>
-      </c>
-      <c r="E8" s="9" t="inlineStr">
         <is>
           <t>animate_retreat() (the single shared function used by every retreat/Whirlwind/Teleport/forced-switch effect in the game) only ever showed 'X RETREATED TO THE BENCH!' and never announced the replacement. Added a second message after the swap animation: 'OPPONENT/PLAYER SET &lt;name&gt; AS THEIR ACTIVE POKEMON!'. Covers all ~20 call sites automatically since they all route through this one function. Watch console for 'ISSUE #7 FIX ACTIVE'.
 FOLLOW-UP: reworked the ordering rather than adding another message. animate_retreat() now takes an is_forced_switch flag (default false). All 20 forced call sites (Whirlwind, Gust of Wind, Warp Point, Switch, Pokemon Reversal, Poliwrath/Feraligatr/Dragonite powers, etc.) pass true; only the two genuine voluntary retreats (CPU_AI.gd:1336 and the player's retreat button) leave it false. Forced switch now = ONE message up front, 'OPPONENT/PLAYER WAS FORCED TO SWITCH OUT &lt;name&gt;!', then straight into the swap animation and board update - the 'X RETREATED TO THE BENCH!' and '...SET X AS THEIR ACTIVE POKEMON!' pair are both suppressed. Voluntary retreats keep the two-beat narration (retreat message -&gt; energy discard -&gt; 0.5s -&gt; swap animation -&gt; set-active message). Callers keep their own flavour lines (e.g. 'HEADS! X SWITCHED IN!'). Watch console for 'ISSUE #6/#7 FIX ACTIVE'.
@@ -993,17 +985,17 @@
 FIX PASS 2026-07-21 (ISSUE #7 regular retreat): the voluntary branch of animate_retreat (Main_Match_Core) now plays the SAME sequential glide as a forced switch — 'X RETREATED TO THE BENCH!' first, then hide Active, glide outgoing card down to Bench, apply swap + refresh board (Active pointer set here since the player caller only reassigns it after the call — its post-retreat cleanup switched to the saved old-active ref), glide incoming card up into Active, reveal, then the closing 'SET X AS THEIR ACTIVE POKEMON!' at the end. Cards no longer fly simultaneously. Debug: 'ISSUE #7 FIX ACTIVE (voluntary sequential)'.</t>
         </is>
       </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Force switching now works perfectly. Using gust of wind all the animations played in the correct order and the field was updated. However make this the same for a regular retreat now as this doesn't quite have the animation fixes we need. Regular retreat does the swap at the same time so follow the forced switch code but have the message instead of being the "X was forced to switch out" have it be "X retreated to bench" &gt; on click of message confirmation have the animation play of it going to the bench, the next pokemon coming in then when the next pokemon is active have the message "X Was placed as their active pokemon". This is the only exception to the rule of always showing the message first for the action about to take place, then playing the animation/updating the board, as of course for this we have the animation play fully then have a message at the end for "X was set as their active pokemon". Check last issue in this log for note on adding 0.5s timer to end of message</t>
+        </is>
+      </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>Force switching now works perfectly. Using gust of wind all the animations played in the correct order and the field was updated. However make this the same for a regular retreat now as this doesn't quite have the animation fixes we need. Regular retreat does the swap at the same time so follow the forced switch code but have the message instead of being the "X was forced to switch out" have it be "X retreated to bench" &gt; on click of message confirmation have the animation play of it going to the bench, the next pokemon coming in then when the next pokemon is active have the message "X Was placed as their active pokemon". This is the only exception to the rule of always showing the message first for the action about to take place, then playing the animation/updating the board, as of course for this we have the animation play fully then have a message at the end for "X was set as their active pokemon". Check last issue in this log for note on adding 0.5s timer to end of message</t>
-        </is>
-      </c>
-      <c r="G8" s="8" t="inlineStr">
-        <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H8" s="9" t="inlineStr">
+      <c r="G8" s="9" t="inlineStr">
         <is>
           <t>16/07/2026</t>
         </is>
@@ -1018,33 +1010,32 @@
           <t>CPU logic</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n"/>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>When retreating, the opponent will still retreat a pokemon that is guarenteed to be knocked out with another pokemon that is guarenteed to be knocked out, wasting an energy to retreat. Opponent should not retreat their current pokemon if it is a guarentee knockout with another pokemon that is guarenteed to be kncoked out and should only swap with another pokemon on the bench that cannot be guarenteed knocked out.</t>
+        </is>
+      </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>When retreating, the opponent will still retreat a pokemon that is guarenteed to be knocked out with another pokemon that is guarenteed to be knocked out, wasting an energy to retreat. Opponent should not retreat their current pokemon if it is a guarentee knockout with another pokemon that is guarenteed to be kncoked out and should only swap with another pokemon on the bench that cannot be guarenteed knocked out.</t>
-        </is>
-      </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
           <t>Confirmed and fixed. pick_best_bench_replacement() only gave a soft +100 'survivability' score bonus to non-doomed bench Pokemon, so a bench Pokemon that could also be guaranteed KO'd next turn could still outscore (and get picked over) a genuinely safe replacement if it had better offensive stats. Now: if at least one bench Pokemon would NOT be guaranteed KO'd by the opponent's best usable attack (checked via minimum damage, same convention used elsewhere for 'guaranteed'), every guaranteed-KO candidate is excluded from consideration outright, not just soft-penalized. Watch console for 'ISSUE #8 FIX ACTIVE'.</t>
         </is>
       </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>Fixed</t>
-        </is>
-      </c>
-      <c r="G9" s="8" t="inlineStr">
-        <is>
           <t>Issue Resolved</t>
         </is>
       </c>
-      <c r="H9" s="9" t="inlineStr">
+      <c r="G9" s="9" t="inlineStr">
         <is>
           <t>16/07/2026</t>
         </is>
       </c>
-      <c r="I9" s="6" t="n">
+      <c r="H9" s="6" t="n">
         <v>46220</v>
       </c>
     </row>
@@ -1057,34 +1048,33 @@
           <t>CPU logic</t>
         </is>
       </c>
-      <c r="C10" s="7" t="n"/>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>If a Pokemon can use metronome (or a similar move) the moves it can copy should be added to their priotiy check. E.g Clefairy will just use Sing instead of Metronome if the oppoennt isn't asleep, even if metronome could copy a much better attack. In fact, metronome appears to always score never, opponent used sing again even though active player pokemon was already asleep</t>
+        </is>
+      </c>
       <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>If a Pokemon can use metronome (or a similar move) the moves it can copy should be added to their priotiy check. E.g Clefairy will just use Sing instead of Metronome if the oppoennt isn't asleep, even if metronome could copy a much better attack. In fact, metronome appears to always score never, opponent used sing again even though active player pokemon was already asleep</t>
-        </is>
-      </c>
-      <c r="E10" s="9" t="inlineStr">
         <is>
           <t>Confirmed and fixed (same root cause as Base1 base1-5 Clefairy). Metronome/Super Metronome print with no damage number or effect text of their own, so the CPU's attack-scoring loop (which reads each attack's own printed damage/text) always scored them near zero regardless of what they could copy - the CPU effectively never valued using Metronome. Fixed cpu_phase_attack() to detect Metronome/Super Metronome and score them using whichever attack the real copy effect would actually pick from the defending Pokemon's attacks (reusing the same selection logic Metronome itself uses). Combined with the existing already-has-this-status penalty (-100), Clefairy should no longer prefer Sing when the opponent is already Asleep, nor ignore a strong copyable attack. Watch console for 'ISSUE #9 FIX ACTIVE'.
 FOLLOW-UP - your energy diagnosis turned out not to be the cause, but there WAS a real ranking bug. Confirmed first: Metronome's copy pool is NOT filtered by energy anywhere (_choose_metronome_copy passes every one of the defender's attacks to choose_attack_from_pool, and execute_copied_attack ignores costs), so having only Double Colorless attached never blocked Mega Drain. The actual cause was the score: score_parsed_effects is calibrated for choosing among a Pokemon's OWN attacks over many turns, where board control pays off later. Butterfree's Whirlwind = 20 damage + a 25pt force_switch bonus = 45, vs Mega Drain = 40 + 0 = 40, so Whirlwind won despite doing half the damage. Fixed _choose_metronome_copy's cpu_rank to (a) weight actual damage 1.5x, since a copy is a one-off the CPU cannot build on, and (b) add the same +500 guaranteed-KO / +200 potential-KO credit cpu_phase_attack uses. Mega Drain now scores 60 vs Whirlwind 55. Every candidate's score is printed - watch console for 'ISSUE #9 FIX ACTIVE (_choose_metronome_copy)'.</t>
         </is>
       </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Check priority works on being able to use any attack with no energy requirements when copying opponents. Clefairy just used metronome correctly but copied Butterfree's whirlwhind, not Mega drain because it had only double colorless energy attached to itself</t>
+        </is>
+      </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>Check priority works on being able to use any attack with no energy requirements when copying opponents. Clefairy just used metronome correctly but copied Butterfree's whirlwhind, not Mega drain because it had only double colorless energy attached to itself</t>
-        </is>
-      </c>
-      <c r="G10" s="8" t="inlineStr">
-        <is>
           <t>Issue Resolved</t>
         </is>
       </c>
-      <c r="H10" s="9" t="inlineStr">
+      <c r="G10" s="9" t="inlineStr">
         <is>
           <t>16/07/2026</t>
         </is>
       </c>
-      <c r="I10" s="6" t="n">
+      <c r="H10" s="6" t="n">
         <v>46220</v>
       </c>
     </row>
@@ -1097,33 +1087,32 @@
           <t>Animation</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n"/>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>When drawing multiple cards at once (e.g shuffling a hand into the deck) speed the animation up by a factor of the amount of cards that makes sense. E.g if the draw animation from player's deck to hand is 0.5 seconds, keep that for 1 card, but for 2 cards make each draw take 0.4 seconds instead, for 3 cards set each draw to be 0.3 seconds, 4 cards 0.25s, 5 cards 0.22s 6 cards 0.2s, 7+cards 0.15s each</t>
+        </is>
+      </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>When drawing multiple cards at once (e.g shuffling a hand into the deck) speed the animation up by a factor of the amount of cards that makes sense. E.g if the draw animation from player's deck to hand is 0.5 seconds, keep that for 1 card, but for 2 cards make each draw take 0.4 seconds instead, for 3 cards set each draw to be 0.3 seconds, 4 cards 0.25s, 5 cards 0.22s 6 cards 0.2s, 7+cards 0.15s each</t>
-        </is>
-      </c>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
           <t>Added draw_animation_speed_multiplier(count) in Main_Match_Core_Gameplay_Script.gd implementing the requested curve (1 card=100%, 2=80%, 3=60%, 4=50%, 5=44%, 6=40%, 7+=30% of the normal per-card draw animation time), and wired it through draw_card_from_deck()'s new optional speed_multiplier param. Card_Ops.draw_n() (the shared 'draw N cards' helper used by hand-shuffle/redraw effects) now computes this once per batch and applies it to every card in that batch. Single draws (turn-start draw, etc.) are unaffected. Watch console for 'ISSUE #10 FIX ACTIVE'.</t>
         </is>
       </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>Fixed</t>
-        </is>
-      </c>
-      <c r="G11" s="8" t="inlineStr">
-        <is>
           <t>Issue Resolved</t>
         </is>
       </c>
-      <c r="H11" s="9" t="inlineStr">
+      <c r="G11" s="9" t="inlineStr">
         <is>
           <t>16/07/2026</t>
         </is>
       </c>
-      <c r="I11" s="6" t="n">
+      <c r="H11" s="6" t="n">
         <v>46220</v>
       </c>
     </row>
@@ -1136,42 +1125,40 @@
           <t>CPU logic</t>
         </is>
       </c>
-      <c r="C12" s="7" t="n"/>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Damage swap seems to never activate. Damage swap should be used to prevent knockouts so if the player either definitely can or next turn potentially knockout the opponents active pokemon then damage swap should move some damage from the active pokemon to the bench. Similarly if the player can damage the opponent's bench with an attack and a bench pokemon may be knocked out by it, damage swap should try and move damage counters from that bench pokemon to another </t>
+        </is>
+      </c>
       <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Damage swap seems to never activate. Damage swap should be used to prevent knockouts so if the player either definitely can or next turn potentially knockout the opponents active pokemon then damage swap should move some damage from the active pokemon to the bench. Similarly if the player can damage the opponent's bench with an attack and a bench pokemon may be knocked out by it, damage swap should try and move damage counters from that bench pokemon to another </t>
-        </is>
-      </c>
-      <c r="E12" s="9" t="inlineStr">
         <is>
           <t>CPU_AI.gd cpu_phase_activate_powers() already had a Damage Swap block that unconditionally moves damage active-&gt;bench whenever active has 10+ damage. Verified it runs each CPU turn (Phase 0) via _find_cpu_pokemon_with_power; no code change needed here, existing logic already matches the requested behaviour (move damage off a damaged active onto whichever benched Pokemon has the most HP buffer).
 FOLLOW-UP - previous pass wrongly concluded 'no code change needed'. Rewrote the CPU Damage Swap block (Powers_And_Bodies_Effects.gd) into a new cpu_damage_swap() + helpers. Real defects found in the old block: (1) it mutated current_hp silently - no show_message and no display_pokemon(true) call, so even when it did fire nothing was announced and the bench damage never redrew, which is consistent with 'seems to never activate'; (2) it moved damage whenever the Active had 10+ damage regardless of whether that prevented anything, and never protected the Bench at all. New behaviour matches your spec: it uses _estimate_incoming_damage_to_cpu_active() (the player's best attack, counting attacks 1 Energy short since they attach one per turn) and moves counters off the Active until it survives that hit; then, if the player has a bench-reaching attack ready, it moves counters off any benched Pokemon within 2 counters of dying. Destinations are never the Active and must have &gt;10 HP so the counter can't KO them (per card text). Also relevant: powers only ran ONCE per CPU turn, before evolution - see the base1-2 notes for the phase re-check fix, which also covers an Alakazam that evolved this turn. Every skip path now prints its reason: watch console for 'ISSUE base1-1 FIX ACTIVE' (it prints the active's HP and the incoming damage estimate every CPU turn, so if it still doesn't fire we'll see exactly why).</t>
         </is>
       </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Alakazam still doesn't seem to use damage swap at all by the opponent.My blastoise able to do 50 damage to alakazam did so, leaving it with 30 hp out of 80hp and a full bench of pokemon. Alakazam was both the active pokemon and opponent had one on bench and neither used damage swap to pull counters off alakazam to the bench</t>
+        </is>
+      </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>Alakazam still doesn't seem to use damage swap at all by the opponent.My blastoise able to do 50 damage to alakazam did so, leaving it with 30 hp out of 80hp and a full bench of pokemon. Alakazam was both the active pokemon and opponent had one on bench and neither used damage swap to pull counters off alakazam to the bench</t>
-        </is>
-      </c>
-      <c r="G12" s="8" t="inlineStr">
-        <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H12" s="9" t="n"/>
+      <c r="G12" s="9" t="n"/>
     </row>
     <row r="13" ht="101.45" customHeight="1">
       <c r="A13" s="7" t="n">
         <v>12</v>
       </c>
       <c r="B13" s="7" t="n"/>
-      <c r="C13" s="7" t="n"/>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Rain dance needs to activate more often. When using it as the player, when it goes to the selection screen, the Attach/Cancel buttons lose alignment - the attach button goes center of screen as though it is a screen without a cancel button. When returning by pressing cancel, the player never gains the ability to click anything (assuming cancel button doesn't hide the input blocker)</t>
+        </is>
+      </c>
       <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>Rain dance needs to activate more often. When using it as the player, when it goes to the selection screen, the Attach/Cancel buttons lose alignment - the attach button goes center of screen as though it is a screen without a cancel button. When returning by pressing cancel, the player never gains the ability to click anything (assuming cancel button doesn't hide the input blocker)</t>
-        </is>
-      </c>
-      <c r="E13" s="9" t="inlineStr">
         <is>
           <t>Root cause of the button misalignment: Card_Ops.gd prompt_select_card() set cancel_button.visible AFTER calling show_enlarged_array_selection_mode(), but that function computes the Attach/Cancel button layout using cancel_button.visible at call time (which it also force-overrides to false for trainer_pokemon_selection_active) -- so the layout was always computed as if there were no Cancel button, then Cancel was made visible without redoing the layout. Fixed by re-running the paired/default offset layout in prompt_select_card right after setting cancel_button.visible = cancelable. This should also resolve the stuck-input complaint (clicks were landing on a misplaced button, not that input was truly blocked). Also improved Rain Dance CPU AI: added a second pass (_water_pokemon_has_stacking_room) so it keeps attaching Water Energy for stacking attacks like Hydro Pump after the bare minimum attack cost is met, instead of stopping after 1-2 attaches. Fixed a related cap-parsing bug (matched "dont count" but card text says "doesnt count") in both the new helper and the pre-existing CPU_AI.gd copy.
 Found the real cause of both remaining complaints. The damage-cap parser in Attack_Effects.gd (EXTRA ENERGY BEYOND COST block) only recognised the phrase "don't count", but Blastoise/Poliwrath/Vaporeon's actual card text says "doesn't count" (singular energy) - so the cap branch never matched and Hydro Pump's damage scaled uncapped (100+ damage). Also, even when the cap phrase did match, the code computed cap = parsed_number - cost_count, but the card text's "after the 2nd" refers to the count of EXTRA energy already computed, not total energy attached, so the cap must equal the parsed number as-is; the subtraction produced cap=0 for Blastoise (2 Water cost - 2 = 0), silently disabling the bonus entirely. Same bug (same-cap-math) existed in Powers_And_Bodies_Effects.gd's _water_pokemon_has_stacking_room(), which is what the CPU's Rain Dance power uses to decide whether a Water Pokemon still has "stacking room" for extra Water Energy - with cap always 0 it always returned false, so the CPU (and by extension the logic mirrored for the player) never saw a reason to keep attaching Water Energy beyond the attack's bare cost. Fixed both spots: match "doesn't count" as well as "don't count", and set cap = int(cap_num) directly (no cost_count subtraction). Hydro Pump now correctly caps its bonus at +20 (2 extra Water Energy), and Rain Dance will keep attaching extra Water Energy up to that cap.
@@ -1182,17 +1169,17 @@
 FIX PASS 2026-07-18: root cause was that the CPU Rain Dance loop only called display_active_pokemon_energies() (which refreshes the ACTIVE's energies), so energy attached to a BENCH Water Pokemon never appeared -&gt; 'board never refreshed between uses'. Added _cpu_rain_dance_attach() (Powers_And_Bodies_Effects.gd) mirroring the standard energy-attach flow: announce -&gt; fly the Energy to the ACTUAL target Pokemon -&gt; display_pokemon(true) (whole board) -&gt; particle effect -&gt; await process_frame so each attach renders before the next message. Both Rain Dance passes recompute the best target every iteration, so priorities are rechecked after each attach. Debug: 'ISSUE #12 FIX ACTIVE'.</t>
         </is>
       </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Play the adding water animation and board refresh after each time opponent uses rain dance. Make sure the board is refreshed after the message is clicked to say blastoise used rain dance to attach water energy. THen popup the message only after. may need an await or process frame as this is still failing. Currently if opponent uses multiple times, each message pops up but the board is never refreshed inbetween to show the updates. ALSO just make sure the opponent rechecks the board status to prioritse any additional water attachments, it's possible it currently only does priority checking first then attaches multiple energy to one pokemon where it should recheck priorities after </t>
+        </is>
+      </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Play the adding water animation and board refresh after each time opponent uses rain dance. Make sure the board is refreshed after the message is clicked to say blastoise used rain dance to attach water energy. THen popup the message only after. may need an await or process frame as this is still failing. Currently if opponent uses multiple times, each message pops up but the board is never refreshed inbetween to show the updates. ALSO just make sure the opponent rechecks the board status to prioritse any additional water attachments, it's possible it currently only does priority checking first then attaches multiple energy to one pokemon where it should recheck priorities after </t>
-        </is>
-      </c>
-      <c r="G13" s="8" t="inlineStr">
-        <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H13" s="9" t="inlineStr">
+      <c r="G13" s="9" t="inlineStr">
         <is>
           <t>18/07/2026</t>
         </is>
@@ -1203,53 +1190,54 @@
         <v>13</v>
       </c>
       <c r="B14" s="7" t="n"/>
-      <c r="C14" s="7" t="n"/>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>Current always uses recover if it can. Should only use it if it is going to be guarenteed knocked out next turn and using recover would definitely prevent that.
 Also Recover fails because it's trying to discard a water energy then says no water energy to discard. Probably routing issue with Starmie's Recover.</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>Found the real bug: the Recover attack dispatch (Attack_Effects.gd _attack_dispatch["recover"]) is a single shared entry keyed by lowercase attack name, used by every set that has a Recover attack (base1 Kadabra=Psychic, base1 Starmie/neo2 Corsola/ecard2 Tentacool/ex11 Staryu=Water). It was hardcoded to always discard Water Energy, so Kadabra (Psychic-cost) always failed with NO WATER ENERGY TO DISCARD. Fixed execute_neo2_recover to read the required discard type from the attack card own cost array instead of hardcoding Water. Separately, CPU_AI.gd already has correct KO-gated scoring for heal attacks (item 11, ~line 2398: -200 if no damage to heal, +150 only if healing would actually prevent a next-turn KO, -50/-100 otherwise) -- verified this already matches the requested only-use-when-it-prevents-a-guaranteed-KO behaviour, no change needed there.</t>
         </is>
       </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>Checking</t>
+        </is>
+      </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>Checking</t>
-        </is>
-      </c>
-      <c r="G14" s="8" t="inlineStr">
-        <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H14" s="9" t="n"/>
+      <c r="G14" s="9" t="n"/>
     </row>
     <row r="15" ht="29.1" customHeight="1">
       <c r="A15" s="7" t="n">
         <v>14</v>
       </c>
       <c r="B15" s="7" t="n"/>
-      <c r="C15" s="7" t="n"/>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For moves like whirlwind that show an array as part of the attack (e.g the bench showing to select a card) have a 1second delay below showing the array after showing the damage label first, so the damage is shown and floats upwards, then the effect of the card kicks in 1 second after the label is shown </t>
+        </is>
+      </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">For moves like whirlwind that show an array as part of the attack (e.g the bench showing to select a card) have a 1second delay below showing the array after showing the damage label first, so the damage is shown and floats upwards, then the effect of the card kicks in 1 second after the label is shown </t>
-        </is>
-      </c>
-      <c r="E15" s="9" t="inlineStr">
-        <is>
           <t>Added a 1-second delay (await get_tree().create_timer(1.0).timeout) in Attack_Effects.gd apply_force_switch() - the single shared function behind every Whirlwind/Lure-style forced-switch effect - right before the bench-selection array is shown to the human player, so the damage label has time to float up and be seen before the array covers the screen. Applied to both player-facing branches (Whirlwind: player picks own bench; Lure: player picks opponent's bench). Watch console for 'ISSUE base2-33 FIX ACTIVE'.</t>
         </is>
       </c>
-      <c r="F15" s="8" t="n"/>
-      <c r="G15" s="8" t="inlineStr">
+      <c r="E15" s="8" t="n"/>
+      <c r="F15" s="8" t="inlineStr">
         <is>
           <t>Issue Resolved</t>
         </is>
       </c>
-      <c r="H15" s="9" t="n"/>
+      <c r="G15" s="9" t="n"/>
+      <c r="H15" s="6" t="n">
+        <v>46223</v>
+      </c>
     </row>
     <row r="16" ht="43.5" customHeight="1">
       <c r="A16" s="7" t="n">
@@ -1260,28 +1248,27 @@
           <t>CPU logic</t>
         </is>
       </c>
-      <c r="C16" s="7" t="n"/>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Inlclude the extra bit of poison damage in scoring. Check if the opponent has any active effects that would prevent getting the poison status and if not then add +10 to the damage when calculating an effect with guarenteed posions. E.g if a card does 0 damage but always posions without a heads flip, if the opponent isn't already poisoned and cannot prevent poison in any way, then that damage is realistically a minimum of 10</t>
+        </is>
+      </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>Inlclude the extra bit of poison damage in scoring. Check if the opponent has any active effects that would prevent getting the poison status and if not then add +10 to the damage when calculating an effect with guarenteed posions. E.g if a card does 0 damage but always posions without a heads flip, if the opponent isn't already poisoned and cannot prevent poison in any way, then that damage is realistically a minimum of 10</t>
-        </is>
-      </c>
-      <c r="E16" s="9" t="inlineStr">
-        <is>
           <t>Added a guaranteed_poison_bonus of +10 in cpu_phase_attack()'s scoring when an attack inflicts Poison with no coin-flip gate (flip='none'), the defender isn't already poisoned, and the defender has no textual poison immunity (new _defender_prevents_poison() helper, scans ability text for phrasing like "can't be poisoned"). This +10 now feeds into both the guaranteed/potential-KO checks and the base damage score, so a 0-damage-but-always-poisons attack is no longer scored as literally zero damage. Watch console for 'ISSUE #11 FIX ACTIVE'.</t>
         </is>
       </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>Checking</t>
+        </is>
+      </c>
       <c r="F16" s="8" t="inlineStr">
         <is>
-          <t>Checking</t>
-        </is>
-      </c>
-      <c r="G16" s="8" t="inlineStr">
-        <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H16" s="9" t="inlineStr">
+      <c r="G16" s="9" t="inlineStr">
         <is>
           <t>16/07/2026</t>
         </is>
@@ -1296,33 +1283,32 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="C17" s="7" t="n"/>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>When showing another array over the main UI, when clicking where the prize cards are shown, the click is eaten by that function even though nothing happens instead of the card in the array. E.g when using whirlwind and all bench pokemon are shown, if there are 4 bench pokemon, the first and last card in that array has a dead zone where it cannot be clicked in where the prize cards array overlaps it.</t>
+        </is>
+      </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>When showing another array over the main UI, when clicking where the prize cards are shown, the click is eaten by that function even though nothing happens instead of the card in the array. E.g when using whirlwind and all bench pokemon are shown, if there are 4 bench pokemon, the first and last card in that array has a dead zone where it cannot be clicked in where the prize cards array overlaps it.</t>
-        </is>
-      </c>
-      <c r="E17" s="9" t="inlineStr">
-        <is>
           <t>Root cause: Card_Image_Loader_Script.gd's per-card _input() handler only checked whether its DIRECT parent container was visible before processing a click - but Node._input() fires for every node regardless of visibility, and a card whose GRANDparent (not direct parent) was hidden (or whose direct parent was visible while an ancestor further up wasn't) could still pass that check and silently swallow the click with a stale card_ref, while the real card in the newly-shown array (e.g. Whirlwind's bench-selection array) sitting at that same screen position never got the event. Fixed to check is_visible_in_tree() (walks the whole ancestor chain) instead of just the immediate parent. Watch console for 'ISSUE #12 FIX ACTIVE'.</t>
         </is>
       </c>
-      <c r="F17" s="8" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>Issue Resolved</t>
+        </is>
+      </c>
       <c r="G17" s="9" t="inlineStr">
         <is>
-          <t>Issue Resolved</t>
-        </is>
-      </c>
-      <c r="H17" s="9" t="inlineStr">
-        <is>
           <t>16/07/2026</t>
         </is>
       </c>
-      <c r="I17" s="6" t="n">
+      <c r="H17" s="6" t="n">
         <v>46220</v>
       </c>
     </row>
@@ -1335,33 +1321,32 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="C18" s="7" t="n"/>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Pressing space bar to preview a card in deck saves the card as a cached variable so when spacebar is pressed again but not hovering over any card, the preview is saved of that card. Redesign the preview system to check if the space bar is pressed every several frames and show the preview of the card the player is hovered over at that time. Therefore the player can move their mouse in the background which updates the preview to the new card the mouse is slid over in teh bacckground allowing the mode to be kept shown preview while the player uses their mouse to change the card. this will also solve the issue when hovering not over a card no card preview is shown and prevents caching issues if moving between sets or menus</t>
+        </is>
+      </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>Pressing space bar to preview a card in deck saves the card as a cached variable so when spacebar is pressed again but not hovering over any card, the preview is saved of that card. Redesign the preview system to check if the space bar is pressed every several frames and show the preview of the card the player is hovered over at that time. Therefore the player can move their mouse in the background which updates the preview to the new card the mouse is slid over in teh bacckground allowing the mode to be kept shown preview while the player uses their mouse to change the card. this will also solve the issue when hovering not over a card no card preview is shown and prevents caching issues if moving between sets or menus</t>
-        </is>
-      </c>
-      <c r="E18" s="9" t="inlineStr">
-        <is>
           <t>Redesigned exactly as described. Deck_Build_And_Card_View_Script.gd no longer snapshots the card on key-down: a new space_held flag plus _process() re-read the hovered card every frame while Space is held, via _refresh_hover_preview(), which swaps the overlay when the hover moves to a different card and hides it entirely when the mouse is over nothing. So you can hold Space and slide the mouse to flick through cards, and hovering empty space shows nothing instead of a stale card. Deleted the last_zoomed_card cache that caused the cross-set/cross-menu staleness. Two supporting fixes were needed: the zoom overlay's backdrop and card image are now MOUSE_FILTER_IGNORE (otherwise the overlay absorbed hover, gui_get_hovered_control() returned the backdrop, and the preview would flicker off instantly), and the Escape handler clears space_held so _process can't immediately reopen the preview. Watch console for 'ISSUE #13 FIX ACTIVE'.</t>
         </is>
       </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>Fixed</t>
-        </is>
-      </c>
-      <c r="G18" s="8" t="inlineStr">
-        <is>
           <t>Issue Resolved</t>
         </is>
       </c>
-      <c r="H18" s="9" t="inlineStr">
+      <c r="G18" s="9" t="inlineStr">
         <is>
           <t>16/07/2026</t>
         </is>
       </c>
-      <c r="I18" s="6" t="n">
+      <c r="H18" s="6" t="n">
         <v>46220</v>
       </c>
     </row>
@@ -1374,28 +1359,27 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="C19" s="7" t="n"/>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For all attacks like Metronome or Mimic that copies an opponents attack, prevent that from being copied by the copying move. E.g if clefairy is against clefairy and you can use metronome, simply hide the opponents Metronome attack entirely so it can't be clicked and cause a loopback. </t>
+        </is>
+      </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">For all attacks like Metronome or Mimic that copies an opponents attack, prevent that from being copied by the copying move. E.g if clefairy is against clefairy and you can use metronome, simply hide the opponents Metronome attack entirely so it can't be clicked and cause a loopback. </t>
-        </is>
-      </c>
-      <c r="E19" s="9" t="inlineStr">
-        <is>
           <t>Done at the shared chokepoint. Added COPY_ATTACK_NAMES + is_copy_attack() to Attack_Effects.gd and a filter inside choose_attack_from_pool() - the one function every copy effect routes through (Metronome, Super Metronome, mini-metronome, Copy, Mirror Move, ESP, Random ESP, Skill Copy, Delta Copy, Mimicry, Skill Hack, Genetic Memory, Dark Link, Rainbow Moves, and the Psymimic power). Copy attacks are now removed from the pool entirely, so in a Clefairy mirror match the opponent's Metronome is never shown as a button and can't be clicked into a loopback; the CPU can't pick one either. ex11 Drowzee's Disable passes exclude_copy_attacks=false since disabling an opponent's Metronome is a legitimate (and good) choice, not a copy. Watch console for 'ISSUE #14 FIX ACTIVE'.</t>
         </is>
       </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>Checking</t>
+        </is>
+      </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>Checking</t>
-        </is>
-      </c>
-      <c r="G19" s="8" t="inlineStr">
-        <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H19" s="9" t="inlineStr">
+      <c r="G19" s="9" t="inlineStr">
         <is>
           <t>16/07/2026</t>
         </is>
@@ -1410,27 +1394,26 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="C20" s="7" t="n"/>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Remove the pop up messages from the cheat keys for drawing, healing, shuffling and attaching energy. Just do the action so the messagebox doesn't slow down debugging</t>
+        </is>
+      </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>Remove the pop up messages from the cheat keys for drawing, healing, shuffling and attaching energy. Just do the action so the messagebox doesn't slow down debugging</t>
-        </is>
-      </c>
-      <c r="E20" s="9" t="inlineStr">
-        <is>
           <t>FIX 2026-07-18: removed the show_message pop-ups from the debug cheat keys in Main_Match_Core_Gameplay_Script.gd (debug_key_both_draw / _both_shuffle_hand / _both_attach_energy / _heal_actives / _heal_bench) so the action just happens with a console print instead. Debug: 'ISSUE #19 FIX ACTIVE'.</t>
         </is>
       </c>
-      <c r="F20" s="8" t="n"/>
-      <c r="G20" s="8" t="inlineStr">
+      <c r="E20" s="8" t="n"/>
+      <c r="F20" s="8" t="inlineStr">
         <is>
           <t>Issue Resolved</t>
         </is>
       </c>
-      <c r="H20" s="10" t="n">
+      <c r="G20" s="10" t="n">
         <v>46221</v>
       </c>
-      <c r="I20" s="6" t="n">
+      <c r="H20" s="6" t="n">
         <v>46224</v>
       </c>
     </row>
@@ -1443,29 +1426,24 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="C21" s="7" t="n"/>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Currently all animations for card moving (evolve, energy attachment, placing on bench, placing as active pokemon) go to the centre of the parent object instead of the actual location of where the card is going to be. Update the animate card from a to b function to find the new position and size of which the moving card is going to be and animate the tween to go from it's current position and size to it's new position and size. Card sizes are different depending where the card is (e.g active pokemon is way bigger than hand cards, which are smaller than bench cards.) With these changes increase the tween speed by 50% (if it's 0.5s now set to 0.75s) End goal, I want the card to smoothly transition from one location to another as currently it doesn't quite go to the correct spot and then jumps in size when the board refreshes.</t>
+        </is>
+      </c>
       <c r="D21" s="8" t="inlineStr">
-        <is>
-          <t>Currently all animations for card moving (evolve, energy attachment, placing on bench, placing as active pokemon) go to the centre of the parent object instead of the actual location of where the card is going to be. Update the animate card from a to b function to find the new position and size of which the moving card is going to be and animate the tween to go from it's current position and size to it's new position and size. Card sizes are different depending where the card is (e.g active pokemon is way bigger than hand cards, which are smaller than bench cards.) With these changes increase the tween speed by 50% (if it's 0.5s now set to 0.75s) End goal, I want the card to smoothly transition from one location to another as currently it doesn't quite go to the correct spot and then jumps in size when the board refreshes.</t>
-        </is>
-      </c>
-      <c r="E21" s="9" t="inlineStr">
         <is>
           <t>FIX 2026-07-18: extended animate_card_a_to_b (Main_Match_Core_Gameplay_Script.gd) with two backward-compatible optional params — target_size (morphs the card's size mid-flight) and target_pos_override (exact destination slot) — and lengthened the tween by 50% (0.3s-&gt;0.45s). Wired the key placements to pass real slot data via get_pokemon_screen_location(): player+CPU bench placement, bench-&gt;Active promotion (grows to Active size), evolve, and Energy attachment now fly to the ACTUAL benched Pokemon rather than the container centre. Cards no longer jump in size on the board refresh. Debug: 'ISSUE #20 FIX ACTIVE'.
 FIX PASS 2026-07-21 (ISSUE #20 energy-to-active position): both the player and CPU energy-attach paths only set the fly-to target for BENCH Pokemon; the ACTIVE fell back to the energy-container centre. Now both use get_pokemon_screen_location(target).position for the Active as well, so energy lands on the real Active slot. Debug: 'ISSUE #20 FIX ACTIVE'.</t>
         </is>
       </c>
+      <c r="E21" s="8" t="n"/>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>This is MOSTLY working. However 1) Attaching an energy to active pokemon still seems to go to middle of the container 2)     Working: Placing or evolving pokemon on bench works perfectly. Evolving active pokemon perfect.</t>
-        </is>
-      </c>
-      <c r="G21" s="8" t="inlineStr">
-        <is>
-          <t>Untested Fix</t>
-        </is>
-      </c>
-      <c r="H21" s="10" t="n">
+          <t>Issue Resolved</t>
+        </is>
+      </c>
+      <c r="G21" s="10" t="n">
         <v>46221</v>
       </c>
     </row>
@@ -1478,24 +1456,23 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="C22" s="7" t="n"/>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>When using oddish sprout and the oddishes are shown, there is an input blocker blocking the player from clicking the confirm button. It covers the whole screen. Potentially a bug for any card that searches deck for a card</t>
+        </is>
+      </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>When using oddish sprout and the oddishes are shown, there is an input blocker blocking the player from clicking the confirm button. It covers the whole screen. Potentially a bug for any card that searches deck for a card</t>
-        </is>
-      </c>
-      <c r="E22" s="9" t="inlineStr">
-        <is>
           <t>FIX 2026-07-18: same root cause as issue #3 — an ATTACK-triggered deck search (Oddish's Sprout) runs while perform_attack() has the full-screen opponent_blocker up, which sat on top of the selection UI and ate the click on the confirm button. Added the same save/hide/restore of opponent_blocker inside card_ops.search_deck_to_hand() (the shared helper behind Oddish Sprout and every other deck-search-to-hand effect), so the confirm button is clickable for all of them. Debug: 'ISSUE #21 FIX ACTIVE'.</t>
         </is>
       </c>
-      <c r="F22" s="8" t="n"/>
-      <c r="G22" s="8" t="inlineStr">
+      <c r="E22" s="8" t="n"/>
+      <c r="F22" s="8" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H22" s="10" t="n">
+      <c r="G22" s="10" t="n">
         <v>46221</v>
       </c>
     </row>
@@ -1508,28 +1485,27 @@
           <t>Player input</t>
         </is>
       </c>
-      <c r="C23" s="7" t="n"/>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>When using cards like recover, don't auto detach the energy. Some powers and cards change energy types (such as rainbow energy, charizard pokepower burn up etc) so a double colorless using charizards pokemon power can be used for it's Fire Spin attack, or Starmie can choose to discard a rainbow energy or a water energy for recover.</t>
+        </is>
+      </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>When using cards like recover, don't auto detach the energy. Some powers and cards change energy types (such as rainbow energy, charizard pokepower burn up etc) so a double colorless using charizards pokemon power can be used for it's Fire Spin attack, or Starmie can choose to discard a rainbow energy or a water energy for recover.</t>
-        </is>
-      </c>
-      <c r="E23" s="9" t="inlineStr">
-        <is>
           <t>FIX 2026-07-18 (Recover energy choice): execute_neo2_recover (Attack_Effects.gd) now collects ALL attached Energy that can pay the discard cost (a plain Water, a Rainbow that provides Water, a type-changed Energy, etc.) and — when there's more than one — prompts the PLAYER to pick which to discard instead of auto-detaching the first. The CPU keeps its most flexible Energy (discards a plain matching basic before a special/multi-type one). Debug: 'ISSUE #22 FIX ACTIVE'.</t>
         </is>
       </c>
-      <c r="F23" s="8" t="n"/>
-      <c r="G23" s="8" t="inlineStr">
+      <c r="E23" s="8" t="n"/>
+      <c r="F23" s="8" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H23" s="10" t="n">
+      <c r="G23" s="10" t="n">
         <v>46221</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" ht="180" customHeight="1">
       <c r="A24" s="7" t="n">
         <v>23</v>
       </c>
@@ -1538,24 +1514,23 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="C24" s="7" t="n"/>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>For recover and any other healing moves that fully heal, ensure the healing animations play (show floating label and colour squares in one at a time)</t>
+        </is>
+      </c>
       <c r="D24" s="8" t="inlineStr">
         <is>
-          <t>For recover and any other healing moves that fully heal, ensure the healing animations play (show floating label and colour squares in one at a time)</t>
-        </is>
-      </c>
-      <c r="E24" s="9" t="inlineStr">
-        <is>
           <t>FIX 2026-07-18 (full-heal animations): routed the generic self-heal chokepoint apply_self_heal (Attack_Effects.gd) through card_ops.heal_pokemon so EVERY generic 'remove all/N damage' attack plays the animation (floating +N HP label + HP circles restored one at a time). Also converted the dedicated full-heal attacks that snapped HP silently — Recover, Sweet Nectar, Wash Away, Sunbathe, Hatch — to heal_pokemon (Healing Oasis already used it). Debug: 'ISSUE #23a FIX ACTIVE'.</t>
         </is>
       </c>
-      <c r="F24" s="8" t="n"/>
-      <c r="G24" s="8" t="inlineStr">
+      <c r="E24" s="8" t="n"/>
+      <c r="F24" s="8" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H24" s="10" t="n">
+      <c r="G24" s="10" t="n">
         <v>46221</v>
       </c>
     </row>
@@ -1568,28 +1543,27 @@
           <t>CPU logic</t>
         </is>
       </c>
-      <c r="C25" s="7" t="n"/>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Player retreated poliwrath against starmie with no energies attached. Starmie only had 20hp left and poliwhrath had 5 energies attached. Poliwrath should not have retreated and definitely shouldn't have seen a "potential ko"</t>
+        </is>
+      </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>Player retreated poliwrath against starmie with no energies attached. Starmie only had 20hp left and poliwhrath had 5 energies attached. Poliwrath should not have retreated and definitely shouldn't have seen a "potential ko"</t>
-        </is>
-      </c>
-      <c r="E25" s="9" t="inlineStr">
-        <is>
           <t>FIX 2026-07-18 (CPU bad retreat/potential-KO): two fixes in CPU_AI.gd. (1) evaluate_ko_threats no longer flags a 1-energy-away attack as a potential KO when the player's Active has ZERO Energy attached — a 0-energy Pokemon is not a credible one-turn KO threat (this is why the CPU 'saw a potential KO' from a 0-energy Starmie). (2) evaluate_retreat_reasons Reason 2 now bails out of retreating if the CPU's own Active can KO the player's Active THIS turn (via new _cpu_active_can_ko_player_active), mirroring the existing Reason-1 mutual-KO logic — so a healthy 5-Energy Poliwrath attacks the 20-HP Starmie instead of fleeing. Debug: 'ISSUE #23b FIX ACTIVE'.</t>
         </is>
       </c>
-      <c r="F25" s="8" t="n"/>
-      <c r="G25" s="8" t="inlineStr">
+      <c r="E25" s="8" t="n"/>
+      <c r="F25" s="8" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H25" s="10" t="n">
+      <c r="G25" s="10" t="n">
         <v>46221</v>
       </c>
     </row>
-    <row r="26" ht="29.1" customHeight="1">
+    <row r="26" ht="210" customHeight="1">
       <c r="A26" s="7" t="n">
         <v>24</v>
       </c>
@@ -1598,24 +1572,28 @@
           <t>Attack effect</t>
         </is>
       </c>
-      <c r="C26" s="7" t="n"/>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>Poliwrath's whirlpool has the user decide the detached energy. Currently if opponent uses this, the player chooses the energy instead of the opponent removing the highest potential choice.</t>
+        </is>
+      </c>
       <c r="D26" s="8" t="inlineStr">
         <is>
-          <t>Poliwrath's whirlpool has the user decide the detached energy. Currently if opponent uses this, the player chooses the energy instead of the opponent removing the highest potential choice.</t>
-        </is>
-      </c>
-      <c r="E26" s="9" t="inlineStr">
-        <is>
-          <t>FIX 2026-07-21 (ISSUE #24 Whirlpool attacker-chooses): generic apply_energy_discard_defender (Attack_Effects.gd) is-defender-player branch made the PLAYER discard their own energy when the OPPONENT attacked, but the card text says the ATTACKER chooses. Now the CPU auto-picks the player's most valuable energy via new cpu_ai.cpu_pick_energy_to_discard_from (special +100, matching an attack cost +20 each, base +5). Covers every attacker-chooses energy_discard_defender attack (Whirlpool, Hyper Beam, etc.). Debug: 'ISSUE #24 FIX ACTIVE'.</t>
-        </is>
-      </c>
-      <c r="F26" s="8" t="n"/>
-      <c r="G26" s="8" t="inlineStr">
+          <t>FIX 2026-07-21 (ISSUE #24 Whirlpool attacker-chooses): generic apply_energy_discard_defender (Attack_Effects.gd) is-defender-player branch made the PLAYER discard their own energy when the OPPONENT attacked, but the card text says the ATTACKER chooses. Now the CPU auto-picks the player's most valuable energy via new cpu_ai.cpu_pick_energy_to_discard_from (special +100, matching an attack cost +20 each, base +5). Covers every attacker-chooses energy_discard_defender attack (Whirlpool, Hyper Beam, etc.). Debug: 'ISSUE #24 FIX ACTIVE'.
+FIX 2026-07-22 (ISSUE #24 retest — refresh board around discard animation): apply_energy_discard_defender (Attack_Effects.gd) now announces the discard, then removes the energy from the Pokemon and refreshes the board (display_active_pokemon_energies) BEFORE the fly-to-discard animation so the energy vanishes from the Pokemon first, then lands in the discard pile and refreshes again. Card is only ever visible in one place. Covers every attacker-chooses energy_discard_defender attack (Whirlpool/Hyper Beam etc.). Debug: 'ISSUE #24 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>Mostly good now, however make sure to refresh the board when the energy is animated to the discard pile. For any animation for any card moving forward, always ensure it is removed from the array it is moving from just before it starts to move and the board is refreshed to show this, then always refresh the board after the card has moved. E.g when whirlpool is used, say "water energy is discarded" then remove it from the attached energies array, update the board, play the animate card a to b showing it going to discard pile, add to discard pile, then update the board again. The card should always be visible in one location only.</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H26" s="9" t="inlineStr">
+      <c r="G26" s="9" t="inlineStr">
         <is>
           <t>21/07/2026</t>
         </is>
@@ -1630,24 +1608,23 @@
           <t>Item Effect</t>
         </is>
       </c>
-      <c r="C27" s="7" t="n"/>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Super potion just removes the top energy instead of allowing the choice. Should also allow cancellation at the point of choosing energy. Ensure every energy detatch that says "choose X energy card" ALLOWS the choice instead of making one automatically</t>
+        </is>
+      </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>Super potion just removes the top energy instead of allowing the choice. Should also allow cancellation at the point of choosing energy. Ensure every energy detatch that says "choose X energy card" ALLOWS the choice instead of making one automatically</t>
-        </is>
-      </c>
-      <c r="E27" s="9" t="inlineStr">
-        <is>
           <t>FIX 2026-07-21 (ISSUE #25 Super Potion energy choice + cancel): effect_super_potion (Trainer_Effects.gd) player branch popped the top energy automatically. Now the player picks the target (cancelable) AND which energy to discard via card_ops.remove_one_energy (new cancelable param); cancelling at either step refunds the card to hand (_refund_trainer_to_hand). Added a defender_energy_discard_active cancel branch in cancel_button_pressed_hide_selection_mode so the choice UI can be cancelled without hanging. Debug: 'ISSUE #25 FIX ACTIVE'.</t>
         </is>
       </c>
-      <c r="F27" s="8" t="n"/>
-      <c r="G27" s="8" t="inlineStr">
+      <c r="E27" s="8" t="n"/>
+      <c r="F27" s="8" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H27" s="9" t="inlineStr">
+      <c r="G27" s="9" t="inlineStr">
         <is>
           <t>21/07/2026</t>
         </is>
@@ -1662,24 +1639,28 @@
           <t>Overworld</t>
         </is>
       </c>
-      <c r="C28" s="7" t="n"/>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Game starts with player "moving_in_completed": false, but the furniture has the visibility wrong so the moved in furniture can be seen and the moving in furniture can't be seen. When game starts, "Moving in" should be visible. "Post Move In" should be hidden. When player has moving_in_completed as true, "Moving In" should be hidden and "Post Move In" should be visible This is true for both of the objects named in the "UPSTAIRS" tile map layer, but also the collision objects in Collision objects need to be removed not just hidden.</t>
+        </is>
+      </c>
       <c r="D28" s="8" t="inlineStr">
         <is>
-          <t>Game starts with player "moving_in_completed": false, but the furniture has the visibility wrong so the moved in furniture can be seen and the moving in furniture can't be seen. When game starts, "Moving in" should be visible. "Post Move In" should be hidden. When player has moving_in_completed as true, "Moving In" should be hidden and "Post Move In" should be visible This is true for both of the objects named in the "UPSTAIRS" tile map layer, but also the collision objects in Collision objects need to be removed not just hidden.</t>
-        </is>
-      </c>
-      <c r="E28" s="9" t="inlineStr">
-        <is>
-          <t>FIX 2026-07-21 (ISSUE #26 upstairs furniture visibility): new _apply_moving_in_state in Player_House_Upstairs.gd drives BOTH the visual layers and the collision bodies from moving_in_completed. Pre-move-in: UPSTAIRS/'Moving In' visible + 'Post Move In' hidden; post: reversed. Collision Objects 'Moving In'/'Post Move In' bodies are queue_free'd (REMOVED, not just hidden) because hiding a StaticBody2D doesn't stop it colliding; SceneCache re-instantiates fresh so removal is safe. Debug: 'ISSUE #26 FIX ACTIVE'.</t>
-        </is>
-      </c>
-      <c r="F28" s="8" t="n"/>
-      <c r="G28" s="8" t="inlineStr">
+          <t>FIX 2026-07-21 (ISSUE #26 upstairs furniture visibility): new _apply_moving_in_state in Player_House_Upstairs.gd drives BOTH the visual layers and the collision bodies from moving_in_completed. Pre-move-in: UPSTAIRS/'Moving In' visible + 'Post Move In' hidden; post: reversed. Collision Objects 'Moving In'/'Post Move In' bodies are queue_free'd (REMOVED, not just hidden) because hiding a StaticBody2D doesn't stop it colliding; SceneCache re-instantiates fresh so removal is safe. Debug: 'ISSUE #26 FIX ACTIVE'.
+FIX 2026-07-22 (ISSUE #26 retest — downstairs): Player_House_Downstairs.gd now uses a new _apply_moving_in_state (mirroring upstairs) instead of the base _apply_moving_in_visibility (which did nothing pre-move-in and never touched collisions). Drives BOTH the DOWNSTAIRS 'Moving In'/'Post Move In' visual tile layers AND the Collision Objects bodies from moving_in_completed, queue_free'ing the inactive collision set (removed, not hidden). Debug: 'ISSUE #26 FIX ACTIVE (downstairs)'.</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>Working for upstairs but downstairs needs the same fixes. Currently downstairs on game start has the move-in-completed furntiture showing and collisions active. The moving in tile layers and invisible but collision is still active</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H28" s="9" t="inlineStr">
+      <c r="G28" s="9" t="inlineStr">
         <is>
           <t>21/07/2026</t>
         </is>
@@ -1694,24 +1675,23 @@
           <t>Text</t>
         </is>
       </c>
-      <c r="C29" s="7" t="n"/>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Change the "Oh. A box of pokemon cards. I definitely didn't bring these with me. There's a note on top" text to just be "Huh? A box of Pokemon cards with a note on top". Then the note text that we already have</t>
+        </is>
+      </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>Change the "Oh. A box of pokemon cards. I definitely didn't bring these with me. There's a note on top" text to just be "Huh? A box of Pokemon cards with a note on top". Then the note text that we already have</t>
-        </is>
-      </c>
-      <c r="E29" s="9" t="inlineStr">
-        <is>
           <t>FIX 2026-07-21 (ISSUE #27 box text): Player_House_Upstairs.gd box message changed to 'Huh? A box of Pokemon cards with a note on top' (the note text follows as before).</t>
         </is>
       </c>
-      <c r="F29" s="8" t="n"/>
-      <c r="G29" s="8" t="inlineStr">
-        <is>
-          <t>Untested Fix</t>
-        </is>
-      </c>
-      <c r="H29" s="9" t="inlineStr">
+      <c r="E29" s="8" t="n"/>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>Issue Resolved</t>
+        </is>
+      </c>
+      <c r="G29" s="9" t="inlineStr">
         <is>
           <t>21/07/2026</t>
         </is>
@@ -1726,30 +1706,29 @@
           <t>Text</t>
         </is>
       </c>
-      <c r="C30" s="7" t="n"/>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Change the "Pokemon Starter Deck Acquired" message to be the same font formatting as a large message in the main core gameplay messagebox. (Large size, kenney font, central alighment vertical and horizontal)</t>
+        </is>
+      </c>
       <c r="D30" s="8" t="inlineStr">
         <is>
-          <t>Change the "Pokemon Starter Deck Acquired" message to be the same font formatting as a large message in the main core gameplay messagebox. (Large size, kenney font, central alighment vertical and horizontal)</t>
-        </is>
-      </c>
-      <c r="E30" s="9" t="inlineStr">
-        <is>
           <t>FIX 2026-07-21 (ISSUE #28 starter deck message format): new MapManager._show_large_message_with_ok — kenney (kenvector_future) font, size 40, centred H (bbcode [center]) and V (VBox ALIGNMENT_CENTER), mirroring the match's large messagebox. Defaults restored in _hide_message so normal overworld messages are unaffected. Player_House_Upstairs 'Pokemon Starter Deck Acquired!' now uses it. Debug: 'ISSUE #28 FIX ACTIVE'.</t>
         </is>
       </c>
-      <c r="F30" s="8" t="n"/>
-      <c r="G30" s="8" t="inlineStr">
-        <is>
-          <t>Untested Fix</t>
-        </is>
-      </c>
-      <c r="H30" s="9" t="inlineStr">
+      <c r="E30" s="8" t="n"/>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>Issue Resolved</t>
+        </is>
+      </c>
+      <c r="G30" s="9" t="inlineStr">
         <is>
           <t>21/07/2026</t>
         </is>
       </c>
     </row>
-    <row r="31">
+    <row r="31" ht="75" customHeight="1">
       <c r="A31" s="7" t="n">
         <v>29</v>
       </c>
@@ -1758,30 +1737,29 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="C31" s="7" t="n"/>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>The sleeves option should be disabled in the main menu the same as cards &amp; deck and coin case at the beginning of the game.</t>
+        </is>
+      </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>The sleeves option should be disabled in the main menu the same as cards &amp; deck and coin case at the beginning of the game.</t>
-        </is>
-      </c>
-      <c r="E31" s="9" t="inlineStr">
-        <is>
           <t>FIX 2026-07-21 (ISSUE #29 sleeves locked at start): Main_Menu_Script.gd adds sleeves to locked_modes when player_collected_starter_box is false, same as deck &amp; coin case. Debug: 'ISSUE #29 FIX ACTIVE'.</t>
         </is>
       </c>
-      <c r="F31" s="8" t="n"/>
-      <c r="G31" s="8" t="inlineStr">
-        <is>
-          <t>Untested Fix</t>
-        </is>
-      </c>
-      <c r="H31" s="9" t="inlineStr">
+      <c r="E31" s="8" t="n"/>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>Issue Resolved</t>
+        </is>
+      </c>
+      <c r="G31" s="9" t="inlineStr">
         <is>
           <t>21/07/2026</t>
         </is>
       </c>
     </row>
-    <row r="32">
+    <row r="32" ht="120" customHeight="1">
       <c r="A32" s="7" t="n">
         <v>30</v>
       </c>
@@ -1790,24 +1768,23 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="C32" s="7" t="n"/>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>Change the Exit game confirmation and buttons pop up from the main menu button be the same confirm UI theme we now have for the empty deck button</t>
+        </is>
+      </c>
       <c r="D32" s="8" t="inlineStr">
         <is>
-          <t>Change the Exit game confirmation and buttons pop up from the main menu button be the same confirm UI theme we now have for the empty deck button</t>
-        </is>
-      </c>
-      <c r="E32" s="9" t="inlineStr">
-        <is>
           <t>FIX 2026-07-21 (ISSUE #30 exit-game confirm theme): Main_Menu_Script.gd _show_quit_dialog rebuilt from the native ConfirmationDialog into the same styled popup as the deck builder's Empty-deck confirm (kenney-themed centred panel, dim overlay, red Quit + green Cancel). Debug: 'ISSUE #30 FIX ACTIVE'.</t>
         </is>
       </c>
-      <c r="F32" s="8" t="n"/>
-      <c r="G32" s="8" t="inlineStr">
-        <is>
-          <t>Untested Fix</t>
-        </is>
-      </c>
-      <c r="H32" s="9" t="inlineStr">
+      <c r="E32" s="8" t="n"/>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>Issue Resolved</t>
+        </is>
+      </c>
+      <c r="G32" s="9" t="inlineStr">
         <is>
           <t>21/07/2026</t>
         </is>
@@ -1822,24 +1799,23 @@
           <t>Player input</t>
         </is>
       </c>
-      <c r="C33" s="7" t="n"/>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>If the player quits out the game at the point of the taxi ride intro, it bypasses the custcene and the next game load the player is put in the overworld before they have collected hteir cards or entered their house. Ensure that if the player leaves the game during the cutscene, the flag is not changed that stops the cutscene on next game load. On next game load, skip the name entry/sprite pick screen but correctly play the taxi animation until it has played fully. Only clear the taxi cutscene played flag after the player enters their house as this is forced at the end of the cutscene</t>
+        </is>
+      </c>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>If the player quits out the game at the point of the taxi ride intro, it bypasses the custcene and the next game load the player is put in the overworld before they have collected hteir cards or entered their house. Ensure that if the player leaves the game during the cutscene, the flag is not changed that stops the cutscene on next game load. On next game load, skip the name entry/sprite pick screen but correctly play the taxi animation until it has played fully. Only clear the taxi cutscene played flag after the player enters their house as this is forced at the end of the cutscene</t>
-        </is>
-      </c>
-      <c r="E33" s="9" t="inlineStr">
-        <is>
           <t>FIX 2026-07-21 (ISSUE #31 taxi cutscene flag): Celeste_Harbour.gd no longer clears taxi_intro_pending at the START of _run_taxi_intro. Quitting mid-cutscene now keeps the flag set so the taxi animation replays in full on next load (name/sprite entry already skipped via first_launch_complete). The flag is cleared only when the cutscene finishes and the player is forced into their house. Debug: 'ISSUE #31 FIX ACTIVE'.</t>
         </is>
       </c>
-      <c r="F33" s="8" t="n"/>
-      <c r="G33" s="8" t="inlineStr">
-        <is>
-          <t>Untested Fix</t>
-        </is>
-      </c>
-      <c r="H33" s="9" t="inlineStr">
+      <c r="E33" s="8" t="n"/>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>Issue Resolved</t>
+        </is>
+      </c>
+      <c r="G33" s="9" t="inlineStr">
         <is>
           <t>21/07/2026</t>
         </is>
@@ -1854,8 +1830,7 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="C34" s="7" t="n"/>
-      <c r="D34" s="8" t="inlineStr">
+      <c r="C34" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">When loading the large libraries such as Sleeves, deck / card view, coin case or costumes, there is a few seconds where everything is loading (longest for sleeves, shortest for coins/cards). The player is still able to click around and even cancel out of that menu to varying results. Instead, block all input and have a small semi transparent black box the same format as we use for the exit game button confirmation, with a spinning loading icon that pops up as soon as the menu option is entered for each of these (coin, costume, deck, sleeves). Hide the loading box when all data is loading and allow player input from then. Allow the player to still hit escape to cancel loading and return to the main menu However this currently has a game breaking bug causing the game to crash if you try to press cancel or escape while the data is still loading in.
  (E 0:04:15:296   Sleeves_Scene_Script.gd:145 @ _load_sleeves(): Parameter "data.tree" is null.
@@ -1868,18 +1843,23 @@
 </t>
         </is>
       </c>
-      <c r="E34" s="9" t="inlineStr">
-        <is>
-          <t>FIX 2026-07-21 (ISSUE #32 loading crash + overlay): the async grid-load loops called get_tree().process_frame after the scene was freed by Escape/Cancel -&gt; null get_tree() crash. Added 'if not is_inside_tree(): return' guards to the load loops in Sleeves, Costume, Coin Case and Deck builder (incl. the two spots the user flagged with ##### ERROR comments). Sleeves also gains a loading overlay (input-blocking dim CanvasLayer + spinning square + 'Loading...'; Escape still cancels via _load_cancelled). NOTE: the loading overlay is currently only wired into Sleeves (worst case); the crash guard covers all four. The preload-at-startup / WebP redesign was intentionally NOT coded (user said so). Debug: 'ISSUE #32 FIX ACTIVE'.</t>
-        </is>
-      </c>
-      <c r="F34" s="8" t="n"/>
-      <c r="G34" s="8" t="inlineStr">
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>FIX 2026-07-21 (ISSUE #32 loading crash + overlay): the async grid-load loops called get_tree().process_frame after the scene was freed by Escape/Cancel -&gt; null get_tree() crash. Added 'if not is_inside_tree(): return' guards to the load loops in Sleeves, Costume, Coin Case and Deck builder (incl. the two spots the user flagged with ##### ERROR comments). Sleeves also gains a loading overlay (input-blocking dim CanvasLayer + spinning square + 'Loading...'; Escape still cancels via _load_cancelled). NOTE: the loading overlay is currently only wired into Sleeves (worst case); the crash guard covers all four. The preload-at-startup / WebP redesign was intentionally NOT coded (user said so). Debug: 'ISSUE #32 FIX ACTIVE'.
+FIX 2026-07-22 (ISSUE #32 retest — spinner on all libraries): extracted the Sleeves loading overlay into a shared MenuLoadingOverlay (Scripts/Menu_Scripts/Menu_Loading_Overlay.gd) and wired it into Costume, Coin Case AND the Deck/Card builder. Deck builder shows it in _display_current_set every set load/switch (show() auto-replaces so rapid switches never stack). Debug: 'ISSUE #32 FIX ACTIVE'. Preload/WebP redesign still intentionally NOT done.</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>Add the loading spinner to decks/card builder mode and have it show every time a new set is attempting to load, add it to costumes and coins</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H34" s="9" t="inlineStr">
+      <c r="G34" s="9" t="inlineStr">
         <is>
           <t>21/07/2026</t>
         </is>
@@ -1894,24 +1874,28 @@
           <t>Animation</t>
         </is>
       </c>
-      <c r="C35" s="7" t="n"/>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>Allow clicking to skip animations for receiving gifts and rewards both at the end of a match and in the overworld. 1) The fly in text animation: If the player clicks while this animation is playing, skip it to show all the rewards at once and then immediately pop up and reward animation messages such as the coin reward. 2) Spinning animations for cards and coins: if this animation is playing and the player clicks, skip the animation and show the coin/card in it's finished state as just visible.</t>
+        </is>
+      </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>Allow clicking to skip animations for receiving gifts and rewards both at the end of a match and in the overworld. 1) The fly in text animation: If the player clicks while this animation is playing, skip it to show all the rewards at once and then immediately pop up and reward animation messages such as the coin reward. 2) Spinning animations for cards and coins: if this animation is playing and the player clicks, skip the animation and show the coin/card in it's finished state as just visible.</t>
-        </is>
-      </c>
-      <c r="E35" s="9" t="inlineStr">
-        <is>
-          <t>FIX 2026-07-21 (ISSUE #33 skip gift reveal): MapManager gift reveal is now click-to-skip. The dim overlay catches a left-click during the coin/card/costume reveal (_on_gift_reveal_input); _finalize_gift_reveal kills the running tweens and snaps every rect to its finished face, then OK appears immediately. NOTE: this covers the overworld GIFT reveal (coin/card spins, costume fade). Debug: 'ISSUE #33 FIX ACTIVE'.</t>
-        </is>
-      </c>
-      <c r="F35" s="8" t="n"/>
-      <c r="G35" s="8" t="inlineStr">
+          <t>FIX 2026-07-21 (ISSUE #33 skip gift reveal): MapManager gift reveal is now click-to-skip. The dim overlay catches a left-click during the coin/card/costume reveal (_on_gift_reveal_input); _finalize_gift_reveal kills the running tweens and snaps every rect to its finished face, then OK appears immediately. NOTE: this covers the overworld GIFT reveal (coin/card spins, costume fade). Debug: 'ISSUE #33 FIX ACTIVE'.
+FIX 2026-07-22 (ISSUE #33 retest — MATCH-END rewards skippable): root cause was click_enabled=true being set AFTER the fly-in, so clicks during it were ignored entirely. Match_End_Outro_Script.gd now has _in_skippable_anim/_skip_anim: a click during the reward fly-in, coin/card flip, or costume fade fast-forwards it to the finished state (_await_tween_or_skip + _snap_rewards_to_final; flips snap to front face, costume snaps fully visible). Debug: 'ISSUE #33 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>Clicking didn't skip any of the animations for rewards after a match. The rewards still flew in and clicking didn't finish the animation immediately as required. Then coin flipped round and clicking didn't force this to stop spinning either.</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H35" s="9" t="inlineStr">
+      <c r="G35" s="9" t="inlineStr">
         <is>
           <t>21/07/2026</t>
         </is>
@@ -1926,8 +1910,7 @@
           <t>Animation</t>
         </is>
       </c>
-      <c r="C36" s="7" t="n"/>
-      <c r="D36" s="8" t="inlineStr">
+      <c r="C36" s="8" t="inlineStr">
         <is>
           <t>Add 3 new global variables that will eventually be changed in the options sub menu for game speeds. 
 1) Card Match Animation Speed - For all animations in a regular card match (such as placing cards on bench, attaching energies, retreating, discarding etc. Set current animation speed to standard (medium) with a speed multiplier of 1, allow all the animations to have the speed multiplier and in options there will be Slow and Fast for 0.5 and 2x speed respectively
@@ -1935,24 +1918,24 @@
 3) Overworld Animation Speed  - for rewards and gift animations and anything else we have (coin spinning time/speed, card spinning time/speed, costume fade in speed etc). For these also set current speed to standard and allow all the speeds to be changed when the options are added (this will be slow at 0.5 and 2)</t>
         </is>
       </c>
-      <c r="E36" s="9" t="inlineStr">
+      <c r="D36" s="8" t="inlineStr">
         <is>
           <t>FIX 2026-07-21 (ISSUE #34 global speed variables): added GameState.card_match_animation_speed / overworld_walking_speed / overworld_animation_speed (all 1.0 = standard) + scaled_duration() helper. Wired: card-match animate_card_a_to_b duration (card_match_animation_speed); player walk+run velocity &amp; anim (overworld_walking_speed); gift reveal flip/costume durations and skip-wait (overworld_animation_speed). These are the globals the future Options submenu will set (slow/standard/fast). Debug prints on the affected paths.</t>
         </is>
       </c>
-      <c r="F36" s="8" t="n"/>
-      <c r="G36" s="8" t="inlineStr">
+      <c r="E36" s="8" t="n"/>
+      <c r="F36" s="8" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H36" s="9" t="inlineStr">
+      <c r="G36" s="9" t="inlineStr">
         <is>
           <t>21/07/2026</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="75" customHeight="1">
+    <row r="37" ht="225" customHeight="1">
       <c r="A37" s="7" t="n">
         <v>35</v>
       </c>
@@ -1961,24 +1944,29 @@
           <t>CPU logic</t>
         </is>
       </c>
-      <c r="C37" s="7" t="n"/>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>Opponent retreated magnemite for raichu, then attached an energy onto their benched magnemite that they just discarded an energy from. Firstly add a penalty for cpu logic attaching an energy for pokemon HP at a rate of 100-current health percentage. E.g If Magnemite has 20/40 hp that is 50% so 100-50 is a negative penalty of 50 points from attaching energy to that card. Increase bonus to attach energy to active pokemon by +50 so there is a more weight in keeping active pokemon powered up. We should already have a penalty on switching in a pokemon that cannot attack this turn, or next turn guaranteed so the CPU should have just kept magnemite in to be knocked out, but evolved and attached an energy to pikachu</t>
+        </is>
+      </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
-          <t>Player retreated magnemite for raichu, then attached an energy onto their benched magnemite that they just discarded an energy from. Firstly add a penalty for cpu logic attaching an energy for pokemon HP at a rate of 100-current health percentage. E.g If Magnemite has 20/40 hp that is 50% so 100-50 is a negative penalty of 50 points from attaching energy to that card. Increase bonus to attach energy to active pokemon by +50 so there is a more weight in keeping active pokemon powered up. We should already have a penalty on switching in a pokemon that cannot attack this turn, or next turn guaranteed so the CPU should have just kept magnemite in to be knocked out, but evolved and attached an energy to pikachu</t>
-        </is>
-      </c>
-      <c r="E37" s="9" t="inlineStr">
-        <is>
-          <t>FIX 2026-07-21 (ISSUE #35 energy-attach HP penalty): score_energy_pair (CPU_AI.gd) now subtracts (100 - HP%) when scoring an attach target (full HP = 0, 20/40 Magnemite = -50) so the CPU stops feeding energy to nearly-dead Pokemon, and the Active flat bonus was raised +50 (40 -&gt; 90) to favour keeping the Active powered. Debug: 'ISSUE #35 FIX ACTIVE'.</t>
-        </is>
-      </c>
-      <c r="F37" s="8" t="n"/>
-      <c r="G37" s="8" t="inlineStr">
+          <t>FIX 2026-07-21 (ISSUE #35 energy-attach HP penalty): score_energy_pair (CPU_AI.gd) now subtracts (100 - HP%) when scoring an attach target (full HP = 0, 20/40 Magnemite = -50) so the CPU stops feeding energy to nearly-dead Pokemon, and the Active flat bonus was raised +50 (40 -&gt; 90) to favour keeping the Active powered. Debug: 'ISSUE #35 FIX ACTIVE'.
+FIX 2026-07-22 (ISSUE #35 retest — CPU energy attach): (1) staleness: rebuild the CPU evaluation immediately before the energy phase so a Phase-5 retreat / Phase-4b trainer that changed the Active/bench is reflected (fixes attaching to the just-retreated Magnemite; stale bench had empty attack_data -&gt; -200 type penalty -&gt; Active kept winning). (2) dominant guards in score_energy_pair: a DOOMED Active that can already attack (guaranteed KO OR poison-will-KO) scores -400 unless the energy secures a KO now (fixes the 10-HP poisoned flying Pikachu getting a 4th energy over 4 empty bench); a fully-powered Active with no evolution/extra-energy benefit scores -300 so surplus goes to a needy bench (Sandshrew case). Debug: 'ISSUE #35 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>Opponent did something similar just now. Sandshrew was active with 2 energy attached. Opp had a bench of 2 other cards (sandshrew and diglett) with no energy attached. Somehow Opp attached the fightning energy to the active sandshrew that already had 2 attached instead of either of the bench pokemon. Console said attaching energy to sandshrew with -10 points so it should have prioritised a bench pokemon. Is the issue that the energy/CPU priority for actions only runs once before any board changes. e.g did it score the energy when there were no bench pokemon, 2 bench pokemon were added then the opp attached energy to the active as it never reevaluated? 
+Similarly I've just done another game and same situation. opponent is poisoned but on a flying pikachu with 3 lightning energy. 10 hp left guarenteed knockout, but instead the opponent attached ANOTHER ENERGY MAKING 4 ENERGIES ON FLYING PIKACHU WHEN HE HAD 4 BENCH POKEMON. I think the above is an incorrect assumption as the bench pokemon already existed in this situation and weren't benched the same turn this happened.</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H37" s="9" t="inlineStr">
+      <c r="G37" s="9" t="inlineStr">
         <is>
           <t>21/07/2026</t>
         </is>
@@ -1993,24 +1981,23 @@
           <t>CPU logic</t>
         </is>
       </c>
-      <c r="C38" s="7" t="n"/>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>Add a negative penalty to evolving a card if 1) Energy attachment has been complete so no further energies can be played this turn. 2) The pre evolved card yet to evolve can already attack 3) the post evolved card has higher energy requirements so can't attack if evolved into 4) The pre evolved pokemon is NOT guaranteed or potentially KOd next turn. E.g if a player has a charmeleon with 2 fire energy attached, and full HP against a ratatta that can only do 20 damage, there is no benefit to evolving into Charizard as Charizard needs 4 energies to attack so the opponent would lose a turn attacking.</t>
+        </is>
+      </c>
       <c r="D38" s="8" t="inlineStr">
         <is>
-          <t>Add a negative penalty to evolving a card if 1) Energy attachment has been complete so no further energies can be played this turn. 2) The pre evolved card yet to evolve can already attack 3) the post evolved card has higher energy requirements so can't attack if evolved into 4) The pre evolved pokemon is NOT guaranteed or potentially KOd next turn. E.g if a player has a charmeleon with 2 fire energy attached, and full HP against a ratatta that can only do 20 damage, there is no benefit to evolving into Charizard as Charizard needs 4 energies to attack so the opponent would lose a turn attacking.</t>
-        </is>
-      </c>
-      <c r="E38" s="9" t="inlineStr">
-        <is>
           <t>FIX 2026-07-21 (ISSUE #36 pointless-evolution penalty): evaluate_evolution_pair (CPU_AI.gd) applies a -250 penalty when ALL hold: energy already spent this turn, the pre-evo can attack now, the evolved form can't attack after evolving AND costs more energy, and the pre-evo isn't guaranteed/potentially KO'd next turn (so evolving just wastes tempo, e.g. Charmeleon-&gt;Charizard vs a Rattata). Debug: 'ISSUE #36 FIX ACTIVE'.</t>
         </is>
       </c>
-      <c r="F38" s="8" t="n"/>
-      <c r="G38" s="8" t="inlineStr">
+      <c r="E38" s="8" t="n"/>
+      <c r="F38" s="8" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H38" s="9" t="inlineStr">
+      <c r="G38" s="9" t="inlineStr">
         <is>
           <t>21/07/2026</t>
         </is>
@@ -2025,24 +2012,28 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="C39" s="7" t="n"/>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>When the opponent is performing multiple actions at once with no animations in between, sometimes it's a lot of info that is hard to know what's new. Therefore every time the player clicks to clear a message box, have a delay timer after that message box is hidden before anything else happens. Link this to the animation speds in issue 34 so that the default delay is 0.5s but can be multiplied by either 0.5 or 2 to make the gap inbetween messages either 0.25s or 1s.</t>
+        </is>
+      </c>
       <c r="D39" s="8" t="inlineStr">
         <is>
-          <t>When the opponent is performing multiple actions at once with no animations in between, sometimes it's a lot of info that is hard to know what's new. Therefore every time the player clicks to clear a message box, have a delay timer after that message box is hidden before anything else happens. Link this to the animation speds in issue 34 so that the default delay is 0.5s but can be multiplied by either 0.5 or 2 to make the gap inbetween messages either 0.25s or 1s.</t>
-        </is>
-      </c>
-      <c r="E39" s="9" t="inlineStr">
-        <is>
-          <t>FIX 2026-07-21 (ISSUE #37 post-message delay): match show_message (Main_Match_Core) now pauses 0.5s / card_match_animation_speed after each message is dismissed (fast 0.25s, slow 1.0s) so bursts of opponent actions are readable. Linked to the ISSUE #34 speed global.</t>
-        </is>
-      </c>
-      <c r="F39" s="8" t="n"/>
-      <c r="G39" s="8" t="inlineStr">
+          <t>FIX 2026-07-21 (ISSUE #37 post-message delay): match show_message (Main_Match_Core) now pauses 0.5s / card_match_animation_speed after each message is dismissed (fast 0.25s, slow 1.0s) so bursts of opponent actions are readable. Linked to the ISSUE #34 speed global.
+FIX 2026-07-22 (ISSUE #37 retest — REVERTED): removed the post-message delay entirely from show_message (Main_Match_Core). It was a bad change (added a pause after EVERY message box). Messages now dismiss instantly again.</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>I was wrong in my suggestion. Remove the delay now, it shouldn't have been added after every text box. Terrible change.</t>
+        </is>
+      </c>
+      <c r="F39" s="8" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H39" s="9" t="inlineStr">
+      <c r="G39" s="9" t="inlineStr">
         <is>
           <t>21/07/2026</t>
         </is>
@@ -2057,24 +2048,28 @@
           <t>Animation</t>
         </is>
       </c>
-      <c r="C40" s="7" t="n"/>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>we need something like x5 the time between labels appearing showing bench damage for attacks like earthquake where all bench is damaged, currently whole thing seems to be 0.05s delay almost instant but instead should be like 0.2s delay between them all so it looks more like a Mexican wave and the player can keep up better ( of course with the animation multiplier)</t>
+        </is>
+      </c>
       <c r="D40" s="8" t="inlineStr">
         <is>
-          <t>we need something like x5 the time between labels appearing showing bench damage for attacks like earthquake where all bench is damaged, currently whole thing seems to be 0.05s delay almost instant but instead should be like 0.2s delay between them all so it looks more like a Mexican wave and the player can keep up better ( of course with the animation multiplier)</t>
-        </is>
-      </c>
-      <c r="E40" s="9" t="inlineStr">
-        <is>
-          <t>FIX 2026-07-21 (ISSUE #38 bench-damage label pacing): apply_bench_damage (Attack_Effects.gd) staggered floating labels by only 0.1s. Now 0.2s scaled by the card-match animation speed (GameState.scaled_duration) so a multi-target hit like Earthquake reads as a Mexican wave. Debug: 'ISSUE #38 FIX ACTIVE'.</t>
-        </is>
-      </c>
-      <c r="F40" s="8" t="n"/>
-      <c r="G40" s="8" t="inlineStr">
+          <t>FIX 2026-07-21 (ISSUE #38 bench-damage label pacing): apply_bench_damage (Attack_Effects.gd) staggered floating labels by only 0.1s. Now 0.2s scaled by the card-match animation speed (GameState.scaled_duration) so a multi-target hit like Earthquake reads as a Mexican wave. Debug: 'ISSUE #38 FIX ACTIVE'.
+FIX 2026-07-22 (ISSUE #38 retest): bench-damage label stagger bumped 0.2s -&gt; 0.3s in apply_bench_damage (Attack_Effects.gd), still scaled by the card-match animation speed. Debug: 'ISSUE #38 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>Increase time to 0.3s</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H40" s="9" t="inlineStr">
+      <c r="G40" s="9" t="inlineStr">
         <is>
           <t>21/07/2026</t>
         </is>
@@ -2089,30 +2084,32 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="C41" s="7" t="n"/>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>When opponent uses a trainer card e.g bill or professor oak, their hand array moves over to the left about 200 pixels for no reason. Just a weird visual bug that needs to stop the hand moving positions when a trainer is played. Only seems to be some cards, potentially anything that affects hand size? Maintenance and bill and prof oak all have this but not all trainers</t>
+        </is>
+      </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>When opponent uses a trainer card e.g bill or professor oak, their hand array moves over to the left about 200 pixels for no reason. Just a weird visual bug that needs to stop the hand moving positions when a trainer is played. Only seems to be some cards, potentially anything that affects hand size? Maintenance and bill and prof oak all have this but not all trainers</t>
-        </is>
-      </c>
-      <c r="E41" s="9" t="inlineStr">
-        <is>
           <t>FIX 2026-07-21 (ISSUE #39 opponent hand shifts left): the opponent hand HBoxContainer (opponent_hand_hbox_container in Main_Match_Core_GamePlay_Scene.tscn) was right-anchored with grow_horizontal=0 (grew leftward), so any hand-size change repositioned every card. Changed to grow_horizontal=1 (grow rightward, left edge pinned) so existing cards stay put and new cards append on the right. Fixes Bill/Prof Oak/Maintenance and any hand-size-changing trainer.</t>
         </is>
       </c>
-      <c r="F41" s="8" t="n"/>
-      <c r="G41" s="8" t="inlineStr">
-        <is>
-          <t>Untested Fix</t>
-        </is>
-      </c>
-      <c r="H41" s="9" t="inlineStr">
+      <c r="E41" s="8" t="n"/>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>Issue Resolved</t>
+        </is>
+      </c>
+      <c r="G41" s="9" t="inlineStr">
         <is>
           <t>21/07/2026</t>
         </is>
       </c>
-    </row>
-    <row r="42">
+      <c r="H41" s="6" t="n">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="42" ht="75" customHeight="1">
       <c r="A42" s="7" t="n">
         <v>40</v>
       </c>
@@ -2121,20 +2118,31 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="C42" s="7" t="n"/>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>Energy card attaching to active pokemon goes to middle of array not the final position</t>
+        </is>
+      </c>
       <c r="D42" s="8" t="inlineStr">
         <is>
-          <t>Energy card attaching to active pokemon goes to middle of array not the final position</t>
-        </is>
-      </c>
-      <c r="E42" s="9" t="n"/>
-      <c r="F42" s="8" t="n"/>
-      <c r="G42" s="8" t="inlineStr">
+          <t>FIX 2026-07-22 (ISSUE #40 retest — exact final slot): energy attaching to the ACTIVE now flies to its EXACT final slot in the energy stack. New Main_Match_Core.measure_and_hide_new_active_energy_slot builds the real stack, reads the just-appended energy's true global_position + size, hides that slot during the flight, and animates there (size tweens hand-&gt;stack size). Applied to BOTH player (Main_Match_Core) and opponent (CPU_AI) active attaches — the opponent case was ~300px off because it flew to the Active CARD position, not the energy stack. Bench unchanged. Debug: 'ISSUE #40 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>Now even worse. When opponent attaches an energy it goes to a completely wrong position 300 pixels to the left of where it should now. Get the position of where the card WILL be in it's final position in it's new array, then have the card move to this position exactly so there is no guessing. Also ensure the code is the same as moving pokemon to the bench and to active and the card size changes from it's old size to it's final size</t>
+        </is>
+      </c>
+      <c r="F42" s="8" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H42" s="9" t="n"/>
+      <c r="G42" s="9" t="inlineStr">
+        <is>
+          <t>22/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="30" customHeight="1">
       <c r="A43" s="7" t="n">
@@ -2145,24 +2153,23 @@
           <t>Animation</t>
         </is>
       </c>
-      <c r="C43" s="7" t="n"/>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>Opponent using maintenance just vanishes two cards from the hand instantly, pops up the message and then shows 1 draw. It should show the message that the card is played first, then animate each cards going to the deck from the hand (1 at a time) then the card being drawn adding to hand animation</t>
+        </is>
+      </c>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>Opponent using maintenance just vanishes two cards from the hand instantly, pops up the message and then shows 1 draw. It should show the message that the card is played first, then animate each cards going to the deck from the hand (1 at a time) then the card being drawn adding to hand animation</t>
-        </is>
-      </c>
-      <c r="E43" s="9" t="inlineStr">
-        <is>
           <t>FIX 2026-07-21 (ISSUE #41 Maintenance flow): opponent Maintenance (effect_maintenance, Trainer_Effects.gd) vanished 2 cards instantly and showed the message after the draw. Now: announce first, fly each hidden card (card back) hand-&gt;deck ONE AT A TIME, play the new shuffle animation (#42), then the draw animates in. Debug: 'ISSUE #41 FIX ACTIVE'.</t>
         </is>
       </c>
-      <c r="F43" s="8" t="n"/>
-      <c r="G43" s="8" t="inlineStr">
-        <is>
-          <t>Untested Fix</t>
-        </is>
-      </c>
-      <c r="H43" s="9" t="inlineStr">
+      <c r="E43" s="8" t="n"/>
+      <c r="F43" s="8" t="inlineStr">
+        <is>
+          <t>Issue Resolved</t>
+        </is>
+      </c>
+      <c r="G43" s="9" t="inlineStr">
         <is>
           <t>21/07/2026</t>
         </is>
@@ -2177,27 +2184,29 @@
           <t>Animation</t>
         </is>
       </c>
-      <c r="C44" s="7" t="n"/>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>We need a shuffle animation, Just put something in for now that shows the deck being shuffled, I was thinking currently the deck is a stack of individual drawn card backs. Animate and move every second card up 100 pixels over 0.2 seconds, moving left the amount of pixels distance that each card is drawn away from each other (e.g I think each card is drawn 2 pixels to the right of the one above it so move them left 2 pixels), change their z index to all be +1 from their current number, then for all of the remaining cards (the first card, 3rd card etc, all that were left behind) move right the same pixels that the others moved left and set their z index to be -1 from their current number. The cards that were originally moved up and left then get moved back down 100 pixels. The whole thing then repeats 3 more times. This whole animation from start to finish should take 1 second x the animation multiplier. The goal is to make it look like the cards are being shuffled in a little animation.</t>
+        </is>
+      </c>
       <c r="D44" s="8" t="inlineStr">
         <is>
-          <t>We need a shuffle animation, Just put something in for now that shows the deck being shuffled, I was thinking currently the deck is a stack of individual drawn card backs. Animate and move every second card up 100 pixels over 0.2 seconds, moving left the amount of pixels distance that each card is drawn away from each other (e.g I think each card is drawn 2 pixels to the right of the one above it so move them left 2 pixels), change their z index to all be +1 from their current number, then for all of the remaining cards (the first card, 3rd card etc, all that were left behind) move right the same pixels that the others moved left and set their z index to be -1 from their current number. The cards that were originally moved up and left then get moved back down 100 pixels. The whole thing then repeats 3 more times. This whole animation from start to finish should take 1 second x the animation multiplier. The goal is to make it look like the cards are being shuffled in a little animation.</t>
-        </is>
-      </c>
-      <c r="E44" s="9" t="inlineStr">
-        <is>
           <t>FIX 2026-07-21 (ISSUE #42 shuffle animation): new reusable Main_Match_Core.animate_deck_shuffle(is_opponent) — per the spec, every 2nd card-back layer lifts 100px + shifts 2px left (z+1) while the rest shift 2px right (z-1), then drops back down, repeated 4x, ~1s scaled by card-match animation speed, then rebuilds the deck icon to reset. Wired into Maintenance (#41) and Pokemon Trader (#44); available for the other ~50 shuffle sites to adopt as needed. Debug: 'ISSUE #42 FIX ACTIVE'.</t>
         </is>
       </c>
-      <c r="F44" s="8" t="n"/>
-      <c r="G44" s="8" t="inlineStr">
-        <is>
-          <t>Untested Fix</t>
-        </is>
-      </c>
-      <c r="H44" s="9" t="inlineStr">
+      <c r="E44" s="8" t="n"/>
+      <c r="F44" s="8" t="inlineStr">
+        <is>
+          <t>Issue Resolved</t>
+        </is>
+      </c>
+      <c r="G44" s="9" t="inlineStr">
         <is>
           <t>21/07/2026</t>
         </is>
+      </c>
+      <c r="H44" s="6" t="n">
+        <v>46225</v>
       </c>
     </row>
     <row r="45" ht="75" customHeight="1">
@@ -2209,24 +2218,23 @@
           <t>Animation</t>
         </is>
       </c>
-      <c r="C45" s="7" t="n"/>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>When opponent retreats, the energy card is immediately discarded and shown in discard pile before the animation plays showing it to the discard pile. Potentially this is actually a bug and the energy is discarded twice? Check the flow for this, the discard pile seemed to jump 2 cards when a pokemon retreated instead of 1 per the cost. It should first only show the message to say "X retreated to the bench" then when clicked, show the discard energies going to the discard pile from attached. Update display to show the change of them in there. Then wait 0.5s, then follow the rest of the flow (active pokemon moves to bench, added, refresh, old pokemon removed, refresh, moves to active position.</t>
+        </is>
+      </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>When opponent retreats, the energy card is immediately discarded and shown in discard pile before the animation plays showing it to the discard pile. Potentially this is actually a bug and the energy is discarded twice? Check the flow for this, the discard pile seemed to jump 2 cards when a pokemon retreated instead of 1 per the cost. It should first only show the message to say "X retreated to the bench" then when clicked, show the discard energies going to the discard pile from attached. Update display to show the change of them in there. Then wait 0.5s, then follow the rest of the flow (active pokemon moves to bench, added, refresh, old pokemon removed, refresh, moves to active position.</t>
-        </is>
-      </c>
-      <c r="E45" s="9" t="inlineStr">
-        <is>
           <t>FIX 2026-07-21 (ISSUE #43 opponent retreat double-discard): the CPU retreat (CPU_AI.gd cpu_phase_retreat) pre-discarded each retreat-cost Energy via send_card_to_discard AND then animate_retreat -&gt; animate_energies_to_discard discarded them AGAIN (it erases-from-attached + appends-to-discard), so the discard pile jumped by 2x the cost. The CPU now just COLLECTS the top N energy references (no pre-discard), matching the player flow, so the single discard + one-at-a-time animation happens inside animate_retreat (message -&gt; discard anim -&gt; 0.5s -&gt; swap). Debug: 'ISSUE #43 FIX ACTIVE'.</t>
         </is>
       </c>
-      <c r="F45" s="8" t="n"/>
-      <c r="G45" s="8" t="inlineStr">
+      <c r="E45" s="8" t="n"/>
+      <c r="F45" s="8" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H45" s="9" t="inlineStr">
+      <c r="G45" s="9" t="inlineStr">
         <is>
           <t>21/07/2026</t>
         </is>
@@ -2241,27 +2249,29 @@
           <t>Animation</t>
         </is>
       </c>
-      <c r="C46" s="7" t="n"/>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>When opponent plays trader, add animations and change flow. 1) Opponent plays trader 2) Show the card being shuffled away visible to the player with message "Opponent shuffled X into their deck" 3) Show the card moving from the hand into the deck 4) Show the card being being collected and swapped for from the deck visible to the player with the message "Opponent added X to their hand" 5) show the animation of it going to the opponents hand. Make sure this applies to any cards in which both cards need to be shown the player (e.g wherever it says "Show this card to your opponent")</t>
+        </is>
+      </c>
       <c r="D46" s="8" t="inlineStr">
         <is>
-          <t>When opponent plays trader, add animations and change flow. 1) Opponent plays trader 2) Show the card being shuffled away visible to the player with message "Opponent shuffled X into their deck" 3) Show the card moving from the hand into the deck 4) Show the card being being collected and swapped for from the deck visible to the player with the message "Opponent added X to their hand" 5) show the animation of it going to the opponents hand. Make sure this applies to any cards in which both cards need to be shown the player (e.g wherever it says "Show this card to your opponent")</t>
-        </is>
-      </c>
-      <c r="E46" s="9" t="inlineStr">
-        <is>
           <t>FIX 2026-07-21 (ISSUE #44 Pokemon Trader flow/animation): opponent Pokemon Trader (effect_pokemon_trader) did no animation and hid both cards despite the 'show them to your opponent' clause. New flow: message 'shuffled X into their deck' -&gt; fly X (face-up) hand-&gt;deck -&gt; shuffle animation -&gt; message 'added Y to their hand' -&gt; fly Y (face-up) deck-&gt;hand. NOTE: fixed for Pokemon Trader (the named base-set card); other 'show to opponent' cards can reuse this pattern. Debug: 'ISSUE #44 FIX ACTIVE'.</t>
         </is>
       </c>
-      <c r="F46" s="8" t="n"/>
-      <c r="G46" s="8" t="inlineStr">
-        <is>
-          <t>Untested Fix</t>
-        </is>
-      </c>
-      <c r="H46" s="9" t="inlineStr">
+      <c r="E46" s="8" t="n"/>
+      <c r="F46" s="8" t="inlineStr">
+        <is>
+          <t>Issue Resolved</t>
+        </is>
+      </c>
+      <c r="G46" s="9" t="inlineStr">
         <is>
           <t>21/07/2026</t>
         </is>
+      </c>
+      <c r="H46" s="6" t="n">
+        <v>46225</v>
       </c>
     </row>
     <row r="47" ht="90" customHeight="1">
@@ -2273,24 +2283,23 @@
           <t>CPU logic</t>
         </is>
       </c>
-      <c r="C47" s="7" t="n"/>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>Venomoth Power shift there is no point ever activating this when on the bench unless there is a power or attack in player that has the text "For each X type in play" or "for each X type on your bench" or "for each X type on your opponents bench". Otherwise just ignore that power if Venomoth is benched. Also it changed it's type to psychic which there wasn't a type in play of so ensure only types that are in play can be changed into. Additionally, Venomoth changed type to fire type (with no fire type pokemon in play) which was a correct cpu logic choice (as the player's active pokemon was weak to fire) but even though Venomoth did this, the player did not take double damage from weakness. i.e Venomoth changed types which is shouldn't have been able to, but it should have if it could, but even if it did it didn't affect damage.</t>
+        </is>
+      </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>Venomoth Power shift there is no point ever activating this when on the bench unless there is a power or attack in player that has the text "For each X type in play" or "for each X type on your bench" or "for each X type on your opponents bench". Otherwise just ignore that power if Venomoth is benched. Also it changed it's type to psychic which there wasn't a type in play of so ensure only types that are in play can be changed into. Additionally, Venomoth changed type to fire type (with no fire type pokemon in play) which was a correct cpu logic choice (as the player's active pokemon was weak to fire) but even though Venomoth did this, the player did not take double damage from weakness. i.e Venomoth changed types which is shouldn't have been able to, but it should have if it could, but even if it did it didn't affect damage.</t>
-        </is>
-      </c>
-      <c r="E47" s="9" t="inlineStr">
-        <is>
           <t>FIX 2026-07-21 (ISSUE #45 Venomoth Shift, 3 bugs): (1) get_effective_types (Card_Class_Object_Script) now returns [temporary_type] when set, so a Shifted type actually triggers Weakness/Resistance (previously the shift changed nothing about damage). (2) CPU trigger (Powers_And_Bodies_Effects.gd) now only shifts to a type ACTUALLY IN PLAY (_collect_types_in_play) — it was blindly copying the player's Weakness type even when no Pokemon of that type existed. (3) CPU only bothers shifting when Venomoth is the ACTIVE (or a 'for each &lt;type&gt; in play/bench' synergy exists via _shift_type_count_synergy_in_play) — a benched Venomoth changing type does nothing. Debug: 'ISSUE #45 FIX ACTIVE'.</t>
         </is>
       </c>
-      <c r="F47" s="8" t="n"/>
-      <c r="G47" s="8" t="inlineStr">
+      <c r="E47" s="8" t="n"/>
+      <c r="F47" s="8" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H47" s="9" t="inlineStr">
+      <c r="G47" s="9" t="inlineStr">
         <is>
           <t>21/07/2026</t>
         </is>
@@ -2305,24 +2314,28 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="C48" s="7" t="n"/>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>When retreating your own pokemon as the player, don't bother showing the energy cards stacked above the active pokemon as they're all being displayed next to it and are selectable anyway. Do show the health though but increase the size of the active pokemon card by 50% so it's larger than the energies being shown next to it</t>
+        </is>
+      </c>
       <c r="D48" s="8" t="inlineStr">
         <is>
-          <t>When retreating your own pokemon as the player, don't bother showing the energy cards stacked above the active pokemon as they're all being displayed next to it and are selectable anyway. Do show the health though but increase the size of the active pokemon card by 50% so it's larger than the energies being shown next to it</t>
-        </is>
-      </c>
-      <c r="E48" s="9" t="inlineStr">
-        <is>
-          <t>FIX 2026-07-21 (ISSUE #46 player retreat display): during the player retreat energy-selection screen the Active card no longer shows its energies stacked above it (they're already listed as selectable cards in the same array). Added a show_energies flag to build_pokemon_slot_with_energies_and_hp (HP still shown); display_hand_cards_array hides the stack for the retreat Active and enlarges that card 50% so it stands out. Debug: 'ISSUE #46 FIX ACTIVE'.</t>
-        </is>
-      </c>
-      <c r="F48" s="8" t="n"/>
-      <c r="G48" s="8" t="inlineStr">
+          <t>FIX 2026-07-21 (ISSUE #46 player retreat display): during the player retreat energy-selection screen the Active card no longer shows its energies stacked above it (they're already listed as selectable cards in the same array). Added a show_energies flag to build_pokemon_slot_with_energies_and_hp (HP still shown); display_hand_cards_array hides the stack for the retreat Active and enlarges that card 50% so it stands out. Debug: 'ISSUE #46 FIX ACTIVE'.
+FIX 2026-07-22 (ISSUE #46 retest — raise energy cards): during the player retreat energy-selection screen the small energy cards are now raised RETREAT_ENERGY_RAISE_PX (300px, tweakable const in Main_Match_Core) so their centre lines up with the enlarged Active card's centre instead of their bottoms sitting on the HP-label line. Done by bottom-aligning each energy card in a VBox with a 300px spacer beneath. Debug: 'ISSUE #46 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>Fix is working, however raise the position of the energy cards up by about 300 pixels so the middle of the energy cards are in line horizontal with the middle of the active pokemon card. Currently the energy card bottom and the HP label underneath the active pokemon are all in a line. Keep active pokemon looking as is but move the energy cards up to be not on the line at the bottom but aligned centrally</t>
+        </is>
+      </c>
+      <c r="F48" s="8" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H48" s="9" t="inlineStr">
+      <c r="G48" s="9" t="inlineStr">
         <is>
           <t>21/07/2026</t>
         </is>
@@ -2337,153 +2350,242 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="C49" s="7" t="n"/>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>When last prize card is taken, immediately check there and then if it's the last prize card. If so, stop the player/opponent switching in a new active pokemon. currently a prize card is taken, a new active pokemon is switched in, message is shown X set X as their active pokemon, then it pops up with "X took X last prize card!", then congratulations: You won/lost!!!!!". Just redundant to swap in a new pokemon when last prize is taken. Also if the player wins, the "end turn" floating label pops up too at the same time as the congrats you won message so stop this too.</t>
+        </is>
+      </c>
       <c r="D49" s="8" t="inlineStr">
         <is>
-          <t>When last prize card is taken, immediately check there and then if it's the last prize card. If so, stop the player/opponent switching in a new active pokemon. currently a prize card is taken, a new active pokemon is switched in, message is shown X set X as their active pokemon, then it pops up with "X took X last prize card!", then congratulations: You won/lost!!!!!". Just redundant to swap in a new pokemon when last prize is taken. Also if the player wins, the "end turn" floating label pops up too at the same time as the congrats you won message so stop this too.</t>
-        </is>
-      </c>
-      <c r="E49" s="9" t="inlineStr">
-        <is>
           <t>FIX 2026-07-21 (ISSUE #47 last prize / win): in check_all_knockouts the last-prize win is now checked BEFORE handle_post_knockout, so when the final prize is taken the game ends immediately instead of pointlessly promoting a new Active + showing 'set X as active'. Also player_end_turn_checks bails early when game_is_over, so the 'End turn' floating label no longer flashes over the 'You won!' message. Debug: 'ISSUE #47 FIX ACTIVE'.</t>
         </is>
       </c>
-      <c r="F49" s="8" t="n"/>
-      <c r="G49" s="8" t="inlineStr">
+      <c r="E49" s="8" t="n"/>
+      <c r="F49" s="8" t="inlineStr">
+        <is>
+          <t>Issue Resolved</t>
+        </is>
+      </c>
+      <c r="G49" s="9" t="inlineStr">
+        <is>
+          <t>21/07/2026</t>
+        </is>
+      </c>
+      <c r="H49" s="6" t="n">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="7" t="n">
+        <v>48</v>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>Blind message plays twice when sand attack is used. Only one message is required for "X must flip a coin to attack next turn"</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>FIX 2026-07-22 (ISSUE #48 — Sand Attack double message): the blind (is_blind) and flip_attack_block (attack_flip_blocked) systems are the SAME mechanic and BOTH are checked in the generic attack path, so Sand-Attack/Smokescreen text matched both parse rules -&gt; two 'must flip' messages AND two coin flips. parse_card_text_effects (Attack_Effects.gd) now records _blind_parsed and only arms flip_attack_block when blind did NOT match, so exactly one system arms per attack. Debug: 'ISSUE #48 FIX ACTIVE' (via parse prints).</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="n"/>
+      <c r="F50" s="8" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H49" s="9" t="inlineStr">
-        <is>
-          <t>21/07/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="7" t="n"/>
-      <c r="B50" s="7" t="n"/>
-      <c r="C50" s="7" t="n"/>
-      <c r="D50" s="8" t="n"/>
-      <c r="E50" s="9" t="n"/>
-      <c r="F50" s="8" t="n"/>
-      <c r="G50" s="8" t="n"/>
-      <c r="H50" s="9" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="7" t="n"/>
-      <c r="B51" s="7" t="n"/>
-      <c r="C51" s="7" t="n"/>
-      <c r="D51" s="8" t="n"/>
-      <c r="E51" s="9" t="n"/>
-      <c r="F51" s="8" t="n"/>
-      <c r="G51" s="8" t="n"/>
-      <c r="H51" s="9" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="7" t="n"/>
-      <c r="B52" s="7" t="n"/>
-      <c r="C52" s="7" t="n"/>
-      <c r="D52" s="8" t="n"/>
-      <c r="E52" s="9" t="n"/>
-      <c r="F52" s="8" t="n"/>
-      <c r="G52" s="8" t="n"/>
-      <c r="H52" s="9" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="7" t="n"/>
-      <c r="B53" s="7" t="n"/>
-      <c r="C53" s="7" t="n"/>
-      <c r="D53" s="8" t="n"/>
-      <c r="E53" s="9" t="n"/>
-      <c r="F53" s="8" t="n"/>
-      <c r="G53" s="8" t="n"/>
-      <c r="H53" s="9" t="n"/>
+      <c r="G50" s="9" t="inlineStr">
+        <is>
+          <t>22/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="90" customHeight="1">
+      <c r="A51" s="7" t="n">
+        <v>49</v>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>CPU logic</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>Opponent didn't retreat when they should have. Opponent had a sandshrew, 10hp, poisoned about to die. Opponent didn't retreat. 
+CPU considering retreat: guaranteed KO threat and cannot KO back
+CPU retreat not worthwhile: would lose 1 energy and cannot attack from bench
+CPU retreat not worthwhile: energy loss too high
+Even though they could attach an energy to the new active pokemon/a bench pokemon. Opp should DEFINITELY have retreated here as poison is a guarntee kill at the end of their turn AND they had 1 prize card left so it lost the game.</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>FIX 2026-07-22 (ISSUE #49 — CPU retreat a doomed Active): is_retreat_cost_worthwhile (CPU_AI.gd) now returns true when the Active is DOOMED where it stands: poisoned with current_hp &lt;= poison_damage (retreating leaves the Active spot which CLEARS the poison, saving it) OR guaranteed KO with a surviving bench (deny the prize). Overrides the R.4 high-HP/high-investment requirement that wrongly excluded low-HP doomed Pokemon like a 10-HP Sandshrew. Debug: 'ISSUE #49 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="n"/>
+      <c r="F51" s="8" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="G51" s="9" t="inlineStr">
+        <is>
+          <t>22/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="60" customHeight="1">
+      <c r="A52" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>Pack opening</t>
+        </is>
+      </c>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>Pack opening fails entirely at the point the pack is "ripped" open and trying to display the cards
+E 0:21:58:261   _start_pack_opening: Cannot call method 'get_width' on a null value.
+  &lt;GDScript Source&gt;Pack_Opening_Manager.gd:260 @ _start_pack_opening()
+  &lt;Stack Trace&gt; Pack_Opening_Manager.gd:260 @ _start_pack_opening()</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>FIX 2026-07-22 (ISSUE #50 — pack opening crash): CARDBACK_PATH pointed at res://Image_Assets/Sleeves/cardback.png which does not exist -&gt; _load_texture returned null -&gt; get_width() on null crashed at Pack_Opening_Manager.gd:260. Now resolves the player's equipped sleeve (new _resolve_player_cardback_path, mirroring the match) and falls back to the default 1_Default_English.png, with a null-guard before get_width(). Fixed the same dead cardback.png path in Holo_Rare_Shop_Script.gd. Debug: 'ISSUE #50 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="n"/>
+      <c r="F52" s="8" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="G52" s="9" t="inlineStr">
+        <is>
+          <t>22/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="60" customHeight="1">
+      <c r="A53" s="7" t="n">
+        <v>51</v>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>Player input</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>Pressing space bar when asked yes or no to open the shop menu errors. Pressing space bar should accept "yes" to opening the shop
+E 0:00:29:143   _unhandled_input: Cannot call method 'set_input_as_handled' on a null value.
+  &lt;GDScript Source&gt;Player_Object_Script.gd:140 @ _unhandled_input()
+  &lt;Stack Trace&gt; Player_Object_Script.gd:140 @ _unhandled_input()</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>FIX 2026-07-22 (ISSUE #51 — spacebar shop crash): Player_Object_Script.gd _unhandled_input called get_viewport().set_input_as_handled() AFTER MapManager.handle_message_spacebar(), which (on 'yes') triggers a scene change that frees the player node -&gt; get_viewport() null -&gt; crash at line 140. Now grabs the viewport and marks the input handled BEFORE calling the handler, guarded for null. Debug: 'ISSUE #51 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="n"/>
+      <c r="F53" s="8" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="G53" s="9" t="inlineStr">
+        <is>
+          <t>22/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="7" t="n"/>
       <c r="B54" s="7" t="n"/>
-      <c r="C54" s="7" t="n"/>
+      <c r="C54" s="8" t="n"/>
       <c r="D54" s="8" t="n"/>
-      <c r="E54" s="9" t="n"/>
+      <c r="E54" s="8" t="n"/>
       <c r="F54" s="8" t="n"/>
-      <c r="G54" s="8" t="n"/>
-      <c r="H54" s="9" t="n"/>
+      <c r="G54" s="9" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="n"/>
       <c r="B55" s="7" t="n"/>
-      <c r="C55" s="7" t="n"/>
+      <c r="C55" s="8" t="n"/>
       <c r="D55" s="8" t="n"/>
-      <c r="E55" s="9" t="n"/>
+      <c r="E55" s="8" t="n"/>
       <c r="F55" s="8" t="n"/>
-      <c r="G55" s="8" t="n"/>
-      <c r="H55" s="9" t="n"/>
+      <c r="G55" s="9" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="n"/>
       <c r="B56" s="7" t="n"/>
-      <c r="C56" s="7" t="n"/>
+      <c r="C56" s="8" t="n"/>
       <c r="D56" s="8" t="n"/>
-      <c r="E56" s="9" t="n"/>
+      <c r="E56" s="8" t="n"/>
       <c r="F56" s="8" t="n"/>
-      <c r="G56" s="8" t="n"/>
-      <c r="H56" s="9" t="n"/>
+      <c r="G56" s="9" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="n"/>
       <c r="B57" s="7" t="n"/>
-      <c r="C57" s="7" t="n"/>
+      <c r="C57" s="8" t="n"/>
       <c r="D57" s="8" t="n"/>
-      <c r="E57" s="9" t="n"/>
+      <c r="E57" s="8" t="n"/>
       <c r="F57" s="8" t="n"/>
-      <c r="G57" s="8" t="n"/>
-      <c r="H57" s="9" t="n"/>
+      <c r="G57" s="9" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="n"/>
       <c r="B58" s="7" t="n"/>
-      <c r="C58" s="7" t="n"/>
+      <c r="C58" s="8" t="n"/>
       <c r="D58" s="8" t="n"/>
-      <c r="E58" s="9" t="n"/>
+      <c r="E58" s="8" t="n"/>
       <c r="F58" s="8" t="n"/>
-      <c r="G58" s="8" t="n"/>
-      <c r="H58" s="9" t="n"/>
+      <c r="G58" s="9" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="n"/>
       <c r="B59" s="7" t="n"/>
-      <c r="C59" s="7" t="n"/>
+      <c r="C59" s="8" t="n"/>
       <c r="D59" s="8" t="n"/>
-      <c r="E59" s="9" t="n"/>
+      <c r="E59" s="8" t="n"/>
       <c r="F59" s="8" t="n"/>
-      <c r="G59" s="8" t="n"/>
-      <c r="H59" s="9" t="n"/>
+      <c r="G59" s="9" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="n"/>
       <c r="B60" s="7" t="n"/>
-      <c r="C60" s="7" t="n"/>
+      <c r="C60" s="8" t="n"/>
       <c r="D60" s="8" t="n"/>
-      <c r="E60" s="9" t="n"/>
+      <c r="E60" s="8" t="n"/>
       <c r="F60" s="8" t="n"/>
-      <c r="G60" s="8" t="n"/>
-      <c r="H60" s="9" t="n"/>
+      <c r="G60" s="9" t="n"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:G1048576">
-    <cfRule type="expression" priority="16" dxfId="2">
-      <formula>$G2="Issue Resolved"</formula>
+  <conditionalFormatting sqref="A2:F1048576">
+    <cfRule type="expression" priority="46" dxfId="2">
+      <formula>$F2="Issue Resolved"</formula>
     </cfRule>
-    <cfRule type="expression" priority="17" dxfId="1">
-      <formula>$G2="Untested Fix"</formula>
+    <cfRule type="expression" priority="47" dxfId="1">
+      <formula>$F2="Untested Fix"</formula>
     </cfRule>
-    <cfRule type="expression" priority="18" dxfId="0">
-      <formula>OR($G2="New Issue",$G2="Fix Failed")</formula>
+    <cfRule type="expression" priority="48" dxfId="0">
+      <formula>OR($F2="New Issue",$F2="Fix Failed",$F2="Improve Further")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>StatusList</formula1>
     </dataValidation>
   </dataValidations>
@@ -5905,7 +6007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14.140625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5942,6 +6044,13 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>Improve Further</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>Fix Failed</t>
         </is>
       </c>

</xml_diff>

<commit_message>
UI: Converted all Sleeves into small and compressed image to help with the sleeve sub menu loading being quicker
</commit_message>
<xml_diff>
--- a/Spreadsheets/Issue_Log.xlsx
+++ b/Spreadsheets/Issue_Log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\Spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65A32022-0957-4244-8A7B-6421C3FE1AA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEB6E44E-C8D2-4837-A795-65565A52F0D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Game_Issues" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1020" uniqueCount="710">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1026" uniqueCount="712">
   <si>
     <t>#</t>
   </si>
@@ -2211,10 +2211,17 @@
     <t>Fix Failed</t>
   </si>
   <si>
-    <t>Make the darkened input blocker on the deck builder mode 1) 46 pixels taller above the rectangle 2) 179 pixels longer below the rectangle 3) 315 pixels width shorter than the right hand side of the screen 4) Make it 50% more transparent. If the opacity is currently 30% make it 15% so easier to see through and less flashing when moving sets quickly</t>
-  </si>
-  <si>
     <t>There is a big black screen delay now when returning to the main menu from a sub menu presumably because it has to load the main map in again from nothing. Coming to think about this further, the only reason I unloaded the map to reload is because going into sub menus may change the overworld in some way but realistically all that CAN change is the player's sprite. All other sub menus are for in match changes (deck/sleeves/coin). Change the sub menu then to never unload the map scene just like how we keep the main menu scene visible over it, so that there is no delay returning then simply refresh the player sprite after the main menu loads in case the player changed their sprite in the sub menu</t>
+  </si>
+  <si>
+    <t>Make the darkened input blocker on the deck builder mode 1) 46 pixels taller above the rectangle 2) 179 pixels longer below the rectangle (bottom of the screen) 3) 315 pixels width shorter than the right hand side of the screen 4) Make it 50% more transparent. If the opacity is currently 30% make it 15% so easier to see through and less flashing when moving sets quickly
+This input blocker needs to be a different size for coins, sleeves and costumes. The deck builder mode is a different layout and size. For the coin sleeve and costume input blocker 1) perform the same transparency change but 2) Increase vertical size above the rectangle 45 pixels taller 3) increase vertical size 42 pixels below the rectangle.</t>
+  </si>
+  <si>
+    <t>When an attack does no damage at all (the attack does not have a damage number), ignore the weakness/resistance labels to ensure weakeness and resistance don't pop up when doing a no damage attack e.g Cubone using snivel against snorlax, a label pops up saying weakness x2 but of course it's a no damage move.</t>
+  </si>
+  <si>
+    <t>In the rewards screen when winning a costume the aspect ratio isn't presevered so the costume is stretched thin</t>
   </si>
 </sst>
 </file>
@@ -2814,14 +2821,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I74"/>
+  <dimension ref="A1:I76"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.85546875" style="2" customWidth="1"/>
     <col min="4" max="4" width="143.42578125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="255.5703125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="255.5703125" style="1" hidden="1" customWidth="1"/>
     <col min="6" max="6" width="188.7109375" style="1" customWidth="1"/>
     <col min="7" max="7" width="19" style="1" customWidth="1"/>
     <col min="8" max="9" width="11.140625" bestFit="1" customWidth="1"/>
@@ -3713,7 +3720,7 @@
         <v>108</v>
       </c>
       <c r="F34" s="8" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="G34" s="8" t="s">
         <v>706</v>
@@ -3768,7 +3775,7 @@
         <v>115</v>
       </c>
       <c r="G36" s="8" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="H36" s="9" t="s">
         <v>85</v>
@@ -4223,7 +4230,7 @@
         <v>160</v>
       </c>
       <c r="F54" s="8" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="G54" s="8" t="s">
         <v>706</v>
@@ -4672,6 +4679,31 @@
       </c>
       <c r="G74" s="1" t="s">
         <v>195</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="A75" s="2">
+        <v>73</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D75" s="1" t="s">
+        <v>710</v>
+      </c>
+      <c r="G75" s="1" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D76" s="1" t="s">
+        <v>711</v>
+      </c>
+      <c r="G76" s="1" t="s">
+        <v>705</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Debug: Bug fixes detailed in Issue Log
</commit_message>
<xml_diff>
--- a/Spreadsheets/Issue_Log.xlsx
+++ b/Spreadsheets/Issue_Log.xlsx
@@ -85,7 +85,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -106,71 +106,21 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="32">
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1F4E79"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBDD7EE"/>
-          <bgColor rgb="FFBDD7EE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1F4E79"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBDD7EE"/>
-          <bgColor rgb="FFBDD7EE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="16">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -304,42 +254,6 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1F4E79"/>
-      </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFBDD7EE"/>
@@ -348,87 +262,10 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFC6EFCE"/>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1F4E79"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBDD7EE"/>
-          <bgColor rgb="FFBDD7EE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -443,16 +280,8 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBDD7EE"/>
-          <bgColor rgb="FFBDD7EE"/>
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -850,7 +679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I84"/>
+  <dimension ref="A1:J95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3.42578125" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
@@ -861,6 +690,7 @@
     <col width="188.7109375" customWidth="1" style="1" min="6" max="6"/>
     <col width="19" customWidth="1" style="1" min="7" max="7"/>
     <col width="11.140625" bestFit="1" customWidth="1" min="8" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -909,6 +739,11 @@
           <t>Fixed</t>
         </is>
       </c>
+      <c r="J1" s="8" t="inlineStr">
+        <is>
+          <t>Debug</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="n">
@@ -993,6 +828,11 @@
       </c>
       <c r="I3" s="9" t="n">
         <v>46220</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
       </c>
     </row>
     <row r="4" ht="120" customHeight="1">
@@ -1223,6 +1063,11 @@
         </is>
       </c>
       <c r="I8" s="8" t="n"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Live: 3</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="6" t="n">
@@ -1391,6 +1236,11 @@
       </c>
       <c r="H12" s="8" t="n"/>
       <c r="I12" s="8" t="n"/>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="345" customHeight="1">
       <c r="A13" s="6" t="n">
@@ -1438,6 +1288,11 @@
         </is>
       </c>
       <c r="I13" s="8" t="n"/>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Live: 2</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="60" customHeight="1">
       <c r="A14" s="6" t="n">
@@ -1476,6 +1331,11 @@
       </c>
       <c r="H14" s="8" t="n"/>
       <c r="I14" s="8" t="n"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="6" t="n">
@@ -1751,7 +1611,7 @@
       <c r="H21" s="9" t="n">
         <v>46221</v>
       </c>
-      <c r="I21" s="11" t="inlineStr">
+      <c r="I21" s="10" t="inlineStr">
         <is>
           <t>24/07/2026</t>
         </is>
@@ -1791,6 +1651,11 @@
         <v>46221</v>
       </c>
       <c r="I22" s="8" t="n"/>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Live: 2</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="45" customHeight="1">
       <c r="A23" s="6" t="n">
@@ -1826,6 +1691,11 @@
         <v>46221</v>
       </c>
       <c r="I23" s="8" t="n"/>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="6" t="n">
@@ -1896,6 +1766,11 @@
         <v>46221</v>
       </c>
       <c r="I25" s="8" t="n"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Live: 4</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="75" customHeight="1">
       <c r="A26" s="6" t="n">
@@ -1938,6 +1813,11 @@
         </is>
       </c>
       <c r="I26" s="8" t="n"/>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Live: 2</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="6" t="n">
@@ -1975,6 +1855,11 @@
         </is>
       </c>
       <c r="I27" s="8" t="n"/>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Live: 2</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="75" customHeight="1">
       <c r="A28" s="6" t="n">
@@ -2055,7 +1940,7 @@
           <t>21/07/2026</t>
         </is>
       </c>
-      <c r="I29" s="11" t="inlineStr">
+      <c r="I29" s="10" t="inlineStr">
         <is>
           <t>24/07/2026</t>
         </is>
@@ -2096,7 +1981,7 @@
           <t>21/07/2026</t>
         </is>
       </c>
-      <c r="I30" s="11" t="inlineStr">
+      <c r="I30" s="10" t="inlineStr">
         <is>
           <t>24/07/2026</t>
         </is>
@@ -2137,7 +2022,7 @@
           <t>21/07/2026</t>
         </is>
       </c>
-      <c r="I31" s="11" t="inlineStr">
+      <c r="I31" s="10" t="inlineStr">
         <is>
           <t>24/07/2026</t>
         </is>
@@ -2178,7 +2063,7 @@
           <t>21/07/2026</t>
         </is>
       </c>
-      <c r="I32" s="11" t="inlineStr">
+      <c r="I32" s="10" t="inlineStr">
         <is>
           <t>24/07/2026</t>
         </is>
@@ -2219,7 +2104,7 @@
           <t>21/07/2026</t>
         </is>
       </c>
-      <c r="I33" s="11" t="inlineStr">
+      <c r="I33" s="10" t="inlineStr">
         <is>
           <t>24/07/2026</t>
         </is>
@@ -2252,18 +2137,19 @@
 </t>
         </is>
       </c>
-      <c r="E34" s="7" t="inlineStr">
+      <c r="E34" s="12" t="inlineStr">
         <is>
           <t>FIX 2026-07-21 (ISSUE #32 loading crash + overlay): the async grid-load loops called get_tree().process_frame after the scene was freed by Escape/Cancel -&gt; null get_tree() crash. Added 'if not is_inside_tree(): return' guards to the load loops in Sleeves, Costume, Coin Case and Deck builder (incl. the two spots the user flagged with ##### ERROR comments). Sleeves also gains a loading overlay (input-blocking dim CanvasLayer + spinning square + 'Loading...'; Escape still cancels via _load_cancelled). NOTE: the loading overlay is currently only wired into Sleeves (worst case); the crash guard covers all four. The preload-at-startup / WebP redesign was intentionally NOT coded (user said so). Debug: 'ISSUE #32 FIX ACTIVE'.
 FIX 2026-07-22 (ISSUE #32 retest — spinner on all libraries): extracted the Sleeves loading overlay into a shared MenuLoadingOverlay (Scripts/Menu_Scripts/Menu_Loading_Overlay.gd) and wired it into Costume, Coin Case AND the Deck/Card builder. Deck builder shows it in _display_current_set every set load/switch (show() auto-replaces so rapid switches never stack). Debug: 'ISSUE #32 FIX ACTIVE'. Preload/WebP redesign still intentionally NOT done.
 FIX 23/07/2026 (ISSUE #32 retest): MenuLoadingOverlay.show() now takes icon_offset_x + blocker top/bottom insets. Deck screen passes (-150, 142, 134) so the loading icon shifts 150px left of the ~300px right banner and the top 142px/bottom 134px stay clickable (Cancel + set-switch). Costume/Coin pass (0,142,134); Sleeves inline overlay dim inset the same 142/134. Debug: ISSUE #32 FIX ACTIVE.
 FIX 24/07/2026 (ISSUE #32 retest — blocker geometry + opacity): all loading-overlay tuning now lives in named constants at the top of Scripts/Menu_Scripts/Menu_Loading_Overlay.gd. DIM_ALPHA 0.55 -&gt; 0.275 (halved, per '50% more transparent'). Added a new blocker_right_inset parameter plus two presets: show_for_deck() = icon_x -150, top inset 96 (46px taller above), bottom inset -45 (179px longer below, i.e. now runs to/past the screen bottom), right inset 315 (stops 315px short of the right edge); show_for_library() = icon_x 0, top inset 97 (45px taller above), bottom inset 92 (42px lower). Deck builder / Coin Case / Costume switched to the presets. ALSO: the Sleeves screen still had its own INLINE copy of the overlay (which is why it kept missing these tweaks) — it now uses the shared MenuLoadingOverlay too, so there is only one place left to tune. Debug: 'ISSUE #32 FIX ACTIVE'.
-FIX 25/07/2026 (ISSUE #32 retest): Menu_Loading_Overlay.show() gained blocker_left_inset + icon_offset_y params. Deck preset now DECK_LEFT_INSET=-78 (blocker extends 78px further left = 78px wider) and DECK_ICON_OFFSET_Y=11 (box moved 11px down). Debug: 'ISSUE #32 FIX ACTIVE'.</t>
+FIX 25/07/2026 (ISSUE #32 retest): Menu_Loading_Overlay.show() gained blocker_left_inset + icon_offset_y params. Deck preset now DECK_LEFT_INSET=-78 (blocker extends 78px further left = 78px wider) and DECK_ICON_OFFSET_Y=11 (box moved 11px down). Debug: 'ISSUE #32 FIX ACTIVE'.
+FIX 26/07/2026 (ISSUE #32 retest — 78px on the RIGHT, not the left): the previous attempt widened the deck blocker leftward. Reverted DECK_LEFT_INSET -78 -&gt; 0 and dropped DECK_RIGHT_INSET 315 -&gt; 237, so the blocker now extends 78px FURTHER RIGHT and the overall width matches what was last tested, just moved to the right edge. All geometry still lives in the named consts at the top of Scripts/Menu_Scripts/Menu_Loading_Overlay.gd. Debug: 'ISSUE #32 FIX ACTIVE'.</t>
         </is>
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>In deck builder mode make the width of the input blocker 78 pixels wider so it extends to the left 78 pixels more. Move the box 11 pixels downwards.</t>
+          <t xml:space="preserve">Sorry - fix failed on this was my fault, I said extend left, I meant extend right.In deck builder mode make the width of the input blocker 78 pixels wider so it extends to the right 78 pixels more. </t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
@@ -2277,6 +2163,11 @@
         </is>
       </c>
       <c r="I34" s="8" t="n"/>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="75" customHeight="1">
       <c r="A35" s="6" t="n">
@@ -2318,7 +2209,7 @@
           <t>21/07/2026</t>
         </is>
       </c>
-      <c r="I35" s="11" t="inlineStr">
+      <c r="I35" s="10" t="inlineStr">
         <is>
           <t>24/07/2026</t>
         </is>
@@ -2367,7 +2258,7 @@
           <t>21/07/2026</t>
         </is>
       </c>
-      <c r="I36" s="11" t="inlineStr">
+      <c r="I36" s="10" t="inlineStr">
         <is>
           <t>24/07/2026</t>
         </is>
@@ -2415,6 +2306,11 @@
         </is>
       </c>
       <c r="I37" s="8" t="n"/>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Live: 4</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="60" customHeight="1">
       <c r="A38" s="6" t="n">
@@ -2452,6 +2348,11 @@
         </is>
       </c>
       <c r="I38" s="8" t="n"/>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="45" customHeight="1">
       <c r="A39" s="6" t="n">
@@ -2493,7 +2394,7 @@
           <t>21/07/2026</t>
         </is>
       </c>
-      <c r="I39" s="11" t="inlineStr">
+      <c r="I39" s="10" t="inlineStr">
         <is>
           <t>24/07/2026</t>
         </is>
@@ -2542,6 +2443,11 @@
         </is>
       </c>
       <c r="I40" s="8" t="n"/>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="45" customHeight="1">
       <c r="A41" s="6" t="n">
@@ -2621,7 +2527,7 @@
           <t>22/07/2026</t>
         </is>
       </c>
-      <c r="I42" s="11" t="inlineStr">
+      <c r="I42" s="10" t="inlineStr">
         <is>
           <t>24/07/2026</t>
         </is>
@@ -2662,7 +2568,7 @@
           <t>21/07/2026</t>
         </is>
       </c>
-      <c r="I43" s="11" t="inlineStr">
+      <c r="I43" s="10" t="inlineStr">
         <is>
           <t>24/07/2026</t>
         </is>
@@ -2743,6 +2649,11 @@
         </is>
       </c>
       <c r="I45" s="8" t="n"/>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="60" customHeight="1">
       <c r="A46" s="6" t="n">
@@ -2787,6 +2698,11 @@
       <c r="I46" s="9" t="n">
         <v>46225</v>
       </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="90" customHeight="1">
       <c r="A47" s="6" t="n">
@@ -2824,6 +2740,11 @@
         </is>
       </c>
       <c r="I47" s="8" t="n"/>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="75" customHeight="1">
       <c r="A48" s="6" t="n">
@@ -2942,7 +2863,7 @@
           <t>22/07/2026</t>
         </is>
       </c>
-      <c r="I50" s="11" t="inlineStr">
+      <c r="I50" s="10" t="inlineStr">
         <is>
           <t>24/07/2026</t>
         </is>
@@ -2988,6 +2909,11 @@
         </is>
       </c>
       <c r="I51" s="8" t="n"/>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Live: 2</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="60" customHeight="1">
       <c r="A52" s="6" t="n">
@@ -3027,7 +2953,7 @@
           <t>22/07/2026</t>
         </is>
       </c>
-      <c r="I52" s="11" t="inlineStr">
+      <c r="I52" s="10" t="inlineStr">
         <is>
           <t>24/07/2026</t>
         </is>
@@ -3071,7 +2997,7 @@
           <t>22/07/2026</t>
         </is>
       </c>
-      <c r="I53" s="11" t="inlineStr">
+      <c r="I53" s="10" t="inlineStr">
         <is>
           <t>24/07/2026</t>
         </is>
@@ -3356,7 +3282,7 @@
       <c r="F60" s="7" t="n"/>
       <c r="G60" s="7" t="inlineStr">
         <is>
-          <t>Untested Fix</t>
+          <t>Issue Resolved</t>
         </is>
       </c>
       <c r="H60" s="8" t="inlineStr">
@@ -3364,7 +3290,11 @@
           <t>23/07/2026</t>
         </is>
       </c>
-      <c r="I60" s="8" t="n"/>
+      <c r="I60" s="8" t="inlineStr">
+        <is>
+          <t>26/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="45" customHeight="1">
       <c r="A61" s="6" t="n">
@@ -3385,15 +3315,19 @@
           <t>Show tool cards above energy cards for bench pokemon so that they are also shown "attached"</t>
         </is>
       </c>
-      <c r="E61" s="8" t="inlineStr">
+      <c r="E61" s="12" t="inlineStr">
         <is>
           <t>FIX 23/07/2026 (ISSUE #59): build_pokemon_slot_with_energies_and_hp now renders attached tool/trainer cards stacked ABOVE the energy cards for BENCH Pokemon (Active shows them via display_attached_trainer_cards). Debug: ISSUE #59 FIX ACTIVE.
-FIX 25/07/2026 (ISSUE #59 retest — 3 sub-issues): (1) Z-ORDER: bench tools now iterate highest-first (reverse), like the energy stack, so the tool closest to the card renders in FRONT instead of behind. (2) REFRESH: tick_defender_counters now also calls display_pokemon(is_opponent) after discarding, so a Defender expiring on a BENCH Pokemon is refreshed immediately (display_attached_trainer_cards only refreshes the ACTIVE) — it no longer lingers until the next defender attaches. (3) Y-ALIGN: player_active_pokemon_attached_cards moved offset_top 413-&gt;366 in the scene to match the opponent's Y. Debug: 'ISSUE #59 FIX ACTIVE'.</t>
+FIX 25/07/2026 (ISSUE #59 retest — 3 sub-issues): (1) Z-ORDER: bench tools now iterate highest-first (reverse), like the energy stack, so the tool closest to the card renders in FRONT instead of behind. (2) REFRESH: tick_defender_counters now also calls display_pokemon(is_opponent) after discarding, so a Defender expiring on a BENCH Pokemon is refreshed immediately (display_attached_trainer_cards only refreshes the ACTIVE) — it no longer lingers until the next defender attaches. (3) Y-ALIGN: player_active_pokemon_attached_cards moved offset_top 413-&gt;366 in the scene to match the opponent's Y. Debug: 'ISSUE #59 FIX ACTIVE'.
+FIX 26/07/2026 (ISSUE #59 retest — both sub-issues):
+(1) Z-ORDER — the real cause. Godot draws sibling Controls in CHILD ORDER (last added = in front), and the bench tool block ran AFTER the energy block, so every tool rendered in front of the topmost energy card even though it sits further up the stack. Reversing the two blocks in build_pokemon_slot_with_energies_and_hp fixes it: the slot is now built strictly back-to-front (highest tool -&gt; lowest tool -&gt; highest energy -&gt; lowest energy -&gt; Pokemon card). Last time only the iteration order WITHIN the tool loop was reversed, which ordered tools against each other but never against the energies.
+(2) REFRESH BEFORE MESSAGE — every tool-attach path now calls main.display_pokemon() before show_message(), so the tool is visibly attached while the message is on screen: PlusPower, Defender (CPU), Defender (player, Active AND Bench). The bench case mattered most since a bench Pokemon's tools are drawn by display_pokemon, not display_attached_trainer_cards (which only rebuilds the Active's tool stack).
+Debug: 'ISSUE #59 FIX ACTIVE' (the z-order print is one-shot per match — it sits in the per-slot draw path, so an unconditional print produced dozens of lines per attack).</t>
         </is>
       </c>
       <c r="F61" s="7" t="inlineStr">
         <is>
-          <t>A few issues. 1) The tool card z index is reveresed so each tool card is placed in front instead of behind 2) the tools don't get refreshed when the screen refreshes at the end of the turn. The defenders did not appear to be discarded and instead only vanished when the next defender was attached to the active pokemon. 3) Tool position is different for player's active pokemon compared to opponent's active pokemon. Ensure the on screen position Y positioning is the same for both player and opponent (use the opponent's Y position for the tools)</t>
+          <t>1) Tool card Z index still not correct.  2) Refresh the board view before displaying the message that the tool was attached to X so it can be visibly seen attached before the message pops up</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
@@ -3407,6 +3341,11 @@
         </is>
       </c>
       <c r="I61" s="8" t="n"/>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>Live: 3</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="30" customHeight="1">
       <c r="A62" s="6" t="n">
@@ -3444,6 +3383,11 @@
         </is>
       </c>
       <c r="I62" s="8" t="n"/>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="135" customHeight="1">
       <c r="A63" s="6" t="n">
@@ -3483,6 +3427,11 @@
         </is>
       </c>
       <c r="I63" s="8" t="n"/>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>Live: 3</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="6" t="n">
@@ -3557,6 +3506,11 @@
         </is>
       </c>
       <c r="I65" s="8" t="n"/>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>Live: 2</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="6" t="n">
@@ -3622,7 +3576,7 @@
       <c r="F67" s="7" t="n"/>
       <c r="G67" s="7" t="inlineStr">
         <is>
-          <t>Untested Fix</t>
+          <t>Issue Resolved</t>
         </is>
       </c>
       <c r="H67" s="8" t="inlineStr">
@@ -3630,7 +3584,11 @@
           <t>23/07/2026</t>
         </is>
       </c>
-      <c r="I67" s="8" t="n"/>
+      <c r="I67" s="8" t="inlineStr">
+        <is>
+          <t>26/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="6" t="n">
@@ -3659,7 +3617,7 @@
         </is>
       </c>
       <c r="H68" s="8" t="n"/>
-      <c r="I68" s="11" t="inlineStr">
+      <c r="I68" s="10" t="inlineStr">
         <is>
           <t>24/07/2026</t>
         </is>
@@ -3759,6 +3717,11 @@
         </is>
       </c>
       <c r="I71" s="8" t="n"/>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>Live: 2</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="6" t="n">
@@ -3787,7 +3750,7 @@
       <c r="F72" s="7" t="n"/>
       <c r="G72" s="7" t="inlineStr">
         <is>
-          <t>Untested Fix</t>
+          <t>Issue Resolved</t>
         </is>
       </c>
       <c r="H72" s="8" t="inlineStr">
@@ -3795,7 +3758,11 @@
           <t>23/07/2026</t>
         </is>
       </c>
-      <c r="I72" s="8" t="n"/>
+      <c r="I72" s="8" t="inlineStr">
+        <is>
+          <t>26/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="6" t="n">
@@ -3833,6 +3800,11 @@
         </is>
       </c>
       <c r="I73" s="8" t="n"/>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="6" t="n">
@@ -3890,15 +3862,19 @@
       <c r="F75" s="7" t="n"/>
       <c r="G75" s="7" t="inlineStr">
         <is>
-          <t>Untested Fix</t>
-        </is>
-      </c>
-      <c r="H75" s="11" t="inlineStr">
+          <t>Issue Resolved</t>
+        </is>
+      </c>
+      <c r="H75" s="10" t="inlineStr">
         <is>
           <t>24/07/2026</t>
         </is>
       </c>
-      <c r="I75" s="8" t="n"/>
+      <c r="I75" s="8" t="inlineStr">
+        <is>
+          <t>26/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="45" customHeight="1">
       <c r="A76" s="6" t="n">
@@ -3930,7 +3906,7 @@
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H76" s="11" t="inlineStr">
+      <c r="H76" s="10" t="inlineStr">
         <is>
           <t>24/07/2026</t>
         </is>
@@ -3956,23 +3932,39 @@
           <t>Opponent used Lass when there were 3 other trainer cards in it's hand. Create a more detailed calculation for when the opponent should play lass. E.g if the player only has less than 3 cards in their hand then most likely no reason to play Lass. Don't play lass if opponent's hand is greater than 1/5th trainers. calculation should be something like P = (#OfCardsInOpponentHand-(#OfTrainersInOpponentHand*2)) * (#OfCardsInPlayerHand)) and then only use Lass if P &gt; 50. Do some calculations on this with some numbers to make sure it roughly lines up with how a human would play this card with gambling if it's worth it or not. Also if the opponent has 2 lasses in their hand then ignore that as a trainer card so when doing the count of amount of trainers, ignore other lasses. Also always use lass LAST before any attack. Run through all the priorities, trainer cards, energy attaching, evolving etc first and then only use lass as the last card before moving to the attack stage. (E.g if the opponnt has energy search, pokemon trader, bill and 2x lass in their hand, no point evaluting lass at that point as they should use all the other trainers they can first and then use lass to force the opponent into shuffling any of their trainers away.</t>
         </is>
       </c>
-      <c r="E77" s="7" t="inlineStr">
-        <is>
-          <t>FIX 24/07/2026 (ISSUE #74 Lass): _cpu_score_lass (CPU_AI.gd) rewritten to the requested profitability model. P = (own hand size - 2 * own Trainers) * player hand size, and Lass is only played when P &gt; 50. Other copies of Lass in the CPU's own hand are NOT counted as Trainers (they'd be shuffled away anyway, so losing a duplicate costs nothing). Two hard gates first: never play it when more than 1/5 of our hand is Trainers, and never against a player holding fewer than 3 cards. Above the bar the score scales 35..65 with how far past 50 P is. Sanity check: 7-card Trainer-light hand vs an 8-card player hand = 56 -&gt; plays; vs a 7-card hand = 49 -&gt; holds; any real Trainer in a 5-6 card hand fails the 1/5 gate -&gt; holds. SECOND HALF: Lass is now always the LAST card played before attacking. It is skipped by both cpu_phase_play_trainer_cards_priority and _remaining (via the new LASS_UID const, base1-75 is the only card with this name) and played by the new cpu_phase_play_lass_last(), inserted into cpu_turn_orchestrator as Phase 7d — after powers, evolutions, bench plays, every other Trainer, energy attachment and both retreat passes, immediately before Phase 8 (attack). Respects the trainer lock, the match-effect trainer_discard_cost threshold and validate_trainer_can_be_played. Debug: 'ISSUE #74 FIX ACTIVE'.</t>
-        </is>
-      </c>
-      <c r="F77" s="7" t="n"/>
+      <c r="E77" s="12" t="inlineStr">
+        <is>
+          <t>FIX 24/07/2026 (ISSUE #74 Lass): _cpu_score_lass (CPU_AI.gd) rewritten to the requested profitability model. P = (own hand size - 2 * own Trainers) * player hand size, and Lass is only played when P &gt; 50. Other copies of Lass in the CPU's own hand are NOT counted as Trainers (they'd be shuffled away anyway, so losing a duplicate costs nothing). Two hard gates first: never play it when more than 1/5 of our hand is Trainers, and never against a player holding fewer than 3 cards. Above the bar the score scales 35..65 with how far past 50 P is. Sanity check: 7-card Trainer-light hand vs an 8-card player hand = 56 -&gt; plays; vs a 7-card hand = 49 -&gt; holds; any real Trainer in a 5-6 card hand fails the 1/5 gate -&gt; holds. SECOND HALF: Lass is now always the LAST card played before attacking. It is skipped by both cpu_phase_play_trainer_cards_priority and _remaining (via the new LASS_UID const, base1-75 is the only card with this name) and played by the new cpu_phase_play_lass_last(), inserted into cpu_turn_orchestrator as Phase 7d — after powers, evolutions, bench plays, every other Trainer, energy attachment and both retreat passes, immediately before Phase 8 (attack). Respects the trainer lock, the match-effect trainer_discard_cost threshold and validate_trainer_can_be_played. Debug: 'ISSUE #74 FIX ACTIVE'.
+FIX 26/07/2026 (ISSUE #74 retest — new formula, as specified): the old P multiplied by our OWN hand size, so the ideal case (a hand of nothing but Lass vs a full player hand) scored 7 and never fired. Own hand size is irrelevant. Now:
+    value = player hand size - 2.5 * (our own Trainers, EXCLUDING copies of Lass)
+    play Lass when value &gt;= 3
+Worked examples: player 7 / our Trainers 0 -&gt; 7.0 PLAY (the reported case); 7 / 1 -&gt; 4.5 play; 7 / 2 -&gt; 2.0 hold; 3 / 0 -&gt; 3.0 play; 2 / 0 -&gt; 2.0 hold. The &gt;= 3 threshold also subsumes the old 'never against a player holding fewer than 3 cards' gate, so that separate gate is gone.
+Kept the hard rule from the original issue text ('don't play Lass if more than 1/5 of the hand is Trainers'), now measured against the hand as it will be AFTER Lass is played (this Lass goes to the discard, so counting it understated the fraction). It uses the same non-Lass Trainer count, so a hand of only Lasses always passes. IF THIS GATE EVER HOLDS LASS WHEN YOU WANTED IT PLAYED, the console says so explicitly and LASS_MAX_TRAINER_FRACTION is the constant to change.
+All three numbers are named constants: LASS_TRAINER_PENALTY 2.5, LASS_MIN_VALUE 3.0, LASS_MAX_TRAINER_FRACTION 0.2. The 'Lass is played LAST, just before attacking' half from the 24/07 fix is unchanged. Debug: 'ISSUE #74 FIX ACTIVE (Lass)' prints the full value calculation every turn.</t>
+        </is>
+      </c>
+      <c r="F77" s="7" t="inlineStr">
+        <is>
+          <t>My formula is poor. Opponent has 1 single card (Lass) in their hand. Player has 7 cards in their hand. This resulted in [ (1 - 2*0) *7 ] which is 7. This should have been the perfect time to use Lass so we need a new formula. Something like:
+ if ((#OfCardsInPlayersHand)-(#OfTrainersInOpponentsHand*2.5) &gt;= 3, (where #OfTrainersInOpponentsHand excludes any copies of lass) then play lass.</t>
+        </is>
+      </c>
       <c r="G77" s="7" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H77" s="11" t="inlineStr">
+      <c r="H77" s="10" t="inlineStr">
         <is>
           <t>24/07/2026</t>
         </is>
       </c>
       <c r="I77" s="8" t="n"/>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>Live: 5</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="30" customHeight="1">
       <c r="A78" s="6" t="n">
@@ -4009,239 +4001,732 @@
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H78" s="11" t="inlineStr">
+      <c r="H78" s="10" t="inlineStr">
         <is>
           <t>24/07/2026</t>
         </is>
       </c>
       <c r="I78" s="8" t="n"/>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>Live: 2</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="30" customHeight="1">
-      <c r="A79" s="2" t="n">
+      <c r="A79" s="6" t="n">
         <v>76</v>
       </c>
-      <c r="B79" s="2" t="inlineStr">
+      <c r="B79" s="6" t="inlineStr">
         <is>
           <t>CPU logic</t>
         </is>
       </c>
-      <c r="C79" s="2" t="inlineStr">
+      <c r="C79" s="6" t="inlineStr">
         <is>
           <t>Prioritisation</t>
         </is>
       </c>
-      <c r="D79" s="10" t="inlineStr">
+      <c r="D79" s="11" t="inlineStr">
         <is>
           <t>Error with some recursive cards such as item finder and lass. Stack overflow (stack size: 1024). Check for infinite recursion in your
   script. seemed to be at "match card_id:</t>
         </is>
       </c>
-      <c r="G79" s="1" t="inlineStr">
+      <c r="E79" s="7" t="n"/>
+      <c r="F79" s="7" t="n"/>
+      <c r="G79" s="7" t="inlineStr">
         <is>
           <t>Issue Resolved</t>
         </is>
       </c>
-      <c r="H79" s="11" t="inlineStr">
+      <c r="H79" s="10" t="inlineStr">
         <is>
           <t>24/07/2026</t>
         </is>
       </c>
-      <c r="I79" s="12" t="inlineStr">
+      <c r="I79" s="10" t="inlineStr">
         <is>
           <t>24/07/2026</t>
         </is>
       </c>
     </row>
     <row r="80" ht="105" customHeight="1">
-      <c r="A80" s="2" t="n">
+      <c r="A80" s="6" t="n">
         <v>77</v>
       </c>
-      <c r="B80" s="2" t="inlineStr">
+      <c r="B80" s="6" t="inlineStr">
         <is>
           <t>Player input</t>
         </is>
       </c>
-      <c r="C80" s="2" t="inlineStr">
+      <c r="C80" s="6" t="inlineStr">
         <is>
           <t>Input</t>
         </is>
       </c>
-      <c r="D80" s="1" t="inlineStr">
+      <c r="D80" s="7" t="inlineStr">
         <is>
           <t>Clicking anywhere on screen when you are playing a card effect or retreating in which multiple cards need to be clicked and selected, clicking a blank space while a card is selected breaks the game UI/Logic/Confirm button. The button goes back to "Select a card" because the last click input there was no card selected even though there is a card selected still (animation plays and message reads 0 cards to be selected). Keep the mouse click clearing functionality for selected cards when selecting a SINGLE card like normal gameplay selecting a card from the hand, or once you have discarded energy to retreat and need to select ONE card from the bench functionality and apply it for all multiple card selections, clear all cards when a blank space is clicked or the right mouse button is clicked. End goal is at any point when a card is selected for an action, if you click a blank space, clear all selected cards (including stopping selection animations, clearing cached variables, updating the OK button to be the select a card etc etc</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr">
+      <c r="E80" s="8" t="inlineStr">
         <is>
           <t>FIX 25/07/2026 (ISSUE #77): added clear_current_action_selection() — a blank-space click now clears ALL selected cards for the in-progress action, SINGLE or MULTI-select (retreat energy discard, trainer discard, Pokedex reorder): stops each selection animation, empties the cached arrays, and resets the action button + hint to that mode's 'nothing selected' state WITHOUT cancelling the mode. Previously multi-select modes either did a partial single-card clear (button reset to 'Select A Card' while cards stayed selected) or bailed without clearing. Debug: 'ISSUE #77 FIX ACTIVE'.</t>
         </is>
       </c>
-      <c r="G80" s="1" t="inlineStr">
+      <c r="F80" s="7" t="n"/>
+      <c r="G80" s="7" t="inlineStr">
+        <is>
+          <t>Issue Resolved</t>
+        </is>
+      </c>
+      <c r="H80" s="10" t="inlineStr">
+        <is>
+          <t>25/07/2026</t>
+        </is>
+      </c>
+      <c r="I80" s="10" t="inlineStr">
+        <is>
+          <t>26/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="45" customHeight="1">
+      <c r="A81" s="6" t="n">
+        <v>78</v>
+      </c>
+      <c r="B81" s="6" t="inlineStr">
+        <is>
+          <t>Player input</t>
+        </is>
+      </c>
+      <c r="C81" s="6" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="D81" s="7" t="inlineStr">
+        <is>
+          <t>Add functionality so that during a match, right clicking is the same as clicking a blank space. When a card is selected and a blank space is clicked, the selected card is cleared. I want the same function so that whenever the right click is pressed it is always treated as clicking a blank space. I don't think anywhere in the game a right click is distinguished from a left click so this shouldn't replace any functionality at all.</t>
+        </is>
+      </c>
+      <c r="E81" s="8" t="inlineStr">
+        <is>
+          <t>FIX 25/07/2026 (ISSUE #78 New Functionality): a right-click during a match is now always treated as clicking a blank space — handled up-front in _input, it calls clear_current_action_selection() (see #77) and consumes the event. Nothing else in the match uses right-click. Debug: 'ISSUE #78 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="F81" s="7" t="n"/>
+      <c r="G81" s="7" t="inlineStr">
+        <is>
+          <t>Issue Resolved</t>
+        </is>
+      </c>
+      <c r="H81" s="10" t="inlineStr">
+        <is>
+          <t>25/07/2026</t>
+        </is>
+      </c>
+      <c r="I81" s="10" t="inlineStr">
+        <is>
+          <t>26/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="30" customHeight="1">
+      <c r="A82" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="inlineStr">
+        <is>
+          <t>Aesthetic</t>
+        </is>
+      </c>
+      <c r="D82" s="7" t="inlineStr">
+        <is>
+          <t>When knocking out or retreating a pokemon and there are multiple energies being discarded, update the board (or at least the discard pile) view so that the discarded energy is shown in the discard pile after every discard</t>
+        </is>
+      </c>
+      <c r="E82" s="8" t="inlineStr">
+        <is>
+          <t>FIX 25/07/2026 (ISSUE #79): animate_energies_to_discard now calls update_discard_pile_display after EVERY energy (not just once at the end), so when multiple energies are discarded during retreat OR knockout (both paths share this function) each one visibly lands on the discard pile as it goes. Debug: 'ISSUE #79 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="F82" s="7" t="n"/>
+      <c r="G82" s="7" t="inlineStr">
+        <is>
+          <t>Issue Resolved</t>
+        </is>
+      </c>
+      <c r="H82" s="8" t="inlineStr">
+        <is>
+          <t>25/07/2026</t>
+        </is>
+      </c>
+      <c r="I82" s="8" t="inlineStr">
+        <is>
+          <t>26/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="60" customHeight="1">
+      <c r="A83" s="6" t="n">
+        <v>81</v>
+      </c>
+      <c r="B83" s="6" t="inlineStr">
+        <is>
+          <t>Player input</t>
+        </is>
+      </c>
+      <c r="C83" s="6" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="D83" s="7" t="inlineStr">
+        <is>
+          <t>When scrolling in the card/deck view mode, it passes the scroll through to the map scene underneath so if you scroll up/down to navigate the card menus (most likely happens with coin case and sleeves too then), when you return to the map the game view zooms in/out. Simply block all input being passed to the map scene when the main menu has been opened until the main menu is closed. Correctly using the movement keys doesn't move the player but scrolling zooms</t>
+        </is>
+      </c>
+      <c r="E83" s="8" t="inlineStr">
+        <is>
+          <t>FIX 25/07/2026 (ISSUE #81): Player_Object_Script._unhandled_input mouse-wheel camera zoom is now gated on can_move. While any menu/sub-menu overlay (deck/card/coin/sleeves) is open the player is locked (lock_movement), so scroll events that fall THROUGH the sub-menu Controls no longer zoom the map underneath (only visible on return). Movement keys were already gated; the zoom was not. Debug: 'ISSUE #81 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="F83" s="7" t="n"/>
+      <c r="G83" s="7" t="inlineStr">
+        <is>
+          <t>Issue Resolved</t>
+        </is>
+      </c>
+      <c r="H83" s="8" t="inlineStr">
+        <is>
+          <t>25/07/2026</t>
+        </is>
+      </c>
+      <c r="I83" s="8" t="inlineStr">
+        <is>
+          <t>26/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="105" customHeight="1">
+      <c r="A84" s="6" t="n">
+        <v>80</v>
+      </c>
+      <c r="B84" s="6" t="inlineStr">
+        <is>
+          <t>Player input</t>
+        </is>
+      </c>
+      <c r="C84" s="6" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="D84" s="7" t="inlineStr">
+        <is>
+          <t>When viewing the player's bench, cards can be selected and the action button updates to "Place card on bench" which is obviously wrong. This is legacy code from when originally I was going to allow pokemon to be set as active directly by clicking on bench instead of clicking retreat. We now dont' have ANY functionality and no requirement to click a card on the bench to select it at all. Therefore, Add new functionality for BOTH the player and opponents BENCH cards (only bench) so that when any of the bench cards are clicked, open the card in a new view that only shows that card and all cards attached to it, with only the single centred cancel button. Remove the action button for viewing the player's bench and in this new preview mode. Reuse the same view when retreating your active pokemon so that all the energy cards are shown to the left of the pokemon, the HP is shown in a label underneath, but also of course show any tool cards attached to that pokemon with the energy cards.</t>
+        </is>
+      </c>
+      <c r="E84" s="8" t="inlineStr">
+        <is>
+          <t>FIX 25/07/2026 (ISSUE #80 New Functionality): removed the bogus 'PLACE ON BENCH' action when viewing a bench. Added a view-only single-card preview (show_pokemon_preview): clicking a card while viewing EITHER bench opens that Pokemon enlarged with its HP label beneath and its attached energies + tool cards laid out as separate cards to the left (only a centred CLOSE button). The retreat screen reuses this exact layout — tools are now shown beside the energies (and are not selectable for the retreat cost). New flags bench_view_active / pokemon_preview_active. Debug: 'ISSUE #80 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="F84" s="7" t="n"/>
+      <c r="G84" s="7" t="inlineStr">
+        <is>
+          <t>Issue Resolved</t>
+        </is>
+      </c>
+      <c r="H84" s="8" t="inlineStr">
+        <is>
+          <t>25/07/2026</t>
+        </is>
+      </c>
+      <c r="I84" s="8" t="inlineStr">
+        <is>
+          <t>26/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="30" customHeight="1">
+      <c r="A85" s="6" t="n">
+        <v>81</v>
+      </c>
+      <c r="B85" s="6" t="inlineStr">
+        <is>
+          <t>Overworld</t>
+        </is>
+      </c>
+      <c r="C85" s="6" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="D85" s="7" t="inlineStr">
+        <is>
+          <t>One of the latest bug fixes has completely broken NPC/Opponent interactions. No Interaction bubble appears above heads, spacebar doesn't interact and some NPCs are facing downwards by default instead of the direction they should be facing.</t>
+        </is>
+      </c>
+      <c r="E85" s="12" t="inlineStr">
+        <is>
+          <t>FIX 26/07/2026 (ISSUE #81): a straightforward but total regression — refresh_sprite() (added for ISSUE #52) was inserted INTO THE MIDDLE of Player_Object_Script._ready(), so everything after the insertion point silently became part of refresh_sprite() instead of _ready(). The orphaned lines were the two interaction_area.body_entered/body_exited connects, the returning_from_battle position restore, and _seed_existing_overlaps(). With the signals never connected, no interaction bubble could ever appear and spacebar did nothing. refresh_sprite() moved below _ready() and the four steps restored.
+NPCs FACING DOWN: separate cause, same root area. The locked idle_left/idle_right/idle_up/idle_down patterns in World_Object_Base._init_movement played the right animation but never set current_facing, leaving it at its "down" default. MapManager.capture_actor_positions() then snapshotted "down" and ISSUE #56's restore_facing forced them to face down on the next spawn. Those four branches now set current_facing, and restore_facing is ignored outright for FIXED_FACING_PATTERNS (the four locked patterns + idle_cycle, whose walk animation an idle_ animation would freeze).
+ALSO fixed the same exposure the ISSUE #81 scroll fix left open for the keyboard: the ui_accept branch of _unhandled_input was not gated on can_move, so since ISSUE #52 keeps the map loaded under sub-menu overlays, an unconsumed Space/Enter inside the deck builder could reach the map and start a battle. Debug: 'ISSUE #81 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="F85" s="7" t="n"/>
+      <c r="G85" s="7" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H80" s="12" t="inlineStr">
-        <is>
-          <t>25/07/2026</t>
-        </is>
-      </c>
-      <c r="I80" s="12" t="n"/>
-    </row>
-    <row r="81" ht="45" customHeight="1">
-      <c r="A81" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="B81" s="2" t="inlineStr">
+      <c r="H85" s="8" t="inlineStr">
+        <is>
+          <t>26/07/2026</t>
+        </is>
+      </c>
+      <c r="I85" s="8" t="n"/>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>Live: 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>Incorrect Logic</t>
+        </is>
+      </c>
+      <c r="D86" s="1" t="inlineStr">
+        <is>
+          <t>Plus power just like defender should increase self damage. If attached and a pokemon does any damage to itself that damage should be increased by 10</t>
+        </is>
+      </c>
+      <c r="E86" s="13" t="inlineStr">
+        <is>
+          <t>FIX 26/07/2026 (ISSUE #82): new shared helper main.apply_self_damage_modifiers(pokemon, damage) in Main_Match_Core_Gameplay_Script.gd (right next to get_defender_reduction) — the mirror image of Defender: +10 per PlusPower attached, then -20 per Defender, floored at 0. It is now THE one place self-damage modifiers are applied, and all 18 self-damage sites route through it: confusion coin-flip, the generic 'does N damage to itself' parser, gym2_self_damage (the shared helper behind dozens of recoil attacks, which applied NEITHER modifier before), Thunderstorm recoil, Weezing Liability 70, Hasty Headbutt 20, Gastly Energy Conversion, Belly Drum, Metal Charge, Make a Wish, Tonnage, Darkness Charge, Bouncy Move, ex10 Pop, ex5/ex7 damage-counter attacks, Unown Hidden Power, Burn Away recoil, the Vermilion Gym self-damage and the confused-retreat penalty. This also completes ISSUE #60's coverage, since most of those sites had no Defender reduction either.
+Counter-attack damage (Mirror Shell, Crosscounter, counter_attack_fixed) gets the Defender reduction but deliberately NOT PlusPower — the DEFENDING Pokemon is dealing that damage, not the attacker.
+NOTE FOR RETEST: because PlusPower now mirrors Defender exactly, it also raises the confused-retreat-failure penalty (20 -&gt; 30 with one PlusPower) and every recoil attack. That follows literally from 'any damage to itself', but say the word if you'd rather it were limited to attack self-damage only. Debug: 'ISSUE #82 FIX ACTIVE' prints the before/after and which modifiers applied.</t>
+        </is>
+      </c>
+      <c r="G86" s="1" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>26/07/2026</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>Debug</t>
+        </is>
+      </c>
+      <c r="D87" s="1" t="inlineStr">
+        <is>
+          <t>When using T to enter a test match, when the match concludes the game crashes due to no meet text message</t>
+        </is>
+      </c>
+      <c r="E87" s="13" t="inlineStr">
+        <is>
+          <t>FIX 26/07/2026 (ISSUE #83): the crash was in MapManager's map load, not the outro. On returning from a battle it re-spawns the last battled opponent from GameState.last_battled_opponent_entry using HARD key indexing (lbe["meet_text"] etc.). The T-key TEST match's entry is synthesized by GameState.build_test_opponent_data(), which carries only the handful of fields the match itself needs — so it died on the first missing key, "meet_text", and would have gone on to fail on position and sprite too. Two changes: (1) the respawn is skipped entirely when GameState.test_match_mode is true, since a TEST match has no opponent in the world at all; (2) every field in BOTH spawn blocks (the day-file loop and the respawn) now uses .get() with a default, so one missing dialogue key can never again abort a whole map load. Debug: 'ISSUE #83 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="G87" s="1" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>26/07/2026</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="75" customHeight="1">
+      <c r="A88" s="2" t="n">
+        <v>84</v>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>Deck Builder</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="D88" s="1" t="inlineStr">
+        <is>
+          <t>I don't think we ever put a check in place to make sure that when saving a deck, the player has to have at least 1 single basic pokemon. If the deck does not have a basic pokemon then the deck cannot be saved. For all the checks we have (some are currently disabled for debugging) can we still have functionality that happens when you try to hit the save button even though it is completely disabled? It would be good to have a floating message (as we have across the game already) that pops up with the reason the deck cannot be saved. "Deck needs at least 1 Basic Pokemon" "Deck does not have enough cards. 60 cards required" "Deck has too many cards. 60 cards required" "No Deck name entered"</t>
+        </is>
+      </c>
+      <c r="E88" s="13" t="inlineStr">
+        <is>
+          <t>FIX 26/07/2026 (ISSUE #84 — new functionality): added the missing Basic Pokemon requirement plus visible reasons for every refused save.
+The key change is that the save button is no longer ever actually `disabled` — a disabled Button emits no `pressed` signal, which is exactly why clicking it gave no feedback. It always accepts the click now; the green/grey theme still shows at a glance whether saving will work, and _on_save_pressed() explains why nothing happened.
+New _deck_save_blocker() is the single source of truth both the button colour and the message read, so they can never disagree. Messages: "Deck does not have enough cards. 60 cards required" / "Deck has too many cards. 60 cards required" / "Deck needs at least 1 Basic Pokemon" / "No Deck name entered" / "No changes to save" (and "Deck is empty" while TESTING_UNLIMITED_DECKS relaxes the 60-card rule).
+The Basic Pokemon check is enforced EVEN in testing mode, since a deck with no Basic cannot be set up at the start of a match at all. It reads card metadata (supertype Pokemon + "Basic" in subtypes), so Basic Energy correctly doesn't count.
+The floating message rises and fades like the in-match labels; all its timings/size/colour/position are named MSG_* constants at the top of that section. Debug: 'ISSUE #84 FIX ACTIVE' names the exact blocker.</t>
+        </is>
+      </c>
+      <c r="G88" s="1" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>26/07/2026</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>Live: 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>Item Effect</t>
+        </is>
+      </c>
+      <c r="D89" s="1" t="inlineStr">
+        <is>
+          <t>Remove the (-20 Damage) from the defender attached text so it's just "Defender attached to X"</t>
+        </is>
+      </c>
+      <c r="E89" s="13" t="inlineStr">
+        <is>
+          <t>FIX 26/07/2026 (ISSUE #85): dropped the " (-20 damage)" suffix from the CPU's Defender attach message, so both sides now just say "Defender attached to X!". Debug: 'ISSUE #85 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="G89" s="1" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>26/07/2026</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="30" customHeight="1">
+      <c r="A90" s="2" t="n">
+        <v>86</v>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>Item Effect</t>
+        </is>
+      </c>
+      <c r="D90" s="1" t="inlineStr">
+        <is>
+          <t>Energy Search does not say "Show this card to your opponent" so the card added to the hand of the opponent shouldn't be stated. It should just say "Opponent played energy search", with no second message, just the animate card a to b showing A card going from the deck to the hand.</t>
+        </is>
+      </c>
+      <c r="E90" s="13" t="inlineStr">
+        <is>
+          <t>FIX 26/07/2026 (ISSUE #86): Energy Search has no "Show this card to your opponent" clause, so the "ENERGY SEARCH: ADDED &lt;NAME&gt; TO HAND!" message leaked hidden information. That message is gone; instead a card glides from the deck to the hand — FACE DOWN (the opponent's sleeve) for the CPU, face up for the player since they picked it themselves. The deck icon is refreshed too. Debug: 'ISSUE #86 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="G90" s="1" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>26/07/2026</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="60" customHeight="1">
+      <c r="A91" s="2" t="n">
+        <v>87</v>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>Aesthetic</t>
+        </is>
+      </c>
+      <c r="D91" s="1" t="inlineStr">
+        <is>
+          <t>During any situation where there is no active pokemon for a player or opponent (e.g retreating, knock out, force switch) at the point that the active pokemon is hidden to show it moving from a to b, also hide that player/opponent HP squares. E.g if player retreats active pokemon, as soon as the active pokemon card is hidden and animated moving to the bench, also hide the HP. End goal is that only show the HP squares when there is an active pokemon visible and not animating moving from a to b</t>
+        </is>
+      </c>
+      <c r="E91" s="13" t="inlineStr">
+        <is>
+          <t>FIX 26/07/2026 (ISSUE #87 — new functionality): new helper main.set_active_slot_visible(is_opponent, visible) is now THE one place the Active slot's visibility is toggled — it hides/shows the Active card container and that side's HP squares together, so they can never get out of step. Wired into every path where the Active card is hidden to fly somewhere: voluntary retreat, forced switch (both the outgoing glide and the re-hide after the mid-animation board refresh), and the knockout animation. The squares come back the moment a replacement Pokemon lands in the slot (both the CPU's automatic pick and the player's bench choice).
+display_hp_circles_above_align also now sets the container's visibility directly from whether there IS an Active Pokemon, so a knocked-out side shows no squares at all rather than an empty grid. Debug: 'ISSUE #87 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="G91" s="1" t="inlineStr">
+        <is>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>26/07/2026</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="75" customHeight="1">
+      <c r="A92" s="2" t="n">
+        <v>88</v>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
         <is>
           <t>Player input</t>
         </is>
       </c>
-      <c r="C81" s="2" t="inlineStr">
+      <c r="C92" s="2" t="inlineStr">
         <is>
           <t>Input</t>
         </is>
       </c>
-      <c r="D81" s="1" t="inlineStr">
-        <is>
-          <t>Add functionality so that during a match, right clicking is the same as clicking a blank space. When a card is selected and a blank space is clicked, the selected card is cleared. I want the same function so that whenever the right click is pressed it is always treated as clicking a blank space. I don't think anywhere in the game a right click is distinguished from a left click so this shouldn't replace any functionality at all.</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>FIX 25/07/2026 (ISSUE #78 New Functionality): a right-click during a match is now always treated as clicking a blank space — handled up-front in _input, it calls clear_current_action_selection() (see #77) and consumes the event. Nothing else in the match uses right-click. Debug: 'ISSUE #78 FIX ACTIVE'.</t>
-        </is>
-      </c>
-      <c r="G81" s="1" t="inlineStr">
+      <c r="D92" s="1" t="inlineStr">
+        <is>
+          <t>We have just distinguished right clicking from left clicking to clear selected cards when they are selected. Also add functionality such that when right click is pressed, if there is a cancel button on screen, it is treated as though cancel is pressed. E.g if you click an energy card in hand and select attach, the attach view appears allowing you to attach it to a pokemon but you can cancel this as there is a cancel button, pressing right click anywhere on screen should "press" the cancel button. I will eventually add controller support in which the space bar will have the same functionality as the (A) or (X) button and right click is the same as (B) or (O) button.</t>
+        </is>
+      </c>
+      <c r="E92" s="13" t="inlineStr">
+        <is>
+          <t>FIX 26/07/2026 (ISSUE #88 — new functionality): right-click now presses the on-screen Cancel button. In Main_Match_Core_Gameplay_Script._input, a right-click emits cancel_button.pressed when that button is visible and enabled — whatever its current label ("Cancel", "Done", "CLOSE") — so it works for energy attach, evolution, retreat, trainer targeting, the bench/preview views and every other mode that puts a Cancel button up. With no Cancel button on screen it falls back to ISSUE #78's behaviour (treated as a blank-space click: clears the selected cards without cancelling the mode). This lines up with the planned controller mapping of right-click = B/O. Debug: 'ISSUE #88 FIX ACTIVE' names the button label it pressed.</t>
+        </is>
+      </c>
+      <c r="G92" s="1" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H81" s="12" t="inlineStr">
-        <is>
-          <t>25/07/2026</t>
-        </is>
-      </c>
-      <c r="I81" s="12" t="n"/>
-    </row>
-    <row r="82" ht="30" customHeight="1">
-      <c r="A82" s="2" t="n">
-        <v>79</v>
-      </c>
-      <c r="B82" s="2" t="inlineStr">
-        <is>
-          <t>UI</t>
-        </is>
-      </c>
-      <c r="C82" s="2" t="inlineStr">
-        <is>
-          <t>Aesthetic</t>
-        </is>
-      </c>
-      <c r="D82" s="1" t="inlineStr">
-        <is>
-          <t>When knocking out or retreating a pokemon and there are multiple energies being discarded, update the board (or at least the discard pile) view so that the discarded energy is shown in the discard pile after every discard</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>FIX 25/07/2026 (ISSUE #79): animate_energies_to_discard now calls update_discard_pile_display after EVERY energy (not just once at the end), so when multiple energies are discarded during retreat OR knockout (both paths share this function) each one visibly lands on the discard pile as it goes. Debug: 'ISSUE #79 FIX ACTIVE'.</t>
-        </is>
-      </c>
-      <c r="G82" s="1" t="inlineStr">
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>26/07/2026</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>Live: 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="45" customHeight="1">
+      <c r="A93" s="2" t="n">
+        <v>89</v>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>Player input</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="D93" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scrolling is treated as a mouse click. We already have distinguished right click from left click forcing right click to act like a cancel and left click for all the actions. Prevent scrolling from acting as a mouse click (e.g if the hand is over 7 cards and therefore they go into a scroll box, allow scrolling without clearing or selecting another card in hand. </t>
+        </is>
+      </c>
+      <c r="E93" s="13" t="inlineStr">
+        <is>
+          <t>FIX 26/07/2026 (ISSUE #89): the cause is that Godot delivers mouse-wheel notches as InputEventMouseButton with pressed == true, so every handler testing "is InputEventMouseButton and event.pressed" treated scrolling as a click. Three handlers were affected and all now ignore the four wheel button indices up front:
+- Main_Match_Core_Gameplay_Script._input — was acknowledging message boxes and, whenever the cursor wasn't over a card, calling clear_current_action_selection() (the "clearing" half of the report).
+- Card_Image_Loader_Script._input — was emitting card_clicked for whichever card sat under the cursor (the "selecting another card in hand" half).
+- array_container_clicked — was opening a container's enlarged selection view on scroll.
+The deck builder's own handlers were checked and are safe: they dispatch explicitly on MOUSE_BUTTON_LEFT/RIGHT, so wheel events already fell through harmlessly. Debug: 'ISSUE #89 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="G93" s="1" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr">
-        <is>
-          <t>25/07/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" ht="60" customHeight="1">
-      <c r="A83" s="2" t="n">
-        <v>81</v>
-      </c>
-      <c r="B83" s="2" t="inlineStr">
-        <is>
-          <t>Player input</t>
-        </is>
-      </c>
-      <c r="C83" s="2" t="inlineStr">
-        <is>
-          <t>Input</t>
-        </is>
-      </c>
-      <c r="D83" s="1" t="inlineStr">
-        <is>
-          <t>When scrolling in the card/deck view mode, it passes the scroll through to the map scene underneath so if you scroll up/down to navigate the card menus (most likely happens with coin case and sleeves too then), when you return to the map the game view zooms in/out. Simply block all input being passed to the map scene when the main menu has been opened until the main menu is closed. Correctly using the movement keys doesn't move the player but scrolling zooms</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>FIX 25/07/2026 (ISSUE #81): Player_Object_Script._unhandled_input mouse-wheel camera zoom is now gated on can_move. While any menu/sub-menu overlay (deck/card/coin/sleeves) is open the player is locked (lock_movement), so scroll events that fall THROUGH the sub-menu Controls no longer zoom the map underneath (only visible on return). Movement keys were already gated; the zoom was not. Debug: 'ISSUE #81 FIX ACTIVE'.</t>
-        </is>
-      </c>
-      <c r="G83" s="1" t="inlineStr">
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>26/07/2026</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="75" customHeight="1">
+      <c r="A94" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>Core Gameplay</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>Item Effect</t>
+        </is>
+      </c>
+      <c r="D94" s="1" t="inlineStr">
+        <is>
+          <t>Defender is acting strange. Sometimes when one defender is attached to the opponent and an attack is used, more damage is blocked than should be. Opponent had one defender on their active and player had 2 defenders on their active. Player hitmonchan did special punch for 40 damage but defender blocked all 40 on the opponent so player did no damage to opponent. Debug message even states "ISSUE #60 FIX ACTIVE: Defender reduced attack damage by 40 on Hitmonchan". This isn't 100% of the time though, is it possibly caching old defenders so it thinks more are attached or possibly counting every defender in play and not just on the attached pokemon?</t>
+        </is>
+      </c>
+      <c r="E94" s="13" t="inlineStr">
+        <is>
+          <t>FIX 26/07/2026 (ISSUE #90): your guess was right — it was caching old Defenders. tick_defender_counters discarded the expiring Defender CARDS but never reset pokemon.defender_count (the PlusPower equivalent immediately above it always zeroed pluspower_count). defender_turns_remaining going to -1 masked the stale count, so nothing looked wrong — until the NEXT Defender was attached to that same Pokemon, which set turns back to 0 and did defender_count += 1 on top of the phantom count. One physical Defender then blocked 40 (or 60+) damage. That also explains why it wasn't 100% of the time: it only happens after an earlier Defender has expired on that same Pokemon.
+Fixed at the source, and swept the whole family — every other place that reset defender_turns_remaining without clearing defender_count now clears both: Scoop Up's returned Basic, the two "shuffle a Pokemon back with everything attached" trainers, and the two return-to-hand/deck powers.
+ALSO found and fixed a genuine double-reduction on the same theme: under base_set_confusion_rules, confusion self-damage was passed through calculate_final_damage with the attacker as the DEFENDING Pokemon (so Defender was applied inside it) and then had get_defender_reduction subtracted again on the next line. calculate_final_damage gained an is_self_damage flag that skips its Defender and PlusPower blocks for exactly this case, and the modifiers are applied once by the new shared helper (see ISSUE #82). Debug: 'ISSUE #90 FIX ACTIVE' prints whenever a stale count is cleared.</t>
+        </is>
+      </c>
+      <c r="G94" s="1" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr">
-        <is>
-          <t>25/07/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="84" ht="105" customHeight="1">
-      <c r="A84" s="2" t="n">
-        <v>80</v>
-      </c>
-      <c r="B84" s="2" t="inlineStr">
-        <is>
-          <t>Player input</t>
-        </is>
-      </c>
-      <c r="C84" s="2" t="inlineStr">
-        <is>
-          <t>Input</t>
-        </is>
-      </c>
-      <c r="D84" s="1" t="inlineStr">
-        <is>
-          <t>When viewing the player's bench, cards can be selected and the action button updates to "Place card on bench" which is obviously wrong. This is legacy code from when originally I was going to allow pokemon to be set as active directly by clicking on bench instead of clicking retreat. We now dont' have ANY functionality and no requirement to click a card on the bench to select it at all. Therefore, Add new functionality for BOTH the player and opponents BENCH cards (only bench) so that when any of the bench cards are clicked, open the card in a new view that only shows that card and all cards attached to it, with only the single centred cancel button. Remove the action button for viewing the player's bench and in this new preview mode. Reuse the same view when retreating your active pokemon so that all the energy cards are shown to the left of the pokemon, the HP is shown in a label underneath, but also of course show any tool cards attached to that pokemon with the energy cards.</t>
-        </is>
-      </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>FIX 25/07/2026 (ISSUE #80 New Functionality): removed the bogus 'PLACE ON BENCH' action when viewing a bench. Added a view-only single-card preview (show_pokemon_preview): clicking a card while viewing EITHER bench opens that Pokemon enlarged with its HP label beneath and its attached energies + tool cards laid out as separate cards to the left (only a centred CLOSE button). The retreat screen reuses this exact layout — tools are now shown beside the energies (and are not selectable for the retreat cost). New flags bench_view_active / pokemon_preview_active. Debug: 'ISSUE #80 FIX ACTIVE'.</t>
-        </is>
-      </c>
-      <c r="G84" s="1" t="inlineStr">
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>26/07/2026</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>Live: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="30" customHeight="1">
+      <c r="A95" s="2" t="n">
+        <v>91</v>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>Animation</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>Item Effect</t>
+        </is>
+      </c>
+      <c r="D95" s="1" t="inlineStr">
+        <is>
+          <t>Animate Scoop up appropriately. Message pops up "X used scoop up". Animate the attached cards of the card selected going to discard pile (1 at a time and refresh board each time). Animate the card going to the hand.</t>
+        </is>
+      </c>
+      <c r="E95" s="13" t="inlineStr">
+        <is>
+          <t>FIX 26/07/2026 (ISSUE #91): Scoop Up used to resolve entirely off-screen — every attachment vanished at once and the Pokemon was simply gone by the time the message appeared. It is now narrated in the order it happens: (1) "PLAYER/OPPONENT USED SCOOP UP ON X!", (2) each attachment flies to the discard pile one at a time with the whole board refreshed after each, (3) the Basic card flies from its board slot up into the hand (face down for the CPU).
+The one-at-a-time stripping lives in a new reusable Card_Ops.discard_all_attachments_animated(pokemon, is_opponent) — the animated twin of discard_all_attachments. Energies reuse the shared animate_energies_to_discard path (already one at a time since ISSUE #79) with a board refresh added for the benched case; tools/attached Trainers and pre-evolution cards then animate the same way. Use it for any future player-visible effect that empties a Pokemon; the synchronous version stays for internal cleanup. Debug: 'ISSUE #91 FIX ACTIVE'.</t>
+        </is>
+      </c>
+      <c r="G95" s="1" t="inlineStr">
         <is>
           <t>Untested Fix</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr">
-        <is>
-          <t>25/07/2026</t>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>26/07/2026</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>Live: 2</t>
         </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I79"/>
-  <conditionalFormatting sqref="A2:I1000">
-    <cfRule type="expression" priority="1" dxfId="28" stopIfTrue="1">
+  <conditionalFormatting sqref="A2:J1000">
+    <cfRule type="expression" priority="1" dxfId="15" stopIfTrue="1">
       <formula>OR($G2="New Issue",$G2="Fix Failed",$G2="Improve Further",$G2="New Functionality")</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="29" stopIfTrue="1">
+    <cfRule type="expression" priority="2" dxfId="14" stopIfTrue="1">
       <formula>$G2="Untested Fix"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" dxfId="30" stopIfTrue="1">
+    <cfRule type="expression" priority="3" dxfId="13" stopIfTrue="1">
       <formula>$G2="Issue Resolved"</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" dxfId="31" stopIfTrue="1">
+    <cfRule type="expression" priority="4" dxfId="12" stopIfTrue="1">
       <formula>$G2="Manual Fix"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5571,13 +6056,13 @@
     </sortState>
   </autoFilter>
   <conditionalFormatting sqref="A2:C1048576">
-    <cfRule type="expression" priority="37" dxfId="0">
+    <cfRule type="expression" priority="37" dxfId="2">
       <formula>OR($C2="Y",#REF!="Issue Resolved")</formula>
     </cfRule>
-    <cfRule type="expression" priority="38" dxfId="3">
+    <cfRule type="expression" priority="38" dxfId="1">
       <formula>#REF!="Untested Fix"</formula>
     </cfRule>
-    <cfRule type="expression" priority="39" dxfId="2">
+    <cfRule type="expression" priority="39" dxfId="0">
       <formula>OR($C2="N",#REF!="New Issue",#REF!="Fix Failed")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6198,13 +6683,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:C17 A19:C1048576">
-    <cfRule type="expression" priority="34" dxfId="0">
+    <cfRule type="expression" priority="34" dxfId="2">
       <formula>OR($C2="Y",#REF!="Issue Resolved")</formula>
     </cfRule>
-    <cfRule type="expression" priority="35" dxfId="3">
+    <cfRule type="expression" priority="35" dxfId="1">
       <formula>#REF!="Untested Fix"</formula>
     </cfRule>
-    <cfRule type="expression" priority="36" dxfId="2">
+    <cfRule type="expression" priority="36" dxfId="0">
       <formula>OR($C2="N",#REF!="New Issue",#REF!="Fix Failed")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6809,13 +7294,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:C1048576">
-    <cfRule type="expression" priority="40" dxfId="0">
+    <cfRule type="expression" priority="40" dxfId="2">
       <formula>OR($C2="Y",#REF!="Issue Resolved")</formula>
     </cfRule>
-    <cfRule type="expression" priority="41" dxfId="3">
+    <cfRule type="expression" priority="41" dxfId="1">
       <formula>#REF!="Untested Fix"</formula>
     </cfRule>
-    <cfRule type="expression" priority="42" dxfId="2">
+    <cfRule type="expression" priority="42" dxfId="0">
       <formula>OR($C2="N",#REF!="New Issue",#REF!="Fix Failed")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7648,13 +8133,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:C1048576">
-    <cfRule type="expression" priority="43" dxfId="0">
+    <cfRule type="expression" priority="43" dxfId="2">
       <formula>OR($C2="Y",#REF!="Issue Resolved")</formula>
     </cfRule>
-    <cfRule type="expression" priority="44" dxfId="3">
+    <cfRule type="expression" priority="44" dxfId="1">
       <formula>#REF!="Untested Fix"</formula>
     </cfRule>
-    <cfRule type="expression" priority="45" dxfId="2">
+    <cfRule type="expression" priority="45" dxfId="0">
       <formula>OR($C2="N",#REF!="New Issue",#REF!="Fix Failed")</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Debug: Fixed issues - mostly display/UI problems with messageboxes
</commit_message>
<xml_diff>
--- a/Spreadsheets/Issue_Log.xlsx
+++ b/Spreadsheets/Issue_Log.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\Spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33290548-FFFA-4FF5-A66C-3F5C73CAAD4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CE991EE-C820-48C8-9CAF-E9362E952FC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1364" uniqueCount="816">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1461" uniqueCount="849">
   <si>
     <t>#</t>
   </si>
@@ -844,6 +844,9 @@
     <t>FIX 26/07/2026 (ISSUE #83): the crash was in MapManager's map load, not the outro. On returning from a battle it re-spawns the last battled opponent from GameState.last_battled_opponent_entry using HARD key indexing (lbe["meet_text"] etc.). The T-key TEST match's entry is synthesized by GameState.build_test_opponent_data(), which carries only the handful of fields the match itself needs — so it died on the first missing key, "meet_text", and would have gone on to fail on position and sprite too. Two changes: (1) the respawn is skipped entirely when GameState.test_match_mode is true, since a TEST match has no opponent in the world at all; (2) every field in BOTH spawn blocks (the day-file loop and the respawn) now uses .get() with a default, so one missing dialogue key can never again abort a whole map load. Debug: 'ISSUE #83 FIX ACTIVE'.</t>
   </si>
   <si>
+    <t>23/08/2026</t>
+  </si>
+  <si>
     <t>Deck Builder</t>
   </si>
   <si>
@@ -989,7 +992,7 @@
     <t xml:space="preserve">When the opponent had a vileplume active, they correctly used it's power Heal. But to the player the game just flipped a coin (got tails) and said vileplume heal: tails! Failed!. The flow for any powers similar to this that need activating and then have an effect should be 1) Messagebox pops up saying "Opponent used [POKEMONS] [POWER NAME] Power 2) Messagebox is clicked to clear, follow the effects of the power (such as for vileplume flip the coin). 3)  Messagebox to explain the effect that is going to happen now the coin flip has happened and the power has been checkjed. 4) Messagebox is clickedf to clear, perform the animations for any actions of the power (heal, damage, drawing, energy move) </t>
   </si>
   <si>
-    <t>Added a shared announce_cpu_power(pokemon, power_name) helper in Powers_And_Bodies_Effects.gd that shows OPPONENT USED &lt;POKEMON&gt;'S &lt;POWER&gt; POWER! and waits for a click - beat 1 of the requested flow. Applied the full announce -&gt; resolve -&gt; explain -&gt; animate ordering to all 18 CPU power activations in cpu_phase_activate_powers(): Special Delivery, Solar Power, Rain Dance, Energy Trans, Heal (the reported Vileplume case), Shift, Damage Swap, Buzzap, Step In, Curse, Strange Behavior, Cowardice, Evolutionary Light, Matter Exchange, Pollen Stench, Gather Fire, Long-Distance Hypnosis, Trickery. Board animations now run AFTER the explanation message rather than before it. Two side bugs fixed on the way: Vileplume burned power_used_this_turn even on turns where there was nothing to heal, and Slowbro's Strange Behavior moved damage counters in complete silence with no message at all. NOT DONE: the ~30 per-set cpu_phase_&lt;set&gt;_powers() functions (neo/ecard/ex/pop) still use their old single-message style - the helper is in place for them but retrofitting several hundred call sites is a separate pass.</t>
+    <t>Added a shared announce_cpu_power(pokemon, power_name) helper in Powers_And_Bodies_Effects.gd that shows OPPONENT USED &lt;POKEMON&gt;'S &lt;POWER&gt; POWER! and waits for a click - beat 1 of the requested flow. Applied the full announce -&gt; resolve -&gt; explain -&gt; animate ordering to all 18 CPU power activations in cpu_phase_activate_powers(): Special Delivery, Solar Power, Rain Dance, Energy Trans, Heal (the reported Vileplume case), Shift, Damage Swap, Buzzap, Step In, Curse, Strange Behavior, Cowardice, Evolutionary Light, Matter Exchange, Pollen Stench, Gather Fire, Long-Distance Hypnosis, Trickery. Board animations now run AFTER the explanation message rather than before it. Two side bugs fixed on the way: Vileplume burned power_used_this_turn even on turns where there was nothing to heal, and Slowbro's Strange Behavior moved damage counters in complete silence with no message at all. NOT DONE: the ~30 per-set cpu_phase_&lt;set&gt;_powers() functions (neo/ecard/ex/pop) still use their old single-message style - the helper is in place for them but retrofitting several hundred call sites is a separate pass. | 2026-08-23 FOLLOW-UP (carry-over task, completed): the per-set retrofit is now DONE. announce_cpu_power() added to all 125 CPU power activations across the 25 per-set phase functions (gym, neo1-3, np, ecard1-3, ex1-ex16) plus trigger_pop_on_bench for the three POP on-bench powers (Time Reversal / Purple Ray / Dark Ray, announced only when it is the CPU benching the Pokemon). Repeat-fire powers announce ONCE via a local flag, never power_used_this_turn, which must stay clear for unlimited-use powers: Energy Charge (gym, while-loop) and Downpour (neo1, up to 3 discards). Per-Pokemon loops (Baby Evolution ex2, Magnetic Call np) correctly announce once per Pokemon. Beats 3+4 fixed in the per-power CPU helpers that animated before explaining: cpu_ex1_firestarter, cpu_ex1_energy_draw, cpu_ex1_psy_shadow, cpu_ex1_water_call, cpu_ex1_drive_off, cpu_ex3_magnetic_field, cpu_ex3_call_for_power - each now shows its explanation BEFORE the display_* calls, and the redundant 'OPPONENT USED X!' trailers were replaced with messages that say what actually happened. cpu_ex3_dragon_wind had NO message at all and now explains before it switches the player's Active. cpu_ex2_fan_away and the three cpu_ex4_* helpers just delegate to shared power_* functions, so the call-site announce covers them. cpu_phase_neo4_powers is deliberately untouched - it activates Stadium cards (Lucky Stadium, Energy Stadium, Radio Tower), not Poke-Powers. Shared power_* functions are used by BOTH sides, so their existing messages were left as the explain beat rather than being reworded for the CPU.</t>
   </si>
   <si>
     <t xml:space="preserve">allways check for poison damage in card priorities. E.g the opponent attached a defender to their active pokemon to save them from being knocked out from an attack on the next turn but the pokemon was poisoned with 10hp left. Similarly they attach energies to them even if it's a guarenteed posion knockout. </t>
@@ -1022,15 +1025,15 @@
     <t>Moved the 5 remaining Misc images (new_battle, new_talk, old_battle, old_talk, shop_talk) to Image_Assets/Icons/Message_Icons/ and updated all 5 GDScript references in World_Object_Base, NPC_Object_Script, Opponent_Object_Script and Shopkeeper_Script - these were lowercase 'res://image_assets/misc/...' paths that only worked because Windows is case-insensitive, so they are correctly cased now too. .import files rewritten as for #105. Image_Assets/Misc is now empty and has been deleted. Verified with a full headless editor import.</t>
   </si>
   <si>
+    <t>Baby pokemon have a little bit of flavour text saying "this card evolves into X" e.g Tyrogue has "This pokemon evolves into hitmonchan, hitmonlee, hitmontop". Is this missing from the card set data entirely? If it already exists we should add this to the preview window.</t>
+  </si>
+  <si>
+    <t>It was already in the data - all 19 Baby cards carry an evolvesTo array. The preview's subtype line now reads BABY - EVOLVES INTO HITMONLEE, HITMONCHAN OR HITMONTOP, using a shared _join_or() helper so one, two or three names all read naturally. Deliberately limited to Baby cards: 1418 non-Baby cards also carry evolvesTo and printing it on all of them would just be noise. The long Tyrogue line auto-shrinks to fit the header width via the existing _fit_text pass.</t>
+  </si>
+  <si>
     <t>21/08/2026</t>
   </si>
   <si>
-    <t>Baby pokemon have a little bit of flavour text saying "this card evolves into X" e.g Tyrogue has "This pokemon evolves into hitmonchan, hitmonlee, hitmontop". Is this missing from the card set data entirely? If it already exists we should add this to the preview window.</t>
-  </si>
-  <si>
-    <t>It was already in the data - all 19 Baby cards carry an evolvesTo array. The preview's subtype line now reads BABY - EVOLVES INTO HITMONLEE, HITMONCHAN OR HITMONTOP, using a shared _join_or() helper so one, two or three names all read naturally. Deliberately limited to Baby cards: 1418 non-Baby cards also carry evolvesTo and printing it on all of them would just be noise. The long Tyrogue line auto-shrinks to fit the header width via the existing _fit_text pass.</t>
-  </si>
-  <si>
     <t>Some pokemon ex can evolve from other pokemon ex or normal. Chansey ex exists so blissey ex states on the card it can evolve from chansey or chansey ex. Scizor is the same can evolve from scyther or scyther ex. The text only states on preview that it evolves from the ex version. If this is missing from the card set data, simply add the chansey or chansey ex, scyther or scyther ex to the card set data and ensure the actual evolves from fields are updated to make them legal plays. This does NOT apply to the rocket scizor ex which can only evolve from rocket scyther ex.</t>
   </si>
   <si>
@@ -1061,6 +1064,99 @@
     <t>Added a SHOW_FILTER_PANEL flag in Card_Search_Overlay.gd, currently false. It makes the panel TRANSPARENT rather than hidden on purpose: a hidden Control is dropped from Godot's input picking entirely, so visible=false would have stopped it swallowing clicks over the filter rows. Row labels were briefly switched to a light colour to suit the dark backdrop, then put back to black on request after seeing it in game - the comment on the flag now says so, to stop it being 'fixed' again later. Flip the one flag to true to bring the panel back, or resize it to cover the whole screen.</t>
   </si>
   <si>
+    <t>In the holo rare shopkeeper, increase the size of the card that you buy by 50%, it's too small on screen, it should be pretty much the same size as when a card is received as a gift</t>
+  </si>
+  <si>
+    <t>Holo Rare shop reveal card enlarged 50%: Holo_Rare_Shop_Script.REVEAL_SIZE 318x437 -&gt; 477x655.5 (aspect unchanged). That lands it alongside the 430x600 a single card gets as an NPC gift (MapManager.GIFT_CARD_SIZES[1]). The 'You got X' label and OK button are positioned off the card's height so they follow it down automatically; the whole stack still fits 1080p.</t>
+  </si>
+  <si>
+    <t>When you buy a holo rare and the OK button pops up, allow space escape and enter to press the OK button</t>
+  </si>
+  <si>
+    <t>The reveal's OK button now answers to Space / Enter / Escape as well as a click. Holo_Rare_Shop_Script keeps the button in _reveal_ok_btn and _input() presses it via UIInput.is_advance(), consuming the event so the press can't also fire ui_accept on a focused button. SIBLING ALSO FIXED: Coin_Shop_Script's purchase reveal is the identical overlay+OK pattern and had the identical problem - same fix applied there. Both screens' raw KEY_ESCAPE tests were also routed through UIInput.is_cancel() per the project convention.</t>
+  </si>
+  <si>
+    <t>For all messageboxes, increase the line spacing ever so slightly. When there is more than one line in a message the lines are too close together harming readability</t>
+  </si>
+  <si>
+    <t>Dynamic_Message_Box.gd: new BODY_LINE_SPACING = 8, applied to the body label as a line_separation theme override. _measured_text_height() adds the same spacing per line gap when measuring, so the shrink-to-fit and the vertical centring both stay honest with the extra leading. Covers every box in the game - overworld, in-match and outro all share this one class.</t>
+  </si>
+  <si>
+    <t>When a gift is received from an NPC, don't show the NPC as the messagebox provider, have it as the plain grey with the "You received X"</t>
+  </si>
+  <si>
+    <t>MapManager._show_gift_display() now calls message_panel.show_as_plain() (new helper in Dynamic_Message_Box.gd) right after showing the 'You received X' notice, which clears the chip row and drops back to the default grey theme. The gift notice is the game talking, not the NPC who handed it over.</t>
+  </si>
+  <si>
+    <t>Remove the bold font in the messageboxes for name prize cards and deck name</t>
+  </si>
+  <si>
+    <t>Chip labels use the plain font, not the bold one. Dynamic_Message_Box._build_chip() draws with _msg_font instead of _msg_font_bold, and _measure_chip_list() measures with the same face so the pill widths still match the text. Covers all chips - NPC/opponent name, deck name and prize count.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For any vendor (juice vendor, card mart, rocket mart, gym pack mart, holo rare, coin vendor etc) we currently have a little label that appears in the bottom right of the screen showing the player's cash. Now we have our new dynamic messagebox system instead, add a new little mini rounded rectangle at the top right of the messagebox, identical in colour and style to when the messagebox shows the prize card box for an opponent. This should result in the name of the NPC being in the top left and in the top right have the similar box style showing the cash value instead of having it outside of the messagebox under it </t>
+  </si>
+  <si>
+    <t>Cash is now a chip on the message box instead of a loose label. Dynamic_Message_Box gained a second, RIGHT-aligned chip row (set_right_chips()): same pill, same corner radius, colours carry on up the same ramp, laid out so the last chip ends flush with the panel's right inset - mirroring how the name chip starts flush with the left. MapManager._apply_cash_chip() fills it with '$&lt;cash&gt;' + the pokedollar icon for vendors only (_npc_is_vendor: npc_type 'shop' - card mart, rocket mart, gym mart, coin mart, holo mart - or 'juice_vendor'), and is refreshed after a juice purchase and after a shop purchase (Shopkeeper_Script). Opponents and ordinary NPCs explicitly clear it. See also #127, which removed the old labels.</t>
+  </si>
+  <si>
+    <t>Thew new dynamic messagebox system is broken inside of a match. It currently shows a HUGE box with two of the headers in the top left, it should instead just be the same size as when talking to a sign or interactable object so it doesn't have the npc name header or anything else other than the main box background</t>
+  </si>
+  <si>
+    <t>ROOT CAUSE: the in-match box was never converted - it was still the old baked PNG (Image_Assets/Messageboxes/bluesquaremessagebox.png) stretched across a 1910x156 TextureRect. That PNG has since been re-cut as a 4353x432 render of the NEW dynamic box, chip row and all, so stretching it drew a huge panel with two dead 'header' chips baked into its top-left corner. Main_Match_Core_Gameplay_Script now builds a real DynamicMessageBox (_ensure_match_msgbox, on first use so it can't race the @onready lookups): configure(138, 40, no buttons) + show_as_plain() - the same plain grey, chipless, buttonless box a sign or interactable gets in the overworld. The old messagebox_texture and messagebox_text_label are hidden for good; messagebox_container still gates input, so every existing visibility check and the click/Space dismissal are untouched.</t>
+  </si>
+  <si>
+    <t>similarly on the match end outro screen, the messagebox is too big and shows the name of the NPC as plain text within the message itself. This messagebox in the outro should replicate the NPC box showing the overworld sprite and name in a header box at the top left of the messagebox with the messagebox being the same size as the rest of the overworld messageboxes</t>
+  </si>
+  <si>
+    <t>Two changes. (1) The name is off the body text: Match_End_Outro_Script no longer prefixes the dialogue with '&lt;NAME&gt;:\n' - the opponent's name and overworld sprite go on a proper chip above the box (_dialogue_panel.set_chips, after apply_theme so it picks up their colour ramp). The 'sprite' key names a file in both the in-battle and overworld sprite folders, so the same value that picks the battle portrait picks the walking sprite for the chip. (2) The box is overworld-sized: MessageBoxHelper.build(138, 28, no buttons) instead of the outsized 220px/36pt one-off, via new DIALOGUE_BOX_HEIGHT / DIALOGUE_FONT_SIZE constants.</t>
+  </si>
+  <si>
+    <t>Increase the size of the reward label text and icons on the outro screen by 50%</t>
+  </si>
+  <si>
+    <t>Match_End_Outro_Script reward rows scaled 50%: font 21 -&gt; REWARD_FONT_SIZE 32, icons 20px -&gt; REWARD_ICON_PX 30, icon+gap 30 -&gt; REWARD_ICON_GAP 45, icon drop 5 -&gt; REWARD_ICON_DROP 7.5, header box 60 -&gt; 90 tall. REWARD_ROW_SPACING also had to go 35 -&gt; 52.5: the rows stack upward on a fixed pitch, and a 32pt line would have overlapped the row above it at the old 35. Applies to the 'Rewards:' header and every row (cash, coin, cards, costumes).</t>
+  </si>
+  <si>
+    <t>Receiving the rewards / gifts at the end of a match has the font "you received X" top aligned instead of center aligned in the messagebox but the size of the box is correct</t>
+  </si>
+  <si>
+    <t>ROOT CAUSE (shared with #125): the box centred its body text by putting a fit_content RichTextLabel in a centre-aligned VBox, but RichTextLabel recomputes its content height lazily - on the frame the box is shown it still reads ~0. The outro's gift panel had worked around that by setting fit_content = false + SIZE_EXPAND_FILL, which made the label fill the whole panel, so the text drew hard against its top edge. Fixed properly in Dynamic_Message_Box: the text area is now a plain Control and _place_body_label() measures the wrapped text with the Font API (_measured_text_height, line spacing included) and positions the label itself. The outro's two workaround lines were removed. Deterministic on the first frame, so both this and #125 are fixed by the one change.</t>
+  </si>
+  <si>
+    <t>The text inside the box when interacting with a sign with only a single line of text also isn't centrally aligned but is just slightly above the bottom of the messagebox</t>
+  </si>
+  <si>
+    <t>Same root cause and same fix as #124 - see that row. The sign symptom was the other half of it: with the content height reading ~0 the VBox centred a zero-height label, so the label's TOP landed on the panel's centre line and the text hung DOWN from there, ending just above the panel's bottom edge. Now measured and centred explicitly.</t>
+  </si>
+  <si>
+    <t>For all NPC interactions in which it's only an "OK" and not a yes/no choice, just remove the ok button. We don't need an ok button when you can just click anywhere on screen or press spacebar/enter/escape. In removing OK ensure the messagebox is moved down</t>
+  </si>
+  <si>
+    <t>The OK button is gone. Dynamic_Message_Box gained an explicit mode (set_mode 'ok' | 'choices'): 'ok' hides the whole button row and drops the panel from PANEL_BOTTOM_Y (1004) to PANEL_BOTTOM_NO_BUTTONS (1068), into the space the button row used to occupy. Panel geometry is no longer baked in at construction - _layout_panel() re-runs on every mode change and re-flows the panel, the text area, the chip row and the fitted body text. Callers can no longer test 'ok_button.visible' to ask whether a dismissable message is up, so MapManager's keyboard handlers use is_ok_mode() / is_choice_mode(), and the gift reveal (which used to hide the OK button while the cards flip) uses the new ok_armed flag instead. Clicking anywhere, Space, Enter and Escape all already dismissed the box, so nothing was lost. Yes/No boxes are unchanged.</t>
+  </si>
+  <si>
+    <t>Instead of having the cash label always be displayed in certain shop buildings (marts and the gym challenge hall) remove it to only be displayed when interacting with an NPC that is a vendor (as mentioned in issue 120)</t>
+  </si>
+  <si>
+    <t>Removed _create_cash_label()/_update_cash_label() from Card_Mart, Rocket_Mart and Gym_Challenge_Reception, deleted the shared helper from Base_Map_Scene (and its _exit_tree call), and deleted the juice vendor's equivalent _show/_update/_hide_cash_overlay block from MapManager. Shopkeeper_Script's post-purchase refresh now calls MapManager._apply_cash_chip(). Cash appears only on the message box while talking to a vendor - see #120.</t>
+  </si>
+  <si>
+    <t>Audio</t>
+  </si>
+  <si>
+    <t>When entering a sub menu from the main escape menu, the main menu audio carries over into the submenu and overlaps. Also there is no audio for the player info screen, set the same audio that plays in all the other sub menus</t>
+  </si>
+  <si>
+    <t>Two separate faults. (1) OVERLAP: since sub-menus became overlays (#52) the main menu is only HIDDEN behind one, not unloaded, so its own AudioStreamPlayer kept playing under the sub-menu's track. Main_Menu_Script gained pause_music()/resume_music() (stream_paused, so the theme resumes where it left off) and Base_Map_Scene calls them from open_submenu_overlay/close_submenu_overlay, alongside the existing set_process_input toggle. (2) SILENT INFO SCREEN: Info_Script now creates the same AudioStreamPlayer + 'coin_mode (TCG GB Water Club).ogg' the Coin Case, Sleeves and Costume screens use. Options_Script got the identical block as well - it had no track of its own and was running on the main menu's music bleeding through, so fixing (1) would have left it silent.</t>
+  </si>
+  <si>
+    <t>When starting the game, grant the player the 1_default_english, 1_default_japanese_new and 1_default_japanese_old. Set the 1_default_english as the default sleeve for the player on game initialization. Ensure these are in the seed files that get copied on game init.</t>
+  </si>
+  <si>
+    <t>Seed files: Player_Data/Player_Game_Progress.json 'sleeves' is now [1_Default_English, 1_Default_Japanese_New, 1_Default_Japanese_Old] and Player_Data/Player_Current_Data.json 'sleeve' is 1_Default_English - both are copied to user:// on first run. GameState gained STARTER_SLEEVES and its migration branch seeds that instead of the old ['default'], which matched no file on disk. ALSO REQUIRED: Sleeves_Scene_Script deliberately filtered every '1_Default*' file out of the grid (because the only starter entry used to be the fake name 'default'), so granting them would have been meaningless - they could never be equipped. That filter is removed. The trainer card's collection counter (Info_Script._sleeve_universe) still excludes them, so the three freebies don't count as collected sleeves. NOTE FOR THE USER: Image_Assets/Sleeves/small/ still holds 1_Default_Ancient.jpg while the full-size folder now has Ancient.jpg - the small/ copy needs the same rename or 'Ancient' won't appear in the grid.</t>
+  </si>
+  <si>
     <t>UID</t>
   </si>
   <si>
@@ -2574,6 +2670,9 @@
   </si>
   <si>
     <t>Fix Failed</t>
+  </si>
+  <si>
+    <t>All good, but actually make the messagebox inside the match the same colour as the opponent being battled, this is already done for the match rewards</t>
   </si>
 </sst>
 </file>
@@ -3164,20 +3263,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J117"/>
+  <dimension ref="A1:J132"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.42578125" style="5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21.42578125" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="143.42578125" style="6" customWidth="1"/>
+    <col min="4" max="4" width="125.28515625" style="6" customWidth="1"/>
     <col min="5" max="5" width="255.5703125" style="6" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="188.7109375" style="6" customWidth="1"/>
+    <col min="6" max="6" width="102" style="6" customWidth="1"/>
     <col min="7" max="7" width="19" style="6" customWidth="1"/>
     <col min="8" max="9" width="11.140625" style="7" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="16" style="7" customWidth="1"/>
-    <col min="11" max="11" width="9.140625" style="7" customWidth="1"/>
-    <col min="12" max="16384" width="9.140625" style="7"/>
+    <col min="11" max="12" width="9.140625" style="7" customWidth="1"/>
+    <col min="13" max="16384" width="9.140625" style="7"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -3212,7 +3311,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="5">
         <v>1</v>
       </c>
@@ -5475,13 +5574,13 @@
         <v>243</v>
       </c>
       <c r="G87" s="6" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="H87" s="7" t="s">
         <v>183</v>
       </c>
-      <c r="J87" s="7" t="s">
-        <v>20</v>
+      <c r="I87" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="88" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.25">
@@ -5489,25 +5588,25 @@
         <v>84</v>
       </c>
       <c r="B88" s="5" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C88" s="5" t="s">
         <v>22</v>
       </c>
       <c r="D88" s="6" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E88" s="11" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G88" s="6" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="H88" s="7" t="s">
         <v>183</v>
       </c>
-      <c r="J88" s="7" t="s">
-        <v>56</v>
+      <c r="I88" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.25">
@@ -5521,10 +5620,10 @@
         <v>91</v>
       </c>
       <c r="D89" s="6" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E89" s="11" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="G89" s="6" t="s">
         <v>14</v>
@@ -5547,10 +5646,10 @@
         <v>91</v>
       </c>
       <c r="D90" s="6" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E90" s="11" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="G90" s="6" t="s">
         <v>19</v>
@@ -5573,10 +5672,10 @@
         <v>45</v>
       </c>
       <c r="D91" s="6" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E91" s="11" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="G91" s="6" t="s">
         <v>14</v>
@@ -5599,10 +5698,10 @@
         <v>22</v>
       </c>
       <c r="D92" s="6" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E92" s="11" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="G92" s="6" t="s">
         <v>14</v>
@@ -5625,10 +5724,10 @@
         <v>22</v>
       </c>
       <c r="D93" s="6" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E93" s="11" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="G93" s="6" t="s">
         <v>14</v>
@@ -5651,10 +5750,10 @@
         <v>91</v>
       </c>
       <c r="D94" s="6" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E94" s="11" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="G94" s="6" t="s">
         <v>19</v>
@@ -5677,10 +5776,10 @@
         <v>91</v>
       </c>
       <c r="D95" s="6" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E95" s="11" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="G95" s="6" t="s">
         <v>19</v>
@@ -5697,13 +5796,13 @@
         <v>92</v>
       </c>
       <c r="B96" s="5" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C96" s="5" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D96" s="6" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="G96" s="6" t="s">
         <v>14</v>
@@ -5712,18 +5811,18 @@
         <v>218</v>
       </c>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A97" s="5">
         <v>92</v>
       </c>
       <c r="B97" s="5" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C97" s="5" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D97" s="6" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="G97" s="6" t="s">
         <v>14</v>
@@ -5743,22 +5842,22 @@
         <v>192</v>
       </c>
       <c r="D98" s="6" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="E98" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="F98" s="6" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="G98" s="6" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="H98" t="s">
         <v>218</v>
       </c>
-      <c r="J98" t="s">
-        <v>56</v>
+      <c r="I98" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="99" spans="1:10" ht="45" customHeight="1" x14ac:dyDescent="0.25">
@@ -5772,7 +5871,7 @@
         <v>45</v>
       </c>
       <c r="D99" s="6" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="G99" s="6" t="s">
         <v>14</v>
@@ -5792,10 +5891,10 @@
         <v>11</v>
       </c>
       <c r="D100" s="6" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E100" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="G100" s="6" t="s">
         <v>19</v>
@@ -5818,10 +5917,10 @@
         <v>78</v>
       </c>
       <c r="D101" s="6" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E101" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="G101" s="6" t="s">
         <v>19</v>
@@ -5833,7 +5932,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A102" s="5">
         <v>97</v>
       </c>
@@ -5844,10 +5943,10 @@
         <v>78</v>
       </c>
       <c r="D102" s="6" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="E102" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="G102" s="6" t="s">
         <v>19</v>
@@ -5867,16 +5966,19 @@
         <v>22</v>
       </c>
       <c r="D103" s="6" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E103" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="G103" s="6" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="H103" t="s">
         <v>218</v>
+      </c>
+      <c r="I103" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="104" spans="1:10" x14ac:dyDescent="0.25">
@@ -5884,16 +5986,16 @@
         <v>99</v>
       </c>
       <c r="B104" s="5" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C104" s="5" t="s">
         <v>78</v>
       </c>
       <c r="D104" s="6" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="E104" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G104" s="6" t="s">
         <v>19</v>
@@ -5913,22 +6015,22 @@
         <v>94</v>
       </c>
       <c r="C105" s="5" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D105" s="6" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="E105" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G105" s="6" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="H105" t="s">
         <v>218</v>
       </c>
-      <c r="J105" t="s">
-        <v>20</v>
+      <c r="I105" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="106" spans="1:10" x14ac:dyDescent="0.25">
@@ -5942,19 +6044,19 @@
         <v>45</v>
       </c>
       <c r="D106" s="6" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="E106" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="G106" s="6" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="H106" t="s">
         <v>218</v>
       </c>
-      <c r="J106" t="s">
-        <v>20</v>
+      <c r="I106" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="107" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.25">
@@ -5968,10 +6070,10 @@
         <v>30</v>
       </c>
       <c r="D107" s="6" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E107" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="G107" s="6" t="s">
         <v>19</v>
@@ -5994,10 +6096,10 @@
         <v>11</v>
       </c>
       <c r="D108" s="6" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="E108" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="G108" s="6" t="s">
         <v>19</v>
@@ -6020,10 +6122,10 @@
         <v>45</v>
       </c>
       <c r="D109" s="6" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="E109" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="G109" s="6" t="s">
         <v>19</v>
@@ -6032,24 +6134,24 @@
         <v>218</v>
       </c>
       <c r="J109" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="110" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A110" s="5">
         <v>105</v>
       </c>
       <c r="B110" s="5" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C110" s="5" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D110" s="6" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="E110" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="G110" s="6" t="s">
         <v>19</v>
@@ -6063,16 +6165,16 @@
         <v>106</v>
       </c>
       <c r="B111" s="5" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C111" s="5" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D111" s="6" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E111" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="G111" s="6" t="s">
         <v>19</v>
@@ -6081,7 +6183,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="112" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="5">
         <v>109</v>
       </c>
@@ -6101,13 +6203,13 @@
         <v>14</v>
       </c>
       <c r="H112" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="I112" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="113" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="113" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="5">
         <v>110</v>
       </c>
@@ -6118,22 +6220,22 @@
         <v>78</v>
       </c>
       <c r="D113" s="6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="E113" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="G113" s="6" t="s">
         <v>14</v>
       </c>
       <c r="H113" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="I113" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="114" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="114" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A114" s="5">
         <v>111</v>
       </c>
@@ -6144,48 +6246,48 @@
         <v>100</v>
       </c>
       <c r="D114" s="6" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="E114" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="G114" s="6" t="s">
         <v>14</v>
       </c>
       <c r="H114" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="I114" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="115" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="115" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115" s="5">
         <v>112</v>
       </c>
       <c r="B115" s="5" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C115" s="5" t="s">
         <v>22</v>
       </c>
       <c r="D115" s="6" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E115" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="G115" s="6" t="s">
         <v>14</v>
       </c>
       <c r="H115" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="I115" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="116" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="116" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="5">
         <v>113</v>
       </c>
@@ -6196,22 +6298,22 @@
         <v>45</v>
       </c>
       <c r="D116" s="6" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E116" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="G116" s="6" t="s">
         <v>14</v>
       </c>
       <c r="H116" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="I116" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="117" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="117" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="5">
         <v>114</v>
       </c>
@@ -6222,19 +6324,382 @@
         <v>45</v>
       </c>
       <c r="D117" s="6" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E117" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="G117" s="6" t="s">
         <v>14</v>
       </c>
       <c r="H117" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="I117" t="s">
-        <v>298</v>
+        <v>301</v>
+      </c>
+    </row>
+    <row r="118" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A118" s="5">
+        <v>115</v>
+      </c>
+      <c r="B118" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C118" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D118" s="6" t="s">
+        <v>312</v>
+      </c>
+      <c r="E118" t="s">
+        <v>313</v>
+      </c>
+      <c r="G118" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="H118" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="119" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A119" s="5">
+        <v>116</v>
+      </c>
+      <c r="B119" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C119" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D119" s="6" t="s">
+        <v>314</v>
+      </c>
+      <c r="E119" t="s">
+        <v>315</v>
+      </c>
+      <c r="G119" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="H119" t="s">
+        <v>244</v>
+      </c>
+      <c r="J119" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="120" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A120" s="5">
+        <v>117</v>
+      </c>
+      <c r="B120" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C120" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D120" s="6" t="s">
+        <v>316</v>
+      </c>
+      <c r="E120" t="s">
+        <v>317</v>
+      </c>
+      <c r="G120" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="H120" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="121" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A121" s="5">
+        <v>118</v>
+      </c>
+      <c r="B121" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C121" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D121" s="6" t="s">
+        <v>318</v>
+      </c>
+      <c r="E121" t="s">
+        <v>319</v>
+      </c>
+      <c r="G121" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="H121" t="s">
+        <v>244</v>
+      </c>
+      <c r="J121" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A122" s="5">
+        <v>119</v>
+      </c>
+      <c r="B122" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C122" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D122" s="6" t="s">
+        <v>320</v>
+      </c>
+      <c r="E122" t="s">
+        <v>321</v>
+      </c>
+      <c r="G122" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="H122" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="123" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A123" s="5">
+        <v>120</v>
+      </c>
+      <c r="B123" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C123" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D123" s="6" t="s">
+        <v>322</v>
+      </c>
+      <c r="E123" t="s">
+        <v>323</v>
+      </c>
+      <c r="G123" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="H123" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="124" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A124" s="5">
+        <v>121</v>
+      </c>
+      <c r="B124" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C124" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D124" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="E124" t="s">
+        <v>325</v>
+      </c>
+      <c r="F124" s="6" t="s">
+        <v>848</v>
+      </c>
+      <c r="G124" s="6" t="s">
+        <v>845</v>
+      </c>
+      <c r="H124" t="s">
+        <v>244</v>
+      </c>
+      <c r="J124" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="125" spans="1:10" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A125" s="5">
+        <v>122</v>
+      </c>
+      <c r="B125" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C125" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D125" s="6" t="s">
+        <v>326</v>
+      </c>
+      <c r="E125" t="s">
+        <v>327</v>
+      </c>
+      <c r="G125" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="H125" t="s">
+        <v>244</v>
+      </c>
+      <c r="J125" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="126" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A126" s="5">
+        <v>123</v>
+      </c>
+      <c r="B126" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C126" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D126" s="6" t="s">
+        <v>328</v>
+      </c>
+      <c r="E126" t="s">
+        <v>329</v>
+      </c>
+      <c r="G126" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="H126" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="127" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A127" s="5">
+        <v>124</v>
+      </c>
+      <c r="B127" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C127" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D127" s="6" t="s">
+        <v>330</v>
+      </c>
+      <c r="E127" t="s">
+        <v>331</v>
+      </c>
+      <c r="G127" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="H127" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="128" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A128" s="5">
+        <v>125</v>
+      </c>
+      <c r="B128" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C128" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D128" s="6" t="s">
+        <v>332</v>
+      </c>
+      <c r="E128" t="s">
+        <v>333</v>
+      </c>
+      <c r="G128" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="H128" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="129" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A129" s="5">
+        <v>126</v>
+      </c>
+      <c r="B129" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C129" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D129" s="6" t="s">
+        <v>334</v>
+      </c>
+      <c r="E129" t="s">
+        <v>335</v>
+      </c>
+      <c r="G129" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="H129" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="130" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A130" s="5">
+        <v>127</v>
+      </c>
+      <c r="B130" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C130" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D130" s="6" t="s">
+        <v>336</v>
+      </c>
+      <c r="E130" t="s">
+        <v>337</v>
+      </c>
+      <c r="G130" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="H130" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="131" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A131" s="5">
+        <v>128</v>
+      </c>
+      <c r="B131" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="C131" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="D131" s="6" t="s">
+        <v>339</v>
+      </c>
+      <c r="E131" t="s">
+        <v>340</v>
+      </c>
+      <c r="G131" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="H131" t="s">
+        <v>244</v>
+      </c>
+      <c r="J131" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="132" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A132" s="5">
+        <v>129</v>
+      </c>
+      <c r="B132" s="5" t="s">
+        <v>293</v>
+      </c>
+      <c r="C132" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="D132" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="E132" t="s">
+        <v>342</v>
+      </c>
+      <c r="G132" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="H132" t="s">
+        <v>244</v>
       </c>
     </row>
   </sheetData>
@@ -6274,862 +6739,862 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>311</v>
+        <v>343</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>312</v>
+        <v>344</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>313</v>
+        <v>345</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>314</v>
+        <v>346</v>
       </c>
       <c r="B2" t="s">
-        <v>315</v>
+        <v>347</v>
       </c>
       <c r="C2" t="s">
-        <v>316</v>
+        <v>348</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>317</v>
+        <v>349</v>
       </c>
       <c r="B3" t="s">
-        <v>318</v>
+        <v>350</v>
       </c>
       <c r="C3" t="s">
-        <v>316</v>
+        <v>348</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>319</v>
+        <v>351</v>
       </c>
       <c r="B4" t="s">
-        <v>320</v>
+        <v>352</v>
       </c>
       <c r="C4" t="s">
-        <v>316</v>
+        <v>348</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>321</v>
+        <v>353</v>
       </c>
       <c r="B5" t="s">
-        <v>322</v>
+        <v>354</v>
       </c>
       <c r="C5" t="s">
-        <v>323</v>
+        <v>355</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>324</v>
+        <v>356</v>
       </c>
       <c r="B6" t="s">
-        <v>325</v>
+        <v>357</v>
       </c>
       <c r="C6" t="s">
-        <v>323</v>
+        <v>355</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>326</v>
+        <v>358</v>
       </c>
       <c r="B7" t="s">
-        <v>327</v>
+        <v>359</v>
       </c>
       <c r="C7" t="s">
-        <v>323</v>
+        <v>355</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>328</v>
+        <v>360</v>
       </c>
       <c r="B8" t="s">
-        <v>329</v>
+        <v>361</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>330</v>
+        <v>362</v>
       </c>
       <c r="B9" t="s">
-        <v>331</v>
+        <v>363</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>332</v>
+        <v>364</v>
       </c>
       <c r="B10" t="s">
-        <v>333</v>
+        <v>365</v>
       </c>
       <c r="C10" t="s">
-        <v>323</v>
+        <v>355</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>334</v>
+        <v>366</v>
       </c>
       <c r="B11" t="s">
-        <v>335</v>
+        <v>367</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>336</v>
+        <v>368</v>
       </c>
       <c r="B12" t="s">
-        <v>337</v>
+        <v>369</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>338</v>
+        <v>370</v>
       </c>
       <c r="B13" t="s">
-        <v>339</v>
+        <v>371</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>340</v>
+        <v>372</v>
       </c>
       <c r="B14" t="s">
-        <v>341</v>
+        <v>373</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>342</v>
+        <v>374</v>
       </c>
       <c r="B15" t="s">
-        <v>343</v>
+        <v>375</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>344</v>
+        <v>376</v>
       </c>
       <c r="B16" t="s">
-        <v>345</v>
+        <v>377</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>346</v>
+        <v>378</v>
       </c>
       <c r="B17" t="s">
-        <v>347</v>
+        <v>379</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>348</v>
+        <v>380</v>
       </c>
       <c r="B18" t="s">
-        <v>349</v>
+        <v>381</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>350</v>
+        <v>382</v>
       </c>
       <c r="B19" t="s">
-        <v>351</v>
+        <v>383</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>352</v>
+        <v>384</v>
       </c>
       <c r="B20" t="s">
-        <v>353</v>
+        <v>385</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>354</v>
+        <v>386</v>
       </c>
       <c r="B21" t="s">
-        <v>355</v>
+        <v>387</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>356</v>
+        <v>388</v>
       </c>
       <c r="B22" t="s">
-        <v>357</v>
+        <v>389</v>
       </c>
       <c r="C22" t="s">
-        <v>323</v>
+        <v>355</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>358</v>
+        <v>390</v>
       </c>
       <c r="B23" t="s">
-        <v>359</v>
+        <v>391</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>360</v>
+        <v>392</v>
       </c>
       <c r="B24" t="s">
-        <v>361</v>
+        <v>393</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>362</v>
+        <v>394</v>
       </c>
       <c r="B25" t="s">
-        <v>363</v>
+        <v>395</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>364</v>
+        <v>396</v>
       </c>
       <c r="B26" t="s">
-        <v>365</v>
+        <v>397</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>366</v>
+        <v>398</v>
       </c>
       <c r="B27" t="s">
-        <v>367</v>
+        <v>399</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>368</v>
+        <v>400</v>
       </c>
       <c r="B28" t="s">
-        <v>369</v>
+        <v>401</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>370</v>
+        <v>402</v>
       </c>
       <c r="B29" t="s">
-        <v>371</v>
+        <v>403</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>372</v>
+        <v>404</v>
       </c>
       <c r="B30" t="s">
-        <v>373</v>
+        <v>405</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>374</v>
+        <v>406</v>
       </c>
       <c r="B31" t="s">
-        <v>375</v>
+        <v>407</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>376</v>
+        <v>408</v>
       </c>
       <c r="B32" t="s">
-        <v>377</v>
+        <v>409</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>378</v>
+        <v>410</v>
       </c>
       <c r="B33" t="s">
-        <v>379</v>
+        <v>411</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>380</v>
+        <v>412</v>
       </c>
       <c r="B34" t="s">
-        <v>381</v>
+        <v>413</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>382</v>
+        <v>414</v>
       </c>
       <c r="B35" t="s">
-        <v>383</v>
+        <v>415</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>384</v>
+        <v>416</v>
       </c>
       <c r="B36" t="s">
-        <v>385</v>
+        <v>417</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>386</v>
+        <v>418</v>
       </c>
       <c r="B37" t="s">
-        <v>387</v>
+        <v>419</v>
       </c>
       <c r="C37" t="s">
-        <v>323</v>
+        <v>355</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>388</v>
+        <v>420</v>
       </c>
       <c r="B38" t="s">
-        <v>389</v>
+        <v>421</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>390</v>
+        <v>422</v>
       </c>
       <c r="B39" t="s">
-        <v>391</v>
+        <v>423</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>392</v>
+        <v>424</v>
       </c>
       <c r="B40" t="s">
-        <v>393</v>
+        <v>425</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>394</v>
+        <v>426</v>
       </c>
       <c r="B41" t="s">
-        <v>395</v>
+        <v>427</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>396</v>
+        <v>428</v>
       </c>
       <c r="B42" t="s">
-        <v>397</v>
+        <v>429</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>398</v>
+        <v>430</v>
       </c>
       <c r="B43" t="s">
-        <v>399</v>
+        <v>431</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>400</v>
+        <v>432</v>
       </c>
       <c r="B44" t="s">
-        <v>401</v>
+        <v>433</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>402</v>
+        <v>434</v>
       </c>
       <c r="B45" t="s">
-        <v>403</v>
+        <v>435</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>404</v>
+        <v>436</v>
       </c>
       <c r="B46" t="s">
-        <v>405</v>
+        <v>437</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>406</v>
+        <v>438</v>
       </c>
       <c r="B47" t="s">
-        <v>407</v>
+        <v>439</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>408</v>
+        <v>440</v>
       </c>
       <c r="B48" t="s">
-        <v>409</v>
+        <v>441</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>410</v>
+        <v>442</v>
       </c>
       <c r="B49" t="s">
-        <v>411</v>
+        <v>443</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>412</v>
+        <v>444</v>
       </c>
       <c r="B50" t="s">
-        <v>413</v>
+        <v>445</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>414</v>
+        <v>446</v>
       </c>
       <c r="B51" t="s">
-        <v>415</v>
+        <v>447</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>416</v>
+        <v>448</v>
       </c>
       <c r="B52" t="s">
-        <v>417</v>
+        <v>449</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>418</v>
+        <v>450</v>
       </c>
       <c r="B53" t="s">
-        <v>419</v>
+        <v>451</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>420</v>
+        <v>452</v>
       </c>
       <c r="B54" t="s">
-        <v>421</v>
+        <v>453</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>422</v>
+        <v>454</v>
       </c>
       <c r="B55" t="s">
-        <v>423</v>
+        <v>455</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>424</v>
+        <v>456</v>
       </c>
       <c r="B56" t="s">
-        <v>425</v>
+        <v>457</v>
       </c>
       <c r="C56" t="s">
-        <v>323</v>
+        <v>355</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>426</v>
+        <v>458</v>
       </c>
       <c r="B57" t="s">
-        <v>427</v>
+        <v>459</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>428</v>
+        <v>460</v>
       </c>
       <c r="B58" t="s">
-        <v>429</v>
+        <v>461</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>430</v>
+        <v>462</v>
       </c>
       <c r="B59" t="s">
-        <v>431</v>
+        <v>463</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>432</v>
+        <v>464</v>
       </c>
       <c r="B60" t="s">
-        <v>433</v>
+        <v>465</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>434</v>
+        <v>466</v>
       </c>
       <c r="B61" t="s">
-        <v>435</v>
+        <v>467</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>436</v>
+        <v>468</v>
       </c>
       <c r="B62" t="s">
-        <v>437</v>
+        <v>469</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>438</v>
+        <v>470</v>
       </c>
       <c r="B63" t="s">
-        <v>439</v>
+        <v>471</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>440</v>
+        <v>472</v>
       </c>
       <c r="B64" t="s">
-        <v>441</v>
+        <v>473</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>442</v>
+        <v>474</v>
       </c>
       <c r="B65" t="s">
-        <v>443</v>
+        <v>475</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>444</v>
+        <v>476</v>
       </c>
       <c r="B66" t="s">
-        <v>445</v>
+        <v>477</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>446</v>
+        <v>478</v>
       </c>
       <c r="B67" t="s">
-        <v>447</v>
+        <v>479</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>448</v>
+        <v>480</v>
       </c>
       <c r="B68" t="s">
-        <v>449</v>
+        <v>481</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>450</v>
+        <v>482</v>
       </c>
       <c r="B69" t="s">
-        <v>451</v>
+        <v>483</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>452</v>
+        <v>484</v>
       </c>
       <c r="B70" t="s">
-        <v>453</v>
+        <v>485</v>
       </c>
       <c r="C70" t="s">
-        <v>323</v>
+        <v>355</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>454</v>
+        <v>486</v>
       </c>
       <c r="B71" t="s">
-        <v>455</v>
+        <v>487</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>456</v>
+        <v>488</v>
       </c>
       <c r="B72" t="s">
-        <v>457</v>
+        <v>489</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>458</v>
+        <v>490</v>
       </c>
       <c r="B73" t="s">
-        <v>459</v>
+        <v>491</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>460</v>
+        <v>492</v>
       </c>
       <c r="B74" t="s">
-        <v>461</v>
+        <v>493</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>462</v>
+        <v>494</v>
       </c>
       <c r="B75" t="s">
-        <v>463</v>
+        <v>495</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>464</v>
+        <v>496</v>
       </c>
       <c r="B76" t="s">
-        <v>465</v>
+        <v>497</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>466</v>
+        <v>498</v>
       </c>
       <c r="B77" t="s">
-        <v>467</v>
+        <v>499</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>468</v>
+        <v>500</v>
       </c>
       <c r="B78" t="s">
-        <v>469</v>
+        <v>501</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>470</v>
+        <v>502</v>
       </c>
       <c r="B79" t="s">
-        <v>471</v>
+        <v>503</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>472</v>
+        <v>504</v>
       </c>
       <c r="B80" t="s">
-        <v>473</v>
+        <v>505</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>474</v>
+        <v>506</v>
       </c>
       <c r="B81" t="s">
-        <v>475</v>
+        <v>507</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>476</v>
+        <v>508</v>
       </c>
       <c r="B82" t="s">
-        <v>477</v>
+        <v>509</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>478</v>
+        <v>510</v>
       </c>
       <c r="B83" t="s">
-        <v>479</v>
+        <v>511</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>480</v>
+        <v>512</v>
       </c>
       <c r="B84" t="s">
-        <v>481</v>
+        <v>513</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>482</v>
+        <v>514</v>
       </c>
       <c r="B85" t="s">
-        <v>483</v>
+        <v>515</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>484</v>
+        <v>516</v>
       </c>
       <c r="B86" t="s">
-        <v>485</v>
+        <v>517</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>486</v>
+        <v>518</v>
       </c>
       <c r="B87" t="s">
-        <v>487</v>
+        <v>519</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>488</v>
+        <v>520</v>
       </c>
       <c r="B88" t="s">
-        <v>489</v>
+        <v>521</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>490</v>
+        <v>522</v>
       </c>
       <c r="B89" t="s">
-        <v>491</v>
+        <v>523</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>492</v>
+        <v>524</v>
       </c>
       <c r="B90" t="s">
-        <v>493</v>
+        <v>525</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>494</v>
+        <v>526</v>
       </c>
       <c r="B91" t="s">
-        <v>495</v>
+        <v>527</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>496</v>
+        <v>528</v>
       </c>
       <c r="B92" t="s">
-        <v>497</v>
+        <v>529</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>498</v>
+        <v>530</v>
       </c>
       <c r="B93" t="s">
-        <v>499</v>
+        <v>531</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>500</v>
+        <v>532</v>
       </c>
       <c r="B94" t="s">
-        <v>501</v>
+        <v>533</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>502</v>
+        <v>534</v>
       </c>
       <c r="B95" t="s">
-        <v>503</v>
+        <v>535</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>504</v>
+        <v>536</v>
       </c>
       <c r="B96" t="s">
-        <v>505</v>
+        <v>537</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>506</v>
+        <v>538</v>
       </c>
       <c r="B97" t="s">
-        <v>507</v>
+        <v>539</v>
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>508</v>
+        <v>540</v>
       </c>
       <c r="B98" t="s">
-        <v>509</v>
+        <v>541</v>
       </c>
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>510</v>
+        <v>542</v>
       </c>
       <c r="B99" t="s">
-        <v>511</v>
+        <v>543</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>512</v>
+        <v>544</v>
       </c>
       <c r="B100" t="s">
-        <v>513</v>
+        <v>545</v>
       </c>
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>514</v>
+        <v>546</v>
       </c>
       <c r="B101" t="s">
-        <v>515</v>
+        <v>547</v>
       </c>
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>516</v>
+        <v>548</v>
       </c>
       <c r="B102" t="s">
-        <v>517</v>
+        <v>549</v>
       </c>
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>518</v>
+        <v>550</v>
       </c>
       <c r="B103" t="s">
-        <v>519</v>
+        <v>551</v>
       </c>
     </row>
   </sheetData>
@@ -7164,400 +7629,400 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>311</v>
+        <v>343</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>312</v>
+        <v>344</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>313</v>
+        <v>345</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>520</v>
+        <v>552</v>
       </c>
       <c r="B2" t="s">
-        <v>521</v>
+        <v>553</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>522</v>
+        <v>554</v>
       </c>
       <c r="B3" t="s">
-        <v>365</v>
+        <v>397</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>523</v>
+        <v>555</v>
       </c>
       <c r="B4" t="s">
-        <v>524</v>
+        <v>556</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>525</v>
+        <v>557</v>
       </c>
       <c r="B5" t="s">
-        <v>526</v>
+        <v>558</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>527</v>
+        <v>559</v>
       </c>
       <c r="B6" t="s">
-        <v>528</v>
+        <v>560</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>529</v>
+        <v>561</v>
       </c>
       <c r="B7" t="s">
-        <v>530</v>
+        <v>562</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>531</v>
+        <v>563</v>
       </c>
       <c r="B8" t="s">
-        <v>532</v>
+        <v>564</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>533</v>
+        <v>565</v>
       </c>
       <c r="B9" t="s">
-        <v>534</v>
+        <v>566</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>535</v>
+        <v>567</v>
       </c>
       <c r="B10" t="s">
-        <v>536</v>
+        <v>568</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>537</v>
+        <v>569</v>
       </c>
       <c r="B11" t="s">
-        <v>538</v>
+        <v>570</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>539</v>
+        <v>571</v>
       </c>
       <c r="B12" t="s">
-        <v>540</v>
+        <v>572</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>541</v>
+        <v>573</v>
       </c>
       <c r="B13" t="s">
-        <v>542</v>
+        <v>574</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>543</v>
+        <v>575</v>
       </c>
       <c r="B14" t="s">
-        <v>544</v>
+        <v>576</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>545</v>
+        <v>577</v>
       </c>
       <c r="B15" t="s">
-        <v>546</v>
+        <v>578</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>547</v>
+        <v>579</v>
       </c>
       <c r="B16" t="s">
-        <v>548</v>
+        <v>580</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>549</v>
+        <v>581</v>
       </c>
       <c r="B17" t="s">
-        <v>550</v>
+        <v>582</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>551</v>
+        <v>583</v>
       </c>
       <c r="B18" t="s">
-        <v>552</v>
+        <v>584</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>323</v>
+        <v>355</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>553</v>
+        <v>585</v>
       </c>
       <c r="B19" t="s">
-        <v>554</v>
+        <v>586</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>555</v>
+        <v>587</v>
       </c>
       <c r="B20" t="s">
-        <v>556</v>
+        <v>588</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>557</v>
+        <v>589</v>
       </c>
       <c r="B21" t="s">
-        <v>558</v>
+        <v>590</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>559</v>
+        <v>591</v>
       </c>
       <c r="B22" t="s">
-        <v>560</v>
+        <v>592</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>561</v>
+        <v>593</v>
       </c>
       <c r="B23" t="s">
-        <v>562</v>
+        <v>594</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>563</v>
+        <v>595</v>
       </c>
       <c r="B24" t="s">
-        <v>564</v>
+        <v>596</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>565</v>
+        <v>597</v>
       </c>
       <c r="B25" t="s">
-        <v>566</v>
+        <v>598</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>567</v>
+        <v>599</v>
       </c>
       <c r="B26" t="s">
-        <v>568</v>
+        <v>600</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>569</v>
+        <v>601</v>
       </c>
       <c r="B27" t="s">
-        <v>570</v>
+        <v>602</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>571</v>
+        <v>603</v>
       </c>
       <c r="B28" t="s">
-        <v>572</v>
+        <v>604</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>573</v>
+        <v>605</v>
       </c>
       <c r="B29" t="s">
-        <v>574</v>
+        <v>606</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>575</v>
+        <v>607</v>
       </c>
       <c r="B30" t="s">
-        <v>576</v>
+        <v>608</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>577</v>
+        <v>609</v>
       </c>
       <c r="B31" t="s">
-        <v>578</v>
+        <v>610</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>579</v>
+        <v>611</v>
       </c>
       <c r="B32" t="s">
-        <v>580</v>
+        <v>612</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>581</v>
+        <v>613</v>
       </c>
       <c r="B33" t="s">
-        <v>582</v>
+        <v>614</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>583</v>
+        <v>615</v>
       </c>
       <c r="B34" t="s">
-        <v>584</v>
+        <v>616</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>585</v>
+        <v>617</v>
       </c>
       <c r="B35" t="s">
-        <v>586</v>
+        <v>618</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>587</v>
+        <v>619</v>
       </c>
       <c r="B36" t="s">
-        <v>588</v>
+        <v>620</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>589</v>
+        <v>621</v>
       </c>
       <c r="B37" t="s">
-        <v>590</v>
+        <v>622</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>591</v>
+        <v>623</v>
       </c>
       <c r="B38" t="s">
-        <v>592</v>
+        <v>624</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>593</v>
+        <v>625</v>
       </c>
       <c r="B39" t="s">
-        <v>594</v>
+        <v>626</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>595</v>
+        <v>627</v>
       </c>
       <c r="B40" t="s">
-        <v>596</v>
+        <v>628</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>597</v>
+        <v>629</v>
       </c>
       <c r="B41" t="s">
-        <v>598</v>
+        <v>630</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>599</v>
+        <v>631</v>
       </c>
       <c r="B42" t="s">
-        <v>600</v>
+        <v>632</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>601</v>
+        <v>633</v>
       </c>
       <c r="B43" t="s">
-        <v>602</v>
+        <v>634</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>603</v>
+        <v>635</v>
       </c>
       <c r="B44" t="s">
-        <v>604</v>
+        <v>636</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>605</v>
+        <v>637</v>
       </c>
       <c r="B45" t="s">
-        <v>433</v>
+        <v>465</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>606</v>
+        <v>638</v>
       </c>
       <c r="B46" t="s">
-        <v>607</v>
+        <v>639</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>608</v>
+        <v>640</v>
       </c>
       <c r="B47" t="s">
-        <v>609</v>
+        <v>641</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>610</v>
+        <v>642</v>
       </c>
       <c r="B48" t="s">
-        <v>611</v>
+        <v>643</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>612</v>
+        <v>644</v>
       </c>
       <c r="B49" t="s">
-        <v>613</v>
+        <v>645</v>
       </c>
     </row>
   </sheetData>
@@ -7588,389 +8053,389 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>311</v>
+        <v>343</v>
       </c>
       <c r="B1" t="s">
-        <v>312</v>
+        <v>344</v>
       </c>
       <c r="C1" t="s">
-        <v>313</v>
+        <v>345</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>614</v>
+        <v>646</v>
       </c>
       <c r="B2" t="s">
-        <v>615</v>
+        <v>647</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>616</v>
+        <v>648</v>
       </c>
       <c r="B3" t="s">
-        <v>617</v>
+        <v>649</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>618</v>
+        <v>650</v>
       </c>
       <c r="B4" t="s">
-        <v>619</v>
+        <v>651</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>620</v>
+        <v>652</v>
       </c>
       <c r="B5" t="s">
-        <v>621</v>
+        <v>653</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>622</v>
+        <v>654</v>
       </c>
       <c r="B6" t="s">
-        <v>623</v>
+        <v>655</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>624</v>
+        <v>656</v>
       </c>
       <c r="B7" t="s">
-        <v>381</v>
+        <v>413</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>625</v>
+        <v>657</v>
       </c>
       <c r="B8" t="s">
-        <v>626</v>
+        <v>658</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>627</v>
+        <v>659</v>
       </c>
       <c r="B9" t="s">
-        <v>628</v>
+        <v>660</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>629</v>
+        <v>661</v>
       </c>
       <c r="B10" t="s">
-        <v>630</v>
+        <v>662</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>631</v>
+        <v>663</v>
       </c>
       <c r="B11" t="s">
-        <v>632</v>
+        <v>664</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>633</v>
+        <v>665</v>
       </c>
       <c r="B12" t="s">
-        <v>341</v>
+        <v>373</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>634</v>
+        <v>666</v>
       </c>
       <c r="B13" t="s">
-        <v>635</v>
+        <v>667</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>636</v>
+        <v>668</v>
       </c>
       <c r="B14" t="s">
-        <v>637</v>
+        <v>669</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>638</v>
+        <v>670</v>
       </c>
       <c r="B15" t="s">
-        <v>351</v>
+        <v>383</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>639</v>
+        <v>671</v>
       </c>
       <c r="B16" t="s">
-        <v>355</v>
+        <v>387</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>640</v>
+        <v>672</v>
       </c>
       <c r="B17" t="s">
-        <v>641</v>
+        <v>673</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>642</v>
+        <v>674</v>
       </c>
       <c r="B18" t="s">
-        <v>643</v>
+        <v>675</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>644</v>
+        <v>676</v>
       </c>
       <c r="B19" t="s">
-        <v>417</v>
+        <v>449</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>645</v>
+        <v>677</v>
       </c>
       <c r="B20" t="s">
-        <v>646</v>
+        <v>678</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>647</v>
+        <v>679</v>
       </c>
       <c r="B21" t="s">
-        <v>648</v>
+        <v>680</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>649</v>
+        <v>681</v>
       </c>
       <c r="B22" t="s">
-        <v>650</v>
+        <v>682</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>651</v>
+        <v>683</v>
       </c>
       <c r="B23" t="s">
-        <v>652</v>
+        <v>684</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>653</v>
+        <v>685</v>
       </c>
       <c r="B24" t="s">
-        <v>654</v>
+        <v>686</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>655</v>
+        <v>687</v>
       </c>
       <c r="B25" t="s">
-        <v>393</v>
+        <v>425</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>656</v>
+        <v>688</v>
       </c>
       <c r="B26" t="s">
-        <v>657</v>
+        <v>689</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>658</v>
+        <v>690</v>
       </c>
       <c r="B27" t="s">
-        <v>659</v>
+        <v>691</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>660</v>
+        <v>692</v>
       </c>
       <c r="B28" t="s">
-        <v>661</v>
+        <v>693</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>662</v>
+        <v>694</v>
       </c>
       <c r="B29" t="s">
-        <v>663</v>
+        <v>695</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>664</v>
+        <v>696</v>
       </c>
       <c r="B30" t="s">
-        <v>665</v>
+        <v>697</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>666</v>
+        <v>698</v>
       </c>
       <c r="B31" t="s">
-        <v>667</v>
+        <v>699</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>668</v>
+        <v>700</v>
       </c>
       <c r="B32" t="s">
-        <v>669</v>
+        <v>701</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>670</v>
+        <v>702</v>
       </c>
       <c r="B33" t="s">
-        <v>671</v>
+        <v>703</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>672</v>
+        <v>704</v>
       </c>
       <c r="B34" t="s">
-        <v>673</v>
+        <v>705</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>674</v>
+        <v>706</v>
       </c>
       <c r="B35" t="s">
-        <v>675</v>
+        <v>707</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>676</v>
+        <v>708</v>
       </c>
       <c r="B36" t="s">
-        <v>677</v>
+        <v>709</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>678</v>
+        <v>710</v>
       </c>
       <c r="B37" t="s">
-        <v>679</v>
+        <v>711</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>680</v>
+        <v>712</v>
       </c>
       <c r="B38" t="s">
-        <v>681</v>
+        <v>713</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>682</v>
+        <v>714</v>
       </c>
       <c r="B39" t="s">
-        <v>683</v>
+        <v>715</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>684</v>
+        <v>716</v>
       </c>
       <c r="B40" t="s">
-        <v>685</v>
+        <v>717</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>686</v>
+        <v>718</v>
       </c>
       <c r="B41" t="s">
-        <v>687</v>
+        <v>719</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>688</v>
+        <v>720</v>
       </c>
       <c r="B42" t="s">
-        <v>689</v>
+        <v>721</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>690</v>
+        <v>722</v>
       </c>
       <c r="B43" t="s">
-        <v>691</v>
+        <v>723</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>692</v>
+        <v>724</v>
       </c>
       <c r="B44" t="s">
-        <v>693</v>
+        <v>725</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>694</v>
+        <v>726</v>
       </c>
       <c r="B45" t="s">
-        <v>695</v>
+        <v>727</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>696</v>
+        <v>728</v>
       </c>
       <c r="B46" t="s">
-        <v>697</v>
+        <v>729</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>698</v>
+        <v>730</v>
       </c>
       <c r="B47" t="s">
-        <v>699</v>
+        <v>731</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>700</v>
+        <v>732</v>
       </c>
       <c r="B48" t="s">
-        <v>701</v>
+        <v>733</v>
       </c>
     </row>
   </sheetData>
@@ -8001,541 +8466,541 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>311</v>
+        <v>343</v>
       </c>
       <c r="B1" t="s">
-        <v>312</v>
+        <v>344</v>
       </c>
       <c r="C1" t="s">
-        <v>313</v>
+        <v>345</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>702</v>
+        <v>734</v>
       </c>
       <c r="B2" t="s">
-        <v>703</v>
+        <v>735</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>704</v>
+        <v>736</v>
       </c>
       <c r="B3" t="s">
-        <v>705</v>
+        <v>737</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>706</v>
+        <v>738</v>
       </c>
       <c r="B4" t="s">
-        <v>707</v>
+        <v>739</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>708</v>
+        <v>740</v>
       </c>
       <c r="B5" t="s">
-        <v>709</v>
+        <v>741</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>710</v>
+        <v>742</v>
       </c>
       <c r="B6" t="s">
-        <v>711</v>
+        <v>743</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>712</v>
+        <v>744</v>
       </c>
       <c r="B7" t="s">
-        <v>713</v>
+        <v>745</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>714</v>
+        <v>746</v>
       </c>
       <c r="B8" t="s">
-        <v>715</v>
+        <v>747</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>716</v>
+        <v>748</v>
       </c>
       <c r="B9" t="s">
-        <v>717</v>
+        <v>749</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>718</v>
+        <v>750</v>
       </c>
       <c r="B10" t="s">
-        <v>719</v>
+        <v>751</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>720</v>
+        <v>752</v>
       </c>
       <c r="B11" t="s">
-        <v>721</v>
+        <v>753</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>722</v>
+        <v>754</v>
       </c>
       <c r="B12" t="s">
-        <v>723</v>
+        <v>755</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>724</v>
+        <v>756</v>
       </c>
       <c r="B13" t="s">
-        <v>725</v>
+        <v>757</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>726</v>
+        <v>758</v>
       </c>
       <c r="B14" t="s">
-        <v>727</v>
+        <v>759</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>728</v>
+        <v>760</v>
       </c>
       <c r="B15" t="s">
-        <v>729</v>
+        <v>761</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>730</v>
+        <v>762</v>
       </c>
       <c r="B16" t="s">
-        <v>731</v>
+        <v>763</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>732</v>
+        <v>764</v>
       </c>
       <c r="B17" t="s">
-        <v>733</v>
+        <v>765</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>734</v>
+        <v>766</v>
       </c>
       <c r="B18" t="s">
-        <v>735</v>
+        <v>767</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>736</v>
+        <v>768</v>
       </c>
       <c r="B19" t="s">
-        <v>737</v>
+        <v>769</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>738</v>
+        <v>770</v>
       </c>
       <c r="B20" t="s">
-        <v>739</v>
+        <v>771</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>740</v>
+        <v>772</v>
       </c>
       <c r="B21" t="s">
-        <v>741</v>
+        <v>773</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>742</v>
+        <v>774</v>
       </c>
       <c r="B22" t="s">
-        <v>743</v>
+        <v>775</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>744</v>
+        <v>776</v>
       </c>
       <c r="B23" t="s">
-        <v>745</v>
+        <v>777</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>746</v>
+        <v>778</v>
       </c>
       <c r="B24" t="s">
-        <v>747</v>
+        <v>779</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>748</v>
+        <v>780</v>
       </c>
       <c r="B25" t="s">
-        <v>749</v>
+        <v>781</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>750</v>
+        <v>782</v>
       </c>
       <c r="B26" t="s">
-        <v>751</v>
+        <v>783</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>752</v>
+        <v>784</v>
       </c>
       <c r="B27" t="s">
-        <v>753</v>
+        <v>785</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>754</v>
+        <v>786</v>
       </c>
       <c r="B28" t="s">
-        <v>755</v>
+        <v>787</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>756</v>
+        <v>788</v>
       </c>
       <c r="B29" t="s">
-        <v>757</v>
+        <v>789</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>758</v>
+        <v>790</v>
       </c>
       <c r="B30" t="s">
-        <v>759</v>
+        <v>791</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>760</v>
+        <v>792</v>
       </c>
       <c r="B31" t="s">
-        <v>761</v>
+        <v>793</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>762</v>
+        <v>794</v>
       </c>
       <c r="B32" t="s">
-        <v>763</v>
+        <v>795</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>764</v>
+        <v>796</v>
       </c>
       <c r="B33" t="s">
-        <v>765</v>
+        <v>797</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>766</v>
+        <v>798</v>
       </c>
       <c r="B34" t="s">
-        <v>391</v>
+        <v>423</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>767</v>
+        <v>799</v>
       </c>
       <c r="B35" t="s">
-        <v>399</v>
+        <v>431</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>768</v>
+        <v>800</v>
       </c>
       <c r="B36" t="s">
-        <v>325</v>
+        <v>357</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>769</v>
+        <v>801</v>
       </c>
       <c r="B37" t="s">
-        <v>409</v>
+        <v>441</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>770</v>
+        <v>802</v>
       </c>
       <c r="B38" t="s">
-        <v>771</v>
+        <v>803</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>772</v>
+        <v>804</v>
       </c>
       <c r="B39" t="s">
-        <v>411</v>
+        <v>443</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>773</v>
+        <v>805</v>
       </c>
       <c r="B40" t="s">
-        <v>375</v>
+        <v>407</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>774</v>
+        <v>806</v>
       </c>
       <c r="B41" t="s">
-        <v>415</v>
+        <v>447</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>775</v>
+        <v>807</v>
       </c>
       <c r="B42" t="s">
-        <v>588</v>
+        <v>620</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>776</v>
+        <v>808</v>
       </c>
       <c r="B43" t="s">
-        <v>669</v>
+        <v>701</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>777</v>
+        <v>809</v>
       </c>
       <c r="B44" t="s">
-        <v>673</v>
+        <v>705</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>778</v>
+        <v>810</v>
       </c>
       <c r="B45" t="s">
-        <v>419</v>
+        <v>451</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>779</v>
+        <v>811</v>
       </c>
       <c r="B46" t="s">
-        <v>421</v>
+        <v>453</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>780</v>
+        <v>812</v>
       </c>
       <c r="B47" t="s">
-        <v>423</v>
+        <v>455</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>781</v>
+        <v>813</v>
       </c>
       <c r="B48" t="s">
-        <v>596</v>
+        <v>628</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>782</v>
+        <v>814</v>
       </c>
       <c r="B49" t="s">
-        <v>598</v>
+        <v>630</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>783</v>
+        <v>815</v>
       </c>
       <c r="B50" t="s">
-        <v>602</v>
+        <v>634</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>784</v>
+        <v>816</v>
       </c>
       <c r="B51" t="s">
-        <v>437</v>
+        <v>469</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>785</v>
+        <v>817</v>
       </c>
       <c r="B52" t="s">
-        <v>683</v>
+        <v>715</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>786</v>
+        <v>818</v>
       </c>
       <c r="B53" t="s">
-        <v>439</v>
+        <v>471</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>787</v>
+        <v>819</v>
       </c>
       <c r="B54" t="s">
-        <v>687</v>
+        <v>719</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>788</v>
+        <v>820</v>
       </c>
       <c r="B55" t="s">
-        <v>327</v>
+        <v>359</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>789</v>
+        <v>821</v>
       </c>
       <c r="B56" t="s">
-        <v>449</v>
+        <v>481</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>790</v>
+        <v>822</v>
       </c>
       <c r="B57" t="s">
-        <v>691</v>
+        <v>723</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>791</v>
+        <v>823</v>
       </c>
       <c r="B58" t="s">
-        <v>792</v>
+        <v>824</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>793</v>
+        <v>825</v>
       </c>
       <c r="B59" t="s">
-        <v>794</v>
+        <v>826</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>795</v>
+        <v>827</v>
       </c>
       <c r="B60" t="s">
-        <v>796</v>
+        <v>828</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>797</v>
+        <v>829</v>
       </c>
       <c r="B61" t="s">
-        <v>798</v>
+        <v>830</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>799</v>
+        <v>831</v>
       </c>
       <c r="B62" t="s">
-        <v>800</v>
+        <v>832</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>801</v>
+        <v>833</v>
       </c>
       <c r="B63" t="s">
-        <v>802</v>
+        <v>834</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>803</v>
+        <v>835</v>
       </c>
       <c r="B64" t="s">
-        <v>804</v>
+        <v>836</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>805</v>
+        <v>837</v>
       </c>
       <c r="B65" t="s">
-        <v>806</v>
+        <v>838</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>807</v>
+        <v>839</v>
       </c>
       <c r="B66" t="s">
-        <v>808</v>
+        <v>840</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>809</v>
+        <v>841</v>
       </c>
       <c r="B67" t="s">
-        <v>810</v>
+        <v>842</v>
       </c>
     </row>
   </sheetData>
@@ -8564,12 +9029,12 @@
   <sheetData>
     <row r="1" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>811</v>
+        <v>843</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>812</v>
+        <v>844</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
@@ -8584,12 +9049,12 @@
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>813</v>
+        <v>845</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>814</v>
+        <v>846</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
@@ -8599,7 +9064,7 @@
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>815</v>
+        <v>847</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ReadMe: Completely overhauled readme
</commit_message>
<xml_diff>
--- a/Spreadsheets/Issue_Log.xlsx
+++ b/Spreadsheets/Issue_Log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\Spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CE991EE-C820-48C8-9CAF-E9362E952FC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B356DF2B-3219-40D2-9DC8-AF64E186116C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1461" uniqueCount="849">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1522" uniqueCount="866">
   <si>
     <t>#</t>
   </si>
@@ -2673,6 +2673,57 @@
   </si>
   <si>
     <t>All good, but actually make the messagebox inside the match the same colour as the opponent being battled, this is already done for the match rewards</t>
+  </si>
+  <si>
+    <t>Add New Cheats "CHT.All_Coins", "CHT.All_Costumes", "CHT.All_Sleeves" to grant all coins costumes and sleeves respectively.</t>
+  </si>
+  <si>
+    <t>Prevent scrolling when a messagebox is visible, currently scrolling acts as a mouse click and clears the message</t>
+  </si>
+  <si>
+    <t>When the starterset from the card mart is purchased, the message pops up saying "You received starter set". The following message is the shopkeeper thanking the player for purchasing it but the messagebox is in the same format as the you received starter set when instead it should show the message from the card mart NPC</t>
+  </si>
+  <si>
+    <t>The "EX Era Rules" button in options is overlapping the fairer retreat rules button instead of all 3 being equally spaced apart</t>
+  </si>
+  <si>
+    <t>Sleeves owned doesn't seem to count the 3 default owned sleeves granted at the beginning of the game. These should count</t>
+  </si>
+  <si>
+    <t>Search</t>
+  </si>
+  <si>
+    <t>In the search/filter mode in deck/card view, hide the background_scroller and top_and_right_border. Make the filter_border and filter_background visible in the filter mode. When the filter mode is exited and the card view is returned to, hide the filter bodrder and background and make the background scroller and top and right border visible again</t>
+  </si>
+  <si>
+    <t>Add a new row in the deck/card search/filter mode for "Has Power/Body". Use the poke-power / poke-body icon in the subtype icons folder. When selected they should turn into the color version the same as the rest of the icons with the growing/shrinking animation like the rest of the icons. These should be "And" type search, meaning if the delta sub type is ticket and has Body is ticked then only delta species WITH a body should be displayed. Add this row under sub type</t>
+  </si>
+  <si>
+    <t>Add a new row in the deck/card search/filter mode for "Illustrator". Have this be a free text box. It should be applied as an "AND" search so if someone searches for Name = "Pikachu" and Illustrator = "Ken Sugimori" only Pikachu cards WITH Ken Sugimori art should be shown. Put this at the bottom just above the sort by name/set buttons</t>
+  </si>
+  <si>
+    <t>With the change above (141) this will now give a larger width to use in the screen, extend all the filter options to make use of the entire width of the screen now that the right border is hidden. For all the label headers on the left hand side, make all the text on one line instead of two lines for most of them. With this same change, we can have "Technical Machine" on one line in the button instead of two</t>
+  </si>
+  <si>
+    <t>ACTUALLY SCRAP THIS, I WILL REVISIT TAB AND SPACEBAR REQUIREMENTS</t>
+  </si>
+  <si>
+    <t>On the costumes screen there's a large amount of space after the last row and the scrollbar near the end of the screen. The last costume has something between 50-100pixels of empty space to the right of it, then the scrollbar, then another 10-20 pixels, then the edge of the screen</t>
+  </si>
+  <si>
+    <t>For the fun of it make the activated cheat codes rainbow coloured font like the "BONUS!" in the card packs</t>
+  </si>
+  <si>
+    <t>The Starting deck (Your First Deck) and the cards gifted by the starter box at the beginning of the game don't line up. In the deck are 4 farfetched but the game gifts 4 voltorb and 2 farfetched. Make both the starter your first deck and starter box have the exact same cards: 2 farfetchd, 4 diglet, 4 doduo, 4 machop, 2 poliwag, 4 rattata, 4 staryu, 2 voltorb, 16 fighting energy, 12 water energy, 2 potion, 2 super potion, 2 bill (all base set)</t>
+  </si>
+  <si>
+    <t>Remove case sensitivity from the cheats so cheat codes can be entered into the name field without worrying about capitals</t>
+  </si>
+  <si>
+    <t>When activating a card cheat, the unlocked sets count doesn't increase, but the sets are marked as completed</t>
+  </si>
+  <si>
+    <t>The two NPCS (Local woman and local man) (the man gifts money) that are stood next to each other have their sprites mixed up. Swap the sprites of these two NPCs</t>
   </si>
 </sst>
 </file>
@@ -3263,7 +3314,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J132"/>
+  <dimension ref="A1:J147"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="5" bestFit="1" customWidth="1"/>
@@ -5923,7 +5974,7 @@
         <v>274</v>
       </c>
       <c r="G101" s="6" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="H101" t="s">
         <v>218</v>
@@ -5948,8 +5999,11 @@
       <c r="E102" t="s">
         <v>276</v>
       </c>
+      <c r="F102" s="6" t="s">
+        <v>859</v>
+      </c>
       <c r="G102" s="6" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="H102" t="s">
         <v>218</v>
@@ -5998,7 +6052,7 @@
         <v>281</v>
       </c>
       <c r="G104" s="6" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="H104" t="s">
         <v>218</v>
@@ -6128,7 +6182,7 @@
         <v>292</v>
       </c>
       <c r="G109" s="6" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="H109" t="s">
         <v>218</v>
@@ -6154,7 +6208,7 @@
         <v>296</v>
       </c>
       <c r="G110" s="6" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="H110" t="s">
         <v>218</v>
@@ -6177,7 +6231,7 @@
         <v>298</v>
       </c>
       <c r="G111" s="6" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="H111" t="s">
         <v>218</v>
@@ -6700,6 +6754,261 @@
       </c>
       <c r="H132" t="s">
         <v>244</v>
+      </c>
+    </row>
+    <row r="133" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="A133" s="5">
+        <v>130</v>
+      </c>
+      <c r="B133" s="5" t="s">
+        <v>293</v>
+      </c>
+      <c r="C133" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="D133" s="6" t="s">
+        <v>862</v>
+      </c>
+      <c r="G133" s="6" t="s">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="134" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A134" s="5">
+        <v>131</v>
+      </c>
+      <c r="B134" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="C134" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="D134" s="6" t="s">
+        <v>863</v>
+      </c>
+      <c r="G134" s="6" t="s">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="135" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A135" s="5">
+        <v>132</v>
+      </c>
+      <c r="B135" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="C135" s="5" t="s">
+        <v>846</v>
+      </c>
+      <c r="D135" s="6" t="s">
+        <v>861</v>
+      </c>
+      <c r="G135" s="6" t="s">
+        <v>846</v>
+      </c>
+    </row>
+    <row r="136" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A136" s="5">
+        <v>133</v>
+      </c>
+      <c r="B136" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="C136" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="D136" s="6" t="s">
+        <v>864</v>
+      </c>
+      <c r="G136" s="6" t="s">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="137" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A137" s="5">
+        <v>134</v>
+      </c>
+      <c r="B137" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="C137" s="5" t="s">
+        <v>846</v>
+      </c>
+      <c r="D137" s="6" t="s">
+        <v>849</v>
+      </c>
+      <c r="G137" s="6" t="s">
+        <v>846</v>
+      </c>
+    </row>
+    <row r="138" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A138" s="5">
+        <v>135</v>
+      </c>
+      <c r="B138" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C138" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D138" s="6" t="s">
+        <v>850</v>
+      </c>
+      <c r="G138" s="6" t="s">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="139" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A139" s="5">
+        <v>136</v>
+      </c>
+      <c r="B139" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C139" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D139" s="6" t="s">
+        <v>851</v>
+      </c>
+      <c r="G139" s="6" t="s">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="140" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A140" s="5">
+        <v>137</v>
+      </c>
+      <c r="B140" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C140" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D140" s="6" t="s">
+        <v>865</v>
+      </c>
+      <c r="G140" s="6" t="s">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="141" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A141" s="5">
+        <v>138</v>
+      </c>
+      <c r="B141" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C141" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D141" s="6" t="s">
+        <v>852</v>
+      </c>
+      <c r="G141" s="6" t="s">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="142" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A142" s="5">
+        <v>139</v>
+      </c>
+      <c r="B142" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C142" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="D142" s="6" t="s">
+        <v>853</v>
+      </c>
+      <c r="G142" s="6" t="s">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="143" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="A143" s="5">
+        <v>140</v>
+      </c>
+      <c r="B143" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C143" s="5" t="s">
+        <v>846</v>
+      </c>
+      <c r="D143" s="6" t="s">
+        <v>856</v>
+      </c>
+      <c r="G143" s="6" t="s">
+        <v>846</v>
+      </c>
+    </row>
+    <row r="144" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A144" s="5">
+        <v>141</v>
+      </c>
+      <c r="B144" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C144" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D144" s="6" t="s">
+        <v>855</v>
+      </c>
+      <c r="G144" s="6" t="s">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="145" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A145" s="5">
+        <v>142</v>
+      </c>
+      <c r="B145" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C145" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D145" s="6" t="s">
+        <v>858</v>
+      </c>
+      <c r="G145" s="6" t="s">
+        <v>846</v>
+      </c>
+    </row>
+    <row r="146" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A146" s="5">
+        <v>143</v>
+      </c>
+      <c r="B146" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C146" s="5" t="s">
+        <v>846</v>
+      </c>
+      <c r="D146" s="6" t="s">
+        <v>857</v>
+      </c>
+      <c r="G146" s="6" t="s">
+        <v>846</v>
+      </c>
+    </row>
+    <row r="147" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A147" s="5">
+        <v>144</v>
+      </c>
+      <c r="B147" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C147" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D147" s="6" t="s">
+        <v>860</v>
+      </c>
+      <c r="G147" s="6" t="s">
+        <v>844</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Search: Added new search items for illustrator, has power and body
</commit_message>
<xml_diff>
--- a/Spreadsheets/Issue_Log.xlsx
+++ b/Spreadsheets/Issue_Log.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Game_Issues" sheetId="1" state="visible" r:id="rId1"/>
@@ -685,8 +685,8 @@
     <col width="19" customWidth="1" style="6" min="7" max="7"/>
     <col width="11.109375" bestFit="1" customWidth="1" style="7" min="8" max="9"/>
     <col width="16" customWidth="1" style="7" min="10" max="10"/>
-    <col width="9.109375" customWidth="1" style="7" min="11" max="12"/>
-    <col width="9.109375" customWidth="1" style="7" min="13" max="16384"/>
+    <col width="9.109375" customWidth="1" style="7" min="11" max="13"/>
+    <col width="9.109375" customWidth="1" style="7" min="14" max="16384"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4828,6 +4828,11 @@
           <t>08/08/2026</t>
         </is>
       </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
       <c r="J101" t="inlineStr">
         <is>
           <t>Live: 2</t>
@@ -4873,6 +4878,11 @@
           <t>08/08/2026</t>
         </is>
       </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="103" ht="90" customHeight="1">
       <c r="A103" s="5" t="n">
@@ -4948,6 +4958,11 @@
           <t>08/08/2026</t>
         </is>
       </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
       <c r="J104" t="inlineStr">
         <is>
           <t>Live: 1</t>
@@ -5148,6 +5163,11 @@
           <t>08/08/2026</t>
         </is>
       </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
       <c r="J109" t="inlineStr">
         <is>
           <t>Live: 1</t>
@@ -5188,6 +5208,11 @@
           <t>08/08/2026</t>
         </is>
       </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="5" t="n">
@@ -5223,6 +5248,11 @@
           <t>08/08/2026</t>
         </is>
       </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="112" ht="30" customHeight="1">
       <c r="A112" s="5" t="n">
@@ -5498,6 +5528,11 @@
           <t>23/08/2026</t>
         </is>
       </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="5" t="n">
@@ -5533,6 +5568,11 @@
           <t>23/08/2026</t>
         </is>
       </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
       <c r="J119" t="inlineStr">
         <is>
           <t>Live: 2</t>
@@ -5573,6 +5613,11 @@
           <t>23/08/2026</t>
         </is>
       </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="5" t="n">
@@ -5608,6 +5653,11 @@
           <t>23/08/2026</t>
         </is>
       </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
       <c r="J121" t="inlineStr">
         <is>
           <t>Live: 1</t>
@@ -5648,6 +5698,11 @@
           <t>23/08/2026</t>
         </is>
       </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="123" ht="60" customHeight="1">
       <c r="A123" s="5" t="n">
@@ -5683,6 +5738,11 @@
           <t>23/08/2026</t>
         </is>
       </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="124" ht="30" customHeight="1">
       <c r="A124" s="5" t="n">
@@ -5763,6 +5823,11 @@
           <t>23/08/2026</t>
         </is>
       </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
       <c r="J125" t="inlineStr">
         <is>
           <t>Live: 1</t>
@@ -5803,6 +5868,11 @@
           <t>23/08/2026</t>
         </is>
       </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="127" ht="30" customHeight="1">
       <c r="A127" s="5" t="n">
@@ -5838,6 +5908,11 @@
           <t>23/08/2026</t>
         </is>
       </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="128" ht="30" customHeight="1">
       <c r="A128" s="5" t="n">
@@ -5873,6 +5948,11 @@
           <t>23/08/2026</t>
         </is>
       </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="129" ht="30" customHeight="1">
       <c r="A129" s="5" t="n">
@@ -5908,6 +5988,11 @@
           <t>23/08/2026</t>
         </is>
       </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="130" ht="30" customHeight="1">
       <c r="A130" s="5" t="n">
@@ -5943,6 +6028,11 @@
           <t>23/08/2026</t>
         </is>
       </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="131" ht="30" customHeight="1">
       <c r="A131" s="5" t="n">
@@ -5978,6 +6068,11 @@
           <t>23/08/2026</t>
         </is>
       </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
       <c r="J131" t="inlineStr">
         <is>
           <t>Live: 1</t>
@@ -6018,6 +6113,11 @@
           <t>23/08/2026</t>
         </is>
       </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="133" ht="43.2" customHeight="1">
       <c r="A133" s="5" t="n">
@@ -6095,10 +6195,15 @@
       </c>
       <c r="G135" s="6" t="inlineStr">
         <is>
-          <t>Untested Fix</t>
+          <t>Issue Resolved</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
         <is>
           <t>24/08/2026</t>
         </is>
@@ -6155,10 +6260,15 @@
       </c>
       <c r="G137" s="6" t="inlineStr">
         <is>
-          <t>Untested Fix</t>
+          <t>Issue Resolved</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
         <is>
           <t>24/08/2026</t>
         </is>
@@ -6308,9 +6418,19 @@
           <t>Add a new row in the deck/card search/filter mode for "Has Power/Body". Use the poke-power / poke-body icon in the subtype icons folder. When selected they should turn into the color version the same as the rest of the icons with the growing/shrinking animation like the rest of the icons. These should be "And" type search, meaning if the delta sub type is ticket and has Body is ticked then only delta species WITH a body should be displayed. Add this row under sub type</t>
         </is>
       </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>New HAS POWER / OR BODY icon row added to the card search screen, directly under POKEMON SUB TYPE (Card_Search_Overlay._build_power_row + POWER_FILTERS table). Uses the existing icon_power/icon_body and color_icon_power/color_icon_body art from Icons/Subtype_Icons, routed through the same _make_icon and _on_icon_input path as every other icon row, so the greyed-&gt;colour swap and the grow/shrink pulse come for free with no new animation code. Matching: Deck_Build_And_Card_View_Script._card_matches_power, fed by two booleans (has_power / has_body) precomputed per card in _ensure_set_metadata_loaded so the 3340 ability arrays are not held in memory. POWER covers 'Poke-Power' AND the older 'Pokemon Power' (Base-&gt;Neo printed every ability under that one name; e-Card split it into the activated Poke-Power and the passive Poke-Body, so the old name belongs with Power) = 463 cards. BODY = 'Poke-Body' = 385 cards. Type strings are matched as a lowercased SUBSTRING so the accented e cannot break the compare. DELIBERATE DECISION 1: the row is NOT part of the Pokemon/Trainer supertype lock, unlike the rows above it - the 8 Claw Fossil / Root Fossil Trainers in ex2/ex12/ex13/ex16 carry a real Poke-Body, and locking Card Type to Pokemon would hide cards that genuinely match. It behaves like the RARITY row: a whole-card property that simply ANDs with everything else, which is the behaviour asked for (delta + body = 33 cards, verified against the data). DELIBERATE DECISION 2: ticking BOTH power and body is OR, not AND, matching the documented 'OR within a category, AND between categories' rule the whole screen follows - only 2 cards in the entire pool have both, so AND-within would be a near-empty result. Say if you want that flipped. BODY is gated on ecard1 (first non-promo set with one, same convention as the trainer sub type gates); POWER is ungated, it exists from base1. Debug: 'ISSUE #140/#143 FIX ACTIVE' print reports the bottom y of the rebuilt row stack against FOOTER_TOP.</t>
+        </is>
+      </c>
       <c r="G143" s="6" t="inlineStr">
         <is>
-          <t>New Functionality</t>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
         </is>
       </c>
     </row>
@@ -6383,9 +6503,19 @@
           <t>Add a new row in the deck/card search/filter mode for "Illustrator". Have this be a free text box. It should be applied as an "AND" search so if someone searches for Name = "Pikachu" and Illustrator = "Ken Sugimori" only Pikachu cards WITH Ken Sugimori art should be shown. Put this at the bottom just above the sort by name/set buttons</t>
         </is>
       </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>New ILLUSTRATOR free-text row added to the card search screen, directly above the SORT BY buttons (Card_Search_Overlay._build_illustrator_row). Same size, font and Enter-to-search behaviour as the NAME box so the two read as a pair; 30 char limit; cleared by RESET; counts towards whether SEARCH is enabled. Matched in Deck_Build_And_Card_View_Script._card_matches_search as a case-insensitive SUBSTRING ANDed against every other filter, exactly like the name box - so Name='Pikachu' + Illustrator='Ken Sugimori' returns the 4 Sugimori Pikachu cards (verified against the data; 'sugimori' alone returns 540). Free text rather than a picker because there are 89 distinct illustrators in the card pool, far too many for an icon or button row. The card's 'artist' field is now cached in _ensure_set_metadata_loaded alongside name/ supertype/subtypes. Note 31 cards in the pool have no artist recorded, so they never match a non-empty illustrator box. Shares the ISSUE #140/#143 layout debug print.</t>
+        </is>
+      </c>
       <c r="G146" s="6" t="inlineStr">
         <is>
-          <t>New Functionality</t>
+          <t>Untested Fix</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
UI: Fixed attack buttons so 5 attacks fit and further paginate.
</commit_message>
<xml_diff>
--- a/Spreadsheets/Issue_Log.xlsx
+++ b/Spreadsheets/Issue_Log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\Spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81A4458A-2A26-4E50-8648-7628D7432C79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B1EEAE3-459F-40BF-860E-84235AD6FD1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Game_Issues" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1657" uniqueCount="907">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1677" uniqueCount="912">
   <si>
     <t>#</t>
   </si>
@@ -2901,6 +2901,21 @@
   </si>
   <si>
     <t>Fix Failed</t>
+  </si>
+  <si>
+    <t>Technical machines simply attach to the active pokemon but some of these TMs explicity state "Choose a pokemon" to attach it to. If any card, tool, technical machine, trainer or anything else say "choose" then the choice should always be offered</t>
+  </si>
+  <si>
+    <t>Similarly, Shining magikarp says "your opponent may draw up to 2 cards". When used by the opponent, this forces the player to draw 2 cards without asking. The player should be prompted to choose 0, 1 or 2 cards. Always ensure a choice offers the choice</t>
+  </si>
+  <si>
+    <t>Similarly, loudreds surprise says "choose 1 card from opponents hand without looking". This just randomly selects one which functionally is the same but again, it says CHOOSE so should offer the choice even if it's still technically random.</t>
+  </si>
+  <si>
+    <t>If multiple TMs are attached to the active pokemon, at the end of the turn only the last one is discarded instead of all of them.</t>
+  </si>
+  <si>
+    <t>Exploud (Ex emerald card 3) has Mega throw. This is a 5 energy attack but the game only seems to count it as 4. It also only displays as 4 so it's as if the game completely ignores anything after the 4th energy and never is aware of a 5th for any attack?</t>
   </si>
 </sst>
 </file>
@@ -3491,23 +3506,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J157"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:J162"/>
+  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.44140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.44140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="125.33203125" style="6" customWidth="1"/>
-    <col min="5" max="5" width="255.5546875" style="6" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="14.453125" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.453125" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="125.36328125" style="6" customWidth="1"/>
+    <col min="5" max="5" width="255.54296875" style="6" hidden="1" customWidth="1"/>
     <col min="6" max="6" width="102" style="6" customWidth="1"/>
     <col min="7" max="7" width="19" style="6" customWidth="1"/>
-    <col min="8" max="9" width="11.109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="11.08984375" style="7" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="16" style="7" customWidth="1"/>
-    <col min="11" max="17" width="9.109375" style="7" customWidth="1"/>
-    <col min="18" max="16384" width="9.109375" style="7"/>
+    <col min="11" max="17" width="9.08984375" style="7" customWidth="1"/>
+    <col min="18" max="16384" width="9.08984375" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -3539,7 +3554,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="5">
         <v>1</v>
       </c>
@@ -3565,7 +3580,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" ht="86.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="5">
         <v>2</v>
       </c>
@@ -3597,7 +3612,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" ht="115.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="5">
         <v>3</v>
       </c>
@@ -3626,7 +3641,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="5">
         <v>4</v>
       </c>
@@ -3655,7 +3670,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
         <v>5</v>
       </c>
@@ -3684,7 +3699,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="172.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" ht="172.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="5">
         <v>6</v>
       </c>
@@ -3713,7 +3728,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="201.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" ht="201.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="5">
         <v>7</v>
       </c>
@@ -3742,7 +3757,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="5">
         <v>8</v>
       </c>
@@ -3771,7 +3786,7 @@
         <v>46220</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="100.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="5">
         <v>9</v>
       </c>
@@ -3800,7 +3815,7 @@
         <v>46220</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="5">
         <v>10</v>
       </c>
@@ -3829,7 +3844,7 @@
         <v>46220</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" ht="100.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="5">
         <v>11</v>
       </c>
@@ -3855,7 +3870,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="302.39999999999998" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" ht="302.39999999999998" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="5">
         <v>12</v>
       </c>
@@ -3884,7 +3899,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="5">
         <v>13</v>
       </c>
@@ -3910,7 +3925,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="5">
         <v>14</v>
       </c>
@@ -3933,7 +3948,7 @@
         <v>46223</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="5">
         <v>15</v>
       </c>
@@ -3959,7 +3974,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="5">
         <v>16</v>
       </c>
@@ -3988,7 +4003,7 @@
         <v>46220</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="5">
         <v>17</v>
       </c>
@@ -4017,7 +4032,7 @@
         <v>46220</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="5">
         <v>18</v>
       </c>
@@ -4043,7 +4058,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="5">
         <v>19</v>
       </c>
@@ -4069,7 +4084,7 @@
         <v>46224</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" ht="86.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="5">
         <v>20</v>
       </c>
@@ -4095,7 +4110,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="5">
         <v>21</v>
       </c>
@@ -4121,7 +4136,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="5">
         <v>22</v>
       </c>
@@ -4147,7 +4162,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="5">
         <v>23</v>
       </c>
@@ -4170,7 +4185,7 @@
         <v>46221</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="5">
         <v>23</v>
       </c>
@@ -4196,7 +4211,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:10" ht="115.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="5">
         <v>24</v>
       </c>
@@ -4225,7 +4240,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="5">
         <v>25</v>
       </c>
@@ -4251,7 +4266,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="5">
         <v>26</v>
       </c>
@@ -4280,7 +4295,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="5">
         <v>27</v>
       </c>
@@ -4306,7 +4321,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="5">
         <v>28</v>
       </c>
@@ -4332,7 +4347,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" s="5">
         <v>29</v>
       </c>
@@ -4358,7 +4373,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32" s="5">
         <v>30</v>
       </c>
@@ -4384,7 +4399,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:10" ht="57.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="5">
         <v>31</v>
       </c>
@@ -4410,7 +4425,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="345.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:10" ht="345.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="5">
         <v>32</v>
       </c>
@@ -4439,7 +4454,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="35" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="5">
         <v>33</v>
       </c>
@@ -4468,7 +4483,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="36" spans="1:10" ht="144" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:10" ht="144" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="5">
         <v>34</v>
       </c>
@@ -4497,7 +4512,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="37" spans="1:10" ht="172.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:10" ht="172.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="5">
         <v>35</v>
       </c>
@@ -4526,7 +4541,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="38" spans="1:10" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:10" ht="57.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="5">
         <v>36</v>
       </c>
@@ -4552,7 +4567,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="39" spans="1:10" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:10" ht="57.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="5">
         <v>37</v>
       </c>
@@ -4581,7 +4596,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="40" spans="1:10" ht="129.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:10" ht="129.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="5">
         <v>38</v>
       </c>
@@ -4610,7 +4625,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="41" spans="1:10" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="5">
         <v>39</v>
       </c>
@@ -4636,7 +4651,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="42" spans="1:10" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:10" ht="57.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="5">
         <v>40</v>
       </c>
@@ -4665,7 +4680,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="43" spans="1:10" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="5">
         <v>41</v>
       </c>
@@ -4691,7 +4706,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="44" spans="1:10" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:10" ht="100.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="5">
         <v>42</v>
       </c>
@@ -4717,7 +4732,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="45" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="5">
         <v>43</v>
       </c>
@@ -4743,7 +4758,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="46" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="5">
         <v>44</v>
       </c>
@@ -4775,7 +4790,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="47" spans="1:10" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:10" ht="86.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="5">
         <v>45</v>
       </c>
@@ -4801,7 +4816,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="48" spans="1:10" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:10" ht="115.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="5">
         <v>46</v>
       </c>
@@ -4827,7 +4842,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="49" spans="1:10" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:10" ht="57.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="5">
         <v>47</v>
       </c>
@@ -4853,7 +4868,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="50" spans="1:10" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="5">
         <v>48</v>
       </c>
@@ -4879,7 +4894,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="51" spans="1:10" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:10" ht="86.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="5">
         <v>49</v>
       </c>
@@ -4905,7 +4920,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="52" spans="1:10" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:10" ht="57.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" s="5">
         <v>50</v>
       </c>
@@ -4931,7 +4946,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="53" spans="1:10" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:10" ht="57.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" s="5">
         <v>51</v>
       </c>
@@ -4957,7 +4972,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="54" spans="1:10" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:10" ht="100.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" s="5">
         <v>52</v>
       </c>
@@ -4986,7 +5001,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="55" spans="1:10" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" s="5">
         <v>53</v>
       </c>
@@ -5012,7 +5027,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="56" spans="1:10" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A56" s="5">
         <v>54</v>
       </c>
@@ -5038,7 +5053,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="57" spans="1:10" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A57" s="5">
         <v>55</v>
       </c>
@@ -5064,7 +5079,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="58" spans="1:10" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:10" ht="86.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A58" s="5">
         <v>56</v>
       </c>
@@ -5090,7 +5105,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="59" spans="1:10" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A59" s="5">
         <v>57</v>
       </c>
@@ -5116,7 +5131,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="60" spans="1:10" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A60" s="5">
         <v>58</v>
       </c>
@@ -5142,7 +5157,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="61" spans="1:10" ht="172.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:10" ht="172.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A61" s="5">
         <v>59</v>
       </c>
@@ -5171,7 +5186,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="62" spans="1:10" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A62" s="5">
         <v>60</v>
       </c>
@@ -5197,7 +5212,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="63" spans="1:10" ht="129.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:10" ht="129.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A63" s="5">
         <v>61</v>
       </c>
@@ -5223,7 +5238,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A64" s="5">
         <v>62</v>
       </c>
@@ -5246,7 +5261,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="65" spans="1:10" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A65" s="5">
         <v>63</v>
       </c>
@@ -5272,7 +5287,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A66" s="5">
         <v>64</v>
       </c>
@@ -5295,7 +5310,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="67" spans="1:10" ht="129.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:10" ht="129.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A67" s="5">
         <v>65</v>
       </c>
@@ -5321,7 +5336,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A68" s="5">
         <v>66</v>
       </c>
@@ -5341,7 +5356,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A69" s="5">
         <v>67</v>
       </c>
@@ -5361,7 +5376,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A70" s="5">
         <v>68</v>
       </c>
@@ -5381,7 +5396,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="71" spans="1:10" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A71" s="5">
         <v>69</v>
       </c>
@@ -5407,7 +5422,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A72" s="5">
         <v>70</v>
       </c>
@@ -5433,7 +5448,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A73" s="5">
         <v>71</v>
       </c>
@@ -5459,7 +5474,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A74" s="5">
         <v>72</v>
       </c>
@@ -5476,7 +5491,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="75" spans="1:10" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75" s="5">
         <v>73</v>
       </c>
@@ -5502,7 +5517,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="76" spans="1:10" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A76" s="5">
         <v>77</v>
       </c>
@@ -5528,7 +5543,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="77" spans="1:10" ht="187.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:10" ht="187.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A77" s="5">
         <v>74</v>
       </c>
@@ -5557,7 +5572,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="78" spans="1:10" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:10" ht="86.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A78" s="5">
         <v>75</v>
       </c>
@@ -5586,7 +5601,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="79" spans="1:10" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A79" s="5">
         <v>76</v>
       </c>
@@ -5609,7 +5624,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="80" spans="1:10" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:10" ht="100.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80" s="5">
         <v>77</v>
       </c>
@@ -5635,7 +5650,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="81" spans="1:10" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A81" s="5">
         <v>78</v>
       </c>
@@ -5661,7 +5676,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="82" spans="1:10" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A82" s="5">
         <v>79</v>
       </c>
@@ -5687,7 +5702,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="83" spans="1:10" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:10" ht="57.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A83" s="5">
         <v>81</v>
       </c>
@@ -5713,7 +5728,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="84" spans="1:10" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:10" ht="100.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A84" s="5">
         <v>80</v>
       </c>
@@ -5739,7 +5754,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="85" spans="1:10" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:10" ht="86.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A85" s="5">
         <v>81</v>
       </c>
@@ -5765,7 +5780,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="86" spans="1:10" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:10" ht="100.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A86" s="5">
         <v>82</v>
       </c>
@@ -5791,7 +5806,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="87" spans="1:10" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A87" s="5">
         <v>83</v>
       </c>
@@ -5817,7 +5832,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="88" spans="1:10" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:10" ht="100.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A88" s="5">
         <v>84</v>
       </c>
@@ -5843,7 +5858,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A89" s="5">
         <v>85</v>
       </c>
@@ -5869,7 +5884,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="90" spans="1:10" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A90" s="5">
         <v>86</v>
       </c>
@@ -5895,7 +5910,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="91" spans="1:10" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:10" ht="57.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A91" s="5">
         <v>87</v>
       </c>
@@ -5921,7 +5936,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="92" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A92" s="5">
         <v>88</v>
       </c>
@@ -5947,7 +5962,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="93" spans="1:10" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:10" ht="86.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A93" s="5">
         <v>89</v>
       </c>
@@ -5973,7 +5988,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="94" spans="1:10" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:10" ht="86.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A94" s="5">
         <v>90</v>
       </c>
@@ -5999,7 +6014,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="95" spans="1:10" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:10" ht="57.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A95" s="5">
         <v>91</v>
       </c>
@@ -6025,7 +6040,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="96" spans="1:10" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A96" s="5">
         <v>92</v>
       </c>
@@ -6045,7 +6060,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="97" spans="1:10" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A97" s="5">
         <v>92</v>
       </c>
@@ -6065,7 +6080,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A98" s="5">
         <v>93</v>
       </c>
@@ -6094,7 +6109,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="99" spans="1:10" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A99" s="5">
         <v>94</v>
       </c>
@@ -6114,7 +6129,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="100" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A100" s="5">
         <v>95</v>
       </c>
@@ -6140,7 +6155,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="101" spans="1:10" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A101" s="5">
         <v>96</v>
       </c>
@@ -6166,7 +6181,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A102" s="5">
         <v>97</v>
       </c>
@@ -6195,7 +6210,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="103" spans="1:10" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:10" ht="86.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A103" s="5">
         <v>98</v>
       </c>
@@ -6221,7 +6236,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A104" s="5">
         <v>99</v>
       </c>
@@ -6247,7 +6262,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="105" spans="1:10" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A105" s="5">
         <v>100</v>
       </c>
@@ -6273,7 +6288,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A106" s="5">
         <v>101</v>
       </c>
@@ -6299,7 +6314,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="107" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A107" s="5">
         <v>102</v>
       </c>
@@ -6325,7 +6340,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="108" spans="1:10" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A108" s="5">
         <v>103</v>
       </c>
@@ -6351,7 +6366,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="109" spans="1:10" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A109" s="5">
         <v>104</v>
       </c>
@@ -6377,7 +6392,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="110" spans="1:10" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A110" s="5">
         <v>105</v>
       </c>
@@ -6403,7 +6418,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A111" s="5">
         <v>106</v>
       </c>
@@ -6429,7 +6444,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="112" spans="1:10" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A112" s="5">
         <v>109</v>
       </c>
@@ -6455,7 +6470,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="113" spans="1:9" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:9" ht="57.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A113" s="5">
         <v>110</v>
       </c>
@@ -6481,7 +6496,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="114" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:9" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A114" s="5">
         <v>111</v>
       </c>
@@ -6507,7 +6522,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="115" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:9" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A115" s="5">
         <v>112</v>
       </c>
@@ -6533,7 +6548,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="116" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:9" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A116" s="5">
         <v>113</v>
       </c>
@@ -6559,7 +6574,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="117" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:9" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A117" s="5">
         <v>114</v>
       </c>
@@ -6585,7 +6600,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="118" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:9" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A118" s="5">
         <v>115</v>
       </c>
@@ -6611,7 +6626,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="119" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A119" s="5">
         <v>116</v>
       </c>
@@ -6637,7 +6652,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="120" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:9" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A120" s="5">
         <v>117</v>
       </c>
@@ -6663,7 +6678,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="121" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A121" s="5">
         <v>118</v>
       </c>
@@ -6689,7 +6704,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="122" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A122" s="5">
         <v>119</v>
       </c>
@@ -6715,7 +6730,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="123" spans="1:9" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:9" ht="57.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A123" s="5">
         <v>120</v>
       </c>
@@ -6741,7 +6756,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="124" spans="1:9" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:9" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A124" s="5">
         <v>121</v>
       </c>
@@ -6770,7 +6785,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="125" spans="1:9" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:9" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A125" s="5">
         <v>122</v>
       </c>
@@ -6796,7 +6811,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="126" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A126" s="5">
         <v>123</v>
       </c>
@@ -6822,7 +6837,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="127" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:9" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A127" s="5">
         <v>124</v>
       </c>
@@ -6848,7 +6863,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="128" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:9" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A128" s="5">
         <v>125</v>
       </c>
@@ -6874,7 +6889,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="129" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:9" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A129" s="5">
         <v>126</v>
       </c>
@@ -6900,7 +6915,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="130" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:9" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A130" s="5">
         <v>127</v>
       </c>
@@ -6926,7 +6941,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="131" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:9" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A131" s="5">
         <v>128</v>
       </c>
@@ -6952,7 +6967,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="132" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:9" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A132" s="5">
         <v>129</v>
       </c>
@@ -6978,7 +6993,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="133" spans="1:9" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:9" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A133" s="5">
         <v>130</v>
       </c>
@@ -7004,7 +7019,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="134" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A134" s="5">
         <v>131</v>
       </c>
@@ -7030,7 +7045,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="135" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:9" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A135" s="5">
         <v>132</v>
       </c>
@@ -7056,7 +7071,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="136" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:9" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A136" s="5">
         <v>133</v>
       </c>
@@ -7085,7 +7100,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="137" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A137" s="5">
         <v>134</v>
       </c>
@@ -7111,7 +7126,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="138" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A138" s="5">
         <v>135</v>
       </c>
@@ -7137,7 +7152,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="139" spans="1:9" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:9" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A139" s="5">
         <v>136</v>
       </c>
@@ -7163,7 +7178,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="140" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:9" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A140" s="5">
         <v>137</v>
       </c>
@@ -7189,7 +7204,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="141" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A141" s="5">
         <v>138</v>
       </c>
@@ -7215,7 +7230,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="142" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A142" s="5">
         <v>139</v>
       </c>
@@ -7241,7 +7256,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="143" spans="1:9" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:9" ht="57.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A143" s="5">
         <v>140</v>
       </c>
@@ -7267,7 +7282,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="144" spans="1:9" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:9" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A144" s="5">
         <v>141</v>
       </c>
@@ -7296,7 +7311,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="145" spans="1:10" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A145" s="5">
         <v>142</v>
       </c>
@@ -7322,7 +7337,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="146" spans="1:10" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A146" s="5">
         <v>143</v>
       </c>
@@ -7348,7 +7363,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="147" spans="1:10" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A147" s="5">
         <v>144</v>
       </c>
@@ -7374,7 +7389,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="148" spans="1:10" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A148" s="5">
         <v>145</v>
       </c>
@@ -7403,7 +7418,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="149" spans="1:10" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:10" ht="57.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A149" s="5">
         <v>146</v>
       </c>
@@ -7432,7 +7447,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="150" spans="1:10" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A150" s="5">
         <v>147</v>
       </c>
@@ -7458,7 +7473,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="151" spans="1:10" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A151" s="5">
         <v>148</v>
       </c>
@@ -7484,7 +7499,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="152" spans="1:10" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:10" ht="100.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A152" s="5">
         <v>149</v>
       </c>
@@ -7513,7 +7528,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="153" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A153" s="5">
         <v>150</v>
       </c>
@@ -7539,7 +7554,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="154" spans="1:10" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A154" s="5">
         <v>151</v>
       </c>
@@ -7565,7 +7580,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="155" spans="1:10" ht="129.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:10" ht="129.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A155" s="5">
         <v>152</v>
       </c>
@@ -7591,7 +7606,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="156" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A156" s="5">
         <v>154</v>
       </c>
@@ -7617,7 +7632,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="157" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A157" s="5">
         <v>155</v>
       </c>
@@ -7641,6 +7656,91 @@
       </c>
       <c r="J157" t="s">
         <v>20</v>
+      </c>
+    </row>
+    <row r="158" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A158" s="5">
+        <v>156</v>
+      </c>
+      <c r="B158" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="C158" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="D158" s="6" t="s">
+        <v>907</v>
+      </c>
+      <c r="G158" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="159" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A159" s="5">
+        <v>157</v>
+      </c>
+      <c r="B159" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="C159" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="D159" s="6" t="s">
+        <v>908</v>
+      </c>
+      <c r="G159" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="160" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A160" s="5">
+        <v>158</v>
+      </c>
+      <c r="B160" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="C160" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="D160" s="6" t="s">
+        <v>909</v>
+      </c>
+      <c r="G160" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="161" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A161" s="5">
+        <v>159</v>
+      </c>
+      <c r="B161" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="C161" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="D161" s="6" t="s">
+        <v>910</v>
+      </c>
+      <c r="G161" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="162" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A162" s="5">
+        <v>160</v>
+      </c>
+      <c r="B162" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="C162" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="D162" s="6" t="s">
+        <v>911</v>
+      </c>
+      <c r="G162" s="6" t="s">
+        <v>904</v>
       </c>
     </row>
   </sheetData>
@@ -7671,14 +7771,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C103"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.5546875" customWidth="1"/>
+    <col min="1" max="1" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.54296875" customWidth="1"/>
     <col min="3" max="3" width="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="2" t="s">
         <v>403</v>
       </c>
@@ -7689,7 +7789,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>406</v>
       </c>
@@ -7700,7 +7800,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>409</v>
       </c>
@@ -7711,7 +7811,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>411</v>
       </c>
@@ -7722,7 +7822,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>413</v>
       </c>
@@ -7733,7 +7833,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>416</v>
       </c>
@@ -7744,7 +7844,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>418</v>
       </c>
@@ -7755,7 +7855,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>420</v>
       </c>
@@ -7763,7 +7863,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>422</v>
       </c>
@@ -7771,7 +7871,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" ht="72.650000000000006" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>424</v>
       </c>
@@ -7782,7 +7882,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>426</v>
       </c>
@@ -7790,7 +7890,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>428</v>
       </c>
@@ -7798,7 +7898,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>430</v>
       </c>
@@ -7806,7 +7906,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>432</v>
       </c>
@@ -7814,7 +7914,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>434</v>
       </c>
@@ -7822,7 +7922,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>436</v>
       </c>
@@ -7830,7 +7930,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>438</v>
       </c>
@@ -7838,7 +7938,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>440</v>
       </c>
@@ -7846,7 +7946,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>442</v>
       </c>
@@ -7854,7 +7954,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>444</v>
       </c>
@@ -7862,7 +7962,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>446</v>
       </c>
@@ -7870,7 +7970,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>448</v>
       </c>
@@ -7881,7 +7981,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>450</v>
       </c>
@@ -7889,7 +7989,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>452</v>
       </c>
@@ -7897,7 +7997,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>454</v>
       </c>
@@ -7905,7 +8005,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>456</v>
       </c>
@@ -7913,7 +8013,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>458</v>
       </c>
@@ -7921,7 +8021,7 @@
         <v>459</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>460</v>
       </c>
@@ -7929,7 +8029,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>462</v>
       </c>
@@ -7937,7 +8037,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>464</v>
       </c>
@@ -7945,7 +8045,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>466</v>
       </c>
@@ -7953,7 +8053,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>468</v>
       </c>
@@ -7961,7 +8061,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>470</v>
       </c>
@@ -7969,7 +8069,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>472</v>
       </c>
@@ -7977,7 +8077,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>474</v>
       </c>
@@ -7985,7 +8085,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>476</v>
       </c>
@@ -7993,7 +8093,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>478</v>
       </c>
@@ -8004,7 +8104,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>480</v>
       </c>
@@ -8012,7 +8112,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>482</v>
       </c>
@@ -8020,7 +8120,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>484</v>
       </c>
@@ -8028,7 +8128,7 @@
         <v>485</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>486</v>
       </c>
@@ -8036,7 +8136,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>488</v>
       </c>
@@ -8044,7 +8144,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>490</v>
       </c>
@@ -8052,7 +8152,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>492</v>
       </c>
@@ -8060,7 +8160,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>494</v>
       </c>
@@ -8068,7 +8168,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>496</v>
       </c>
@@ -8076,7 +8176,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>498</v>
       </c>
@@ -8084,7 +8184,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>500</v>
       </c>
@@ -8092,7 +8192,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>502</v>
       </c>
@@ -8100,7 +8200,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>504</v>
       </c>
@@ -8108,7 +8208,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>506</v>
       </c>
@@ -8116,7 +8216,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>508</v>
       </c>
@@ -8124,7 +8224,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>510</v>
       </c>
@@ -8132,7 +8232,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>512</v>
       </c>
@@ -8140,7 +8240,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>514</v>
       </c>
@@ -8148,7 +8248,7 @@
         <v>515</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>516</v>
       </c>
@@ -8159,7 +8259,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>518</v>
       </c>
@@ -8167,7 +8267,7 @@
         <v>519</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>520</v>
       </c>
@@ -8175,7 +8275,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>522</v>
       </c>
@@ -8183,7 +8283,7 @@
         <v>523</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>524</v>
       </c>
@@ -8191,7 +8291,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>526</v>
       </c>
@@ -8199,7 +8299,7 @@
         <v>527</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>528</v>
       </c>
@@ -8207,7 +8307,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>530</v>
       </c>
@@ -8215,7 +8315,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>532</v>
       </c>
@@ -8223,7 +8323,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>534</v>
       </c>
@@ -8231,7 +8331,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>536</v>
       </c>
@@ -8239,7 +8339,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>538</v>
       </c>
@@ -8247,7 +8347,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>540</v>
       </c>
@@ -8255,7 +8355,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>542</v>
       </c>
@@ -8263,7 +8363,7 @@
         <v>543</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>544</v>
       </c>
@@ -8274,7 +8374,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>546</v>
       </c>
@@ -8282,7 +8382,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>548</v>
       </c>
@@ -8290,7 +8390,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>550</v>
       </c>
@@ -8298,7 +8398,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>552</v>
       </c>
@@ -8306,7 +8406,7 @@
         <v>553</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>554</v>
       </c>
@@ -8314,7 +8414,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>556</v>
       </c>
@@ -8322,7 +8422,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>558</v>
       </c>
@@ -8330,7 +8430,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>560</v>
       </c>
@@ -8338,7 +8438,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>562</v>
       </c>
@@ -8346,7 +8446,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>564</v>
       </c>
@@ -8354,7 +8454,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>566</v>
       </c>
@@ -8362,7 +8462,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>568</v>
       </c>
@@ -8370,7 +8470,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>570</v>
       </c>
@@ -8378,7 +8478,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>572</v>
       </c>
@@ -8386,7 +8486,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>574</v>
       </c>
@@ -8394,7 +8494,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>576</v>
       </c>
@@ -8402,7 +8502,7 @@
         <v>577</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>578</v>
       </c>
@@ -8410,7 +8510,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>580</v>
       </c>
@@ -8418,7 +8518,7 @@
         <v>581</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>582</v>
       </c>
@@ -8426,7 +8526,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>584</v>
       </c>
@@ -8434,7 +8534,7 @@
         <v>585</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>586</v>
       </c>
@@ -8442,7 +8542,7 @@
         <v>587</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>588</v>
       </c>
@@ -8450,7 +8550,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>590</v>
       </c>
@@ -8458,7 +8558,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>592</v>
       </c>
@@ -8466,7 +8566,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>594</v>
       </c>
@@ -8474,7 +8574,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>596</v>
       </c>
@@ -8482,7 +8582,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>598</v>
       </c>
@@ -8490,7 +8590,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>600</v>
       </c>
@@ -8498,7 +8598,7 @@
         <v>601</v>
       </c>
     </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>602</v>
       </c>
@@ -8506,7 +8606,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>604</v>
       </c>
@@ -8514,7 +8614,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>606</v>
       </c>
@@ -8522,7 +8622,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>608</v>
       </c>
@@ -8530,7 +8630,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>610</v>
       </c>
@@ -8562,13 +8662,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C49"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="29.5546875" customWidth="1"/>
-    <col min="3" max="3" width="5.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="29.54296875" customWidth="1"/>
+    <col min="3" max="3" width="5.453125" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
         <v>403</v>
       </c>
@@ -8579,7 +8679,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>612</v>
       </c>
@@ -8587,7 +8687,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>614</v>
       </c>
@@ -8595,7 +8695,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>615</v>
       </c>
@@ -8603,7 +8703,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>617</v>
       </c>
@@ -8611,7 +8711,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>619</v>
       </c>
@@ -8619,7 +8719,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>621</v>
       </c>
@@ -8627,7 +8727,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>623</v>
       </c>
@@ -8635,7 +8735,7 @@
         <v>624</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>625</v>
       </c>
@@ -8643,7 +8743,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>627</v>
       </c>
@@ -8651,7 +8751,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>629</v>
       </c>
@@ -8659,7 +8759,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>631</v>
       </c>
@@ -8667,7 +8767,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>633</v>
       </c>
@@ -8675,7 +8775,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>635</v>
       </c>
@@ -8683,7 +8783,7 @@
         <v>636</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>637</v>
       </c>
@@ -8691,7 +8791,7 @@
         <v>638</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>639</v>
       </c>
@@ -8699,7 +8799,7 @@
         <v>640</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>641</v>
       </c>
@@ -8707,7 +8807,7 @@
         <v>642</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>643</v>
       </c>
@@ -8718,7 +8818,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>645</v>
       </c>
@@ -8726,7 +8826,7 @@
         <v>646</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>647</v>
       </c>
@@ -8734,7 +8834,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>649</v>
       </c>
@@ -8742,7 +8842,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>651</v>
       </c>
@@ -8750,7 +8850,7 @@
         <v>652</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>653</v>
       </c>
@@ -8758,7 +8858,7 @@
         <v>654</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>655</v>
       </c>
@@ -8766,7 +8866,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>657</v>
       </c>
@@ -8774,7 +8874,7 @@
         <v>658</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>659</v>
       </c>
@@ -8782,7 +8882,7 @@
         <v>660</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>661</v>
       </c>
@@ -8790,7 +8890,7 @@
         <v>662</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>663</v>
       </c>
@@ -8798,7 +8898,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>665</v>
       </c>
@@ -8806,7 +8906,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>667</v>
       </c>
@@ -8814,7 +8914,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>669</v>
       </c>
@@ -8822,7 +8922,7 @@
         <v>670</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>671</v>
       </c>
@@ -8830,7 +8930,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>673</v>
       </c>
@@ -8838,7 +8938,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>675</v>
       </c>
@@ -8846,7 +8946,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>677</v>
       </c>
@@ -8854,7 +8954,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>679</v>
       </c>
@@ -8862,7 +8962,7 @@
         <v>680</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>681</v>
       </c>
@@ -8870,7 +8970,7 @@
         <v>682</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>683</v>
       </c>
@@ -8878,7 +8978,7 @@
         <v>684</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>685</v>
       </c>
@@ -8886,7 +8986,7 @@
         <v>686</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>687</v>
       </c>
@@ -8894,7 +8994,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>689</v>
       </c>
@@ -8902,7 +9002,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>691</v>
       </c>
@@ -8910,7 +9010,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>693</v>
       </c>
@@ -8918,7 +9018,7 @@
         <v>694</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>695</v>
       </c>
@@ -8926,7 +9026,7 @@
         <v>696</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>697</v>
       </c>
@@ -8934,7 +9034,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>698</v>
       </c>
@@ -8942,7 +9042,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>700</v>
       </c>
@@ -8950,7 +9050,7 @@
         <v>701</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>702</v>
       </c>
@@ -8958,7 +9058,7 @@
         <v>703</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>704</v>
       </c>
@@ -8985,14 +9085,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:C48"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="8.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>403</v>
       </c>
@@ -9003,7 +9103,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>706</v>
       </c>
@@ -9011,7 +9111,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>708</v>
       </c>
@@ -9019,7 +9119,7 @@
         <v>709</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>710</v>
       </c>
@@ -9027,7 +9127,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>712</v>
       </c>
@@ -9035,7 +9135,7 @@
         <v>713</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>714</v>
       </c>
@@ -9043,7 +9143,7 @@
         <v>715</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>716</v>
       </c>
@@ -9051,7 +9151,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>717</v>
       </c>
@@ -9059,7 +9159,7 @@
         <v>718</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>719</v>
       </c>
@@ -9067,7 +9167,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>721</v>
       </c>
@@ -9075,7 +9175,7 @@
         <v>722</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>723</v>
       </c>
@@ -9083,7 +9183,7 @@
         <v>724</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>725</v>
       </c>
@@ -9091,7 +9191,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>726</v>
       </c>
@@ -9099,7 +9199,7 @@
         <v>727</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>728</v>
       </c>
@@ -9107,7 +9207,7 @@
         <v>729</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>730</v>
       </c>
@@ -9115,7 +9215,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>731</v>
       </c>
@@ -9123,7 +9223,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>732</v>
       </c>
@@ -9131,7 +9231,7 @@
         <v>733</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>734</v>
       </c>
@@ -9139,7 +9239,7 @@
         <v>735</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>736</v>
       </c>
@@ -9147,7 +9247,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>737</v>
       </c>
@@ -9155,7 +9255,7 @@
         <v>738</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>739</v>
       </c>
@@ -9163,7 +9263,7 @@
         <v>740</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>741</v>
       </c>
@@ -9171,7 +9271,7 @@
         <v>742</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>743</v>
       </c>
@@ -9179,7 +9279,7 @@
         <v>744</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>745</v>
       </c>
@@ -9187,7 +9287,7 @@
         <v>746</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>747</v>
       </c>
@@ -9195,7 +9295,7 @@
         <v>485</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>748</v>
       </c>
@@ -9203,7 +9303,7 @@
         <v>749</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>750</v>
       </c>
@@ -9211,7 +9311,7 @@
         <v>751</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>752</v>
       </c>
@@ -9219,7 +9319,7 @@
         <v>753</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>754</v>
       </c>
@@ -9227,7 +9327,7 @@
         <v>755</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>756</v>
       </c>
@@ -9235,7 +9335,7 @@
         <v>757</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>758</v>
       </c>
@@ -9243,7 +9343,7 @@
         <v>759</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>760</v>
       </c>
@@ -9251,7 +9351,7 @@
         <v>761</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>762</v>
       </c>
@@ -9259,7 +9359,7 @@
         <v>763</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>764</v>
       </c>
@@ -9267,7 +9367,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>766</v>
       </c>
@@ -9275,7 +9375,7 @@
         <v>767</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>768</v>
       </c>
@@ -9283,7 +9383,7 @@
         <v>769</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>770</v>
       </c>
@@ -9291,7 +9391,7 @@
         <v>771</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>772</v>
       </c>
@@ -9299,7 +9399,7 @@
         <v>773</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>774</v>
       </c>
@@ -9307,7 +9407,7 @@
         <v>775</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>776</v>
       </c>
@@ -9315,7 +9415,7 @@
         <v>777</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>778</v>
       </c>
@@ -9323,7 +9423,7 @@
         <v>779</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>780</v>
       </c>
@@ -9331,7 +9431,7 @@
         <v>781</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>782</v>
       </c>
@@ -9339,7 +9439,7 @@
         <v>783</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>784</v>
       </c>
@@ -9347,7 +9447,7 @@
         <v>785</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>786</v>
       </c>
@@ -9355,7 +9455,7 @@
         <v>787</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>788</v>
       </c>
@@ -9363,7 +9463,7 @@
         <v>789</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>790</v>
       </c>
@@ -9371,7 +9471,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>792</v>
       </c>
@@ -9398,14 +9498,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:C67"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="8.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>403</v>
       </c>
@@ -9416,7 +9516,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>794</v>
       </c>
@@ -9424,7 +9524,7 @@
         <v>795</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>796</v>
       </c>
@@ -9432,7 +9532,7 @@
         <v>797</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>798</v>
       </c>
@@ -9440,7 +9540,7 @@
         <v>799</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>800</v>
       </c>
@@ -9448,7 +9548,7 @@
         <v>801</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>802</v>
       </c>
@@ -9456,7 +9556,7 @@
         <v>803</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>804</v>
       </c>
@@ -9464,7 +9564,7 @@
         <v>805</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>806</v>
       </c>
@@ -9472,7 +9572,7 @@
         <v>807</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>808</v>
       </c>
@@ -9480,7 +9580,7 @@
         <v>809</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>810</v>
       </c>
@@ -9488,7 +9588,7 @@
         <v>811</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>812</v>
       </c>
@@ -9496,7 +9596,7 @@
         <v>813</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>814</v>
       </c>
@@ -9504,7 +9604,7 @@
         <v>815</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>816</v>
       </c>
@@ -9512,7 +9612,7 @@
         <v>817</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>818</v>
       </c>
@@ -9520,7 +9620,7 @@
         <v>819</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>820</v>
       </c>
@@ -9528,7 +9628,7 @@
         <v>821</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>822</v>
       </c>
@@ -9536,7 +9636,7 @@
         <v>823</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>824</v>
       </c>
@@ -9544,7 +9644,7 @@
         <v>825</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>826</v>
       </c>
@@ -9552,7 +9652,7 @@
         <v>827</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>828</v>
       </c>
@@ -9560,7 +9660,7 @@
         <v>829</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>830</v>
       </c>
@@ -9568,7 +9668,7 @@
         <v>831</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>832</v>
       </c>
@@ -9576,7 +9676,7 @@
         <v>833</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>834</v>
       </c>
@@ -9584,7 +9684,7 @@
         <v>835</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>836</v>
       </c>
@@ -9592,7 +9692,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>838</v>
       </c>
@@ -9600,7 +9700,7 @@
         <v>839</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>840</v>
       </c>
@@ -9608,7 +9708,7 @@
         <v>841</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>842</v>
       </c>
@@ -9616,7 +9716,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>844</v>
       </c>
@@ -9624,7 +9724,7 @@
         <v>845</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>846</v>
       </c>
@@ -9632,7 +9732,7 @@
         <v>847</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>848</v>
       </c>
@@ -9640,7 +9740,7 @@
         <v>849</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>850</v>
       </c>
@@ -9648,7 +9748,7 @@
         <v>851</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>852</v>
       </c>
@@ -9656,7 +9756,7 @@
         <v>853</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>854</v>
       </c>
@@ -9664,7 +9764,7 @@
         <v>855</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>856</v>
       </c>
@@ -9672,7 +9772,7 @@
         <v>857</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>858</v>
       </c>
@@ -9680,7 +9780,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>859</v>
       </c>
@@ -9688,7 +9788,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>860</v>
       </c>
@@ -9696,7 +9796,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>861</v>
       </c>
@@ -9704,7 +9804,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>862</v>
       </c>
@@ -9712,7 +9812,7 @@
         <v>863</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>864</v>
       </c>
@@ -9720,7 +9820,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>865</v>
       </c>
@@ -9728,7 +9828,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>866</v>
       </c>
@@ -9736,7 +9836,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>867</v>
       </c>
@@ -9744,7 +9844,7 @@
         <v>680</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>868</v>
       </c>
@@ -9752,7 +9852,7 @@
         <v>761</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>869</v>
       </c>
@@ -9760,7 +9860,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>870</v>
       </c>
@@ -9768,7 +9868,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>871</v>
       </c>
@@ -9776,7 +9876,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>872</v>
       </c>
@@ -9784,7 +9884,7 @@
         <v>515</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>873</v>
       </c>
@@ -9792,7 +9892,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>874</v>
       </c>
@@ -9800,7 +9900,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>875</v>
       </c>
@@ -9808,7 +9908,7 @@
         <v>694</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>876</v>
       </c>
@@ -9816,7 +9916,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>877</v>
       </c>
@@ -9824,7 +9924,7 @@
         <v>775</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>878</v>
       </c>
@@ -9832,7 +9932,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>879</v>
       </c>
@@ -9840,7 +9940,7 @@
         <v>779</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>880</v>
       </c>
@@ -9848,7 +9948,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>881</v>
       </c>
@@ -9856,7 +9956,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>882</v>
       </c>
@@ -9864,7 +9964,7 @@
         <v>783</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>883</v>
       </c>
@@ -9872,7 +9972,7 @@
         <v>884</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>885</v>
       </c>
@@ -9880,7 +9980,7 @@
         <v>886</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>887</v>
       </c>
@@ -9888,7 +9988,7 @@
         <v>888</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>889</v>
       </c>
@@ -9896,7 +9996,7 @@
         <v>890</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>891</v>
       </c>
@@ -9904,7 +10004,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>893</v>
       </c>
@@ -9912,7 +10012,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>895</v>
       </c>
@@ -9920,7 +10020,7 @@
         <v>896</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>897</v>
       </c>
@@ -9928,7 +10028,7 @@
         <v>898</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>899</v>
       </c>
@@ -9936,7 +10036,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>901</v>
       </c>
@@ -9963,47 +10063,47 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:A8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="2" t="s">
         <v>903</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>904</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>905</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>350</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>906</v>
       </c>

</xml_diff>

<commit_message>
UI: redesigned shop UI wallet and cost visuals
</commit_message>
<xml_diff>
--- a/Spreadsheets/Issue_Log.xlsx
+++ b/Spreadsheets/Issue_Log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\Spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B1EEAE3-459F-40BF-860E-84235AD6FD1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB1B0CD0-7411-4F22-BFF7-03CA9EB29DBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-132" yWindow="-132" windowWidth="30984" windowHeight="18744" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Game_Issues" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1677" uniqueCount="912">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1713" uniqueCount="924">
   <si>
     <t>#</t>
   </si>
@@ -2916,6 +2916,42 @@
   </si>
   <si>
     <t>Exploud (Ex emerald card 3) has Mega throw. This is a 5 energy attack but the game only seems to count it as 4. It also only displays as 4 so it's as if the game completely ignores anything after the 4th energy and never is aware of a 5th for any attack?</t>
+  </si>
+  <si>
+    <t>The in match full message log (pressing caps lock) should show the little opponent overworld sprite in the top left next to the name, the same way it does for main messages outside of the battle</t>
+  </si>
+  <si>
+    <t>Opponent should know not to discard a double colorless energy if other energies are attached. E.g to retreat or to use an attack. This goes for reverse, if the opponent uses an energy removal or attack like hyper beam, double colorless tends to be twice as valuable as a normal basic energy. This goes for any other special energies with bonus effects such as rainbow, multi, darkness, metal energy etc. Basic energies are less valuable normally (UNLESS LOSING THAT ENERGY PREVENTS AN ATTACK FROM BEING USED BUT THE OTHER ENERGY DOES NOT. If both energies prevent an attack being used, the special/double is still more valuable)</t>
+  </si>
+  <si>
+    <t>Opponent played potion to heal a benched pokemon that 30/70hp. While this had less fractional health percentage, the active pokemon had 30/60 and the player had an attack that did 30 damage meaning a guarenteed knockout next turn. Opponent should have healed the active pokemon not the bench</t>
+  </si>
+  <si>
+    <t>Typo</t>
+  </si>
+  <si>
+    <t>Birdspotter tamsin grants dodou coin not doduo</t>
+  </si>
+  <si>
+    <t>For selected costumes, in both shop and selection in owned, increase the growing shrinking size by 20% to make it more obvious</t>
+  </si>
+  <si>
+    <t>All new shopkeepers have just the normal […] dialogue box above their head instead of [  $  ] icon the original pack shopkeepers use</t>
+  </si>
+  <si>
+    <t>Data</t>
+  </si>
+  <si>
+    <t>Values</t>
+  </si>
+  <si>
+    <t>The coins in the shop are too expensive really, they should be less than $500. Price of the coins should be $100</t>
+  </si>
+  <si>
+    <t>Replace the coins in the shop with more "boring" choices. It's too early in game to offer the good coins. This will work in tandem with the lowered price</t>
+  </si>
+  <si>
+    <t>Change the colour in this issue log spreadsheet for new issues. Instead of Blue, set it to an orange to be closer to the red. Blue is closer to green indiciating manual issue resolved. Setting to orange makes it appear more like an issue I will spot</t>
   </si>
 </sst>
 </file>
@@ -3506,7 +3542,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J162"/>
+  <dimension ref="A1:J171"/>
   <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5" style="5" bestFit="1" customWidth="1"/>
@@ -7740,6 +7776,159 @@
         <v>911</v>
       </c>
       <c r="G162" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="163" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A163" s="5">
+        <v>161</v>
+      </c>
+      <c r="B163" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C163" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D163" s="6" t="s">
+        <v>912</v>
+      </c>
+      <c r="G163" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="164" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A164" s="5">
+        <v>162</v>
+      </c>
+      <c r="B164" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C164" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D164" s="6" t="s">
+        <v>917</v>
+      </c>
+      <c r="G164" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="165" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A165" s="5">
+        <v>163</v>
+      </c>
+      <c r="B165" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="C165" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="D165" s="6" t="s">
+        <v>913</v>
+      </c>
+      <c r="G165" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="166" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A166" s="5">
+        <v>164</v>
+      </c>
+      <c r="B166" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C166" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D166" s="6" t="s">
+        <v>914</v>
+      </c>
+      <c r="G166" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="167" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A167" s="5">
+        <v>165</v>
+      </c>
+      <c r="B167" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C167" s="5" t="s">
+        <v>915</v>
+      </c>
+      <c r="D167" s="6" t="s">
+        <v>916</v>
+      </c>
+      <c r="G167" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="168" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A168" s="5">
+        <v>166</v>
+      </c>
+      <c r="B168" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C168" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D168" s="6" t="s">
+        <v>918</v>
+      </c>
+      <c r="G168" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="169" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A169" s="5">
+        <v>167</v>
+      </c>
+      <c r="B169" s="5" t="s">
+        <v>919</v>
+      </c>
+      <c r="C169" s="5" t="s">
+        <v>920</v>
+      </c>
+      <c r="D169" s="6" t="s">
+        <v>921</v>
+      </c>
+      <c r="G169" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="170" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A170" s="5">
+        <v>168</v>
+      </c>
+      <c r="B170" s="5" t="s">
+        <v>919</v>
+      </c>
+      <c r="C170" s="5" t="s">
+        <v>920</v>
+      </c>
+      <c r="D170" s="6" t="s">
+        <v>922</v>
+      </c>
+      <c r="G170" s="6" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="171" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A171" s="5">
+        <v>169</v>
+      </c>
+      <c r="B171" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C171" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D171" s="6" t="s">
+        <v>923</v>
+      </c>
+      <c r="G171" s="6" t="s">
         <v>904</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Collision: Added collision data for Gym Plaza
</commit_message>
<xml_diff>
--- a/Spreadsheets/Issue_Log.xlsx
+++ b/Spreadsheets/Issue_Log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\Spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB1B0CD0-7411-4F22-BFF7-03CA9EB29DBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33BA1B36-5FDB-4A33-AA2F-A3D7CE9D9B76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-132" yWindow="-132" windowWidth="30984" windowHeight="18744" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Game_Issues" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1713" uniqueCount="924">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1741" uniqueCount="931">
   <si>
     <t>#</t>
   </si>
@@ -2952,6 +2952,27 @@
   </si>
   <si>
     <t>Change the colour in this issue log spreadsheet for new issues. Instead of Blue, set it to an orange to be closer to the red. Blue is closer to green indiciating manual issue resolved. Setting to orange makes it appear more like an issue I will spot</t>
+  </si>
+  <si>
+    <t>When the opponent uses Bill, we had a previous issue that the hand changes location and goes to around the center of the screen. I thought this issue was resolved but it's still happening so when opponent plays bill, the hand shifts location, then the cards get added and the hand moves back to the correct location</t>
+  </si>
+  <si>
+    <t>For any attack that doesn't apply weakness and resistance (such as meowth coin hurl), remove the (no W/R) text from the message</t>
+  </si>
+  <si>
+    <t>When player had tools attached in this order: Defender, PlusPower, Defender: at the end of the turn when plus power was discarded, the screen refreshed only showing 1 defender card. Then the next turn when defender was discarded it showed 2 being discarded. THis could be linked to the issue number 159</t>
+  </si>
+  <si>
+    <t>When rainbow energy was attached to a benched pokemon, the damage for the floating label appeared on the active pokemon and the active pokemon's HP updated to be the benched pokemon. The benched pokemon HP still showed 50/50 but now the active pokemon went from 10/40 to 40/50 showing the benched pokemon's instead incorrectly</t>
+  </si>
+  <si>
+    <t>When a card effect prevents a card being used from the hand such as hay fever preventing trainers being played, the play button works which is fine, and the message appears saying hay fever: no trainer cards can be played. But the card stays selected after the message is cleared and the play button goes back to "select a card" even though the trainer LOOKs selected.</t>
+  </si>
+  <si>
+    <t>For hay fever preventing trainers, change the message to "Dark Vileplume's Hay fever prevents trainer cards being played"</t>
+  </si>
+  <si>
+    <t>Opponent attached a full heal energy to a benched dark primeape. This provides colorless energy to heal statuses. Bench pokemon can't have statuses and dark primeape has no use for colorless energy. Full heal energy should only be played when it provides no energy benefit when it DOES heal a status condition. This is the same for Potion energy, it should only be used if the colorless energy provided actually helps AND OR the 10hp recovery is needed. Otherwise, any other energy should be prioritised instead.</t>
   </si>
 </sst>
 </file>
@@ -3542,23 +3563,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J171"/>
-  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:J178"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.453125" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.453125" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="125.36328125" style="6" customWidth="1"/>
-    <col min="5" max="5" width="255.54296875" style="6" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="14.42578125" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.42578125" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="125.42578125" style="6" customWidth="1"/>
+    <col min="5" max="5" width="255.5703125" style="6" hidden="1" customWidth="1"/>
     <col min="6" max="6" width="102" style="6" customWidth="1"/>
     <col min="7" max="7" width="19" style="6" customWidth="1"/>
-    <col min="8" max="9" width="11.08984375" style="7" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="11.140625" style="7" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="16" style="7" customWidth="1"/>
-    <col min="11" max="17" width="9.08984375" style="7" customWidth="1"/>
-    <col min="18" max="16384" width="9.08984375" style="7"/>
+    <col min="11" max="17" width="9.140625" style="7" customWidth="1"/>
+    <col min="18" max="16384" width="9.140625" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -3590,7 +3611,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="5">
         <v>1</v>
       </c>
@@ -3616,7 +3637,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="86.4" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" ht="86.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5">
         <v>2</v>
       </c>
@@ -3648,7 +3669,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="115.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" ht="115.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
         <v>3</v>
       </c>
@@ -3677,7 +3698,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
         <v>4</v>
       </c>
@@ -3706,7 +3727,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
         <v>5</v>
       </c>
@@ -3735,7 +3756,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="172.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" ht="172.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
         <v>6</v>
       </c>
@@ -3764,7 +3785,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="201.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" ht="201.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
         <v>7</v>
       </c>
@@ -3793,7 +3814,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" ht="43.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
         <v>8</v>
       </c>
@@ -3822,7 +3843,7 @@
         <v>46220</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="100.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" ht="100.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
         <v>9</v>
       </c>
@@ -3851,7 +3872,7 @@
         <v>46220</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" ht="43.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5">
         <v>10</v>
       </c>
@@ -3880,7 +3901,7 @@
         <v>46220</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="100.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" ht="100.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
         <v>11</v>
       </c>
@@ -3906,7 +3927,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="302.39999999999998" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" ht="302.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5">
         <v>12</v>
       </c>
@@ -3935,7 +3956,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" ht="43.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
         <v>13</v>
       </c>
@@ -3961,7 +3982,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5">
         <v>14</v>
       </c>
@@ -3984,7 +4005,7 @@
         <v>46223</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" ht="43.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5">
         <v>15</v>
       </c>
@@ -4010,7 +4031,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" ht="43.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="5">
         <v>16</v>
       </c>
@@ -4039,7 +4060,7 @@
         <v>46220</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5">
         <v>17</v>
       </c>
@@ -4068,7 +4089,7 @@
         <v>46220</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" ht="43.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5">
         <v>18</v>
       </c>
@@ -4094,7 +4115,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="5">
         <v>19</v>
       </c>
@@ -4120,7 +4141,7 @@
         <v>46224</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="86.4" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" ht="86.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="5">
         <v>20</v>
       </c>
@@ -4146,7 +4167,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5">
         <v>21</v>
       </c>
@@ -4172,7 +4193,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" ht="43.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="5">
         <v>22</v>
       </c>
@@ -4198,7 +4219,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5">
         <v>23</v>
       </c>
@@ -4221,7 +4242,7 @@
         <v>46221</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10" ht="43.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="5">
         <v>23</v>
       </c>
@@ -4247,7 +4268,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="115.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" ht="115.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="5">
         <v>24</v>
       </c>
@@ -4276,7 +4297,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="5">
         <v>25</v>
       </c>
@@ -4302,7 +4323,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="5">
         <v>26</v>
       </c>
@@ -4331,7 +4352,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5">
         <v>27</v>
       </c>
@@ -4357,7 +4378,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="5">
         <v>28</v>
       </c>
@@ -4383,7 +4404,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="5">
         <v>29</v>
       </c>
@@ -4409,7 +4430,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="5">
         <v>30</v>
       </c>
@@ -4435,7 +4456,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ht="57.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="5">
         <v>31</v>
       </c>
@@ -4461,7 +4482,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="345.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:10" ht="345.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="5">
         <v>32</v>
       </c>
@@ -4490,7 +4511,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="35" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="5">
         <v>33</v>
       </c>
@@ -4519,7 +4540,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="36" spans="1:10" ht="144" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:10" ht="144" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="5">
         <v>34</v>
       </c>
@@ -4548,7 +4569,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="37" spans="1:10" ht="172.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:10" ht="172.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="5">
         <v>35</v>
       </c>
@@ -4577,7 +4598,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="38" spans="1:10" ht="57.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:10" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="5">
         <v>36</v>
       </c>
@@ -4603,7 +4624,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="39" spans="1:10" ht="57.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:10" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="5">
         <v>37</v>
       </c>
@@ -4632,7 +4653,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="40" spans="1:10" ht="129.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:10" ht="129.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="5">
         <v>38</v>
       </c>
@@ -4661,7 +4682,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="41" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:10" ht="43.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="5">
         <v>39</v>
       </c>
@@ -4687,7 +4708,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="42" spans="1:10" ht="57.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:10" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="5">
         <v>40</v>
       </c>
@@ -4716,7 +4737,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="43" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:10" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="5">
         <v>41</v>
       </c>
@@ -4742,7 +4763,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="44" spans="1:10" ht="100.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:10" ht="100.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="5">
         <v>42</v>
       </c>
@@ -4768,7 +4789,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="45" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="5">
         <v>43</v>
       </c>
@@ -4794,7 +4815,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="46" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="5">
         <v>44</v>
       </c>
@@ -4826,7 +4847,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="47" spans="1:10" ht="86.4" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:10" ht="86.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="5">
         <v>45</v>
       </c>
@@ -4852,7 +4873,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="48" spans="1:10" ht="115.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:10" ht="115.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="5">
         <v>46</v>
       </c>
@@ -4878,7 +4899,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="49" spans="1:10" ht="57.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:10" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="5">
         <v>47</v>
       </c>
@@ -4904,7 +4925,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="50" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:10" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="5">
         <v>48</v>
       </c>
@@ -4930,7 +4951,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="51" spans="1:10" ht="86.4" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:10" ht="86.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="5">
         <v>49</v>
       </c>
@@ -4956,7 +4977,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="52" spans="1:10" ht="57.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:10" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="5">
         <v>50</v>
       </c>
@@ -4982,7 +5003,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="53" spans="1:10" ht="57.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:10" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="5">
         <v>51</v>
       </c>
@@ -5008,7 +5029,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="54" spans="1:10" ht="100.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:10" ht="100.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="5">
         <v>52</v>
       </c>
@@ -5037,7 +5058,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="55" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:10" ht="43.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="5">
         <v>53</v>
       </c>
@@ -5063,7 +5084,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="56" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:10" ht="43.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="5">
         <v>54</v>
       </c>
@@ -5089,7 +5110,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="57" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:10" ht="43.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="5">
         <v>55</v>
       </c>
@@ -5115,7 +5136,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="58" spans="1:10" ht="86.4" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:10" ht="86.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="5">
         <v>56</v>
       </c>
@@ -5141,7 +5162,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="59" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:10" ht="43.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="5">
         <v>57</v>
       </c>
@@ -5167,7 +5188,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="60" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:10" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="5">
         <v>58</v>
       </c>
@@ -5193,7 +5214,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="61" spans="1:10" ht="172.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:10" ht="172.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="5">
         <v>59</v>
       </c>
@@ -5222,7 +5243,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="62" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:10" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="5">
         <v>60</v>
       </c>
@@ -5248,7 +5269,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="63" spans="1:10" ht="129.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:10" ht="129.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="5">
         <v>61</v>
       </c>
@@ -5274,7 +5295,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64" s="5">
         <v>62</v>
       </c>
@@ -5297,7 +5318,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="65" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:10" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="5">
         <v>63</v>
       </c>
@@ -5323,7 +5344,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66" s="5">
         <v>64</v>
       </c>
@@ -5346,7 +5367,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="67" spans="1:10" ht="129.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:10" ht="129.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="5">
         <v>65</v>
       </c>
@@ -5372,7 +5393,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68" s="5">
         <v>66</v>
       </c>
@@ -5392,7 +5413,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A69" s="5">
         <v>67</v>
       </c>
@@ -5412,7 +5433,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70" s="5">
         <v>68</v>
       </c>
@@ -5432,7 +5453,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="71" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:10" ht="43.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="5">
         <v>69</v>
       </c>
@@ -5458,7 +5479,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A72" s="5">
         <v>70</v>
       </c>
@@ -5484,7 +5505,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A73" s="5">
         <v>71</v>
       </c>
@@ -5510,7 +5531,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A74" s="5">
         <v>72</v>
       </c>
@@ -5527,7 +5548,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="75" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:10" ht="43.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="5">
         <v>73</v>
       </c>
@@ -5553,7 +5574,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="76" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:10" ht="43.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="5">
         <v>77</v>
       </c>
@@ -5579,7 +5600,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="77" spans="1:10" ht="187.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:10" ht="187.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="5">
         <v>74</v>
       </c>
@@ -5608,7 +5629,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="78" spans="1:10" ht="86.4" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:10" ht="86.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="5">
         <v>75</v>
       </c>
@@ -5637,7 +5658,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="79" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:10" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="5">
         <v>76</v>
       </c>
@@ -5660,7 +5681,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="80" spans="1:10" ht="100.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:10" ht="100.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="5">
         <v>77</v>
       </c>
@@ -5686,7 +5707,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="81" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:10" ht="43.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="5">
         <v>78</v>
       </c>
@@ -5712,7 +5733,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="82" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:10" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="5">
         <v>79</v>
       </c>
@@ -5738,7 +5759,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="83" spans="1:10" ht="57.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:10" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="5">
         <v>81</v>
       </c>
@@ -5764,7 +5785,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="84" spans="1:10" ht="100.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:10" ht="100.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="5">
         <v>80</v>
       </c>
@@ -5790,7 +5811,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="85" spans="1:10" ht="86.4" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:10" ht="86.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="5">
         <v>81</v>
       </c>
@@ -5816,7 +5837,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="86" spans="1:10" ht="100.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:10" ht="100.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="5">
         <v>82</v>
       </c>
@@ -5842,7 +5863,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="87" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:10" ht="43.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="5">
         <v>83</v>
       </c>
@@ -5868,7 +5889,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="88" spans="1:10" ht="100.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:10" ht="100.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="5">
         <v>84</v>
       </c>
@@ -5894,7 +5915,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A89" s="5">
         <v>85</v>
       </c>
@@ -5920,7 +5941,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="90" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:10" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="5">
         <v>86</v>
       </c>
@@ -5946,7 +5967,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="91" spans="1:10" ht="57.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:10" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="5">
         <v>87</v>
       </c>
@@ -5972,7 +5993,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="92" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="5">
         <v>88</v>
       </c>
@@ -5998,7 +6019,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="93" spans="1:10" ht="86.4" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:10" ht="86.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="5">
         <v>89</v>
       </c>
@@ -6024,7 +6045,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="94" spans="1:10" ht="86.4" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:10" ht="86.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="5">
         <v>90</v>
       </c>
@@ -6050,7 +6071,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="95" spans="1:10" ht="57.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:10" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="5">
         <v>91</v>
       </c>
@@ -6076,7 +6097,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="96" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:10" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="5">
         <v>92</v>
       </c>
@@ -6096,7 +6117,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="97" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:10" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="5">
         <v>92</v>
       </c>
@@ -6116,7 +6137,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A98" s="5">
         <v>93</v>
       </c>
@@ -6145,7 +6166,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="99" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:10" ht="43.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="5">
         <v>94</v>
       </c>
@@ -6165,7 +6186,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="100" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="5">
         <v>95</v>
       </c>
@@ -6191,7 +6212,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="101" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:10" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="5">
         <v>96</v>
       </c>
@@ -6217,7 +6238,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A102" s="5">
         <v>97</v>
       </c>
@@ -6246,7 +6267,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="103" spans="1:10" ht="86.4" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:10" ht="86.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="5">
         <v>98</v>
       </c>
@@ -6272,7 +6293,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A104" s="5">
         <v>99</v>
       </c>
@@ -6298,7 +6319,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="105" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:10" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="5">
         <v>100</v>
       </c>
@@ -6324,7 +6345,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A106" s="5">
         <v>101</v>
       </c>
@@ -6350,7 +6371,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="107" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="5">
         <v>102</v>
       </c>
@@ -6376,7 +6397,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="108" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:10" ht="43.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="5">
         <v>103</v>
       </c>
@@ -6402,7 +6423,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="109" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:10" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="5">
         <v>104</v>
       </c>
@@ -6428,7 +6449,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="110" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:10" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="5">
         <v>105</v>
       </c>
@@ -6454,7 +6475,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A111" s="5">
         <v>106</v>
       </c>
@@ -6480,7 +6501,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="112" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:10" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="5">
         <v>109</v>
       </c>
@@ -6506,7 +6527,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="113" spans="1:9" ht="57.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:9" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="5">
         <v>110</v>
       </c>
@@ -6532,7 +6553,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="114" spans="1:9" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:9" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A114" s="5">
         <v>111</v>
       </c>
@@ -6558,7 +6579,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="115" spans="1:9" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:9" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115" s="5">
         <v>112</v>
       </c>
@@ -6584,7 +6605,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="116" spans="1:9" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:9" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="5">
         <v>113</v>
       </c>
@@ -6610,7 +6631,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="117" spans="1:9" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:9" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="5">
         <v>114</v>
       </c>
@@ -6636,7 +6657,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="118" spans="1:9" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:9" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A118" s="5">
         <v>115</v>
       </c>
@@ -6662,7 +6683,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="119" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A119" s="5">
         <v>116</v>
       </c>
@@ -6688,7 +6709,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="120" spans="1:9" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:9" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="5">
         <v>117</v>
       </c>
@@ -6714,7 +6735,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="121" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A121" s="5">
         <v>118</v>
       </c>
@@ -6740,7 +6761,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="122" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A122" s="5">
         <v>119</v>
       </c>
@@ -6766,7 +6787,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="123" spans="1:9" ht="57.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:9" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A123" s="5">
         <v>120</v>
       </c>
@@ -6792,7 +6813,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="124" spans="1:9" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:9" ht="43.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A124" s="5">
         <v>121</v>
       </c>
@@ -6821,7 +6842,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="125" spans="1:9" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:9" ht="43.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125" s="5">
         <v>122</v>
       </c>
@@ -6847,7 +6868,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="126" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A126" s="5">
         <v>123</v>
       </c>
@@ -6873,7 +6894,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="127" spans="1:9" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:9" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A127" s="5">
         <v>124</v>
       </c>
@@ -6899,7 +6920,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="128" spans="1:9" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:9" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A128" s="5">
         <v>125</v>
       </c>
@@ -6925,7 +6946,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="129" spans="1:9" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:9" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129" s="5">
         <v>126</v>
       </c>
@@ -6951,7 +6972,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="130" spans="1:9" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:9" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" s="5">
         <v>127</v>
       </c>
@@ -6977,7 +6998,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="131" spans="1:9" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:9" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="5">
         <v>128</v>
       </c>
@@ -7003,7 +7024,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="132" spans="1:9" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:9" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132" s="5">
         <v>129</v>
       </c>
@@ -7029,7 +7050,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="133" spans="1:9" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:9" ht="43.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A133" s="5">
         <v>130</v>
       </c>
@@ -7055,7 +7076,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="134" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A134" s="5">
         <v>131</v>
       </c>
@@ -7081,7 +7102,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="135" spans="1:9" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:9" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A135" s="5">
         <v>132</v>
       </c>
@@ -7107,7 +7128,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="136" spans="1:9" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:9" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A136" s="5">
         <v>133</v>
       </c>
@@ -7136,7 +7157,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="137" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A137" s="5">
         <v>134</v>
       </c>
@@ -7162,7 +7183,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="138" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A138" s="5">
         <v>135</v>
       </c>
@@ -7188,7 +7209,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="139" spans="1:9" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:9" ht="43.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A139" s="5">
         <v>136</v>
       </c>
@@ -7214,7 +7235,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="140" spans="1:9" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:9" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A140" s="5">
         <v>137</v>
       </c>
@@ -7240,7 +7261,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="141" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A141" s="5">
         <v>138</v>
       </c>
@@ -7266,7 +7287,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="142" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A142" s="5">
         <v>139</v>
       </c>
@@ -7292,7 +7313,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="143" spans="1:9" ht="57.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:9" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A143" s="5">
         <v>140</v>
       </c>
@@ -7318,7 +7339,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="144" spans="1:9" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:9" ht="43.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A144" s="5">
         <v>141</v>
       </c>
@@ -7347,7 +7368,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="145" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:10" ht="43.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A145" s="5">
         <v>142</v>
       </c>
@@ -7373,7 +7394,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="146" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:10" ht="43.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A146" s="5">
         <v>143</v>
       </c>
@@ -7399,7 +7420,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="147" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:10" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A147" s="5">
         <v>144</v>
       </c>
@@ -7425,7 +7446,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="148" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:10" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A148" s="5">
         <v>145</v>
       </c>
@@ -7454,7 +7475,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="149" spans="1:10" ht="57.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:10" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A149" s="5">
         <v>146</v>
       </c>
@@ -7483,7 +7504,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="150" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:10" ht="43.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A150" s="5">
         <v>147</v>
       </c>
@@ -7509,7 +7530,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="151" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:10" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A151" s="5">
         <v>148</v>
       </c>
@@ -7535,7 +7556,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="152" spans="1:10" ht="100.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:10" ht="100.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A152" s="5">
         <v>149</v>
       </c>
@@ -7564,7 +7585,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="153" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153" s="5">
         <v>150</v>
       </c>
@@ -7590,7 +7611,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="154" spans="1:10" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:10" ht="43.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A154" s="5">
         <v>151</v>
       </c>
@@ -7616,7 +7637,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="155" spans="1:10" ht="129.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:10" ht="129.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A155" s="5">
         <v>152</v>
       </c>
@@ -7642,7 +7663,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="156" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A156" s="5">
         <v>154</v>
       </c>
@@ -7668,7 +7689,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="157" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A157" s="5">
         <v>155</v>
       </c>
@@ -7694,7 +7715,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="158" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A158" s="5">
         <v>156</v>
       </c>
@@ -7711,7 +7732,7 @@
         <v>904</v>
       </c>
     </row>
-    <row r="159" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A159" s="5">
         <v>157</v>
       </c>
@@ -7728,7 +7749,7 @@
         <v>904</v>
       </c>
     </row>
-    <row r="160" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A160" s="5">
         <v>158</v>
       </c>
@@ -7745,7 +7766,7 @@
         <v>904</v>
       </c>
     </row>
-    <row r="161" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A161" s="5">
         <v>159</v>
       </c>
@@ -7762,7 +7783,7 @@
         <v>904</v>
       </c>
     </row>
-    <row r="162" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A162" s="5">
         <v>160</v>
       </c>
@@ -7779,7 +7800,7 @@
         <v>904</v>
       </c>
     </row>
-    <row r="163" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A163" s="5">
         <v>161</v>
       </c>
@@ -7796,7 +7817,7 @@
         <v>904</v>
       </c>
     </row>
-    <row r="164" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A164" s="5">
         <v>162</v>
       </c>
@@ -7813,7 +7834,7 @@
         <v>904</v>
       </c>
     </row>
-    <row r="165" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:7" ht="75" x14ac:dyDescent="0.25">
       <c r="A165" s="5">
         <v>163</v>
       </c>
@@ -7830,7 +7851,7 @@
         <v>904</v>
       </c>
     </row>
-    <row r="166" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A166" s="5">
         <v>164</v>
       </c>
@@ -7847,7 +7868,7 @@
         <v>904</v>
       </c>
     </row>
-    <row r="167" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A167" s="5">
         <v>165</v>
       </c>
@@ -7864,7 +7885,7 @@
         <v>904</v>
       </c>
     </row>
-    <row r="168" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A168" s="5">
         <v>166</v>
       </c>
@@ -7881,7 +7902,7 @@
         <v>904</v>
       </c>
     </row>
-    <row r="169" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A169" s="5">
         <v>167</v>
       </c>
@@ -7898,7 +7919,7 @@
         <v>904</v>
       </c>
     </row>
-    <row r="170" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A170" s="5">
         <v>168</v>
       </c>
@@ -7915,7 +7936,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="171" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A171" s="5">
         <v>169</v>
       </c>
@@ -7929,6 +7950,125 @@
         <v>923</v>
       </c>
       <c r="G171" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="172" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A172" s="5">
+        <v>170</v>
+      </c>
+      <c r="B172" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C172" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D172" s="6" t="s">
+        <v>924</v>
+      </c>
+      <c r="G172" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="173" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A173" s="5">
+        <v>171</v>
+      </c>
+      <c r="B173" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C173" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D173" s="6" t="s">
+        <v>925</v>
+      </c>
+      <c r="G173" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="174" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A174" s="5">
+        <v>172</v>
+      </c>
+      <c r="B174" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C174" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D174" s="6" t="s">
+        <v>926</v>
+      </c>
+      <c r="G174" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="175" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A175" s="5">
+        <v>173</v>
+      </c>
+      <c r="B175" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C175" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="D175" s="6" t="s">
+        <v>927</v>
+      </c>
+      <c r="G175" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="176" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A176" s="5">
+        <v>174</v>
+      </c>
+      <c r="B176" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C176" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="D176" s="6" t="s">
+        <v>928</v>
+      </c>
+      <c r="G176" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="177" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A177" s="5">
+        <v>175</v>
+      </c>
+      <c r="B177" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C177" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D177" s="6" t="s">
+        <v>929</v>
+      </c>
+      <c r="G177" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="178" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A178" s="5">
+        <v>176</v>
+      </c>
+      <c r="B178" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="C178" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="D178" s="6" t="s">
+        <v>930</v>
+      </c>
+      <c r="G178" s="6" t="s">
         <v>904</v>
       </c>
     </row>
@@ -7960,14 +8100,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C103"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.54296875" customWidth="1"/>
+    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.5703125" customWidth="1"/>
     <col min="3" max="3" width="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>403</v>
       </c>
@@ -7978,7 +8118,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>406</v>
       </c>
@@ -7989,7 +8129,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>409</v>
       </c>
@@ -8000,7 +8140,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>411</v>
       </c>
@@ -8011,7 +8151,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>413</v>
       </c>
@@ -8022,7 +8162,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>416</v>
       </c>
@@ -8033,7 +8173,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>418</v>
       </c>
@@ -8044,7 +8184,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>420</v>
       </c>
@@ -8052,7 +8192,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>422</v>
       </c>
@@ -8060,7 +8200,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="72.650000000000006" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>424</v>
       </c>
@@ -8071,7 +8211,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>426</v>
       </c>
@@ -8079,7 +8219,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>428</v>
       </c>
@@ -8087,7 +8227,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>430</v>
       </c>
@@ -8095,7 +8235,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>432</v>
       </c>
@@ -8103,7 +8243,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>434</v>
       </c>
@@ -8111,7 +8251,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>436</v>
       </c>
@@ -8119,7 +8259,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>438</v>
       </c>
@@ -8127,7 +8267,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>440</v>
       </c>
@@ -8135,7 +8275,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>442</v>
       </c>
@@ -8143,7 +8283,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>444</v>
       </c>
@@ -8151,7 +8291,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>446</v>
       </c>
@@ -8159,7 +8299,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>448</v>
       </c>
@@ -8170,7 +8310,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>450</v>
       </c>
@@ -8178,7 +8318,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>452</v>
       </c>
@@ -8186,7 +8326,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>454</v>
       </c>
@@ -8194,7 +8334,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>456</v>
       </c>
@@ -8202,7 +8342,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>458</v>
       </c>
@@ -8210,7 +8350,7 @@
         <v>459</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>460</v>
       </c>
@@ -8218,7 +8358,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>462</v>
       </c>
@@ -8226,7 +8366,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>464</v>
       </c>
@@ -8234,7 +8374,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>466</v>
       </c>
@@ -8242,7 +8382,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>468</v>
       </c>
@@ -8250,7 +8390,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:3" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>470</v>
       </c>
@@ -8258,7 +8398,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>472</v>
       </c>
@@ -8266,7 +8406,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>474</v>
       </c>
@@ -8274,7 +8414,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>476</v>
       </c>
@@ -8282,7 +8422,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>478</v>
       </c>
@@ -8293,7 +8433,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>480</v>
       </c>
@@ -8301,7 +8441,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>482</v>
       </c>
@@ -8309,7 +8449,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>484</v>
       </c>
@@ -8317,7 +8457,7 @@
         <v>485</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>486</v>
       </c>
@@ -8325,7 +8465,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>488</v>
       </c>
@@ -8333,7 +8473,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>490</v>
       </c>
@@ -8341,7 +8481,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>492</v>
       </c>
@@ -8349,7 +8489,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>494</v>
       </c>
@@ -8357,7 +8497,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>496</v>
       </c>
@@ -8365,7 +8505,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>498</v>
       </c>
@@ -8373,7 +8513,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>500</v>
       </c>
@@ -8381,7 +8521,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>502</v>
       </c>
@@ -8389,7 +8529,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>504</v>
       </c>
@@ -8397,7 +8537,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>506</v>
       </c>
@@ -8405,7 +8545,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>508</v>
       </c>
@@ -8413,7 +8553,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>510</v>
       </c>
@@ -8421,7 +8561,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>512</v>
       </c>
@@ -8429,7 +8569,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>514</v>
       </c>
@@ -8437,7 +8577,7 @@
         <v>515</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>516</v>
       </c>
@@ -8448,7 +8588,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>518</v>
       </c>
@@ -8456,7 +8596,7 @@
         <v>519</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>520</v>
       </c>
@@ -8464,7 +8604,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>522</v>
       </c>
@@ -8472,7 +8612,7 @@
         <v>523</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>524</v>
       </c>
@@ -8480,7 +8620,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>526</v>
       </c>
@@ -8488,7 +8628,7 @@
         <v>527</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>528</v>
       </c>
@@ -8496,7 +8636,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>530</v>
       </c>
@@ -8504,7 +8644,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>532</v>
       </c>
@@ -8512,7 +8652,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>534</v>
       </c>
@@ -8520,7 +8660,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>536</v>
       </c>
@@ -8528,7 +8668,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>538</v>
       </c>
@@ -8536,7 +8676,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>540</v>
       </c>
@@ -8544,7 +8684,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>542</v>
       </c>
@@ -8552,7 +8692,7 @@
         <v>543</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>544</v>
       </c>
@@ -8563,7 +8703,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>546</v>
       </c>
@@ -8571,7 +8711,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>548</v>
       </c>
@@ -8579,7 +8719,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>550</v>
       </c>
@@ -8587,7 +8727,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>552</v>
       </c>
@@ -8595,7 +8735,7 @@
         <v>553</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>554</v>
       </c>
@@ -8603,7 +8743,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>556</v>
       </c>
@@ -8611,7 +8751,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>558</v>
       </c>
@@ -8619,7 +8759,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>560</v>
       </c>
@@ -8627,7 +8767,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>562</v>
       </c>
@@ -8635,7 +8775,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>564</v>
       </c>
@@ -8643,7 +8783,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>566</v>
       </c>
@@ -8651,7 +8791,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>568</v>
       </c>
@@ -8659,7 +8799,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>570</v>
       </c>
@@ -8667,7 +8807,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>572</v>
       </c>
@@ -8675,7 +8815,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>574</v>
       </c>
@@ -8683,7 +8823,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>576</v>
       </c>
@@ -8691,7 +8831,7 @@
         <v>577</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>578</v>
       </c>
@@ -8699,7 +8839,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>580</v>
       </c>
@@ -8707,7 +8847,7 @@
         <v>581</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>582</v>
       </c>
@@ -8715,7 +8855,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>584</v>
       </c>
@@ -8723,7 +8863,7 @@
         <v>585</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>586</v>
       </c>
@@ -8731,7 +8871,7 @@
         <v>587</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>588</v>
       </c>
@@ -8739,7 +8879,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>590</v>
       </c>
@@ -8747,7 +8887,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>592</v>
       </c>
@@ -8755,7 +8895,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>594</v>
       </c>
@@ -8763,7 +8903,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>596</v>
       </c>
@@ -8771,7 +8911,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>598</v>
       </c>
@@ -8779,7 +8919,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>600</v>
       </c>
@@ -8787,7 +8927,7 @@
         <v>601</v>
       </c>
     </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>602</v>
       </c>
@@ -8795,7 +8935,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>604</v>
       </c>
@@ -8803,7 +8943,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>606</v>
       </c>
@@ -8811,7 +8951,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>608</v>
       </c>
@@ -8819,7 +8959,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>610</v>
       </c>
@@ -8851,13 +8991,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C49"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="29.54296875" customWidth="1"/>
-    <col min="3" max="3" width="5.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="29.5703125" customWidth="1"/>
+    <col min="3" max="3" width="5.42578125" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>403</v>
       </c>
@@ -8868,7 +9008,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>612</v>
       </c>
@@ -8876,7 +9016,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>614</v>
       </c>
@@ -8884,7 +9024,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>615</v>
       </c>
@@ -8892,7 +9032,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>617</v>
       </c>
@@ -8900,7 +9040,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>619</v>
       </c>
@@ -8908,7 +9048,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>621</v>
       </c>
@@ -8916,7 +9056,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>623</v>
       </c>
@@ -8924,7 +9064,7 @@
         <v>624</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>625</v>
       </c>
@@ -8932,7 +9072,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>627</v>
       </c>
@@ -8940,7 +9080,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>629</v>
       </c>
@@ -8948,7 +9088,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>631</v>
       </c>
@@ -8956,7 +9096,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>633</v>
       </c>
@@ -8964,7 +9104,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>635</v>
       </c>
@@ -8972,7 +9112,7 @@
         <v>636</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>637</v>
       </c>
@@ -8980,7 +9120,7 @@
         <v>638</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>639</v>
       </c>
@@ -8988,7 +9128,7 @@
         <v>640</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>641</v>
       </c>
@@ -8996,7 +9136,7 @@
         <v>642</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>643</v>
       </c>
@@ -9007,7 +9147,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>645</v>
       </c>
@@ -9015,7 +9155,7 @@
         <v>646</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>647</v>
       </c>
@@ -9023,7 +9163,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>649</v>
       </c>
@@ -9031,7 +9171,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>651</v>
       </c>
@@ -9039,7 +9179,7 @@
         <v>652</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>653</v>
       </c>
@@ -9047,7 +9187,7 @@
         <v>654</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>655</v>
       </c>
@@ -9055,7 +9195,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>657</v>
       </c>
@@ -9063,7 +9203,7 @@
         <v>658</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>659</v>
       </c>
@@ -9071,7 +9211,7 @@
         <v>660</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>661</v>
       </c>
@@ -9079,7 +9219,7 @@
         <v>662</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>663</v>
       </c>
@@ -9087,7 +9227,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>665</v>
       </c>
@@ -9095,7 +9235,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>667</v>
       </c>
@@ -9103,7 +9243,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>669</v>
       </c>
@@ -9111,7 +9251,7 @@
         <v>670</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>671</v>
       </c>
@@ -9119,7 +9259,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>673</v>
       </c>
@@ -9127,7 +9267,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>675</v>
       </c>
@@ -9135,7 +9275,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>677</v>
       </c>
@@ -9143,7 +9283,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>679</v>
       </c>
@@ -9151,7 +9291,7 @@
         <v>680</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>681</v>
       </c>
@@ -9159,7 +9299,7 @@
         <v>682</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>683</v>
       </c>
@@ -9167,7 +9307,7 @@
         <v>684</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>685</v>
       </c>
@@ -9175,7 +9315,7 @@
         <v>686</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>687</v>
       </c>
@@ -9183,7 +9323,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>689</v>
       </c>
@@ -9191,7 +9331,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>691</v>
       </c>
@@ -9199,7 +9339,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>693</v>
       </c>
@@ -9207,7 +9347,7 @@
         <v>694</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>695</v>
       </c>
@@ -9215,7 +9355,7 @@
         <v>696</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>697</v>
       </c>
@@ -9223,7 +9363,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>698</v>
       </c>
@@ -9231,7 +9371,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>700</v>
       </c>
@@ -9239,7 +9379,7 @@
         <v>701</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>702</v>
       </c>
@@ -9247,7 +9387,7 @@
         <v>703</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>704</v>
       </c>
@@ -9274,14 +9414,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:C48"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>403</v>
       </c>
@@ -9292,7 +9432,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>706</v>
       </c>
@@ -9300,7 +9440,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>708</v>
       </c>
@@ -9308,7 +9448,7 @@
         <v>709</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>710</v>
       </c>
@@ -9316,7 +9456,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>712</v>
       </c>
@@ -9324,7 +9464,7 @@
         <v>713</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>714</v>
       </c>
@@ -9332,7 +9472,7 @@
         <v>715</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>716</v>
       </c>
@@ -9340,7 +9480,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>717</v>
       </c>
@@ -9348,7 +9488,7 @@
         <v>718</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>719</v>
       </c>
@@ -9356,7 +9496,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>721</v>
       </c>
@@ -9364,7 +9504,7 @@
         <v>722</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>723</v>
       </c>
@@ -9372,7 +9512,7 @@
         <v>724</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>725</v>
       </c>
@@ -9380,7 +9520,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>726</v>
       </c>
@@ -9388,7 +9528,7 @@
         <v>727</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>728</v>
       </c>
@@ -9396,7 +9536,7 @@
         <v>729</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>730</v>
       </c>
@@ -9404,7 +9544,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>731</v>
       </c>
@@ -9412,7 +9552,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>732</v>
       </c>
@@ -9420,7 +9560,7 @@
         <v>733</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>734</v>
       </c>
@@ -9428,7 +9568,7 @@
         <v>735</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>736</v>
       </c>
@@ -9436,7 +9576,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>737</v>
       </c>
@@ -9444,7 +9584,7 @@
         <v>738</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>739</v>
       </c>
@@ -9452,7 +9592,7 @@
         <v>740</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>741</v>
       </c>
@@ -9460,7 +9600,7 @@
         <v>742</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>743</v>
       </c>
@@ -9468,7 +9608,7 @@
         <v>744</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>745</v>
       </c>
@@ -9476,7 +9616,7 @@
         <v>746</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>747</v>
       </c>
@@ -9484,7 +9624,7 @@
         <v>485</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>748</v>
       </c>
@@ -9492,7 +9632,7 @@
         <v>749</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>750</v>
       </c>
@@ -9500,7 +9640,7 @@
         <v>751</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>752</v>
       </c>
@@ -9508,7 +9648,7 @@
         <v>753</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>754</v>
       </c>
@@ -9516,7 +9656,7 @@
         <v>755</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>756</v>
       </c>
@@ -9524,7 +9664,7 @@
         <v>757</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>758</v>
       </c>
@@ -9532,7 +9672,7 @@
         <v>759</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>760</v>
       </c>
@@ -9540,7 +9680,7 @@
         <v>761</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>762</v>
       </c>
@@ -9548,7 +9688,7 @@
         <v>763</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>764</v>
       </c>
@@ -9556,7 +9696,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>766</v>
       </c>
@@ -9564,7 +9704,7 @@
         <v>767</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>768</v>
       </c>
@@ -9572,7 +9712,7 @@
         <v>769</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>770</v>
       </c>
@@ -9580,7 +9720,7 @@
         <v>771</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>772</v>
       </c>
@@ -9588,7 +9728,7 @@
         <v>773</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>774</v>
       </c>
@@ -9596,7 +9736,7 @@
         <v>775</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>776</v>
       </c>
@@ -9604,7 +9744,7 @@
         <v>777</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>778</v>
       </c>
@@ -9612,7 +9752,7 @@
         <v>779</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>780</v>
       </c>
@@ -9620,7 +9760,7 @@
         <v>781</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>782</v>
       </c>
@@ -9628,7 +9768,7 @@
         <v>783</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>784</v>
       </c>
@@ -9636,7 +9776,7 @@
         <v>785</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>786</v>
       </c>
@@ -9644,7 +9784,7 @@
         <v>787</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>788</v>
       </c>
@@ -9652,7 +9792,7 @@
         <v>789</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>790</v>
       </c>
@@ -9660,7 +9800,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>792</v>
       </c>
@@ -9687,14 +9827,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:C67"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>403</v>
       </c>
@@ -9705,7 +9845,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>794</v>
       </c>
@@ -9713,7 +9853,7 @@
         <v>795</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>796</v>
       </c>
@@ -9721,7 +9861,7 @@
         <v>797</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>798</v>
       </c>
@@ -9729,7 +9869,7 @@
         <v>799</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>800</v>
       </c>
@@ -9737,7 +9877,7 @@
         <v>801</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>802</v>
       </c>
@@ -9745,7 +9885,7 @@
         <v>803</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>804</v>
       </c>
@@ -9753,7 +9893,7 @@
         <v>805</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>806</v>
       </c>
@@ -9761,7 +9901,7 @@
         <v>807</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>808</v>
       </c>
@@ -9769,7 +9909,7 @@
         <v>809</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>810</v>
       </c>
@@ -9777,7 +9917,7 @@
         <v>811</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>812</v>
       </c>
@@ -9785,7 +9925,7 @@
         <v>813</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>814</v>
       </c>
@@ -9793,7 +9933,7 @@
         <v>815</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>816</v>
       </c>
@@ -9801,7 +9941,7 @@
         <v>817</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>818</v>
       </c>
@@ -9809,7 +9949,7 @@
         <v>819</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>820</v>
       </c>
@@ -9817,7 +9957,7 @@
         <v>821</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>822</v>
       </c>
@@ -9825,7 +9965,7 @@
         <v>823</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>824</v>
       </c>
@@ -9833,7 +9973,7 @@
         <v>825</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>826</v>
       </c>
@@ -9841,7 +9981,7 @@
         <v>827</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>828</v>
       </c>
@@ -9849,7 +9989,7 @@
         <v>829</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>830</v>
       </c>
@@ -9857,7 +9997,7 @@
         <v>831</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>832</v>
       </c>
@@ -9865,7 +10005,7 @@
         <v>833</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>834</v>
       </c>
@@ -9873,7 +10013,7 @@
         <v>835</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>836</v>
       </c>
@@ -9881,7 +10021,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>838</v>
       </c>
@@ -9889,7 +10029,7 @@
         <v>839</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>840</v>
       </c>
@@ -9897,7 +10037,7 @@
         <v>841</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>842</v>
       </c>
@@ -9905,7 +10045,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>844</v>
       </c>
@@ -9913,7 +10053,7 @@
         <v>845</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>846</v>
       </c>
@@ -9921,7 +10061,7 @@
         <v>847</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>848</v>
       </c>
@@ -9929,7 +10069,7 @@
         <v>849</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>850</v>
       </c>
@@ -9937,7 +10077,7 @@
         <v>851</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>852</v>
       </c>
@@ -9945,7 +10085,7 @@
         <v>853</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>854</v>
       </c>
@@ -9953,7 +10093,7 @@
         <v>855</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>856</v>
       </c>
@@ -9961,7 +10101,7 @@
         <v>857</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>858</v>
       </c>
@@ -9969,7 +10109,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>859</v>
       </c>
@@ -9977,7 +10117,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>860</v>
       </c>
@@ -9985,7 +10125,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>861</v>
       </c>
@@ -9993,7 +10133,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>862</v>
       </c>
@@ -10001,7 +10141,7 @@
         <v>863</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>864</v>
       </c>
@@ -10009,7 +10149,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>865</v>
       </c>
@@ -10017,7 +10157,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>866</v>
       </c>
@@ -10025,7 +10165,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>867</v>
       </c>
@@ -10033,7 +10173,7 @@
         <v>680</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>868</v>
       </c>
@@ -10041,7 +10181,7 @@
         <v>761</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>869</v>
       </c>
@@ -10049,7 +10189,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>870</v>
       </c>
@@ -10057,7 +10197,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>871</v>
       </c>
@@ -10065,7 +10205,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>872</v>
       </c>
@@ -10073,7 +10213,7 @@
         <v>515</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>873</v>
       </c>
@@ -10081,7 +10221,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>874</v>
       </c>
@@ -10089,7 +10229,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>875</v>
       </c>
@@ -10097,7 +10237,7 @@
         <v>694</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>876</v>
       </c>
@@ -10105,7 +10245,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>877</v>
       </c>
@@ -10113,7 +10253,7 @@
         <v>775</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>878</v>
       </c>
@@ -10121,7 +10261,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>879</v>
       </c>
@@ -10129,7 +10269,7 @@
         <v>779</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>880</v>
       </c>
@@ -10137,7 +10277,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>881</v>
       </c>
@@ -10145,7 +10285,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>882</v>
       </c>
@@ -10153,7 +10293,7 @@
         <v>783</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>883</v>
       </c>
@@ -10161,7 +10301,7 @@
         <v>884</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>885</v>
       </c>
@@ -10169,7 +10309,7 @@
         <v>886</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>887</v>
       </c>
@@ -10177,7 +10317,7 @@
         <v>888</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>889</v>
       </c>
@@ -10185,7 +10325,7 @@
         <v>890</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>891</v>
       </c>
@@ -10193,7 +10333,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>893</v>
       </c>
@@ -10201,7 +10341,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>895</v>
       </c>
@@ -10209,7 +10349,7 @@
         <v>896</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>897</v>
       </c>
@@ -10217,7 +10357,7 @@
         <v>898</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>899</v>
       </c>
@@ -10225,7 +10365,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>901</v>
       </c>
@@ -10252,47 +10392,47 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:A8"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>903</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>904</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>905</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>350</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>906</v>
       </c>

</xml_diff>

<commit_message>
NPC Data: Started to create starter gym decks for opponents & logged 20+ issues
</commit_message>
<xml_diff>
--- a/Spreadsheets/Issue_Log.xlsx
+++ b/Spreadsheets/Issue_Log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\Spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33BA1B36-5FDB-4A33-AA2F-A3D7CE9D9B76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE97D2C7-8EFB-4078-AEFC-A6B701DE61D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="30912" windowHeight="18672" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Game_Issues" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1741" uniqueCount="931">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1949" uniqueCount="985">
   <si>
     <t>#</t>
   </si>
@@ -2973,6 +2973,168 @@
   </si>
   <si>
     <t>Opponent attached a full heal energy to a benched dark primeape. This provides colorless energy to heal statuses. Bench pokemon can't have statuses and dark primeape has no use for colorless energy. Full heal energy should only be played when it provides no energy benefit when it DOES heal a status condition. This is the same for Potion energy, it should only be used if the colorless energy provided actually helps AND OR the 10hp recovery is needed. Otherwise, any other energy should be prioritised instead.</t>
+  </si>
+  <si>
+    <t>New UI Update</t>
+  </si>
+  <si>
+    <t>In Search and filter mode for deck mode, Search category texts font needs to be white.</t>
+  </si>
+  <si>
+    <t>In Search and filter mode for deck mode, the set buttons, pokemon sub type, has pokepower body and rarity buttons are all overlapping and need to be more separated. This is easy for everything but set buttons which may potentially force the ex sets onto a new line. However there is a little bit of space to the left of all the search buttons next to the header texts so if needed they can all be moved slightly over to the left and potentially resized 5%-10% Smaller making room</t>
+  </si>
+  <si>
+    <t>Rename the buttons that "has a pokemon power/pokepower" and "has a poke -body"  to just "Poke-Power" "Poke-Body"</t>
+  </si>
+  <si>
+    <t>The text in the textbox for name and illustrator name start at the edge of the left hand side of the textbox, they need a little bit of space before the text is in the box</t>
+  </si>
+  <si>
+    <t>The text in the textbox for name and illustrator name when a player types Is black. Font should be pure white.</t>
+  </si>
+  <si>
+    <t>When entering either view deck mode or search mode then returning to the main deck screen, there is a large XX / XX deck total counter in the top center of the screen. This does not exist unless you go into a sub menu and return and shouldn't exist at all.</t>
+  </si>
+  <si>
+    <t>Increase the size of the arrow font by about double and bolden it. Make the button itself about 10 pixels taller expanding downward</t>
+  </si>
+  <si>
+    <t>Make all buttons in the new UI even more rounded so they're more of a pill vs a rounded rectangle</t>
+  </si>
+  <si>
+    <t>The "View Deck" button text font size is larger than the other button texts.</t>
+  </si>
+  <si>
+    <t>in the View Deck mode, the close button does not work. It cannot be clicked or highlighted at all. (Escape cancels out correctly)</t>
+  </si>
+  <si>
+    <t>Move  the deck count pill box to underneath the composition box, making it wider to match the width of the compositon box. Move the deck name box slightly to the right to make room for a label to the left of the deck name box. Create the new label to the left of the now moved deck name box with text of "Name:"</t>
+  </si>
+  <si>
+    <t>Headers should be consistently central aligned, including the "composition" and "energies in decks" text</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Increase the font size in the composition box for the header "composition"  and the category texts "Basic" "stage 1" "stage 2" "trainer" and "energy" by about 20%. </t>
+  </si>
+  <si>
+    <t>In the View deck mode, for the individual entries in the right hand bar, the text needs moving inwards both ways so the card name needs moving to the rigtht a few pixels, and the count needs moving left a few pixels</t>
+  </si>
+  <si>
+    <t>in the view deck mode, remove the categories in the top right, these are repeated data from the composition box in the main deck view mode</t>
+  </si>
+  <si>
+    <t>Game startup with the first load set of the name costume and date of birth is not in the new UI format entirely. It has the new buttons and textboxes and font but still has the old blue black header footer and white background. This needs setting to the new UI format.</t>
+  </si>
+  <si>
+    <t>Sometimes when in the card shop and moving between sets, the price pills randomly go in the top right corner and arent' showing in the corner of the cards</t>
+  </si>
+  <si>
+    <t>Reduce the bonus rare chance rate by half. When the bonus rare appears, instead of having it as a bonus 11th card, instead replace one of the random commons in the pack with the rare but keeping the order the same so if you get the bonus rare pack, you only get 5 commons, 3 uncommons, the normal rare then the bonus rare</t>
+  </si>
+  <si>
+    <t>The Sleeve shop should use the "large" sleeve images, it looks like it uses the small images as the images don't look crisp</t>
+  </si>
+  <si>
+    <t>For the cards you don't own, instead of having the blacked out cards be a grey opaque rectangle, it should look like translucent glass like the mockup and exactly the same as how the sleeves are shown when they are missing</t>
+  </si>
+  <si>
+    <t>In costume view of unowned costumes, the boxes are all the wrong size and overlap. Most of the sprites are too big for the box and overlap so the costume size needs to be slightly decreased and the boxes are very wide instead of being square,. The boxes are also missing for the default costumes</t>
+  </si>
+  <si>
+    <t>In the trainer card view, the player's in battle sprite (costume) is stretched thinly so it doesn't look right it needs to keep it's aspect</t>
+  </si>
+  <si>
+    <t>in the trainer card view, you can't edit the player's name at all, the box isn't clickable</t>
+  </si>
+  <si>
+    <t>in the trainer card "equipped" should be centrally aligned</t>
+  </si>
+  <si>
+    <t>in the trainer card, all the font needs increasing 50% Except for the "Trainer card" header and the button text fonts</t>
+  </si>
+  <si>
+    <t>in the trainer card, the "trainer since" and cash needs to be moved down away from the name textbox a few pixels</t>
+  </si>
+  <si>
+    <t>The quit the game UI pop up still uses the old kenney theme not the new UI</t>
+  </si>
+  <si>
+    <t>When opening a pack, the cards shouldn't have the player's sleeve, it should use the default card back</t>
+  </si>
+  <si>
+    <t>When in the discount card weighted pack shop, when moving from fossil to rocket or base to rocket, there is a slight noticeable delay in the packs loading</t>
+  </si>
+  <si>
+    <t>With the new UI, the cash label is in the top right of the screen. When selling your bulk, the +$XXX label pops upwards from the bottom right, instead it should move downwards from the top right now and decrease the font size by half</t>
+  </si>
+  <si>
+    <t>In the confirm page of selling bulk, the information box in the top right has all the text aligned to the edge of the box (this has been an issue listed above for other screens.) The box can be made bigger on this screen to give more space to the side of all the text inside</t>
+  </si>
+  <si>
+    <t>Swap the music in the gym plaza out. The music that plays here should be the music at the game startup only (first launch setup screen). The music in gym plaza should instead be the same as inside the gym challenge hall.</t>
+  </si>
+  <si>
+    <t>In the main match screen, the action buttons (Place as activ e) (place on bench) (done) needs moving up to be central in the footer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nearly everything from the mock up is missing from the main match screen. No placeholders for the empty bench, messagebox can't be seen,  hand can't be seen,  no placeholder for missing prize cards, HP blocks overlap the player active pokemon, no card details next to the active cards, </t>
+  </si>
+  <si>
+    <t>When a trainer is played in the main match, it's still shown on a white screen instead of the new UI, instead of it being white, everythign should just be hidden and the trainer card should be shown on the new UI background</t>
+  </si>
+  <si>
+    <t>When the main match starts, the [turn 1] pill, the middle of screen turn split line, the stadium text and placeholder can be seen even though the hand is being shown. All of these should be hidden anytime other than just the main screen is shown. When a card is set as active pokemon, the attack buttons can be seen too.</t>
+  </si>
+  <si>
+    <t>in the main match, the energy icons for attacks are just coloured pills, they shoul dbe the actual energy icons instead</t>
+  </si>
+  <si>
+    <t>in the main match, player attached energies (and proabably tools) are too far right and overlap the attack buttons</t>
+  </si>
+  <si>
+    <t>In the main match, the attack buttons can just be freely pressed at any time so the player can just keep hitting the attack button to do damage</t>
+  </si>
+  <si>
+    <t>in the main match, status condition icons are absolutely massive and too wide.</t>
+  </si>
+  <si>
+    <t>In the main match, the opponent's bench pokemon HP damage counters are slightly too low and the active pokemon cover them slightly, the active pokemon can simply be moved down slightyl as there is spare space under them</t>
+  </si>
+  <si>
+    <t>The discard pile cards are larger than the deck, they should be the same size, but also they're too close and need a few pixels of seperation</t>
+  </si>
+  <si>
+    <t>The lines above and below YOUR TURN should be a lot shorter, closer to the text and thicker.</t>
+  </si>
+  <si>
+    <t>The text in the attack buttons should be more centrally aligned instead of aligned to the right next to the energy costs</t>
+  </si>
+  <si>
+    <t>The attack buttons should be shorter in width</t>
+  </si>
+  <si>
+    <t>The active pokemon HP counters should be in the new style the same as the bench pokemon</t>
+  </si>
+  <si>
+    <t>In all of the shops, the new drop shadow requested is stupidly large and well out of alignment. This drop shadow should only be 5% bigger than the item the shadow is being cast by and should be a lot closer only a few pixels to the right and underneath the item. The drop shadow actually works for the main pack shops but not for anything else</t>
+  </si>
+  <si>
+    <t>In the view deck mode, I assume the card holding container goes all the way to the bottom of the screen which hides the cards behind the footer. The bottom of the container needs to stop at the top of the footer like in regular deck mode. Similarly the top of the container has a small bit of wasted space resulting in  a thin black band at the top of the cards, again this should just match deck mode view. This also applies to the bulk sell confirm page</t>
+  </si>
+  <si>
+    <t>Logic</t>
+  </si>
+  <si>
+    <t>Add "Type" to sort by in the search and filter in deck mode so cards can be sorted by Name, Set or Type. When sorting by type, sort by pokemon energy type first (like fire fighting grass water lightning) then trainers then special energy</t>
+  </si>
+  <si>
+    <t>The reset button on the search and filter page has the old issue that it's only pressed on mouse release instead of on mouse click. It should click on click</t>
+  </si>
+  <si>
+    <t>Change the size of the cards in the deck card view so that the rows are only 7 pokemon cards wide, increasing all the cards to make up the extra room.</t>
+  </si>
+  <si>
+    <t>In deck builder mode, we know if the player has changes that needs to be saved, if the player hits escape or cancel, pop up a confirmation that asks "You have unsaved changes, are you sure you want to leave?"</t>
   </si>
 </sst>
 </file>
@@ -3069,6 +3231,38 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="16">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFBDD7EE"/>
+          <bgColor rgb="FFBDD7EE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -3198,38 +3392,6 @@
         <patternFill patternType="solid">
           <fgColor rgb="FFC6EFCE"/>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBDD7EE"/>
-          <bgColor rgb="FFBDD7EE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3563,7 +3725,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J178"/>
+  <dimension ref="A1:J290"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="5" bestFit="1" customWidth="1"/>
@@ -3573,8 +3735,8 @@
     <col min="5" max="5" width="255.5703125" style="6" hidden="1" customWidth="1"/>
     <col min="6" max="6" width="102" style="6" customWidth="1"/>
     <col min="7" max="7" width="19" style="6" customWidth="1"/>
-    <col min="8" max="9" width="11.140625" style="7" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16" style="7" customWidth="1"/>
+    <col min="8" max="9" width="11.140625" style="7" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="16" style="7" hidden="1" customWidth="1"/>
     <col min="11" max="17" width="9.140625" style="7" customWidth="1"/>
     <col min="18" max="16384" width="9.140625" style="7"/>
   </cols>
@@ -8072,19 +8234,1203 @@
         <v>904</v>
       </c>
     </row>
+    <row r="179" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A179" s="5">
+        <v>177</v>
+      </c>
+      <c r="B179" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C179" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D179" s="6" t="s">
+        <v>932</v>
+      </c>
+      <c r="G179" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="180" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A180" s="5">
+        <v>178</v>
+      </c>
+      <c r="B180" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C180" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D180" s="6" t="s">
+        <v>933</v>
+      </c>
+      <c r="G180" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="181" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A181" s="5">
+        <v>179</v>
+      </c>
+      <c r="B181" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C181" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D181" s="6" t="s">
+        <v>934</v>
+      </c>
+      <c r="G181" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="182" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A182" s="5">
+        <v>180</v>
+      </c>
+      <c r="B182" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C182" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D182" s="6" t="s">
+        <v>935</v>
+      </c>
+      <c r="G182" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="183" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A183" s="5">
+        <v>181</v>
+      </c>
+      <c r="B183" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C183" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D183" s="6" t="s">
+        <v>936</v>
+      </c>
+      <c r="G183" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="184" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A184" s="5">
+        <v>182</v>
+      </c>
+      <c r="B184" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C184" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D184" s="6" t="s">
+        <v>937</v>
+      </c>
+      <c r="G184" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="185" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A185" s="5">
+        <v>183</v>
+      </c>
+      <c r="B185" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C185" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D185" s="6" t="s">
+        <v>938</v>
+      </c>
+      <c r="G185" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="186" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A186" s="5">
+        <v>184</v>
+      </c>
+      <c r="B186" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C186" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D186" s="6" t="s">
+        <v>939</v>
+      </c>
+      <c r="G186" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="187" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A187" s="5">
+        <v>185</v>
+      </c>
+      <c r="B187" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C187" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D187" s="6" t="s">
+        <v>940</v>
+      </c>
+      <c r="G187" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="188" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A188" s="5">
+        <v>186</v>
+      </c>
+      <c r="B188" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C188" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D188" s="6" t="s">
+        <v>941</v>
+      </c>
+      <c r="G188" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="189" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A189" s="5">
+        <v>187</v>
+      </c>
+      <c r="B189" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C189" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D189" s="6" t="s">
+        <v>942</v>
+      </c>
+      <c r="G189" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="190" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A190" s="5">
+        <v>188</v>
+      </c>
+      <c r="B190" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C190" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D190" s="6" t="s">
+        <v>944</v>
+      </c>
+      <c r="G190" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="191" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A191" s="5">
+        <v>189</v>
+      </c>
+      <c r="B191" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C191" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D191" s="6" t="s">
+        <v>943</v>
+      </c>
+      <c r="G191" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="192" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A192" s="5">
+        <v>190</v>
+      </c>
+      <c r="B192" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C192" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D192" s="6" t="s">
+        <v>945</v>
+      </c>
+      <c r="G192" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="193" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A193" s="5">
+        <v>191</v>
+      </c>
+      <c r="B193" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C193" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D193" s="6" t="s">
+        <v>946</v>
+      </c>
+      <c r="G193" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="194" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A194" s="5">
+        <v>192</v>
+      </c>
+      <c r="B194" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C194" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D194" s="6" t="s">
+        <v>947</v>
+      </c>
+      <c r="G194" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="195" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A195" s="5">
+        <v>193</v>
+      </c>
+      <c r="B195" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C195" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D195" s="6" t="s">
+        <v>951</v>
+      </c>
+      <c r="G195" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="196" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A196" s="5">
+        <v>194</v>
+      </c>
+      <c r="B196" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C196" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D196" s="6" t="s">
+        <v>979</v>
+      </c>
+      <c r="G196" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="197" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A197" s="5">
+        <v>195</v>
+      </c>
+      <c r="B197" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C197" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D197" s="6" t="s">
+        <v>948</v>
+      </c>
+      <c r="G197" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="198" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A198" s="5">
+        <v>196</v>
+      </c>
+      <c r="B198" s="5" t="s">
+        <v>919</v>
+      </c>
+      <c r="C198" s="5" t="s">
+        <v>920</v>
+      </c>
+      <c r="D198" s="6" t="s">
+        <v>949</v>
+      </c>
+      <c r="G198" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="199" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A199" s="5">
+        <v>197</v>
+      </c>
+      <c r="B199" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C199" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D199" s="6" t="s">
+        <v>978</v>
+      </c>
+      <c r="G199" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="200" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A200" s="5">
+        <v>198</v>
+      </c>
+      <c r="B200" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C200" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D200" s="6" t="s">
+        <v>950</v>
+      </c>
+      <c r="G200" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="201" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A201" s="5">
+        <v>199</v>
+      </c>
+      <c r="B201" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C201" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D201" s="6" t="s">
+        <v>952</v>
+      </c>
+      <c r="G201" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="202" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A202" s="5">
+        <v>200</v>
+      </c>
+      <c r="B202" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C202" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D202" s="6" t="s">
+        <v>953</v>
+      </c>
+      <c r="G202" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="203" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A203" s="5">
+        <v>201</v>
+      </c>
+      <c r="B203" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C203" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D203" s="6" t="s">
+        <v>954</v>
+      </c>
+      <c r="G203" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="204" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A204" s="5">
+        <v>202</v>
+      </c>
+      <c r="B204" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C204" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D204" s="6" t="s">
+        <v>955</v>
+      </c>
+      <c r="G204" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="205" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A205" s="5">
+        <v>203</v>
+      </c>
+      <c r="B205" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C205" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D205" s="6" t="s">
+        <v>956</v>
+      </c>
+      <c r="G205" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="206" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A206" s="5">
+        <v>204</v>
+      </c>
+      <c r="B206" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C206" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D206" s="6" t="s">
+        <v>957</v>
+      </c>
+      <c r="G206" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="207" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A207" s="5">
+        <v>205</v>
+      </c>
+      <c r="B207" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C207" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D207" s="6" t="s">
+        <v>958</v>
+      </c>
+      <c r="G207" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="208" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A208" s="5">
+        <v>206</v>
+      </c>
+      <c r="B208" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C208" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="D208" s="6" t="s">
+        <v>959</v>
+      </c>
+      <c r="G208" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="209" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A209" s="5">
+        <v>207</v>
+      </c>
+      <c r="B209" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C209" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D209" s="6" t="s">
+        <v>960</v>
+      </c>
+      <c r="G209" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="210" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A210" s="5">
+        <v>208</v>
+      </c>
+      <c r="B210" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C210" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D210" s="6" t="s">
+        <v>961</v>
+      </c>
+      <c r="G210" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="211" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A211" s="5">
+        <v>209</v>
+      </c>
+      <c r="B211" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C211" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D211" s="6" t="s">
+        <v>962</v>
+      </c>
+      <c r="G211" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="212" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A212" s="5">
+        <v>210</v>
+      </c>
+      <c r="B212" s="5" t="s">
+        <v>919</v>
+      </c>
+      <c r="C212" s="5" t="s">
+        <v>920</v>
+      </c>
+      <c r="D212" s="6" t="s">
+        <v>963</v>
+      </c>
+      <c r="G212" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="213" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A213" s="5">
+        <v>211</v>
+      </c>
+      <c r="B213" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C213" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D213" s="6" t="s">
+        <v>964</v>
+      </c>
+      <c r="G213" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="214" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A214" s="5">
+        <v>212</v>
+      </c>
+      <c r="B214" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C214" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D214" s="6" t="s">
+        <v>967</v>
+      </c>
+      <c r="G214" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="215" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A215" s="5">
+        <v>213</v>
+      </c>
+      <c r="B215" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C215" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D215" s="6" t="s">
+        <v>965</v>
+      </c>
+      <c r="G215" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="216" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A216" s="5">
+        <v>214</v>
+      </c>
+      <c r="B216" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C216" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D216" s="6" t="s">
+        <v>966</v>
+      </c>
+      <c r="G216" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="217" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A217" s="5">
+        <v>215</v>
+      </c>
+      <c r="B217" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C217" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D217" s="6" t="s">
+        <v>968</v>
+      </c>
+      <c r="G217" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="218" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A218" s="5">
+        <v>216</v>
+      </c>
+      <c r="B218" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C218" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D218" s="6" t="s">
+        <v>969</v>
+      </c>
+      <c r="G218" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="219" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A219" s="5">
+        <v>217</v>
+      </c>
+      <c r="B219" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C219" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D219" s="6" t="s">
+        <v>970</v>
+      </c>
+      <c r="G219" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="220" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A220" s="5">
+        <v>218</v>
+      </c>
+      <c r="B220" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C220" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D220" s="6" t="s">
+        <v>971</v>
+      </c>
+      <c r="G220" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="221" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A221" s="5">
+        <v>219</v>
+      </c>
+      <c r="B221" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C221" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D221" s="6" t="s">
+        <v>972</v>
+      </c>
+      <c r="G221" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="222" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A222" s="5">
+        <v>220</v>
+      </c>
+      <c r="B222" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C222" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D222" s="6" t="s">
+        <v>973</v>
+      </c>
+      <c r="G222" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="223" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A223" s="5">
+        <v>221</v>
+      </c>
+      <c r="B223" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C223" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D223" s="6" t="s">
+        <v>974</v>
+      </c>
+      <c r="G223" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="224" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A224" s="5">
+        <v>222</v>
+      </c>
+      <c r="B224" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C224" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D224" s="6" t="s">
+        <v>975</v>
+      </c>
+      <c r="G224" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="225" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A225" s="5">
+        <v>223</v>
+      </c>
+      <c r="B225" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C225" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D225" s="6" t="s">
+        <v>976</v>
+      </c>
+      <c r="G225" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="226" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A226" s="5">
+        <v>224</v>
+      </c>
+      <c r="B226" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C226" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="D226" s="6" t="s">
+        <v>977</v>
+      </c>
+      <c r="G226" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="227" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A227" s="5">
+        <v>225</v>
+      </c>
+      <c r="B227" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C227" s="5" t="s">
+        <v>980</v>
+      </c>
+      <c r="D227" s="6" t="s">
+        <v>981</v>
+      </c>
+      <c r="G227" s="6" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="228" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A228" s="5">
+        <v>226</v>
+      </c>
+      <c r="B228" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C228" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D228" s="6" t="s">
+        <v>982</v>
+      </c>
+      <c r="G228" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="229" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A229" s="5">
+        <v>227</v>
+      </c>
+      <c r="B229" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C229" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D229" s="6" t="s">
+        <v>983</v>
+      </c>
+      <c r="G229" s="6" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="230" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A230" s="5">
+        <v>228</v>
+      </c>
+      <c r="B230" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C230" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D230" s="6" t="s">
+        <v>984</v>
+      </c>
+      <c r="G230" s="6" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="231" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A231" s="5">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="232" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A232" s="5">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="233" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A233" s="5">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="234" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A234" s="5">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="235" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A235" s="5">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="236" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A236" s="5">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="237" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A237" s="5">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="238" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A238" s="5">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="239" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A239" s="5">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="240" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A240" s="5">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="241" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A241" s="5">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="242" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A242" s="5">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="243" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A243" s="5">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="244" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A244" s="5">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="245" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A245" s="5">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="246" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A246" s="5">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="247" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A247" s="5">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="248" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A248" s="5">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="249" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A249" s="5">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="250" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A250" s="5">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="251" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A251" s="5">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="252" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A252" s="5">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="253" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A253" s="5">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="254" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A254" s="5">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="255" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A255" s="5">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="256" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A256" s="5">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="257" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A257" s="5">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="258" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A258" s="5">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="259" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A259" s="5">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="260" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A260" s="5">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="261" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A261" s="5">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="262" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A262" s="5">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="263" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A263" s="5">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="264" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A264" s="5">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="265" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A265" s="5">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="266" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A266" s="5">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="267" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A267" s="5">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="268" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A268" s="5">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="269" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A269" s="5">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="270" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A270" s="5">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="271" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A271" s="5">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="272" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A272" s="5">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="273" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A273" s="5">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="274" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A274" s="5">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="275" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A275" s="5">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="276" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A276" s="5">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="277" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A277" s="5">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="278" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A278" s="5">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="279" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A279" s="5">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="280" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A280" s="5">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="281" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A281" s="5">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="282" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A282" s="5">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="283" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A283" s="5">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="284" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A284" s="5">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="285" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A285" s="5">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="286" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A286" s="5">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="287" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A287" s="5">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="288" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A288" s="5">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="289" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A289" s="5">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="290" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A290" s="5">
+        <v>288</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I79" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <conditionalFormatting sqref="A2:J998">
-    <cfRule type="expression" dxfId="15" priority="1" stopIfTrue="1">
+    <cfRule type="expression" dxfId="3" priority="1" stopIfTrue="1">
       <formula>OR($G2="New Issue",$G2="Fix Failed",$G2="Improve Further",$G2="New Functionality")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="14" priority="2" stopIfTrue="1">
+    <cfRule type="expression" dxfId="2" priority="2" stopIfTrue="1">
       <formula>$G2="Untested Fix"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="13" priority="3" stopIfTrue="1">
+    <cfRule type="expression" dxfId="1" priority="3" stopIfTrue="1">
       <formula>$G2="Issue Resolved"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="4" stopIfTrue="1">
+    <cfRule type="expression" dxfId="0" priority="4" stopIfTrue="1">
       <formula>$G2="Manual Fix"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8974,13 +10320,13 @@
     </sortState>
   </autoFilter>
   <conditionalFormatting sqref="A2:C1048576">
-    <cfRule type="expression" dxfId="11" priority="37">
+    <cfRule type="expression" dxfId="15" priority="37">
       <formula>OR($C2="Y",#REF!="Issue Resolved")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="38">
+    <cfRule type="expression" dxfId="14" priority="38">
       <formula>#REF!="Untested Fix"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="39">
+    <cfRule type="expression" dxfId="13" priority="39">
       <formula>OR($C2="N",#REF!="New Issue",#REF!="Fix Failed")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9397,13 +10743,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:C17 A19:C1048576">
-    <cfRule type="expression" dxfId="8" priority="34">
+    <cfRule type="expression" dxfId="12" priority="34">
       <formula>OR($C2="Y",#REF!="Issue Resolved")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="35">
+    <cfRule type="expression" dxfId="11" priority="35">
       <formula>#REF!="Untested Fix"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="36">
+    <cfRule type="expression" dxfId="10" priority="36">
       <formula>OR($C2="N",#REF!="New Issue",#REF!="Fix Failed")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9810,13 +11156,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:C1048576">
-    <cfRule type="expression" dxfId="5" priority="40">
+    <cfRule type="expression" dxfId="9" priority="40">
       <formula>OR($C2="Y",#REF!="Issue Resolved")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="41">
+    <cfRule type="expression" dxfId="8" priority="41">
       <formula>#REF!="Untested Fix"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="42">
+    <cfRule type="expression" dxfId="7" priority="42">
       <formula>OR($C2="N",#REF!="New Issue",#REF!="Fix Failed")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10375,13 +11721,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:C1048576">
-    <cfRule type="expression" dxfId="2" priority="43">
+    <cfRule type="expression" dxfId="6" priority="43">
       <formula>OR($C2="Y",#REF!="Issue Resolved")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="44">
+    <cfRule type="expression" dxfId="5" priority="44">
       <formula>#REF!="Untested Fix"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="45">
+    <cfRule type="expression" dxfId="4" priority="45">
       <formula>OR($C2="N",#REF!="New Issue",#REF!="Fix Failed")</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>